<commit_message>
Expand reviewed source dossier
</commit_message>
<xml_diff>
--- a/dossier/source_dossier.xlsx
+++ b/dossier/source_dossier.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="555" uniqueCount="358">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="555" uniqueCount="354">
   <si>
     <t>id</t>
   </si>
@@ -148,6 +148,33 @@
     <t>{{cite web |last=Schaffhauser |first=Dian |title=Eduventures Publishes Report on Learning Management Systems |url=https://campustechnology.com/articles/2016/01/28/eduventures-publishes-report-on-learning-management-systems.aspx |website=Campus Technology |date=January 28, 2016 |access-date=June 8, 2026}}</t>
   </si>
   <si>
+    <t>CT2</t>
+  </si>
+  <si>
+    <t>Laying the Groundwork for Big Data</t>
+  </si>
+  <si>
+    <t>https://campustechnology.com/articles/2016/02/25/laying-the-groundwork-for-big-data.aspx?Page=3&amp;p=1</t>
+  </si>
+  <si>
+    <t>Minor to moderate. Article about higher-education analytics identifies Alderson as an Eduventures principal analyst and uses his analysis of analytics vendors, data integration, and data governance challenges as context.</t>
+  </si>
+  <si>
+    <t>Alderson was principal analyst for Eduventures; he commented publicly on higher-education analytics vendor-market and data-governance challenges.</t>
+  </si>
+  <si>
+    <t>Low to Medium</t>
+  </si>
+  <si>
+    <t>Optional professional-context source if expanding the Eduventures or analytics section.</t>
+  </si>
+  <si>
+    <t>Reviewed in sources/campus_technology_sources.md; local file data/campus_technology_big_data_groundwork.html</t>
+  </si>
+  <si>
+    <t>{{cite web |last=Raths |first=David |title=Laying the Groundwork for Big Data |url=https://campustechnology.com/articles/2016/02/25/laying-the-groundwork-for-big-data.aspx?Page=3&amp;p=1 |website=Campus Technology |date=February 25, 2016 |access-date=June 8, 2026}}</t>
+  </si>
+  <si>
     <t>M1</t>
   </si>
   <si>
@@ -241,9 +268,6 @@
     <t>Alderson received 4,764 votes for a three-year Town Moderator term; 7,775 ballots were cast according to Town Clerk results.</t>
   </si>
   <si>
-    <t>Low to Medium</t>
-  </si>
-  <si>
     <t>Useful corroboration for election result; stronger than the election preview for vote/result detail.</t>
   </si>
   <si>
@@ -443,42 +467,6 @@
   </si>
   <si>
     <t>Potentially useful if it includes substantive interview/profile coverage.</t>
-  </si>
-  <si>
-    <t>S12</t>
-  </si>
-  <si>
-    <t>ChatGPT shared transcript</t>
-  </si>
-  <si>
-    <t>Wikipedia Biography Creation Plan</t>
-  </si>
-  <si>
-    <t>https://chatgpt.com/share/6a26e762-11cc-83ea-813b-6c705ee3cf73</t>
-  </si>
-  <si>
-    <t>Planning context only</t>
-  </si>
-  <si>
-    <t>Not a Wikipedia source</t>
-  </si>
-  <si>
-    <t>Planning notes and candidate source list.</t>
-  </si>
-  <si>
-    <t>None for article content.</t>
-  </si>
-  <si>
-    <t>None</t>
-  </si>
-  <si>
-    <t>Do not cite in article</t>
-  </si>
-  <si>
-    <t>Saved locally as data/chatgpt_transcript.html</t>
-  </si>
-  <si>
-    <t>Used only to seed source review.</t>
   </si>
   <si>
     <t>N1</t>
@@ -1166,7 +1154,7 @@
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -1471,21 +1459,19 @@
   <dimension ref="A1:O37"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="8.7109375" customWidth="1"/>
-    <col min="2" max="2" width="10.7109375" customWidth="1"/>
-    <col min="3" max="3" width="28.7109375" customWidth="1"/>
-    <col min="4" max="4" width="54.7109375" customWidth="1"/>
-    <col min="5" max="5" width="65.7109375" customWidth="1"/>
-    <col min="6" max="6" width="30.7109375" customWidth="1"/>
+    <col min="1" max="2" width="10.7109375" customWidth="1"/>
+    <col min="3" max="3" width="26.7109375" customWidth="1"/>
+    <col min="4" max="4" width="44.7109375" customWidth="1"/>
+    <col min="5" max="5" width="60.7109375" customWidth="1"/>
+    <col min="6" max="6" width="24.7109375" customWidth="1"/>
     <col min="7" max="7" width="18.7109375" customWidth="1"/>
-    <col min="8" max="8" width="42.7109375" customWidth="1"/>
-    <col min="9" max="9" width="64.7109375" customWidth="1"/>
-    <col min="10" max="10" width="70.7109375" customWidth="1"/>
-    <col min="11" max="11" width="18.7109375" customWidth="1"/>
-    <col min="12" max="12" width="65.7109375" customWidth="1"/>
-    <col min="13" max="13" width="44.7109375" customWidth="1"/>
-    <col min="14" max="14" width="70.7109375" customWidth="1"/>
-    <col min="15" max="15" width="90.7109375" customWidth="1"/>
+    <col min="8" max="8" width="28.7109375" customWidth="1"/>
+    <col min="9" max="10" width="60.7109375" customWidth="1"/>
+    <col min="11" max="11" width="20.7109375" customWidth="1"/>
+    <col min="12" max="12" width="44.7109375" customWidth="1"/>
+    <col min="13" max="13" width="30.7109375" customWidth="1"/>
+    <col min="14" max="14" width="50.7109375" customWidth="1"/>
+    <col min="15" max="15" width="80.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15">
@@ -1634,119 +1620,119 @@
         <v>43</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="E4" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="F4" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="I4" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="J4" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="K4" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="L4" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="H4" s="2" t="s">
+      <c r="M4" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="N4" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="I4" s="2" t="s">
+      <c r="O4" s="2" t="s">
         <v>51</v>
-      </c>
-      <c r="J4" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="K4" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="L4" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="M4" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="N4" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="O4" s="2" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="5" spans="1:15">
       <c r="A5" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="G5" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="D5" s="2" t="s">
+      <c r="H5" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="I5" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="J5" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="G5" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H5" s="2" t="s">
+      <c r="K5" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="I5" s="2" t="s">
+      <c r="L5" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="J5" s="2" t="s">
+      <c r="M5" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="K5" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="L5" s="2" t="s">
+      <c r="N5" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="M5" s="2" t="s">
+      <c r="O5" s="2" t="s">
         <v>66</v>
-      </c>
-      <c r="N5" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="O5" s="2" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="6" spans="1:15">
       <c r="A6" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="E6" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="D6" s="2" t="s">
+      <c r="F6" s="2" t="s">
         <v>70</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>61</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="I6" s="2" t="s">
         <v>72</v>
@@ -1755,13 +1741,13 @@
         <v>73</v>
       </c>
       <c r="K6" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="L6" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="L6" s="2" t="s">
+      <c r="M6" s="2" t="s">
         <v>75</v>
-      </c>
-      <c r="M6" s="2" t="s">
-        <v>66</v>
       </c>
       <c r="N6" s="2" t="s">
         <v>76</v>
@@ -1775,1456 +1761,1456 @@
         <v>78</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="E7" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="F7" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="I7" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="J7" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="F7" s="2" t="s">
+      <c r="K7" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="L7" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="G7" s="2" t="s">
+      <c r="M7" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="N7" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="H7" s="2" t="s">
+      <c r="O7" s="2" t="s">
         <v>85</v>
-      </c>
-      <c r="I7" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="J7" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="K7" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="L7" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="M7" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="N7" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="O7" s="2" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="8" spans="1:15">
       <c r="A8" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="F8" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="G8" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="H8" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="I8" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="J8" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="K8" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="L8" s="2" t="s">
         <v>96</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="I8" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="J8" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="K8" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="L8" s="2" t="s">
-        <v>101</v>
       </c>
       <c r="M8" s="2" t="s">
         <v>40</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="O8" s="2" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
     </row>
     <row r="9" spans="1:15">
       <c r="A9" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="F9" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="G9" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="H9" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="I9" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="J9" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="F9" s="2" t="s">
+      <c r="K9" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="L9" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="G9" s="2" t="s">
+      <c r="M9" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="N9" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="H9" s="2" t="s">
+      <c r="O9" s="2" t="s">
         <v>111</v>
-      </c>
-      <c r="I9" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="J9" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="K9" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="L9" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="M9" s="2" t="s">
-        <v>116</v>
-      </c>
-      <c r="N9" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="O9" s="2" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="10" spans="1:15">
       <c r="A10" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="H10" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="B10" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="C10" s="2" t="s">
+      <c r="I10" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="J10" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="E10" s="3" t="s">
+      <c r="K10" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="F10" s="2" t="s">
+      <c r="L10" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="G10" s="2" t="s">
+      <c r="M10" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="H10" s="2" t="s">
+      <c r="N10" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="I10" s="2" t="s">
+      <c r="O10" s="2" t="s">
         <v>126</v>
-      </c>
-      <c r="J10" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="K10" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="L10" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="M10" s="2" t="s">
-        <v>129</v>
-      </c>
-      <c r="N10" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="O10" s="2" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="11" spans="1:15">
       <c r="A11" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="F11" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="G11" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="H11" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="I11" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="E11" s="3" t="s">
+      <c r="J11" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="F11" s="2" t="s">
+      <c r="K11" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="L11" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="G11" s="2" t="s">
+      <c r="M11" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="H11" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="I11" s="2" t="s">
+      <c r="N11" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="J11" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="K11" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="L11" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="M11" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="N11" s="2" t="s">
-        <v>141</v>
-      </c>
       <c r="O11" s="2" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
     </row>
     <row r="12" spans="1:15">
       <c r="A12" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="B12" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="C12" s="2" t="s">
+      <c r="E12" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="F12" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="E12" s="3" t="s">
+      <c r="G12" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="F12" s="2" t="s">
+      <c r="H12" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="I12" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="G12" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="H12" s="2" t="s">
+      <c r="J12" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="I12" s="2" t="s">
+      <c r="K12" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="L12" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="M12" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="J12" s="2" t="s">
+      <c r="N12" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="K12" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="L12" s="2" t="s">
-        <v>151</v>
-      </c>
-      <c r="M12" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="N12" s="2" t="s">
-        <v>153</v>
-      </c>
       <c r="O12" s="2" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
     </row>
     <row r="13" spans="1:15">
       <c r="A13" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="F13" s="2" t="s">
         <v>154</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>156</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>157</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>158</v>
       </c>
       <c r="G13" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H13" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="J13" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="K13" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="L13" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="M13" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="I13" s="2" t="s">
+      <c r="N13" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="J13" s="2" t="s">
+      <c r="O13" s="2" t="s">
         <v>161</v>
-      </c>
-      <c r="K13" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="L13" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="M13" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="N13" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="O13" s="2" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="14" spans="1:15">
       <c r="A14" s="2" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="G14" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H14" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="J14" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="K14" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="L14" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="M14" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="I14" s="2" t="s">
+      <c r="N14" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="O14" s="2" t="s">
         <v>169</v>
-      </c>
-      <c r="J14" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="K14" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="L14" s="2" t="s">
-        <v>171</v>
-      </c>
-      <c r="M14" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="N14" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="O14" s="2" t="s">
-        <v>173</v>
       </c>
     </row>
     <row r="15" spans="1:15">
       <c r="A15" s="2" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="G15" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H15" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="I15" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="J15" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="K15" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="L15" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="M15" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="I15" s="2" t="s">
+      <c r="N15" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="O15" s="2" t="s">
         <v>177</v>
-      </c>
-      <c r="J15" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="K15" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="L15" s="2" t="s">
-        <v>179</v>
-      </c>
-      <c r="M15" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="N15" s="2" t="s">
-        <v>180</v>
-      </c>
-      <c r="O15" s="2" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="16" spans="1:15">
       <c r="A16" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="I16" s="2" t="s">
         <v>182</v>
       </c>
-      <c r="B16" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="D16" s="2" t="s">
+      <c r="J16" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="E16" s="3" t="s">
+      <c r="K16" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="F16" s="2" t="s">
+      <c r="L16" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="G16" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="H16" s="2" t="s">
+      <c r="M16" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="I16" s="2" t="s">
+      <c r="N16" s="2" t="s">
         <v>186</v>
       </c>
-      <c r="J16" s="2" t="s">
+      <c r="O16" s="2" t="s">
         <v>187</v>
-      </c>
-      <c r="K16" s="2" t="s">
-        <v>188</v>
-      </c>
-      <c r="L16" s="2" t="s">
-        <v>189</v>
-      </c>
-      <c r="M16" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="N16" s="2" t="s">
-        <v>190</v>
-      </c>
-      <c r="O16" s="2" t="s">
-        <v>191</v>
       </c>
     </row>
     <row r="17" spans="1:15">
       <c r="A17" s="2" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="G17" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H17" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="I17" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="J17" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="K17" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="L17" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="M17" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="I17" s="2" t="s">
+      <c r="N17" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="O17" s="2" t="s">
         <v>195</v>
-      </c>
-      <c r="J17" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="K17" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="L17" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="M17" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="N17" s="2" t="s">
-        <v>198</v>
-      </c>
-      <c r="O17" s="2" t="s">
-        <v>199</v>
       </c>
     </row>
     <row r="18" spans="1:15">
       <c r="A18" s="2" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="G18" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H18" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="I18" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="J18" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="K18" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="L18" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="M18" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="I18" s="2" t="s">
+      <c r="N18" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="O18" s="2" t="s">
         <v>203</v>
-      </c>
-      <c r="J18" s="2" t="s">
-        <v>204</v>
-      </c>
-      <c r="K18" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="L18" s="2" t="s">
-        <v>205</v>
-      </c>
-      <c r="M18" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="N18" s="2" t="s">
-        <v>206</v>
-      </c>
-      <c r="O18" s="2" t="s">
-        <v>207</v>
       </c>
     </row>
     <row r="19" spans="1:15">
       <c r="A19" s="2" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="G19" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H19" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="I19" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="J19" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="K19" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="L19" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="M19" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="I19" s="2" t="s">
+      <c r="N19" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="O19" s="2" t="s">
         <v>211</v>
-      </c>
-      <c r="J19" s="2" t="s">
-        <v>212</v>
-      </c>
-      <c r="K19" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="L19" s="2" t="s">
-        <v>213</v>
-      </c>
-      <c r="M19" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="N19" s="2" t="s">
-        <v>214</v>
-      </c>
-      <c r="O19" s="2" t="s">
-        <v>215</v>
       </c>
     </row>
     <row r="20" spans="1:15">
       <c r="A20" s="2" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="G20" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H20" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="I20" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="J20" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="K20" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="L20" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="M20" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="I20" s="2" t="s">
+      <c r="N20" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="O20" s="2" t="s">
         <v>219</v>
-      </c>
-      <c r="J20" s="2" t="s">
-        <v>220</v>
-      </c>
-      <c r="K20" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="L20" s="2" t="s">
-        <v>221</v>
-      </c>
-      <c r="M20" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="N20" s="2" t="s">
-        <v>222</v>
-      </c>
-      <c r="O20" s="2" t="s">
-        <v>223</v>
       </c>
     </row>
     <row r="21" spans="1:15">
       <c r="A21" s="2" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="G21" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H21" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="I21" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="J21" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="K21" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="L21" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="M21" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="I21" s="2" t="s">
+      <c r="N21" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="O21" s="2" t="s">
         <v>227</v>
-      </c>
-      <c r="J21" s="2" t="s">
-        <v>228</v>
-      </c>
-      <c r="K21" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="L21" s="2" t="s">
-        <v>229</v>
-      </c>
-      <c r="M21" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="N21" s="2" t="s">
-        <v>230</v>
-      </c>
-      <c r="O21" s="2" t="s">
-        <v>231</v>
       </c>
     </row>
     <row r="22" spans="1:15">
       <c r="A22" s="2" t="s">
-        <v>232</v>
+        <v>228</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="G22" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H22" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="I22" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="J22" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="K22" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="L22" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="M22" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="I22" s="2" t="s">
+      <c r="N22" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="O22" s="2" t="s">
         <v>235</v>
-      </c>
-      <c r="J22" s="2" t="s">
-        <v>236</v>
-      </c>
-      <c r="K22" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="L22" s="2" t="s">
-        <v>237</v>
-      </c>
-      <c r="M22" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="N22" s="2" t="s">
-        <v>238</v>
-      </c>
-      <c r="O22" s="2" t="s">
-        <v>239</v>
       </c>
     </row>
     <row r="23" spans="1:15">
       <c r="A23" s="2" t="s">
-        <v>240</v>
+        <v>236</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="G23" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H23" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="I23" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="J23" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="K23" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="L23" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="M23" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="I23" s="2" t="s">
+      <c r="N23" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="O23" s="2" t="s">
         <v>243</v>
-      </c>
-      <c r="J23" s="2" t="s">
-        <v>244</v>
-      </c>
-      <c r="K23" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="L23" s="2" t="s">
-        <v>245</v>
-      </c>
-      <c r="M23" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="N23" s="2" t="s">
-        <v>246</v>
-      </c>
-      <c r="O23" s="2" t="s">
-        <v>247</v>
       </c>
     </row>
     <row r="24" spans="1:15">
       <c r="A24" s="2" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="G24" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H24" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="I24" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="J24" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="K24" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="L24" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="M24" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="I24" s="2" t="s">
-        <v>251</v>
-      </c>
-      <c r="J24" s="2" t="s">
-        <v>252</v>
-      </c>
-      <c r="K24" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="L24" s="2" t="s">
-        <v>237</v>
-      </c>
-      <c r="M24" s="2" t="s">
-        <v>163</v>
-      </c>
       <c r="N24" s="2" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="O24" s="2" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
     </row>
     <row r="25" spans="1:15">
       <c r="A25" s="2" t="s">
-        <v>255</v>
+        <v>251</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>257</v>
+        <v>253</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="G25" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H25" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="I25" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="J25" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="K25" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="L25" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="M25" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="I25" s="2" t="s">
+      <c r="N25" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="O25" s="2" t="s">
         <v>258</v>
-      </c>
-      <c r="J25" s="2" t="s">
-        <v>259</v>
-      </c>
-      <c r="K25" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="L25" s="2" t="s">
-        <v>260</v>
-      </c>
-      <c r="M25" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="N25" s="2" t="s">
-        <v>261</v>
-      </c>
-      <c r="O25" s="2" t="s">
-        <v>262</v>
       </c>
     </row>
     <row r="26" spans="1:15">
       <c r="A26" s="2" t="s">
-        <v>263</v>
+        <v>259</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>264</v>
+        <v>260</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>265</v>
+        <v>261</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="G26" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H26" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="I26" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="J26" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="K26" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="L26" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="M26" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="I26" s="2" t="s">
+      <c r="N26" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="O26" s="2" t="s">
         <v>266</v>
-      </c>
-      <c r="J26" s="2" t="s">
-        <v>267</v>
-      </c>
-      <c r="K26" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="L26" s="2" t="s">
-        <v>268</v>
-      </c>
-      <c r="M26" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="N26" s="2" t="s">
-        <v>269</v>
-      </c>
-      <c r="O26" s="2" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="27" spans="1:15">
       <c r="A27" s="2" t="s">
-        <v>271</v>
+        <v>267</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>272</v>
+        <v>268</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="G27" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H27" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="I27" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="J27" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="K27" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="L27" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="M27" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="I27" s="2" t="s">
-        <v>274</v>
-      </c>
-      <c r="J27" s="2" t="s">
-        <v>275</v>
-      </c>
-      <c r="K27" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="L27" s="2" t="s">
-        <v>237</v>
-      </c>
-      <c r="M27" s="2" t="s">
-        <v>163</v>
-      </c>
       <c r="N27" s="2" t="s">
-        <v>276</v>
+        <v>272</v>
       </c>
       <c r="O27" s="2" t="s">
-        <v>277</v>
+        <v>273</v>
       </c>
     </row>
     <row r="28" spans="1:15">
       <c r="A28" s="2" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>279</v>
+        <v>275</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>280</v>
+        <v>276</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="G28" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H28" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="I28" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="J28" s="2" t="s">
+        <v>278</v>
+      </c>
+      <c r="K28" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="L28" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="M28" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="I28" s="2" t="s">
+      <c r="N28" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="O28" s="2" t="s">
         <v>281</v>
-      </c>
-      <c r="J28" s="2" t="s">
-        <v>282</v>
-      </c>
-      <c r="K28" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="L28" s="2" t="s">
-        <v>283</v>
-      </c>
-      <c r="M28" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="N28" s="2" t="s">
-        <v>284</v>
-      </c>
-      <c r="O28" s="2" t="s">
-        <v>285</v>
       </c>
     </row>
     <row r="29" spans="1:15">
       <c r="A29" s="2" t="s">
-        <v>286</v>
+        <v>282</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>287</v>
+        <v>283</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>288</v>
+        <v>284</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="G29" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H29" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="I29" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="J29" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="K29" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="L29" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="M29" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="I29" s="2" t="s">
+      <c r="N29" s="2" t="s">
+        <v>288</v>
+      </c>
+      <c r="O29" s="2" t="s">
         <v>289</v>
-      </c>
-      <c r="J29" s="2" t="s">
-        <v>290</v>
-      </c>
-      <c r="K29" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="L29" s="2" t="s">
-        <v>291</v>
-      </c>
-      <c r="M29" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="N29" s="2" t="s">
-        <v>292</v>
-      </c>
-      <c r="O29" s="2" t="s">
-        <v>293</v>
       </c>
     </row>
     <row r="30" spans="1:15">
       <c r="A30" s="2" t="s">
-        <v>294</v>
+        <v>290</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>295</v>
+        <v>291</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>296</v>
+        <v>292</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>297</v>
+        <v>293</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="G30" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H30" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="I30" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="J30" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="K30" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="L30" s="2" t="s">
+        <v>296</v>
+      </c>
+      <c r="M30" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="I30" s="2" t="s">
+      <c r="N30" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="O30" s="2" t="s">
         <v>298</v>
-      </c>
-      <c r="J30" s="2" t="s">
-        <v>299</v>
-      </c>
-      <c r="K30" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="L30" s="2" t="s">
-        <v>300</v>
-      </c>
-      <c r="M30" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="N30" s="2" t="s">
-        <v>301</v>
-      </c>
-      <c r="O30" s="2" t="s">
-        <v>302</v>
       </c>
     </row>
     <row r="31" spans="1:15">
       <c r="A31" s="2" t="s">
-        <v>303</v>
+        <v>299</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>306</v>
+        <v>302</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="G31" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H31" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="I31" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="J31" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="K31" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="L31" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="M31" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="I31" s="2" t="s">
+      <c r="N31" s="2" t="s">
+        <v>306</v>
+      </c>
+      <c r="O31" s="2" t="s">
         <v>307</v>
-      </c>
-      <c r="J31" s="2" t="s">
-        <v>308</v>
-      </c>
-      <c r="K31" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="L31" s="2" t="s">
-        <v>309</v>
-      </c>
-      <c r="M31" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="N31" s="2" t="s">
-        <v>310</v>
-      </c>
-      <c r="O31" s="2" t="s">
-        <v>311</v>
       </c>
     </row>
     <row r="32" spans="1:15">
       <c r="A32" s="2" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>313</v>
+        <v>309</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="G32" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H32" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="I32" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="J32" s="2" t="s">
+        <v>312</v>
+      </c>
+      <c r="K32" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="L32" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="M32" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="I32" s="2" t="s">
+      <c r="N32" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="O32" s="2" t="s">
         <v>315</v>
-      </c>
-      <c r="J32" s="2" t="s">
-        <v>316</v>
-      </c>
-      <c r="K32" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="L32" s="2" t="s">
-        <v>317</v>
-      </c>
-      <c r="M32" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="N32" s="2" t="s">
-        <v>318</v>
-      </c>
-      <c r="O32" s="2" t="s">
-        <v>319</v>
       </c>
     </row>
     <row r="33" spans="1:15">
       <c r="A33" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>317</v>
+      </c>
+      <c r="E33" s="3" t="s">
+        <v>318</v>
+      </c>
+      <c r="F33" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="G33" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="H33" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="I33" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="J33" s="2" t="s">
         <v>320</v>
       </c>
-      <c r="B33" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="C33" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="D33" s="2" t="s">
+      <c r="K33" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="L33" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="M33" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="N33" s="2" t="s">
         <v>321</v>
       </c>
-      <c r="E33" s="3" t="s">
+      <c r="O33" s="2" t="s">
         <v>322</v>
-      </c>
-      <c r="F33" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="G33" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="H33" s="2" t="s">
-        <v>159</v>
-      </c>
-      <c r="I33" s="2" t="s">
-        <v>323</v>
-      </c>
-      <c r="J33" s="2" t="s">
-        <v>324</v>
-      </c>
-      <c r="K33" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="L33" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="M33" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="N33" s="2" t="s">
-        <v>325</v>
-      </c>
-      <c r="O33" s="2" t="s">
-        <v>326</v>
       </c>
     </row>
     <row r="34" spans="1:15">
       <c r="A34" s="2" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="G34" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H34" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="I34" s="2" t="s">
+        <v>326</v>
+      </c>
+      <c r="J34" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="K34" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="L34" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="M34" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="I34" s="2" t="s">
+      <c r="N34" s="2" t="s">
+        <v>329</v>
+      </c>
+      <c r="O34" s="2" t="s">
         <v>330</v>
-      </c>
-      <c r="J34" s="2" t="s">
-        <v>331</v>
-      </c>
-      <c r="K34" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="L34" s="2" t="s">
-        <v>332</v>
-      </c>
-      <c r="M34" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="N34" s="2" t="s">
-        <v>333</v>
-      </c>
-      <c r="O34" s="2" t="s">
-        <v>334</v>
       </c>
     </row>
     <row r="35" spans="1:15">
       <c r="A35" s="2" t="s">
-        <v>335</v>
+        <v>331</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>295</v>
+        <v>291</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>336</v>
+        <v>332</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>337</v>
+        <v>333</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="G35" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H35" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="I35" s="2" t="s">
+        <v>334</v>
+      </c>
+      <c r="J35" s="2" t="s">
+        <v>335</v>
+      </c>
+      <c r="K35" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="L35" s="2" t="s">
+        <v>336</v>
+      </c>
+      <c r="M35" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="I35" s="2" t="s">
+      <c r="N35" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="O35" s="2" t="s">
         <v>338</v>
-      </c>
-      <c r="J35" s="2" t="s">
-        <v>339</v>
-      </c>
-      <c r="K35" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="L35" s="2" t="s">
-        <v>340</v>
-      </c>
-      <c r="M35" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="N35" s="2" t="s">
-        <v>341</v>
-      </c>
-      <c r="O35" s="2" t="s">
-        <v>342</v>
       </c>
     </row>
     <row r="36" spans="1:15">
       <c r="A36" s="2" t="s">
-        <v>343</v>
+        <v>339</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>344</v>
+        <v>340</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>345</v>
+        <v>341</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="G36" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H36" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="I36" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="J36" s="2" t="s">
+        <v>343</v>
+      </c>
+      <c r="K36" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="L36" s="2" t="s">
+        <v>344</v>
+      </c>
+      <c r="M36" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="I36" s="2" t="s">
+      <c r="N36" s="2" t="s">
+        <v>345</v>
+      </c>
+      <c r="O36" s="2" t="s">
         <v>346</v>
-      </c>
-      <c r="J36" s="2" t="s">
-        <v>347</v>
-      </c>
-      <c r="K36" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="L36" s="2" t="s">
-        <v>348</v>
-      </c>
-      <c r="M36" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="N36" s="2" t="s">
-        <v>349</v>
-      </c>
-      <c r="O36" s="2" t="s">
-        <v>350</v>
       </c>
     </row>
     <row r="37" spans="1:15">
       <c r="A37" s="2" t="s">
-        <v>351</v>
+        <v>347</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>352</v>
+        <v>348</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>353</v>
+        <v>349</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="G37" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H37" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="I37" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="J37" s="2" t="s">
+        <v>351</v>
+      </c>
+      <c r="K37" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="L37" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="M37" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="I37" s="2" t="s">
-        <v>354</v>
-      </c>
-      <c r="J37" s="2" t="s">
-        <v>355</v>
-      </c>
-      <c r="K37" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="L37" s="2" t="s">
-        <v>237</v>
-      </c>
-      <c r="M37" s="2" t="s">
-        <v>163</v>
-      </c>
       <c r="N37" s="2" t="s">
-        <v>356</v>
+        <v>352</v>
       </c>
       <c r="O37" s="2" t="s">
-        <v>357</v>
+        <v>353</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Expand source dossier clusters
</commit_message>
<xml_diff>
--- a/dossier/source_dossier.xlsx
+++ b/dossier/source_dossier.xlsx
@@ -7,17 +7,17 @@
     <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="Source dossier" sheetId="1" r:id="rId1"/>
+    <sheet name="Source Dossier" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Source dossier'!$A$1:$O$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Source Dossier'!$A$1:$O$46</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="555" uniqueCount="354">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="690" uniqueCount="456">
   <si>
     <t>id</t>
   </si>
@@ -109,6 +109,93 @@
     <t>{{cite report |last1=Bulger |first1=Monica |last2=McCormick |first2=Patrick |last3=Pitcan |first3=Mikaela |title=The Legacy of inBloom |publisher=Data &amp; Society Research Institute |date=February 2, 2017 |url=https://datasociety.net/pubs/ecl/InBloom_feb_2017.pdf |access-date=June 8, 2026}}</t>
   </si>
   <si>
+    <t>GF1</t>
+  </si>
+  <si>
+    <t>2013</t>
+  </si>
+  <si>
+    <t>Gates Foundation</t>
+  </si>
+  <si>
+    <t>ConnectEDU, Inc. / OPP1092353</t>
+  </si>
+  <si>
+    <t>https://www.gatesfoundation.org/about/committed-grants/2013/07/opp1092353</t>
+  </si>
+  <si>
+    <t>Primary grant database record</t>
+  </si>
+  <si>
+    <t>No / primary</t>
+  </si>
+  <si>
+    <t>High for Gates Foundation grant details; primary for funding context</t>
+  </si>
+  <si>
+    <t>Minor. Lists ConnectEDU, Inc. as grantee and provides grant details; does not mention Alderson or inBloom by name.</t>
+  </si>
+  <si>
+    <t>Gates Foundation committed $499,375 in July 2013 to ConnectEDU, Inc. for an 18-month K-12 Education grant to build a technology platform for Common Core literacy standards.</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>Use only for ConnectEDU/Gates Foundation funding context if needed; do not use as notability support or for Alderson-specific facts.</t>
+  </si>
+  <si>
+    <t>Verified from downloaded HTML</t>
+  </si>
+  <si>
+    <t>Reviewed in sources/data_society_inbloom_sources.md; local file data/gates_foundation_grant_opp1092353.html</t>
+  </si>
+  <si>
+    <t>{{cite web |title=ConnectEDU, Inc. |url=https://www.gatesfoundation.org/about/committed-grants/2013/07/opp1092353 |website=Gates Foundation |date=July 2013 |access-date=June 8, 2026}}</t>
+  </si>
+  <si>
+    <t>SI1</t>
+  </si>
+  <si>
+    <t>2026</t>
+  </si>
+  <si>
+    <t>Startup Intros</t>
+  </si>
+  <si>
+    <t>ConnectEdu: Funding, Team &amp; Investors</t>
+  </si>
+  <si>
+    <t>https://startupintros.com/orgs/connectedu</t>
+  </si>
+  <si>
+    <t>Company directory/profile summary</t>
+  </si>
+  <si>
+    <t>Partial</t>
+  </si>
+  <si>
+    <t>Medium for company-background orientation; verify facts against underlying sources before article use</t>
+  </si>
+  <si>
+    <t>Company-background summary. Describes ConnectEDU as a Boston-based edtech company founded in 2002 with K-12, college, and career-planning technology; summarizes products, scale, funding, bankruptcy, asset sales, and data-privacy context. Does not mention Alderson.</t>
+  </si>
+  <si>
+    <t>ConnectEDU company context only; not Alderson-specific. Useful as a readable summary and source lead list.</t>
+  </si>
+  <si>
+    <t>None to Low</t>
+  </si>
+  <si>
+    <t>Use only for ConnectEDU background orientation; do not use for Alderson notability and prefer underlying sources for article facts.</t>
+  </si>
+  <si>
+    <t>Reviewed in sources/connectedu_company_sources.md; local file data/startupintros_connectedu.html</t>
+  </si>
+  <si>
+    <t>{{cite web |title=ConnectEdu: Funding, Team &amp; Investors |url=https://startupintros.com/orgs/connectedu |website=Startup Intros |access-date=June 8, 2026}}</t>
+  </si>
+  <si>
     <t>S2</t>
   </si>
   <si>
@@ -139,9 +226,6 @@
     <t>Eduventures analyst role</t>
   </si>
   <si>
-    <t>Verified from downloaded HTML</t>
-  </si>
-  <si>
     <t>Useful secondary source; not a profile.</t>
   </si>
   <si>
@@ -280,9 +364,6 @@
     <t>S7</t>
   </si>
   <si>
-    <t>2026</t>
-  </si>
-  <si>
     <t>Natick Veterans Oral History Project</t>
   </si>
   <si>
@@ -295,9 +376,6 @@
     <t>Local oral history/archive profile</t>
   </si>
   <si>
-    <t>Partial</t>
-  </si>
-  <si>
     <t>Medium for non-contentious service facts; likely based on subject interview/archive intake</t>
   </si>
   <si>
@@ -355,6 +433,45 @@
     <t>{{cite web |title=Awards - PESC Board of Directors Recipients |url=https://pesc.org/awards/ |website=PESC |access-date=June 8, 2026}}</t>
   </si>
   <si>
+    <t>CB1</t>
+  </si>
+  <si>
+    <t>2014</t>
+  </si>
+  <si>
+    <t>Scribd / U.S. Bankruptcy Court filing copy</t>
+  </si>
+  <si>
+    <t>Connectedu Bankruptcy Petition</t>
+  </si>
+  <si>
+    <t>https://www.scribd.com/doc/220960006/Connectedu-Bankruptcy-Petition</t>
+  </si>
+  <si>
+    <t>Legal filing copy / bankruptcy petition</t>
+  </si>
+  <si>
+    <t>Potentially high for narrow filing facts after direct review; weak as hosted copy</t>
+  </si>
+  <si>
+    <t>Unknown until direct filing review. Search indexing identifies the document as ConnectEDU's Chapter 11 bankruptcy petition filed April 28, 2014, but Scribd returned a client-challenge page during local capture.</t>
+  </si>
+  <si>
+    <t>Potentially verifies whether Alderson was listed as a ConnectEDU shareholder or equity security holder at the time of the bankruptcy filing; not yet directly extracted locally.</t>
+  </si>
+  <si>
+    <t>Do not cite until accessible filing text or an official court copy is reviewed.</t>
+  </si>
+  <si>
+    <t>Located but not verified from filing text</t>
+  </si>
+  <si>
+    <t>Reviewed in sources/legal_bankruptcy_sources.md; local files data/connectedu_bankruptcy_petition_scribd.html and data/search_ddg_connectedu_bankruptcy_petition_jina.txt</t>
+  </si>
+  <si>
+    <t>{{cite web |title=Connectedu Bankruptcy Petition |url=https://www.scribd.com/doc/220960006/Connectedu-Bankruptcy-Petition |website=Scribd |date=April 28, 2014 |access-date=June 8, 2026}}</t>
+  </si>
+  <si>
     <t>S9</t>
   </si>
   <si>
@@ -394,7 +511,7 @@
     <t>Located but not verified</t>
   </si>
   <si>
-    <t>Transcript and LinkedIn suggest relevance, but not used in draft.</t>
+    <t>Retained as a publication lead, but not used in draft.</t>
   </si>
   <si>
     <t>Do not cite until verified</t>
@@ -403,37 +520,229 @@
     <t>S10</t>
   </si>
   <si>
-    <t>Encoura</t>
-  </si>
-  <si>
-    <t>Encoura Wake-Up Call Author - Jeffrey Alderson</t>
+    <t>2015-2017</t>
+  </si>
+  <si>
+    <t>Encoura / Eduventures</t>
+  </si>
+  <si>
+    <t>Encoura Wake-Up Call Author - Jeffrey Alderson and linked Wake-Up Call articles</t>
   </si>
   <si>
     <t>https://www.encoura.org/people/jeffery-alderson/</t>
   </si>
   <si>
-    <t>Corporate author profile</t>
+    <t>Corporate author profile / affiliated authored articles</t>
   </si>
   <si>
     <t>No</t>
   </si>
   <si>
-    <t>Medium for affiliation if current at publication time</t>
-  </si>
-  <si>
-    <t>Very sparse on downloaded page.</t>
-  </si>
-  <si>
-    <t>Name/profile existence only from reviewed HTML.</t>
-  </si>
-  <si>
-    <t>Do not use unless richer archived content is found</t>
-  </si>
-  <si>
-    <t>Verified page, insufficient content</t>
-  </si>
-  <si>
-    <t>Primary/corporate profile.</t>
+    <t>Medium for profile and authorship facts; not independent for notability</t>
+  </si>
+  <si>
+    <t>Sparse profile plus 33 linked affiliated authored Wake-Up Call articles verified from the live author page's Builder content API.</t>
+  </si>
+  <si>
+    <t>Profile existence; article titles/dates/URLs for Alderson-attributed Encoura/Eduventures Wake-Up Call posts.</t>
+  </si>
+  <si>
+    <t>Do not use for AfC notability; retain as publication-history evidence and leads for independent coverage.</t>
+  </si>
+  <si>
+    <t>Verified page and article list; no webinar or Enrollminute items returned for the author ID.</t>
+  </si>
+  <si>
+    <t>Reviewed in sources/encoura_eduventures_sources.md; local files data/encoura_people_alderson.html and data/encoura_alderson_articles.json</t>
+  </si>
+  <si>
+    <t>Do not cite for notability</t>
+  </si>
+  <si>
+    <t>FB1</t>
+  </si>
+  <si>
+    <t>Facebook</t>
+  </si>
+  <si>
+    <t>Jeffrey Alderson / Committee to Elect Jeff Alderson for Natick School Committee</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/jeff4natick/</t>
+  </si>
+  <si>
+    <t>Campaign social media / self-published page</t>
+  </si>
+  <si>
+    <t>Low for encyclopedic sourcing; primary/self-published</t>
+  </si>
+  <si>
+    <t>Very sparse campaign-page metadata.</t>
+  </si>
+  <si>
+    <t>A Facebook page existed for the Committee to Elect Jeff Alderson for Natick School Committee.</t>
+  </si>
+  <si>
+    <t>Do not use for notability; retain as campaign-context evidence only.</t>
+  </si>
+  <si>
+    <t>Verified from downloaded HTML metadata</t>
+  </si>
+  <si>
+    <t>Reviewed in sources/campaign_social_media_sources.md; local file data/facebook_jeff4natick.html</t>
+  </si>
+  <si>
+    <t>NP1</t>
+  </si>
+  <si>
+    <t>Natick Patch</t>
+  </si>
+  <si>
+    <t>ICYMI: Who's Running In The 2017 Natick Town Election?</t>
+  </si>
+  <si>
+    <t>https://patch.com/massachusetts/natick/icymi-whos-running-2017-natick-town-election</t>
+  </si>
+  <si>
+    <t>Minor. Article lists candidates for Natick's March 28 2017 town election and identifies Alderson as a School Committee candidate.</t>
+  </si>
+  <si>
+    <t>Alderson was listed with Donna M. McKenzie and Hayley I. Sonneborn as candidates for two three-year School Committee seats.</t>
+  </si>
+  <si>
+    <t>Useful for verifying 2017 candidacy; not notability support.</t>
+  </si>
+  <si>
+    <t>Reviewed in sources/natick_patch_sources.md; local file data/natick_patch_2017_town_election_candidates.html</t>
+  </si>
+  <si>
+    <t>{{cite web |last=Arsenault |first=Charlene |title=ICYMI: Who's Running In The 2017 Natick Town Election? |url=https://patch.com/massachusetts/natick/icymi-whos-running-2017-natick-town-election |website=Natick Patch |date=March 11, 2017 |access-date=June 8, 2026}}</t>
+  </si>
+  <si>
+    <t>WL1</t>
+  </si>
+  <si>
+    <t>Wicked Local</t>
+  </si>
+  <si>
+    <t>NATICK LETTER: Support for School Committee candidate Jeff Alderson</t>
+  </si>
+  <si>
+    <t>https://www.wickedlocal.com/story/bulletin-tab/2017/03/23/natick-letter-support-for-school/21906287007/</t>
+  </si>
+  <si>
+    <t>Letter of support recommending Alderson for Natick School Committee and discussing Waypoint Adventure board service.</t>
+  </si>
+  <si>
+    <t>Supporter publicly endorsed Alderson for School Committee; potential lead for Waypoint/community-service facts.</t>
+  </si>
+  <si>
+    <t>Do not use for notability; avoid unless carefully attributed as opinion.</t>
+  </si>
+  <si>
+    <t>Reviewed in sources/wicked_local_sources.md; local file data/wickedlocal_2017_letter_support_school_committee.html</t>
+  </si>
+  <si>
+    <t>{{cite web |title=NATICK LETTER: Support for School Committee candidate Jeff Alderson |url=https://www.wickedlocal.com/story/bulletin-tab/2017/03/23/natick-letter-support-for-school/21906287007/ |website=Wicked Local |date=March 23, 2017 |access-date=June 8, 2026}}</t>
+  </si>
+  <si>
+    <t>WL2</t>
+  </si>
+  <si>
+    <t>Question for the candidates</t>
+  </si>
+  <si>
+    <t>https://www.wickedlocal.com/story/bulletin-tab/2017/03/24/question-for-candidates/21899647007/</t>
+  </si>
+  <si>
+    <t>Local election news / candidate questionnaire</t>
+  </si>
+  <si>
+    <t>Moderate for campaign context. Article presents School Committee candidate responses and includes Alderson's response on school social issues and policy process.</t>
+  </si>
+  <si>
+    <t>Alderson was a 2017 Natick School Committee candidate; he publicly answered a candidate question about school response to social topics and hate crimes.</t>
+  </si>
+  <si>
+    <t>Useful for civic-background context if the draft expands prior town-government engagement; not a major notability source.</t>
+  </si>
+  <si>
+    <t>Reviewed in sources/wicked_local_sources.md; local file data/wickedlocal_2017_question_for_candidates.html</t>
+  </si>
+  <si>
+    <t>{{cite web |title=Question for the candidates |url=https://www.wickedlocal.com/story/bulletin-tab/2017/03/24/question-for-candidates/21899647007/ |website=Wicked Local |date=March 24, 2017 |access-date=June 8, 2026}}</t>
+  </si>
+  <si>
+    <t>NLTP1</t>
+  </si>
+  <si>
+    <t>Natick Local Town Pages</t>
+  </si>
+  <si>
+    <t>Meet the Candidates for Town Committees / Natick March 2017</t>
+  </si>
+  <si>
+    <t>https://www.yumpu.com/en/document/view/57088486/natick-march-2017</t>
+  </si>
+  <si>
+    <t>Local monthly publication / candidate statements</t>
+  </si>
+  <si>
+    <t>Medium for local election facts; candidate statement is primary</t>
+  </si>
+  <si>
+    <t>Moderate for campaign context. Article identifies the School Committee candidates and includes a candidate-submitted statement by Alderson.</t>
+  </si>
+  <si>
+    <t>Alderson ran for one of two three-year Natick School Committee seats in 2017; his candidate statement discussed public schools, Air Force service, education technology, nonprofit boards, mentoring, disability inclusion, and social justice.</t>
+  </si>
+  <si>
+    <t>Use cautiously for candidate-context facts; candidate-authored material is not independent coverage.</t>
+  </si>
+  <si>
+    <t>Verified from downloaded Yumpu HTML pages 1 and 2/3</t>
+  </si>
+  <si>
+    <t>Reviewed in sources/natick_local_town_pages_sources.md; local files data/natick_local_town_pages_march_2017.html and data/natick_local_town_pages_march_2017_pages_2_3.html</t>
+  </si>
+  <si>
+    <t>{{cite web |last=Whitty |first=Cynthia |title=Meet the Candidates for Town Committees |url=https://www.yumpu.com/en/document/view/57088486/natick-march-2017 |website=Natick Local Town Pages |date=March 2017 |access-date=June 8, 2026}}</t>
+  </si>
+  <si>
+    <t>TN1</t>
+  </si>
+  <si>
+    <t>Town of Natick</t>
+  </si>
+  <si>
+    <t>Official Election Results - March 28 2017</t>
+  </si>
+  <si>
+    <t>https://www.natickma.gov/DocumentCenter/View/4563/Official-Election-Results---March-28-2017?bidId=</t>
+  </si>
+  <si>
+    <t>Official election results</t>
+  </si>
+  <si>
+    <t>High for official election result</t>
+  </si>
+  <si>
+    <t>Minor. Official PDF lists March 28 2017 School Committee vote totals.</t>
+  </si>
+  <si>
+    <t>Alderson received 1012 votes; Donna M. Mckenzie received 1020 votes; Hayley I. Sonneborn received 1402 votes. Official margin between McKenzie and Alderson was 8 votes.</t>
+  </si>
+  <si>
+    <t>Use only to verify official 2017 election result and vote totals; not notability support.</t>
+  </si>
+  <si>
+    <t>Verified from downloaded PDF and extracted text</t>
+  </si>
+  <si>
+    <t>Reviewed in sources/town_of_natick_sources.md; local files data/town_of_natick_2017_official_election_results.pdf and data/town_of_natick_2017_official_election_results.txt</t>
+  </si>
+  <si>
+    <t>{{cite web |title=Official Election Results - March 28, 2017 |url=https://www.natickma.gov/DocumentCenter/View/4563/Official-Election-Results---March-28-2017?bidId= |website=Town of Natick |date=April 4, 2017 |access-date=June 8, 2026}}</t>
   </si>
   <si>
     <t>S11</t>
@@ -569,9 +878,6 @@
   </si>
   <si>
     <t>Alderson authored or supplied a statement as Town Moderator.</t>
-  </si>
-  <si>
-    <t>None to Low</t>
   </si>
   <si>
     <t>Do not use for notability; only use as primary evidence if the statement itself becomes relevant.</t>
@@ -1456,22 +1762,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O37"/>
+  <dimension ref="A1:O46"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="2" width="10.7109375" customWidth="1"/>
-    <col min="3" max="3" width="26.7109375" customWidth="1"/>
-    <col min="4" max="4" width="44.7109375" customWidth="1"/>
-    <col min="5" max="5" width="60.7109375" customWidth="1"/>
-    <col min="6" max="6" width="24.7109375" customWidth="1"/>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="2" width="10.7109375" customWidth="1"/>
+    <col min="3" max="3" width="28.7109375" customWidth="1"/>
+    <col min="4" max="4" width="45.7109375" customWidth="1"/>
+    <col min="5" max="5" width="55.7109375" customWidth="1"/>
+    <col min="6" max="6" width="28.7109375" customWidth="1"/>
     <col min="7" max="7" width="18.7109375" customWidth="1"/>
-    <col min="8" max="8" width="28.7109375" customWidth="1"/>
-    <col min="9" max="10" width="60.7109375" customWidth="1"/>
+    <col min="8" max="8" width="32.7109375" customWidth="1"/>
+    <col min="9" max="10" width="55.7109375" customWidth="1"/>
     <col min="11" max="11" width="20.7109375" customWidth="1"/>
-    <col min="12" max="12" width="44.7109375" customWidth="1"/>
-    <col min="13" max="13" width="30.7109375" customWidth="1"/>
-    <col min="14" max="14" width="50.7109375" customWidth="1"/>
-    <col min="15" max="15" width="80.7109375" customWidth="1"/>
+    <col min="12" max="12" width="45.7109375" customWidth="1"/>
+    <col min="13" max="13" width="35.7109375" customWidth="1"/>
+    <col min="14" max="14" width="55.7109375" customWidth="1"/>
+    <col min="15" max="15" width="65.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15">
@@ -1588,336 +1895,336 @@
         <v>35</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="O3" s="2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="4" spans="1:15">
       <c r="A4" s="2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>31</v>
+        <v>46</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>32</v>
+        <v>47</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>35</v>
+        <v>50</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>21</v>
+        <v>51</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>25</v>
+        <v>52</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="O4" s="2" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
     </row>
     <row r="5" spans="1:15">
       <c r="A5" s="2" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>58</v>
+        <v>21</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>59</v>
+        <v>25</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>64</v>
+        <v>42</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="O5" s="2" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
     </row>
     <row r="6" spans="1:15">
       <c r="A6" s="2" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>71</v>
+        <v>25</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>62</v>
+        <v>76</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>75</v>
+        <v>42</v>
       </c>
       <c r="N6" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="O6" s="2" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="7" spans="1:15">
       <c r="A7" s="2" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>53</v>
+        <v>81</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>54</v>
+        <v>82</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>70</v>
+        <v>85</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>21</v>
+        <v>86</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>71</v>
+        <v>87</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>48</v>
+        <v>90</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="M7" s="2" t="s">
-        <v>75</v>
+        <v>92</v>
       </c>
       <c r="N7" s="2" t="s">
-        <v>84</v>
+        <v>93</v>
       </c>
       <c r="O7" s="2" t="s">
-        <v>85</v>
+        <v>94</v>
       </c>
     </row>
     <row r="8" spans="1:15">
       <c r="A8" s="2" t="s">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="E8" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="K8" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="F8" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="I8" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="J8" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="K8" s="2" t="s">
-        <v>48</v>
-      </c>
       <c r="L8" s="2" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>40</v>
+        <v>103</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="O8" s="2" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
     </row>
     <row r="9" spans="1:15">
       <c r="A9" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H9" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="B9" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="E9" s="3" t="s">
+      <c r="I9" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="J9" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="K9" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="L9" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="M9" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="F9" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="G9" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="H9" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="I9" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="J9" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="K9" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="L9" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="M9" s="2" t="s">
-        <v>40</v>
-      </c>
       <c r="N9" s="2" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="O9" s="2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="10" spans="1:15">
       <c r="A10" s="2" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>113</v>
+        <v>46</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>118</v>
+        <v>51</v>
       </c>
       <c r="H10" s="2" t="s">
         <v>119</v>
@@ -1929,104 +2236,104 @@
         <v>121</v>
       </c>
       <c r="K10" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="L10" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="L10" s="2" t="s">
+      <c r="M10" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="N10" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="M10" s="2" t="s">
+      <c r="O10" s="2" t="s">
         <v>124</v>
-      </c>
-      <c r="N10" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="O10" s="2" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="11" spans="1:15">
       <c r="A11" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="B11" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="C11" s="2" t="s">
+      <c r="D11" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="E11" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="E11" s="3" t="s">
+      <c r="F11" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="F11" s="2" t="s">
+      <c r="G11" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="G11" s="2" t="s">
+      <c r="H11" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="H11" s="2" t="s">
+      <c r="I11" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="I11" s="2" t="s">
+      <c r="J11" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="J11" s="2" t="s">
+      <c r="K11" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="L11" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="K11" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="L11" s="2" t="s">
+      <c r="M11" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="N11" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="M11" s="2" t="s">
+      <c r="O11" s="2" t="s">
         <v>137</v>
-      </c>
-      <c r="N11" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="O11" s="2" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="12" spans="1:15">
       <c r="A12" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="B12" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="C12" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="D12" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="E12" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="E12" s="3" t="s">
+      <c r="F12" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="F12" s="2" t="s">
+      <c r="G12" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="H12" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="G12" s="2" t="s">
+      <c r="I12" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="H12" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="I12" s="2" t="s">
+      <c r="J12" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="J12" s="2" t="s">
+      <c r="K12" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="L12" s="2" t="s">
         <v>147</v>
-      </c>
-      <c r="K12" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="L12" s="2" t="s">
-        <v>123</v>
       </c>
       <c r="M12" s="2" t="s">
         <v>148</v>
@@ -2035,1186 +2342,1609 @@
         <v>149</v>
       </c>
       <c r="O12" s="2" t="s">
-        <v>126</v>
+        <v>150</v>
       </c>
     </row>
     <row r="13" spans="1:15">
       <c r="A13" s="2" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>87</v>
+        <v>152</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>21</v>
+        <v>157</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="K13" s="2" t="s">
-        <v>48</v>
+        <v>161</v>
       </c>
       <c r="L13" s="2" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="M13" s="2" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="N13" s="2" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="O13" s="2" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
     </row>
     <row r="14" spans="1:15">
       <c r="A14" s="2" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>87</v>
+        <v>167</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>151</v>
+        <v>168</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>154</v>
+        <v>171</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>21</v>
+        <v>172</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>155</v>
+        <v>173</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>165</v>
+        <v>174</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="L14" s="2" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="M14" s="2" t="s">
-        <v>159</v>
+        <v>177</v>
       </c>
       <c r="N14" s="2" t="s">
-        <v>168</v>
+        <v>178</v>
       </c>
       <c r="O14" s="2" t="s">
-        <v>169</v>
+        <v>179</v>
       </c>
     </row>
     <row r="15" spans="1:15">
       <c r="A15" s="2" t="s">
-        <v>170</v>
+        <v>180</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>87</v>
+        <v>16</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>151</v>
+        <v>181</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>171</v>
+        <v>182</v>
       </c>
       <c r="E15" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="G15" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="F15" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="G15" s="2" t="s">
-        <v>21</v>
-      </c>
       <c r="H15" s="2" t="s">
-        <v>155</v>
+        <v>185</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>173</v>
+        <v>186</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>174</v>
+        <v>187</v>
       </c>
       <c r="K15" s="2" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="L15" s="2" t="s">
-        <v>175</v>
+        <v>188</v>
       </c>
       <c r="M15" s="2" t="s">
-        <v>159</v>
+        <v>189</v>
       </c>
       <c r="N15" s="2" t="s">
-        <v>176</v>
+        <v>190</v>
       </c>
       <c r="O15" s="2" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
     </row>
     <row r="16" spans="1:15">
       <c r="A16" s="2" t="s">
-        <v>178</v>
+        <v>191</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>87</v>
+        <v>16</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>151</v>
+        <v>192</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>179</v>
+        <v>193</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>180</v>
+        <v>194</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>181</v>
+        <v>98</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>58</v>
+        <v>21</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>155</v>
+        <v>99</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>182</v>
+        <v>195</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>183</v>
+        <v>196</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>184</v>
+        <v>90</v>
       </c>
       <c r="L16" s="2" t="s">
-        <v>185</v>
+        <v>197</v>
       </c>
       <c r="M16" s="2" t="s">
-        <v>159</v>
+        <v>42</v>
       </c>
       <c r="N16" s="2" t="s">
-        <v>186</v>
+        <v>198</v>
       </c>
       <c r="O16" s="2" t="s">
-        <v>187</v>
+        <v>199</v>
       </c>
     </row>
     <row r="17" spans="1:15">
       <c r="A17" s="2" t="s">
-        <v>188</v>
+        <v>200</v>
       </c>
       <c r="B17" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>203</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="H17" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="C17" s="2" t="s">
-        <v>151</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>189</v>
-      </c>
-      <c r="E17" s="3" t="s">
-        <v>190</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="G17" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H17" s="2" t="s">
-        <v>155</v>
-      </c>
       <c r="I17" s="2" t="s">
-        <v>191</v>
+        <v>204</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>192</v>
+        <v>205</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>48</v>
+        <v>90</v>
       </c>
       <c r="L17" s="2" t="s">
-        <v>193</v>
+        <v>206</v>
       </c>
       <c r="M17" s="2" t="s">
-        <v>159</v>
+        <v>42</v>
       </c>
       <c r="N17" s="2" t="s">
-        <v>194</v>
+        <v>207</v>
       </c>
       <c r="O17" s="2" t="s">
-        <v>195</v>
+        <v>208</v>
       </c>
     </row>
     <row r="18" spans="1:15">
       <c r="A18" s="2" t="s">
-        <v>196</v>
+        <v>209</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>53</v>
+        <v>16</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>151</v>
+        <v>201</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>197</v>
+        <v>210</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>198</v>
+        <v>211</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>154</v>
+        <v>212</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>21</v>
+        <v>51</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>155</v>
+        <v>99</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>199</v>
+        <v>213</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>200</v>
+        <v>214</v>
       </c>
       <c r="K18" s="2" t="s">
-        <v>48</v>
+        <v>76</v>
       </c>
       <c r="L18" s="2" t="s">
-        <v>201</v>
+        <v>215</v>
       </c>
       <c r="M18" s="2" t="s">
-        <v>159</v>
+        <v>42</v>
       </c>
       <c r="N18" s="2" t="s">
-        <v>202</v>
+        <v>216</v>
       </c>
       <c r="O18" s="2" t="s">
-        <v>203</v>
+        <v>217</v>
       </c>
     </row>
     <row r="19" spans="1:15">
       <c r="A19" s="2" t="s">
-        <v>204</v>
+        <v>218</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>53</v>
+        <v>16</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>151</v>
+        <v>219</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>205</v>
+        <v>220</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>206</v>
+        <v>221</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>154</v>
+        <v>222</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>21</v>
+        <v>51</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>155</v>
+        <v>223</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>207</v>
+        <v>224</v>
       </c>
       <c r="J19" s="2" t="s">
-        <v>208</v>
+        <v>225</v>
       </c>
       <c r="K19" s="2" t="s">
-        <v>62</v>
+        <v>76</v>
       </c>
       <c r="L19" s="2" t="s">
-        <v>209</v>
+        <v>226</v>
       </c>
       <c r="M19" s="2" t="s">
-        <v>159</v>
+        <v>227</v>
       </c>
       <c r="N19" s="2" t="s">
-        <v>210</v>
+        <v>228</v>
       </c>
       <c r="O19" s="2" t="s">
-        <v>211</v>
+        <v>229</v>
       </c>
     </row>
     <row r="20" spans="1:15">
       <c r="A20" s="2" t="s">
-        <v>212</v>
+        <v>230</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>53</v>
+        <v>16</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>151</v>
+        <v>231</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>213</v>
+        <v>232</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>214</v>
+        <v>233</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>154</v>
+        <v>234</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>155</v>
+        <v>235</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>215</v>
+        <v>236</v>
       </c>
       <c r="J20" s="2" t="s">
-        <v>216</v>
+        <v>237</v>
       </c>
       <c r="K20" s="2" t="s">
-        <v>48</v>
+        <v>90</v>
       </c>
       <c r="L20" s="2" t="s">
-        <v>217</v>
+        <v>238</v>
       </c>
       <c r="M20" s="2" t="s">
-        <v>159</v>
+        <v>239</v>
       </c>
       <c r="N20" s="2" t="s">
-        <v>218</v>
+        <v>240</v>
       </c>
       <c r="O20" s="2" t="s">
-        <v>219</v>
+        <v>241</v>
       </c>
     </row>
     <row r="21" spans="1:15">
       <c r="A21" s="2" t="s">
-        <v>220</v>
+        <v>242</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>53</v>
+        <v>243</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>151</v>
+        <v>244</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>221</v>
+        <v>245</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>222</v>
+        <v>246</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>154</v>
+        <v>247</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>21</v>
+        <v>248</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>223</v>
+        <v>249</v>
       </c>
       <c r="J21" s="2" t="s">
-        <v>224</v>
+        <v>250</v>
       </c>
       <c r="K21" s="2" t="s">
-        <v>62</v>
+        <v>161</v>
       </c>
       <c r="L21" s="2" t="s">
-        <v>225</v>
+        <v>162</v>
       </c>
       <c r="M21" s="2" t="s">
-        <v>159</v>
+        <v>251</v>
       </c>
       <c r="N21" s="2" t="s">
-        <v>226</v>
+        <v>252</v>
       </c>
       <c r="O21" s="2" t="s">
-        <v>227</v>
+        <v>165</v>
       </c>
     </row>
     <row r="22" spans="1:15">
       <c r="A22" s="2" t="s">
-        <v>228</v>
+        <v>253</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>151</v>
+        <v>254</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>229</v>
+        <v>255</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>230</v>
+        <v>256</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>154</v>
+        <v>257</v>
       </c>
       <c r="G22" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>155</v>
+        <v>258</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>231</v>
+        <v>259</v>
       </c>
       <c r="J22" s="2" t="s">
-        <v>232</v>
+        <v>260</v>
       </c>
       <c r="K22" s="2" t="s">
-        <v>62</v>
+        <v>76</v>
       </c>
       <c r="L22" s="2" t="s">
-        <v>233</v>
+        <v>261</v>
       </c>
       <c r="M22" s="2" t="s">
-        <v>159</v>
+        <v>262</v>
       </c>
       <c r="N22" s="2" t="s">
-        <v>234</v>
+        <v>263</v>
       </c>
       <c r="O22" s="2" t="s">
-        <v>235</v>
+        <v>264</v>
       </c>
     </row>
     <row r="23" spans="1:15">
       <c r="A23" s="2" t="s">
-        <v>236</v>
+        <v>265</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>151</v>
+        <v>254</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>237</v>
+        <v>266</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>238</v>
+        <v>267</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>154</v>
+        <v>257</v>
       </c>
       <c r="G23" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>155</v>
+        <v>258</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>239</v>
+        <v>268</v>
       </c>
       <c r="J23" s="2" t="s">
-        <v>240</v>
+        <v>269</v>
       </c>
       <c r="K23" s="2" t="s">
-        <v>48</v>
+        <v>90</v>
       </c>
       <c r="L23" s="2" t="s">
-        <v>241</v>
+        <v>270</v>
       </c>
       <c r="M23" s="2" t="s">
-        <v>159</v>
+        <v>262</v>
       </c>
       <c r="N23" s="2" t="s">
-        <v>242</v>
+        <v>271</v>
       </c>
       <c r="O23" s="2" t="s">
-        <v>243</v>
+        <v>272</v>
       </c>
     </row>
     <row r="24" spans="1:15">
       <c r="A24" s="2" t="s">
-        <v>244</v>
+        <v>273</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>151</v>
+        <v>254</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>245</v>
+        <v>274</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>246</v>
+        <v>275</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>154</v>
+        <v>257</v>
       </c>
       <c r="G24" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>155</v>
+        <v>258</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>247</v>
+        <v>276</v>
       </c>
       <c r="J24" s="2" t="s">
-        <v>248</v>
+        <v>277</v>
       </c>
       <c r="K24" s="2" t="s">
-        <v>62</v>
+        <v>76</v>
       </c>
       <c r="L24" s="2" t="s">
-        <v>233</v>
+        <v>278</v>
       </c>
       <c r="M24" s="2" t="s">
-        <v>159</v>
+        <v>262</v>
       </c>
       <c r="N24" s="2" t="s">
-        <v>249</v>
+        <v>279</v>
       </c>
       <c r="O24" s="2" t="s">
-        <v>250</v>
+        <v>280</v>
       </c>
     </row>
     <row r="25" spans="1:15">
       <c r="A25" s="2" t="s">
-        <v>251</v>
+        <v>281</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>151</v>
+        <v>254</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>252</v>
+        <v>282</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>253</v>
+        <v>283</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>154</v>
+        <v>284</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>21</v>
+        <v>86</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>155</v>
+        <v>258</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>254</v>
+        <v>285</v>
       </c>
       <c r="J25" s="2" t="s">
-        <v>255</v>
+        <v>286</v>
       </c>
       <c r="K25" s="2" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="L25" s="2" t="s">
-        <v>256</v>
+        <v>287</v>
       </c>
       <c r="M25" s="2" t="s">
-        <v>159</v>
+        <v>262</v>
       </c>
       <c r="N25" s="2" t="s">
-        <v>257</v>
+        <v>288</v>
       </c>
       <c r="O25" s="2" t="s">
-        <v>258</v>
+        <v>289</v>
       </c>
     </row>
     <row r="26" spans="1:15">
       <c r="A26" s="2" t="s">
-        <v>259</v>
+        <v>290</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>151</v>
+        <v>254</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>260</v>
+        <v>291</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>261</v>
+        <v>292</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>154</v>
+        <v>257</v>
       </c>
       <c r="G26" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>155</v>
+        <v>258</v>
       </c>
       <c r="I26" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="J26" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="K26" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="L26" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="M26" s="2" t="s">
         <v>262</v>
       </c>
-      <c r="J26" s="2" t="s">
-        <v>263</v>
-      </c>
-      <c r="K26" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="L26" s="2" t="s">
-        <v>264</v>
-      </c>
-      <c r="M26" s="2" t="s">
-        <v>159</v>
-      </c>
       <c r="N26" s="2" t="s">
-        <v>265</v>
+        <v>296</v>
       </c>
       <c r="O26" s="2" t="s">
-        <v>266</v>
+        <v>297</v>
       </c>
     </row>
     <row r="27" spans="1:15">
       <c r="A27" s="2" t="s">
-        <v>267</v>
+        <v>298</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>53</v>
+        <v>81</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>151</v>
+        <v>254</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>268</v>
+        <v>299</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>269</v>
+        <v>300</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>154</v>
+        <v>257</v>
       </c>
       <c r="G27" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>155</v>
+        <v>258</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>270</v>
+        <v>301</v>
       </c>
       <c r="J27" s="2" t="s">
-        <v>271</v>
+        <v>302</v>
       </c>
       <c r="K27" s="2" t="s">
-        <v>62</v>
+        <v>76</v>
       </c>
       <c r="L27" s="2" t="s">
-        <v>233</v>
+        <v>303</v>
       </c>
       <c r="M27" s="2" t="s">
-        <v>159</v>
+        <v>262</v>
       </c>
       <c r="N27" s="2" t="s">
-        <v>272</v>
+        <v>304</v>
       </c>
       <c r="O27" s="2" t="s">
-        <v>273</v>
+        <v>305</v>
       </c>
     </row>
     <row r="28" spans="1:15">
       <c r="A28" s="2" t="s">
-        <v>274</v>
+        <v>306</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>53</v>
+        <v>81</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>151</v>
+        <v>254</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>275</v>
+        <v>307</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>276</v>
+        <v>308</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>154</v>
+        <v>257</v>
       </c>
       <c r="G28" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>155</v>
+        <v>258</v>
       </c>
       <c r="I28" s="2" t="s">
-        <v>277</v>
+        <v>309</v>
       </c>
       <c r="J28" s="2" t="s">
-        <v>278</v>
+        <v>310</v>
       </c>
       <c r="K28" s="2" t="s">
-        <v>48</v>
+        <v>90</v>
       </c>
       <c r="L28" s="2" t="s">
-        <v>279</v>
+        <v>311</v>
       </c>
       <c r="M28" s="2" t="s">
-        <v>159</v>
+        <v>262</v>
       </c>
       <c r="N28" s="2" t="s">
-        <v>280</v>
+        <v>312</v>
       </c>
       <c r="O28" s="2" t="s">
-        <v>281</v>
+        <v>313</v>
       </c>
     </row>
     <row r="29" spans="1:15">
       <c r="A29" s="2" t="s">
-        <v>282</v>
+        <v>314</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>53</v>
+        <v>81</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>151</v>
+        <v>254</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>283</v>
+        <v>315</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>284</v>
+        <v>316</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>154</v>
+        <v>257</v>
       </c>
       <c r="G29" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>155</v>
+        <v>258</v>
       </c>
       <c r="I29" s="2" t="s">
-        <v>285</v>
+        <v>317</v>
       </c>
       <c r="J29" s="2" t="s">
-        <v>286</v>
+        <v>318</v>
       </c>
       <c r="K29" s="2" t="s">
-        <v>62</v>
+        <v>76</v>
       </c>
       <c r="L29" s="2" t="s">
-        <v>287</v>
+        <v>319</v>
       </c>
       <c r="M29" s="2" t="s">
-        <v>159</v>
+        <v>262</v>
       </c>
       <c r="N29" s="2" t="s">
-        <v>288</v>
+        <v>320</v>
       </c>
       <c r="O29" s="2" t="s">
-        <v>289</v>
+        <v>321</v>
       </c>
     </row>
     <row r="30" spans="1:15">
       <c r="A30" s="2" t="s">
-        <v>290</v>
+        <v>322</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>291</v>
+        <v>81</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>151</v>
+        <v>254</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>292</v>
+        <v>323</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>293</v>
+        <v>324</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>154</v>
+        <v>257</v>
       </c>
       <c r="G30" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>155</v>
+        <v>258</v>
       </c>
       <c r="I30" s="2" t="s">
-        <v>294</v>
+        <v>325</v>
       </c>
       <c r="J30" s="2" t="s">
-        <v>295</v>
+        <v>326</v>
       </c>
       <c r="K30" s="2" t="s">
-        <v>62</v>
+        <v>90</v>
       </c>
       <c r="L30" s="2" t="s">
-        <v>296</v>
+        <v>327</v>
       </c>
       <c r="M30" s="2" t="s">
-        <v>159</v>
+        <v>262</v>
       </c>
       <c r="N30" s="2" t="s">
-        <v>297</v>
+        <v>328</v>
       </c>
       <c r="O30" s="2" t="s">
-        <v>298</v>
+        <v>329</v>
       </c>
     </row>
     <row r="31" spans="1:15">
       <c r="A31" s="2" t="s">
-        <v>299</v>
+        <v>330</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>300</v>
+        <v>81</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>151</v>
+        <v>254</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>301</v>
+        <v>331</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>302</v>
+        <v>332</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>154</v>
+        <v>257</v>
       </c>
       <c r="G31" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>155</v>
+        <v>258</v>
       </c>
       <c r="I31" s="2" t="s">
-        <v>303</v>
+        <v>333</v>
       </c>
       <c r="J31" s="2" t="s">
-        <v>304</v>
+        <v>334</v>
       </c>
       <c r="K31" s="2" t="s">
-        <v>48</v>
+        <v>90</v>
       </c>
       <c r="L31" s="2" t="s">
-        <v>305</v>
+        <v>335</v>
       </c>
       <c r="M31" s="2" t="s">
-        <v>159</v>
+        <v>262</v>
       </c>
       <c r="N31" s="2" t="s">
-        <v>306</v>
+        <v>336</v>
       </c>
       <c r="O31" s="2" t="s">
-        <v>307</v>
+        <v>337</v>
       </c>
     </row>
     <row r="32" spans="1:15">
       <c r="A32" s="2" t="s">
-        <v>308</v>
+        <v>338</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>53</v>
+        <v>81</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>151</v>
+        <v>254</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>309</v>
+        <v>339</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>310</v>
+        <v>340</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>154</v>
+        <v>257</v>
       </c>
       <c r="G32" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H32" s="2" t="s">
-        <v>155</v>
+        <v>258</v>
       </c>
       <c r="I32" s="2" t="s">
-        <v>311</v>
+        <v>341</v>
       </c>
       <c r="J32" s="2" t="s">
-        <v>312</v>
+        <v>342</v>
       </c>
       <c r="K32" s="2" t="s">
-        <v>62</v>
+        <v>76</v>
       </c>
       <c r="L32" s="2" t="s">
-        <v>313</v>
+        <v>343</v>
       </c>
       <c r="M32" s="2" t="s">
-        <v>159</v>
+        <v>262</v>
       </c>
       <c r="N32" s="2" t="s">
-        <v>314</v>
+        <v>344</v>
       </c>
       <c r="O32" s="2" t="s">
-        <v>315</v>
+        <v>345</v>
       </c>
     </row>
     <row r="33" spans="1:15">
       <c r="A33" s="2" t="s">
-        <v>316</v>
+        <v>346</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>53</v>
+        <v>81</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>151</v>
+        <v>254</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>317</v>
+        <v>347</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>318</v>
+        <v>348</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>181</v>
+        <v>257</v>
       </c>
       <c r="G33" s="2" t="s">
-        <v>58</v>
+        <v>21</v>
       </c>
       <c r="H33" s="2" t="s">
-        <v>155</v>
+        <v>258</v>
       </c>
       <c r="I33" s="2" t="s">
-        <v>319</v>
+        <v>349</v>
       </c>
       <c r="J33" s="2" t="s">
-        <v>320</v>
+        <v>350</v>
       </c>
       <c r="K33" s="2" t="s">
-        <v>62</v>
+        <v>90</v>
       </c>
       <c r="L33" s="2" t="s">
-        <v>63</v>
+        <v>335</v>
       </c>
       <c r="M33" s="2" t="s">
-        <v>159</v>
+        <v>262</v>
       </c>
       <c r="N33" s="2" t="s">
-        <v>321</v>
+        <v>351</v>
       </c>
       <c r="O33" s="2" t="s">
-        <v>322</v>
+        <v>352</v>
       </c>
     </row>
     <row r="34" spans="1:15">
       <c r="A34" s="2" t="s">
-        <v>323</v>
+        <v>353</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>53</v>
+        <v>81</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>151</v>
+        <v>254</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>324</v>
+        <v>354</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>325</v>
+        <v>355</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>154</v>
+        <v>257</v>
       </c>
       <c r="G34" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>155</v>
+        <v>258</v>
       </c>
       <c r="I34" s="2" t="s">
-        <v>326</v>
+        <v>356</v>
       </c>
       <c r="J34" s="2" t="s">
-        <v>327</v>
+        <v>357</v>
       </c>
       <c r="K34" s="2" t="s">
-        <v>62</v>
+        <v>90</v>
       </c>
       <c r="L34" s="2" t="s">
-        <v>328</v>
+        <v>358</v>
       </c>
       <c r="M34" s="2" t="s">
-        <v>159</v>
+        <v>262</v>
       </c>
       <c r="N34" s="2" t="s">
-        <v>329</v>
+        <v>359</v>
       </c>
       <c r="O34" s="2" t="s">
-        <v>330</v>
+        <v>360</v>
       </c>
     </row>
     <row r="35" spans="1:15">
       <c r="A35" s="2" t="s">
-        <v>331</v>
+        <v>361</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>291</v>
+        <v>81</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>151</v>
+        <v>254</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>332</v>
+        <v>362</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>333</v>
+        <v>363</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>154</v>
+        <v>257</v>
       </c>
       <c r="G35" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H35" s="2" t="s">
-        <v>155</v>
+        <v>258</v>
       </c>
       <c r="I35" s="2" t="s">
-        <v>334</v>
+        <v>364</v>
       </c>
       <c r="J35" s="2" t="s">
-        <v>335</v>
+        <v>365</v>
       </c>
       <c r="K35" s="2" t="s">
-        <v>62</v>
+        <v>76</v>
       </c>
       <c r="L35" s="2" t="s">
-        <v>336</v>
+        <v>366</v>
       </c>
       <c r="M35" s="2" t="s">
-        <v>159</v>
+        <v>262</v>
       </c>
       <c r="N35" s="2" t="s">
-        <v>337</v>
+        <v>367</v>
       </c>
       <c r="O35" s="2" t="s">
-        <v>338</v>
+        <v>368</v>
       </c>
     </row>
     <row r="36" spans="1:15">
       <c r="A36" s="2" t="s">
-        <v>339</v>
+        <v>369</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>300</v>
+        <v>81</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>151</v>
+        <v>254</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>340</v>
+        <v>370</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>341</v>
+        <v>371</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>154</v>
+        <v>257</v>
       </c>
       <c r="G36" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H36" s="2" t="s">
-        <v>155</v>
+        <v>258</v>
       </c>
       <c r="I36" s="2" t="s">
-        <v>342</v>
+        <v>372</v>
       </c>
       <c r="J36" s="2" t="s">
-        <v>343</v>
+        <v>373</v>
       </c>
       <c r="K36" s="2" t="s">
-        <v>48</v>
+        <v>90</v>
       </c>
       <c r="L36" s="2" t="s">
-        <v>344</v>
+        <v>335</v>
       </c>
       <c r="M36" s="2" t="s">
-        <v>159</v>
+        <v>262</v>
       </c>
       <c r="N36" s="2" t="s">
-        <v>345</v>
+        <v>374</v>
       </c>
       <c r="O36" s="2" t="s">
-        <v>346</v>
+        <v>375</v>
       </c>
     </row>
     <row r="37" spans="1:15">
       <c r="A37" s="2" t="s">
-        <v>347</v>
+        <v>376</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>300</v>
+        <v>81</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>151</v>
+        <v>254</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>348</v>
+        <v>377</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>349</v>
+        <v>378</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>154</v>
+        <v>257</v>
       </c>
       <c r="G37" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H37" s="2" t="s">
-        <v>155</v>
+        <v>258</v>
       </c>
       <c r="I37" s="2" t="s">
-        <v>350</v>
+        <v>379</v>
       </c>
       <c r="J37" s="2" t="s">
-        <v>351</v>
+        <v>380</v>
       </c>
       <c r="K37" s="2" t="s">
-        <v>62</v>
+        <v>76</v>
       </c>
       <c r="L37" s="2" t="s">
-        <v>233</v>
+        <v>381</v>
       </c>
       <c r="M37" s="2" t="s">
-        <v>159</v>
+        <v>262</v>
       </c>
       <c r="N37" s="2" t="s">
-        <v>352</v>
+        <v>382</v>
       </c>
       <c r="O37" s="2" t="s">
-        <v>353</v>
+        <v>383</v>
+      </c>
+    </row>
+    <row r="38" spans="1:15">
+      <c r="A38" s="2" t="s">
+        <v>384</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>385</v>
+      </c>
+      <c r="E38" s="3" t="s">
+        <v>386</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="G38" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H38" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="I38" s="2" t="s">
+        <v>387</v>
+      </c>
+      <c r="J38" s="2" t="s">
+        <v>388</v>
+      </c>
+      <c r="K38" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="L38" s="2" t="s">
+        <v>389</v>
+      </c>
+      <c r="M38" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="N38" s="2" t="s">
+        <v>390</v>
+      </c>
+      <c r="O38" s="2" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="39" spans="1:15">
+      <c r="A39" s="2" t="s">
+        <v>392</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>394</v>
+      </c>
+      <c r="E39" s="3" t="s">
+        <v>395</v>
+      </c>
+      <c r="F39" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="G39" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H39" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="I39" s="2" t="s">
+        <v>396</v>
+      </c>
+      <c r="J39" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="K39" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="L39" s="2" t="s">
+        <v>398</v>
+      </c>
+      <c r="M39" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="N39" s="2" t="s">
+        <v>399</v>
+      </c>
+      <c r="O39" s="2" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="40" spans="1:15">
+      <c r="A40" s="2" t="s">
+        <v>401</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>402</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>403</v>
+      </c>
+      <c r="E40" s="3" t="s">
+        <v>404</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="G40" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H40" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="I40" s="2" t="s">
+        <v>405</v>
+      </c>
+      <c r="J40" s="2" t="s">
+        <v>406</v>
+      </c>
+      <c r="K40" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="L40" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="M40" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="N40" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="O40" s="2" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="41" spans="1:15">
+      <c r="A41" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>411</v>
+      </c>
+      <c r="E41" s="3" t="s">
+        <v>412</v>
+      </c>
+      <c r="F41" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="G41" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H41" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="I41" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="J41" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="K41" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="L41" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="M41" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="N41" s="2" t="s">
+        <v>416</v>
+      </c>
+      <c r="O41" s="2" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="42" spans="1:15">
+      <c r="A42" s="2" t="s">
+        <v>418</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="E42" s="3" t="s">
+        <v>420</v>
+      </c>
+      <c r="F42" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="G42" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="H42" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="I42" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="J42" s="2" t="s">
+        <v>422</v>
+      </c>
+      <c r="K42" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="L42" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="M42" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="N42" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="O42" s="2" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="43" spans="1:15">
+      <c r="A43" s="2" t="s">
+        <v>425</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>426</v>
+      </c>
+      <c r="E43" s="3" t="s">
+        <v>427</v>
+      </c>
+      <c r="F43" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="G43" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H43" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="I43" s="2" t="s">
+        <v>428</v>
+      </c>
+      <c r="J43" s="2" t="s">
+        <v>429</v>
+      </c>
+      <c r="K43" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="L43" s="2" t="s">
+        <v>430</v>
+      </c>
+      <c r="M43" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="N43" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="O43" s="2" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="44" spans="1:15">
+      <c r="A44" s="2" t="s">
+        <v>433</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>434</v>
+      </c>
+      <c r="E44" s="3" t="s">
+        <v>435</v>
+      </c>
+      <c r="F44" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="G44" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H44" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="I44" s="2" t="s">
+        <v>436</v>
+      </c>
+      <c r="J44" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="K44" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="L44" s="2" t="s">
+        <v>438</v>
+      </c>
+      <c r="M44" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="N44" s="2" t="s">
+        <v>439</v>
+      </c>
+      <c r="O44" s="2" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="45" spans="1:15">
+      <c r="A45" s="2" t="s">
+        <v>441</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>402</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>442</v>
+      </c>
+      <c r="E45" s="3" t="s">
+        <v>443</v>
+      </c>
+      <c r="F45" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="G45" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H45" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="I45" s="2" t="s">
+        <v>444</v>
+      </c>
+      <c r="J45" s="2" t="s">
+        <v>445</v>
+      </c>
+      <c r="K45" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="L45" s="2" t="s">
+        <v>446</v>
+      </c>
+      <c r="M45" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="N45" s="2" t="s">
+        <v>447</v>
+      </c>
+      <c r="O45" s="2" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="46" spans="1:15">
+      <c r="A46" s="2" t="s">
+        <v>449</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>402</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>450</v>
+      </c>
+      <c r="E46" s="3" t="s">
+        <v>451</v>
+      </c>
+      <c r="F46" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="G46" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H46" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="I46" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="J46" s="2" t="s">
+        <v>453</v>
+      </c>
+      <c r="K46" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="L46" s="2" t="s">
+        <v>335</v>
+      </c>
+      <c r="M46" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="N46" s="2" t="s">
+        <v>454</v>
+      </c>
+      <c r="O46" s="2" t="s">
+        <v>455</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O37"/>
+  <autoFilter ref="A1:O46"/>
   <hyperlinks>
     <hyperlink ref="E2" r:id="rId1"/>
     <hyperlink ref="E3" r:id="rId2"/>
@@ -3252,6 +3982,15 @@
     <hyperlink ref="E35" r:id="rId34"/>
     <hyperlink ref="E36" r:id="rId35"/>
     <hyperlink ref="E37" r:id="rId36"/>
+    <hyperlink ref="E38" r:id="rId37"/>
+    <hyperlink ref="E39" r:id="rId38"/>
+    <hyperlink ref="E40" r:id="rId39"/>
+    <hyperlink ref="E41" r:id="rId40"/>
+    <hyperlink ref="E42" r:id="rId41"/>
+    <hyperlink ref="E43" r:id="rId42"/>
+    <hyperlink ref="E44" r:id="rId43"/>
+    <hyperlink ref="E45" r:id="rId44"/>
+    <hyperlink ref="E46" r:id="rId45"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Verify ConnectEDU bankruptcy source
</commit_message>
<xml_diff>
--- a/dossier/source_dossier.xlsx
+++ b/dossier/source_dossier.xlsx
@@ -451,22 +451,22 @@
     <t>Legal filing copy / bankruptcy petition</t>
   </si>
   <si>
-    <t>Potentially high for narrow filing facts after direct review; weak as hosted copy</t>
-  </si>
-  <si>
-    <t>Unknown until direct filing review. Search indexing identifies the document as ConnectEDU's Chapter 11 bankruptcy petition filed April 28, 2014, but Scribd returned a client-challenge page during local capture.</t>
-  </si>
-  <si>
-    <t>Potentially verifies whether Alderson was listed as a ConnectEDU shareholder or equity security holder at the time of the bankruptcy filing; not yet directly extracted locally.</t>
-  </si>
-  <si>
-    <t>Do not cite until accessible filing text or an official court copy is reviewed.</t>
-  </si>
-  <si>
-    <t>Located but not verified from filing text</t>
-  </si>
-  <si>
-    <t>Reviewed in sources/legal_bankruptcy_sources.md; local files data/connectedu_bankruptcy_petition_scribd.html and data/search_ddg_connectedu_bankruptcy_petition_jina.txt</t>
+    <t>High for narrow filing facts; weak as hosted copy</t>
+  </si>
+  <si>
+    <t>Minor. Primary bankruptcy filing for ConnectEDU, Inc., case 14-11238-scc, Doc. 1. Page 8 is the List of Equity Security Holders cover page; page 10 is Schedule A and lists Jeff Alderson.</t>
+  </si>
+  <si>
+    <t>Alderson was listed in Schedule A of ConnectEDU's List of Equity Security Holders with 139 ordinary common options, 139 total preferred and common, and 0.01% diluted ownership.</t>
+  </si>
+  <si>
+    <t>Use only for the narrow equity-security-holder fact; do not use for notability and prefer an official court copy if available.</t>
+  </si>
+  <si>
+    <t>Verified from downloaded PDF and rendered page images</t>
+  </si>
+  <si>
+    <t>Reviewed in sources/legal_bankruptcy_sources.md; local files data/connectedu_bankruptcy_petition.pdf; data/connectedu_bankruptcy_petition_download_text.txt; data/connectedu_bankruptcy_petition_page_08.png; data/connectedu_bankruptcy_petition_page_10.png</t>
   </si>
   <si>
     <t>{{cite web |title=Connectedu Bankruptcy Petition |url=https://www.scribd.com/doc/220960006/Connectedu-Bankruptcy-Petition |website=Scribd |date=April 28, 2014 |access-date=June 8, 2026}}</t>

</xml_diff>

<commit_message>
Expand source dossier with PESC and MathWorks sources
</commit_message>
<xml_diff>
--- a/dossier/source_dossier.xlsx
+++ b/dossier/source_dossier.xlsx
@@ -10,14 +10,14 @@
     <sheet name="Source Dossier" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Source Dossier'!$A$1:$O$46</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Source Dossier'!$A$1:$O$60</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="690" uniqueCount="456">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="900" uniqueCount="616">
   <si>
     <t>id</t>
   </si>
@@ -259,6 +259,279 @@
     <t>{{cite web |last=Raths |first=David |title=Laying the Groundwork for Big Data |url=https://campustechnology.com/articles/2016/02/25/laying-the-groundwork-for-big-data.aspx?Page=3&amp;p=1 |website=Campus Technology |date=February 25, 2016 |access-date=June 8, 2026}}</t>
   </si>
   <si>
+    <t>MOL1</t>
+  </si>
+  <si>
+    <t>2021</t>
+  </si>
+  <si>
+    <t>MIT Open Learning</t>
+  </si>
+  <si>
+    <t>The Evolution of Engineering Education Post-COVID-19</t>
+  </si>
+  <si>
+    <t>https://openlearning.mit.edu/events/evolution-engineering-education-post-covid-19</t>
+  </si>
+  <si>
+    <t>Event page / panelist bio</t>
+  </si>
+  <si>
+    <t>High for event listing and public affiliation; limited as biographical source</t>
+  </si>
+  <si>
+    <t>Short professional bio. Event page lists Alderson as Product Manager for MATLAB Grader, MathWorks, and describes his role with MATLAB Grader and online teaching and learning at MathWorks.</t>
+  </si>
+  <si>
+    <t>Alderson was product manager for MATLAB Grader at MathWorks in Natick, Massachusetts; led MathWorks marketing efforts in online teaching and learning; was previously Principal Analyst for Technology at Eduventures and Lead Architect for Houghton Mifflin Harcourt / Choice P20 Solutions.</t>
+  </si>
+  <si>
+    <t>Use for narrow MathWorks and MATLAB Grader professional-context facts; do not use as major notability support.</t>
+  </si>
+  <si>
+    <t>Reviewed in sources/mit_open_learning_sources.md; local file data/mit_openlearning_engineering_education_post_covid.html</t>
+  </si>
+  <si>
+    <t>{{cite web |title=The Evolution of Engineering Education Post-COVID-19 |url=https://openlearning.mit.edu/events/evolution-engineering-education-post-covid-19 |website=MIT Open Learning |date=March 22, 2021 |access-date=June 8, 2026}}</t>
+  </si>
+  <si>
+    <t>IEEE1</t>
+  </si>
+  <si>
+    <t>2018</t>
+  </si>
+  <si>
+    <t>IEEE vTools Events / IEEE Education Society</t>
+  </si>
+  <si>
+    <t>WEBINAR: MATLAB Grader for automaticallygraded computational assignments</t>
+  </si>
+  <si>
+    <t>https://events.vtools.ieee.org/m/183771</t>
+  </si>
+  <si>
+    <t>Event page / webinar listing</t>
+  </si>
+  <si>
+    <t>Medium to High for event metadata; limited as biographical source</t>
+  </si>
+  <si>
+    <t>Minor to moderate. Event page lists Jeff Alderson of MathWorks as speaker and gives a short professional bio tied to MATLAB Grader.</t>
+  </si>
+  <si>
+    <t>Alderson presented on MATLAB Grader for automatically graded computational assignments; he was described as Online Learning Product Marketing at MathWorks and product manager for MATLAB's autograding solution, MATLAB Grader.</t>
+  </si>
+  <si>
+    <t>Use only for narrow professional-context evidence; do not use as notability support.</t>
+  </si>
+  <si>
+    <t>Reviewed in sources/mathworks_matlab_grader_sources.md; local file data/ieee_vtools_183771.html</t>
+  </si>
+  <si>
+    <t>{{cite web |title=WEBINAR: MATLAB Grader for automaticallygraded computational assignments |url=https://events.vtools.ieee.org/m/183771 |website=IEEE vTools Events |date=December 13, 2018 |access-date=June 8, 2026}}</t>
+  </si>
+  <si>
+    <t>IN4OBE1</t>
+  </si>
+  <si>
+    <t>2022 / 2025 page</t>
+  </si>
+  <si>
+    <t>IN4OBE</t>
+  </si>
+  <si>
+    <t>Detailed Program / Autograded Programming Assignments with MATLAB Grade</t>
+  </si>
+  <si>
+    <t>https://in4obe.org/detailed-program/</t>
+  </si>
+  <si>
+    <t>Conference program / event listing</t>
+  </si>
+  <si>
+    <t>Medium for event metadata; limited as biographical source</t>
+  </si>
+  <si>
+    <t>Minor to moderate. Detailed program lists an autograded programming assignments session with Jeff Alderson as speaker; LinkedIn metadata provides a recorded-webinar trail.</t>
+  </si>
+  <si>
+    <t>Alderson was listed as speaker for `Autograded Programming Assignments with MATLAB Grade` in Day 1, Track 2: Computing, Engineering &amp; Technology, Theme 3, Topic 4: Automating Assessment and Evaluation.</t>
+  </si>
+  <si>
+    <t>Use only for narrow professional-context evidence of presenter role; do not use as notability support.</t>
+  </si>
+  <si>
+    <t>Reviewed in sources/mathworks_matlab_grader_sources.md; local files data/in4obe_detailed_program.html and data/linkedin_in4obe_empowering_education.html</t>
+  </si>
+  <si>
+    <t>{{cite web |title=Detailed Program |url=https://in4obe.org/detailed-program/ |website=IN4OBE |access-date=June 8, 2026}}</t>
+  </si>
+  <si>
+    <t>YT1</t>
+  </si>
+  <si>
+    <t>2024</t>
+  </si>
+  <si>
+    <t>YouTube / IN4OBE LLC</t>
+  </si>
+  <si>
+    <t>Autograded Programming Assignments with MATLAB Grade</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=C-GlXr3MxvQ</t>
+  </si>
+  <si>
+    <t>Video platform page / recorded webinar</t>
+  </si>
+  <si>
+    <t>No / platform-hosted</t>
+  </si>
+  <si>
+    <t>Medium for video metadata; use with event-page corroboration</t>
+  </si>
+  <si>
+    <t>Minor. YouTube oEmbed identifies the video title and author as IN4OBE LLC; fetched watch-page data includes Alderson, while LinkedIn and IN4OBE sources provide clearer attribution.</t>
+  </si>
+  <si>
+    <t>Recorded IN4OBE webinar title and publisher; supporting trail for Alderson's speaker role when paired with IN4OBE/LinkedIn metadata.</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>Use only as supporting evidence for the recorded webinar, paired with clearer event metadata.</t>
+  </si>
+  <si>
+    <t>Verified from oEmbed and downloaded watch HTML</t>
+  </si>
+  <si>
+    <t>Reviewed in sources/mathworks_matlab_grader_sources.md; local files data/youtube_in4obe_c_glxr3mxvq.html and data/youtube_in4obe_c_glxr3mxvq_oembed.json</t>
+  </si>
+  <si>
+    <t>{{cite web |title=Autograded Programming Assignments with MATLAB Grade |url=https://www.youtube.com/watch?v=C-GlXr3MxvQ |website=YouTube |publisher=IN4OBE LLC |access-date=June 8, 2026}}</t>
+  </si>
+  <si>
+    <t>MWYT1</t>
+  </si>
+  <si>
+    <t>Current page access June 8 2026</t>
+  </si>
+  <si>
+    <t>YouTube / MATLAB channel</t>
+  </si>
+  <si>
+    <t>Teaching with MATLAB and Simulink</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/playlist?list=PLn8PRpmsu08oV_uJZBB7jIemn4-lxN7yL</t>
+  </si>
+  <si>
+    <t>Official channel playlist</t>
+  </si>
+  <si>
+    <t>No / affiliated platform source</t>
+  </si>
+  <si>
+    <t>Medium for playlist metadata; insufficient for Alderson attribution</t>
+  </si>
+  <si>
+    <t>Source lead only. Official MATLAB channel playlist contains teaching and MATLAB Grader topics, but fetched playlist metadata does not name Alderson.</t>
+  </si>
+  <si>
+    <t>Potential lead to MathWorks education-technology videos; does not independently verify Alderson as presenter.</t>
+  </si>
+  <si>
+    <t>Retain as a source-discovery lead; do not cite for Alderson presenter attribution until individual videos or transcripts are reviewed.</t>
+  </si>
+  <si>
+    <t>Verified playlist metadata; Alderson attribution not verified</t>
+  </si>
+  <si>
+    <t>Reviewed in sources/mathworks_matlab_grader_sources.md; local file data/youtube_mathworks_playlist_educational_technology.html</t>
+  </si>
+  <si>
+    <t>Do not cite until individual video attribution is verified</t>
+  </si>
+  <si>
+    <t>MWS1</t>
+  </si>
+  <si>
+    <t>MathWorks</t>
+  </si>
+  <si>
+    <t>Search MATLAB and Simulink Videos: Alderson</t>
+  </si>
+  <si>
+    <t>https://www.mathworks.com/videos/search.html?q=Alderson&amp;page=1</t>
+  </si>
+  <si>
+    <t>Affiliated site search / source lead</t>
+  </si>
+  <si>
+    <t>No / affiliated</t>
+  </si>
+  <si>
+    <t>Medium for source discovery; rendered results not fully available in downloaded HTML</t>
+  </si>
+  <si>
+    <t>Source lead only. MathWorks search page shell and broader search API response were fetched; API response included MathWorks video results but was broader than the rendered video-only results.</t>
+  </si>
+  <si>
+    <t>Potential lead to MathWorks video pages associated with Alderson; exact page-level presenter metadata remains to be verified.</t>
+  </si>
+  <si>
+    <t>Retain as a source-discovery lead; use exact video detail pages only after verification.</t>
+  </si>
+  <si>
+    <t>Partially verified from downloaded page shell and local API response</t>
+  </si>
+  <si>
+    <t>Reviewed in sources/mathworks_matlab_grader_sources.md; local files data/mathworks_video_search_alderson_page1.html and data/mathworks_video_search_alderson_results.json</t>
+  </si>
+  <si>
+    <t>Do not cite until exact video pages are verified</t>
+  </si>
+  <si>
+    <t>RG1</t>
+  </si>
+  <si>
+    <t>ResearchGate</t>
+  </si>
+  <si>
+    <t>Jeffrey Alderson scientific contributions</t>
+  </si>
+  <si>
+    <t>https://www.researchgate.net/scientific-contributions/Jeffrey-Alderson-2273994673</t>
+  </si>
+  <si>
+    <t>Publication-list / profile source lead</t>
+  </si>
+  <si>
+    <t>No / profile platform</t>
+  </si>
+  <si>
+    <t>Low for article facts; direct local fetch blocked</t>
+  </si>
+  <si>
+    <t>Source lead only. ResearchGate page was identified as a publication-list/profile lead, but direct local fetch returned HTTP 403 and page details were not verified locally.</t>
+  </si>
+  <si>
+    <t>Potential lead to Alderson's published articles; use underlying publication records instead of the profile page when possible.</t>
+  </si>
+  <si>
+    <t>Retain only as a publication-list lead; do not cite in article until page or underlying publication records are reviewed.</t>
+  </si>
+  <si>
+    <t>Blocked / unverified; HTTP 403 on direct local fetch</t>
+  </si>
+  <si>
+    <t>Reviewed in sources/affiliated_profile_sources.md and sources/mathworks_matlab_grader_sources.md; no local HTML saved</t>
+  </si>
+  <si>
+    <t>Do not cite until verified</t>
+  </si>
+  <si>
     <t>M1</t>
   </si>
   <si>
@@ -289,9 +562,6 @@
     <t>Foss publicly supported Alderson as successor; use only as attributed opinion.</t>
   </si>
   <si>
-    <t>Low</t>
-  </si>
-  <si>
     <t>Do not use for notability; avoid in draft unless carefully attributed as Foss opinion.</t>
   </si>
   <si>
@@ -433,43 +703,265 @@
     <t>{{cite web |title=Awards - PESC Board of Directors Recipients |url=https://pesc.org/awards/ |website=PESC |access-date=June 8, 2026}}</t>
   </si>
   <si>
+    <t>PESCBOARD2011</t>
+  </si>
+  <si>
+    <t>2011</t>
+  </si>
+  <si>
+    <t>PESC / South Carolina Transfer &amp; Articulation Center</t>
+  </si>
+  <si>
+    <t>PESC Award Letter to South Carolina</t>
+  </si>
+  <si>
+    <t>https://www.sctrac.org/portals/8/SCFiles/PESC_AwardLetterSC.pdf</t>
+  </si>
+  <si>
+    <t>Award letter / organizational record</t>
+  </si>
+  <si>
+    <t>Medium for board-listing facts; primary/organizational for PESC context</t>
+  </si>
+  <si>
+    <t>Minor. Letter includes a sidebar headed `2010-2011 Board of Directors` listing `JEFFREY ALDERSON, ConnectEDU, Inc.`.</t>
+  </si>
+  <si>
+    <t>Alderson was listed as a member of the PESC 2010-2011 Board of Directors while affiliated with ConnectEDU.</t>
+  </si>
+  <si>
+    <t>Use only for narrow PESC board-membership evidence; not a notability anchor.</t>
+  </si>
+  <si>
+    <t>Verified from downloaded PDF and extracted text</t>
+  </si>
+  <si>
+    <t>Reviewed in sources/pesc_sources.md; local files data/pesc_2010_2011_board_award_letter_sc.pdf and data/pesc_2010_2011_board_award_letter_sc.txt</t>
+  </si>
+  <si>
+    <t>{{cite web |title=PESC Award Letter to South Carolina |url=https://www.sctrac.org/portals/8/SCFiles/PESC_AwardLetterSC.pdf |website=South Carolina Transfer &amp; Articulation Center |publisher=Postsecondary Electronic Standards Council |date=March 24, 2011 |access-date=June 8, 2026}}</t>
+  </si>
+  <si>
+    <t>PESC2011</t>
+  </si>
+  <si>
+    <t>Spring 2011 Program Full - Boston</t>
+  </si>
+  <si>
+    <t>https://pesc.org/wp-content/uploads/2024/07/Spring-2011-Program-Full-Boston.pdf</t>
+  </si>
+  <si>
+    <t>Conference program / organizational event record</t>
+  </si>
+  <si>
+    <t>Medium for event-program facts; primary/organizational for PESC context</t>
+  </si>
+  <si>
+    <t>Minor. Program lists Alderson as Director of Development at ConnectEDU and a PESC Board of Directors member in the general session `Welcome to the Commonwealth of Massachusetts`; the same session also lists Jane Swift as Senior Vice President of Government Relations at ConnectEDU and former Massachusetts governor.</t>
+  </si>
+  <si>
+    <t>Alderson was listed as Director of Development at ConnectEDU and PESC Board of Directors member in the PESC Spring 2011 Data Summit program; Jane Swift was also listed as a ConnectEDU executive in the same session.</t>
+  </si>
+  <si>
+    <t>Use only for narrow PESC board / ConnectEDU role context; do not describe Alderson as keynote speaker based on this source.</t>
+  </si>
+  <si>
+    <t>Reviewed in sources/pesc_sources.md; local files data/pesc_spring_2011_program_full_boston.pdf and data/pesc_spring_2011_program_full_boston.txt</t>
+  </si>
+  <si>
+    <t>{{cite conference |title=Spring 2011 Program Full - Boston |conference=PESC Spring 2011 Data Summit |publisher=Postsecondary Electronic Standards Council |date=2011 |url=https://pesc.org/wp-content/uploads/2024/07/Spring-2011-Program-Full-Boston.pdf |access-date=June 8, 2026}}</t>
+  </si>
+  <si>
+    <t>NCES2011</t>
+  </si>
+  <si>
+    <t>NCES / STATS-DC</t>
+  </si>
+  <si>
+    <t>2011 STATS-DC Data Conference agenda</t>
+  </si>
+  <si>
+    <t>https://nces.ed.gov/whatsnew/conferences/PDF/STATSDC2011Agenda.pdf</t>
+  </si>
+  <si>
+    <t>Government conference agenda</t>
+  </si>
+  <si>
+    <t>High for agenda metadata; event listing only for biographical facts</t>
+  </si>
+  <si>
+    <t>Minor to moderate. Agenda lists session `VII-C Best Practices in Linking PK-12 and Higher Education` with Michael Sessa of PESC, David Moldoff of AcademyOne, and Jeffrey Alderson of ConnectEDU. The session description says PESC would present recent best practices using PESC-approved standards and technologies.</t>
+  </si>
+  <si>
+    <t>Alderson co-presented in a STATS-DC session on linking PK-12 and higher education data, in a session framed around PESC-approved standards and technologies.</t>
+  </si>
+  <si>
+    <t>Use only for narrow PESC/data-standards conference context; do not state that the agenda lists him as a PESC employee or board representative.</t>
+  </si>
+  <si>
+    <t>Reviewed in sources/pesc_sources.md; local files data/nces_statsdc_2011_agenda.pdf and data/nces_statsdc_2011_agenda.txt</t>
+  </si>
+  <si>
+    <t>{{cite conference |title=2011 STATS-DC Data Conference agenda |conference=STATS-DC Data Conference |publisher=National Center for Education Statistics |date=2011 |url=https://nces.ed.gov/whatsnew/conferences/PDF/STATSDC2011Agenda.pdf |access-date=June 8, 2026}}</t>
+  </si>
+  <si>
+    <t>PESC2012</t>
+  </si>
+  <si>
+    <t>2012</t>
+  </si>
+  <si>
+    <t>PESC Spring 2012 Data Summit program</t>
+  </si>
+  <si>
+    <t>https://nebula.wsimg.com/ab98b6bb89dd32b40efd76843c5817aa?AccessKeyId=4CF7FAE11697F99C9E6B&amp;disposition=0&amp;alloworigin=1</t>
+  </si>
+  <si>
+    <t>Minor to moderate. Program lists `MyDataButton | Jeffrey Alderson, Senior Director of Product Innovation, ConnectEDU` and says PESC Board Member Alderson would discuss the role he and ConnectEDU were playing in a joint White House/U.S. Department of Education initiative.</t>
+  </si>
+  <si>
+    <t>Alderson presented on MyDataButton at the PESC Spring 2012 Data Summit; the program tied him and ConnectEDU to a joint White House/U.S. Department of Education initiative about student access to data.</t>
+  </si>
+  <si>
+    <t>Use only for narrow MyDataButton / ConnectEDU / PESC professional-context facts; not a notability anchor.</t>
+  </si>
+  <si>
+    <t>Reviewed in sources/pesc_sources.md; local files data/pesc_2012_data_summit_program_my_data_button.pdf and data/pesc_2012_data_summit_program_my_data_button.txt</t>
+  </si>
+  <si>
+    <t>{{cite conference |title=PESC Spring 2012 Data Summit program |conference=PESC Spring 2012 Data Summit |publisher=Postsecondary Electronic Standards Council |date=2012 |url=https://nebula.wsimg.com/ab98b6bb89dd32b40efd76843c5817aa?AccessKeyId=4CF7FAE11697F99C9E6B&amp;disposition=0&amp;alloworigin=1 |access-date=June 8, 2026}}</t>
+  </si>
+  <si>
+    <t>ERUG1</t>
+  </si>
+  <si>
+    <t>PESC / Education Record User Group</t>
+  </si>
+  <si>
+    <t>PESC ERUG Conference Call Notes for April 24 2012</t>
+  </si>
+  <si>
+    <t>https://cdn.cocodoc.com/cocodoc-form-pdf/pdf/44678435--2012-04-24-PESC-ERUG-Call-Notespdf-pesc-.pdf</t>
+  </si>
+  <si>
+    <t>Call notes / organizational working-group record</t>
+  </si>
+  <si>
+    <t>Medium for call-note facts; primary/organizational for ERUG context</t>
+  </si>
+  <si>
+    <t>Moderate for narrow ERUG involvement. Call notes list Alderson as Director of Development at ConnectEDU and PESC Board of Directors member; they say he had suggested potential use of MyData in PESC XML work and briefed ERUG on the White House/U.S. Department of Education initiative.</t>
+  </si>
+  <si>
+    <t>Alderson was involved with the PESC Education Record User Group discussion of MyData; he briefed the group on the White House/U.S. Department of Education initiative and answered technical/product questions.</t>
+  </si>
+  <si>
+    <t>Use only for narrow ERUG / MyData involvement facts; not a notability anchor.</t>
+  </si>
+  <si>
+    <t>Reviewed in sources/pesc_sources.md; local files data/pesc_2012_erug_call_notes.pdf and data/pesc_2012_erug_call_notes.txt</t>
+  </si>
+  <si>
+    <t>{{cite web |title=PESC ERUG Conference Call Notes for April 24, 2012 |url=https://cdn.cocodoc.com/cocodoc-form-pdf/pdf/44678435--2012-04-24-PESC-ERUG-Call-Notespdf-pesc-.pdf |website=PESC Education Record User Group |date=April 24, 2012 |access-date=June 8, 2026}}</t>
+  </si>
+  <si>
+    <t>PESC2016</t>
+  </si>
+  <si>
+    <t>PESC Fall Data Symposium &amp; Summit program</t>
+  </si>
+  <si>
+    <t>https://nebula.wsimg.com/af9365ebe142935671ccd9d9f7258d0c?AccessKeyId=4CF7FAE11697F99C9E6B&amp;disposition=0&amp;alloworigin=1</t>
+  </si>
+  <si>
+    <t>Medium for event-program and award-listing facts; primary/organizational for PESC context</t>
+  </si>
+  <si>
+    <t>Minor to moderate. Program lists Alderson as Principal Analyst, Enterprise Software, Eduventures and speaker in `Global Data Strategy Perspectives | State &amp; PK12 and Evolving E-Portfolio`; it says Alderson of Eduventures would present findings from a review of 30 portfolio vendors. The same program lists `Jeffrey Alderson, Eduventures` under `Service Awards 2014-2015`.</t>
+  </si>
+  <si>
+    <t>Alderson presented Eduventures portfolio-vendor market research at the PESC Fall 2016 Data Symposium &amp; Summit; the program also corroborates a 2014-2015 PESC service-award listing for Alderson while affiliated with Eduventures.</t>
+  </si>
+  <si>
+    <t>Use only for narrow Eduventures ePortfolio research/presenter and PESC service-award facts; not a notability anchor.</t>
+  </si>
+  <si>
+    <t>Reviewed in sources/pesc_sources.md; local files data/pesc_2016_data_summit_eportfolio_vendors.pdf and data/pesc_2016_data_summit_eportfolio_vendors.txt</t>
+  </si>
+  <si>
+    <t>{{cite conference |title=PESC Fall Data Symposium &amp; Summit program |conference=PESC Fall Data Symposium &amp; Summit |publisher=Postsecondary Electronic Standards Council |date=2016 |url=https://nebula.wsimg.com/af9365ebe142935671ccd9d9f7258d0c?AccessKeyId=4CF7FAE11697F99C9E6B&amp;disposition=0&amp;alloworigin=1 |access-date=June 8, 2026}}</t>
+  </si>
+  <si>
+    <t>ACEL1</t>
+  </si>
+  <si>
+    <t>2016 / 2017</t>
+  </si>
+  <si>
+    <t>Academic Credential &amp; Experiential Learning Implementation Guide</t>
+  </si>
+  <si>
+    <t>https://cache.nebula.phx3.secureserver.net/78bacabe0c17ff11c6ee2e735abaa371?AccessKeyId=4CF7FAE11697F99C9E6B&amp;disposition=0&amp;alloworigin=1</t>
+  </si>
+  <si>
+    <t>Implementation guide / technical standard documentation</t>
+  </si>
+  <si>
+    <t>Medium for contributor-listing facts; primary/organizational for PESC context</t>
+  </si>
+  <si>
+    <t>Minor. Implementation guide lists `Jeffrey Alderson, Eduventures` among contributors in the acknowledgments.</t>
+  </si>
+  <si>
+    <t>Alderson was recognized as a contributor to PESC's Academic Credential &amp; Experiential Learning Implementation Guide while affiliated with Eduventures.</t>
+  </si>
+  <si>
+    <t>Use only for narrow PESC implementation-guide contributor evidence; not a notability anchor.</t>
+  </si>
+  <si>
+    <t>Reviewed in sources/pesc_sources.md; local files data/pesc_acel_implementation_guide.pdf and data/pesc_acel_implementation_guide.txt</t>
+  </si>
+  <si>
+    <t>{{cite web |title=Academic Credential &amp; Experiential Learning Implementation Guide |url=https://cache.nebula.phx3.secureserver.net/78bacabe0c17ff11c6ee2e735abaa371?AccessKeyId=4CF7FAE11697F99C9E6B&amp;disposition=0&amp;alloworigin=1 |website=PESC |date=November 2016 |access-date=June 8, 2026}}</t>
+  </si>
+  <si>
     <t>CB1</t>
   </si>
   <si>
     <t>2014</t>
   </si>
   <si>
-    <t>Scribd / U.S. Bankruptcy Court filing copy</t>
-  </si>
-  <si>
-    <t>Connectedu Bankruptcy Petition</t>
-  </si>
-  <si>
-    <t>https://www.scribd.com/doc/220960006/Connectedu-Bankruptcy-Petition</t>
-  </si>
-  <si>
-    <t>Legal filing copy / bankruptcy petition</t>
-  </si>
-  <si>
-    <t>High for narrow filing facts; weak as hosted copy</t>
-  </si>
-  <si>
-    <t>Minor. Primary bankruptcy filing for ConnectEDU, Inc., case 14-11238-scc, Doc. 1. Page 8 is the List of Equity Security Holders cover page; page 10 is Schedule A and lists Jeff Alderson.</t>
-  </si>
-  <si>
-    <t>Alderson was listed in Schedule A of ConnectEDU's List of Equity Security Holders with 139 ordinary common options, 139 total preferred and common, and 0.01% diluted ownership.</t>
-  </si>
-  <si>
-    <t>Use only for the narrow equity-security-holder fact; do not use for notability and prefer an official court copy if available.</t>
-  </si>
-  <si>
-    <t>Verified from downloaded PDF and rendered page images</t>
-  </si>
-  <si>
-    <t>Reviewed in sources/legal_bankruptcy_sources.md; local files data/connectedu_bankruptcy_petition.pdf; data/connectedu_bankruptcy_petition_download_text.txt; data/connectedu_bankruptcy_petition_page_08.png; data/connectedu_bankruptcy_petition_page_10.png</t>
-  </si>
-  <si>
-    <t>{{cite web |title=Connectedu Bankruptcy Petition |url=https://www.scribd.com/doc/220960006/Connectedu-Bankruptcy-Petition |website=Scribd |date=April 28, 2014 |access-date=June 8, 2026}}</t>
+    <t>PACERMonitor / U.S. Bankruptcy Court filing copy</t>
+  </si>
+  <si>
+    <t>ConnectEdu, Inc. Bankruptcy (1:14-bk-11238), New York Southern Bankruptcy Court</t>
+  </si>
+  <si>
+    <t>https://www.pacermonitor.com/public/case/3402250/ConnectEdu,_Inc</t>
+  </si>
+  <si>
+    <t>Public docket page plus legal filing copy</t>
+  </si>
+  <si>
+    <t>High for narrow docket and filing facts; primary legal-source context</t>
+  </si>
+  <si>
+    <t>Minor. PACERMonitor verifies ConnectEDU, Inc. bankruptcy case 1:14-bk-11238 in New York Southern Bankruptcy Court, filed April 28 2014, converted September 12 2014, terminated June 28 2017, and lists Doc. 1 as the Voluntary Petition. The reviewed petition copy shows page 8 as the List of Equity Security Holders cover page and page 10 as Schedule A listing Jeff Alderson.</t>
+  </si>
+  <si>
+    <t>Alderson was listed in Schedule A of ConnectEDU's List of Equity Security Holders with 139 ordinary common options, 139 total preferred and common, and 0.01% diluted ownership; PACERMonitor verifies the docket and Doc. 1 filing metadata.</t>
+  </si>
+  <si>
+    <t>Use only for the narrow equity-security-holder fact and docket context; do not use for notability.</t>
+  </si>
+  <si>
+    <t>Verified from PACERMonitor docket HTML and rendered petition page images</t>
+  </si>
+  <si>
+    <t>Reviewed in sources/legal_bankruptcy_sources.md; local files data/pacermonitor_connectedu_case.html; data/pacermonitor_connectedu_voluntary_petition_doc1.pdf HTML access page; data/connectedu_bankruptcy_petition.pdf; data/connectedu_bankruptcy_petition_download_text.txt; data/connectedu_bankruptcy_petition_page_08.png; data/connectedu_bankruptcy_petition_page_10.png</t>
+  </si>
+  <si>
+    <t>{{cite web |title=ConnectEdu, Inc. Bankruptcy (1:14-bk-11238), New York Southern Bankruptcy Court |url=https://www.pacermonitor.com/public/case/3402250/ConnectEdu,_Inc |website=PACERMonitor |date=April 28, 2014 |access-date=June 8, 2026}}</t>
   </si>
   <si>
     <t>S9</t>
@@ -514,9 +1006,6 @@
     <t>Retained as a publication lead, but not used in draft.</t>
   </si>
   <si>
-    <t>Do not cite until verified</t>
-  </si>
-  <si>
     <t>S10</t>
   </si>
   <si>
@@ -736,9 +1225,6 @@
     <t>Use only to verify official 2017 election result and vote totals; not notability support.</t>
   </si>
   <si>
-    <t>Verified from downloaded PDF and extracted text</t>
-  </si>
-  <si>
     <t>Reviewed in sources/town_of_natick_sources.md; local files data/town_of_natick_2017_official_election_results.pdf and data/town_of_natick_2017_official_election_results.txt</t>
   </si>
   <si>
@@ -748,9 +1234,6 @@
     <t>S11</t>
   </si>
   <si>
-    <t>2021</t>
-  </si>
-  <si>
     <t>ASME Mechanical Engineering</t>
   </si>
   <si>
@@ -1196,9 +1679,6 @@
   </si>
   <si>
     <t>N18</t>
-  </si>
-  <si>
-    <t>2024</t>
   </si>
   <si>
     <t>Natick Town Meeting week #1: MBTA Communities articles pass</t>
@@ -1762,7 +2242,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O46"/>
+  <dimension ref="A1:O60"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -2083,89 +2563,89 @@
         <v>85</v>
       </c>
       <c r="G7" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="H7" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="H7" s="2" t="s">
+      <c r="I7" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="I7" s="2" t="s">
+      <c r="J7" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="J7" s="2" t="s">
+      <c r="K7" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="L7" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="K7" s="2" t="s">
+      <c r="M7" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="N7" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="L7" s="2" t="s">
+      <c r="O7" s="2" t="s">
         <v>91</v>
-      </c>
-      <c r="M7" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="N7" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="O7" s="2" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="8" spans="1:15">
       <c r="A8" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="D8" s="2" t="s">
+      <c r="E8" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="F8" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="G8" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="H8" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="G8" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H8" s="2" t="s">
+      <c r="I8" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="I8" s="2" t="s">
+      <c r="J8" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="J8" s="2" t="s">
+      <c r="K8" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="L8" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="K8" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="L8" s="2" t="s">
+      <c r="M8" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="N8" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="M8" s="2" t="s">
+      <c r="O8" s="2" t="s">
         <v>103</v>
-      </c>
-      <c r="N8" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="O8" s="2" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="9" spans="1:15">
       <c r="A9" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>106</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>82</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>107</v>
@@ -2174,1777 +2654,2435 @@
         <v>108</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>98</v>
+        <v>109</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>21</v>
+        <v>51</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>99</v>
+        <v>110</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="K9" s="2" t="s">
         <v>76</v>
       </c>
       <c r="L9" s="2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>103</v>
+        <v>42</v>
       </c>
       <c r="N9" s="2" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="O9" s="2" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
     </row>
     <row r="10" spans="1:15">
       <c r="A10" s="2" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>46</v>
+        <v>117</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>51</v>
+        <v>122</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>76</v>
+        <v>126</v>
       </c>
       <c r="L10" s="2" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>42</v>
+        <v>128</v>
       </c>
       <c r="N10" s="2" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="O10" s="2" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
     </row>
     <row r="11" spans="1:15">
       <c r="A11" s="2" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>90</v>
+        <v>55</v>
       </c>
       <c r="L11" s="2" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="M11" s="2" t="s">
-        <v>42</v>
+        <v>142</v>
       </c>
       <c r="N11" s="2" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="O11" s="2" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
     </row>
     <row r="12" spans="1:15">
       <c r="A12" s="2" t="s">
-        <v>138</v>
+        <v>145</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>36</v>
+        <v>150</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>144</v>
+        <v>151</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>40</v>
+        <v>55</v>
       </c>
       <c r="L12" s="2" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="M12" s="2" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="N12" s="2" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="O12" s="2" t="s">
-        <v>150</v>
+        <v>157</v>
       </c>
     </row>
     <row r="13" spans="1:15">
       <c r="A13" s="2" t="s">
-        <v>151</v>
+        <v>158</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>152</v>
+        <v>132</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="K13" s="2" t="s">
-        <v>161</v>
+        <v>40</v>
       </c>
       <c r="L13" s="2" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="M13" s="2" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="N13" s="2" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="O13" s="2" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
     </row>
     <row r="14" spans="1:15">
       <c r="A14" s="2" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>55</v>
+        <v>126</v>
       </c>
       <c r="L14" s="2" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="M14" s="2" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="N14" s="2" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="O14" s="2" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
     </row>
     <row r="15" spans="1:15">
       <c r="A15" s="2" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>16</v>
+        <v>172</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>181</v>
+        <v>173</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>172</v>
+        <v>21</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="K15" s="2" t="s">
-        <v>40</v>
+        <v>126</v>
       </c>
       <c r="L15" s="2" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="M15" s="2" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="N15" s="2" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="O15" s="2" t="s">
-        <v>179</v>
+        <v>195</v>
       </c>
     </row>
     <row r="16" spans="1:15">
       <c r="A16" s="2" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>16</v>
+        <v>172</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>192</v>
+        <v>173</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>98</v>
+        <v>188</v>
       </c>
       <c r="G16" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>99</v>
+        <v>189</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>90</v>
+        <v>76</v>
       </c>
       <c r="L16" s="2" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="M16" s="2" t="s">
-        <v>42</v>
+        <v>193</v>
       </c>
       <c r="N16" s="2" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="O16" s="2" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
     </row>
     <row r="17" spans="1:15">
       <c r="A17" s="2" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>16</v>
+        <v>46</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>85</v>
+        <v>208</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>86</v>
+        <v>51</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>87</v>
+        <v>209</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>204</v>
+        <v>210</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>205</v>
+        <v>211</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>90</v>
+        <v>76</v>
       </c>
       <c r="L17" s="2" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
       <c r="M17" s="2" t="s">
         <v>42</v>
       </c>
       <c r="N17" s="2" t="s">
-        <v>207</v>
+        <v>213</v>
       </c>
       <c r="O17" s="2" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
     </row>
     <row r="18" spans="1:15">
       <c r="A18" s="2" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>16</v>
+        <v>216</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>201</v>
+        <v>217</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>210</v>
+        <v>218</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>211</v>
+        <v>219</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>212</v>
+        <v>220</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>51</v>
+        <v>221</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>99</v>
+        <v>222</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>213</v>
+        <v>223</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>214</v>
+        <v>224</v>
       </c>
       <c r="K18" s="2" t="s">
-        <v>76</v>
+        <v>126</v>
       </c>
       <c r="L18" s="2" t="s">
-        <v>215</v>
+        <v>225</v>
       </c>
       <c r="M18" s="2" t="s">
         <v>42</v>
       </c>
       <c r="N18" s="2" t="s">
-        <v>216</v>
+        <v>226</v>
       </c>
       <c r="O18" s="2" t="s">
-        <v>217</v>
+        <v>227</v>
       </c>
     </row>
     <row r="19" spans="1:15">
       <c r="A19" s="2" t="s">
-        <v>218</v>
+        <v>228</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>16</v>
+        <v>229</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>219</v>
+        <v>230</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>220</v>
+        <v>231</v>
       </c>
       <c r="E19" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="G19" s="2" t="s">
         <v>221</v>
       </c>
-      <c r="F19" s="2" t="s">
-        <v>222</v>
-      </c>
-      <c r="G19" s="2" t="s">
-        <v>51</v>
-      </c>
       <c r="H19" s="2" t="s">
-        <v>223</v>
+        <v>234</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>224</v>
+        <v>235</v>
       </c>
       <c r="J19" s="2" t="s">
-        <v>225</v>
+        <v>236</v>
       </c>
       <c r="K19" s="2" t="s">
-        <v>76</v>
+        <v>126</v>
       </c>
       <c r="L19" s="2" t="s">
-        <v>226</v>
+        <v>237</v>
       </c>
       <c r="M19" s="2" t="s">
-        <v>227</v>
+        <v>238</v>
       </c>
       <c r="N19" s="2" t="s">
-        <v>228</v>
+        <v>239</v>
       </c>
       <c r="O19" s="2" t="s">
-        <v>229</v>
+        <v>240</v>
       </c>
     </row>
     <row r="20" spans="1:15">
       <c r="A20" s="2" t="s">
-        <v>230</v>
+        <v>241</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>16</v>
+        <v>229</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>231</v>
+        <v>217</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>232</v>
+        <v>242</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>233</v>
+        <v>243</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>234</v>
+        <v>244</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>36</v>
+        <v>221</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>235</v>
+        <v>245</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>236</v>
+        <v>246</v>
       </c>
       <c r="J20" s="2" t="s">
-        <v>237</v>
+        <v>247</v>
       </c>
       <c r="K20" s="2" t="s">
-        <v>90</v>
+        <v>126</v>
       </c>
       <c r="L20" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="M20" s="2" t="s">
         <v>238</v>
       </c>
-      <c r="M20" s="2" t="s">
-        <v>239</v>
-      </c>
       <c r="N20" s="2" t="s">
-        <v>240</v>
+        <v>249</v>
       </c>
       <c r="O20" s="2" t="s">
-        <v>241</v>
+        <v>250</v>
       </c>
     </row>
     <row r="21" spans="1:15">
       <c r="A21" s="2" t="s">
-        <v>242</v>
+        <v>251</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>243</v>
+        <v>229</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>244</v>
+        <v>252</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>245</v>
+        <v>253</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>246</v>
+        <v>254</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>247</v>
+        <v>255</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>248</v>
+        <v>51</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>158</v>
+        <v>256</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>249</v>
+        <v>257</v>
       </c>
       <c r="J21" s="2" t="s">
-        <v>250</v>
+        <v>258</v>
       </c>
       <c r="K21" s="2" t="s">
-        <v>161</v>
+        <v>76</v>
       </c>
       <c r="L21" s="2" t="s">
-        <v>162</v>
+        <v>259</v>
       </c>
       <c r="M21" s="2" t="s">
-        <v>251</v>
+        <v>238</v>
       </c>
       <c r="N21" s="2" t="s">
-        <v>252</v>
+        <v>260</v>
       </c>
       <c r="O21" s="2" t="s">
-        <v>165</v>
+        <v>261</v>
       </c>
     </row>
     <row r="22" spans="1:15">
       <c r="A22" s="2" t="s">
-        <v>253</v>
+        <v>262</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>46</v>
+        <v>263</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>254</v>
+        <v>217</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>255</v>
+        <v>264</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>256</v>
+        <v>265</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>257</v>
+        <v>244</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>21</v>
+        <v>221</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>258</v>
+        <v>245</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>259</v>
+        <v>266</v>
       </c>
       <c r="J22" s="2" t="s">
-        <v>260</v>
+        <v>267</v>
       </c>
       <c r="K22" s="2" t="s">
         <v>76</v>
       </c>
       <c r="L22" s="2" t="s">
-        <v>261</v>
+        <v>268</v>
       </c>
       <c r="M22" s="2" t="s">
-        <v>262</v>
+        <v>238</v>
       </c>
       <c r="N22" s="2" t="s">
-        <v>263</v>
+        <v>269</v>
       </c>
       <c r="O22" s="2" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
     </row>
     <row r="23" spans="1:15">
       <c r="A23" s="2" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>46</v>
+        <v>263</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>254</v>
+        <v>272</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>266</v>
+        <v>273</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>267</v>
+        <v>274</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>257</v>
+        <v>275</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>21</v>
+        <v>221</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>258</v>
+        <v>276</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>268</v>
+        <v>277</v>
       </c>
       <c r="J23" s="2" t="s">
-        <v>269</v>
+        <v>278</v>
       </c>
       <c r="K23" s="2" t="s">
-        <v>90</v>
+        <v>76</v>
       </c>
       <c r="L23" s="2" t="s">
-        <v>270</v>
+        <v>279</v>
       </c>
       <c r="M23" s="2" t="s">
-        <v>262</v>
+        <v>238</v>
       </c>
       <c r="N23" s="2" t="s">
-        <v>271</v>
+        <v>280</v>
       </c>
       <c r="O23" s="2" t="s">
-        <v>272</v>
+        <v>281</v>
       </c>
     </row>
     <row r="24" spans="1:15">
       <c r="A24" s="2" t="s">
-        <v>273</v>
+        <v>282</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>46</v>
+        <v>60</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>254</v>
+        <v>217</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>274</v>
+        <v>283</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>275</v>
+        <v>284</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>257</v>
+        <v>244</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>21</v>
+        <v>221</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>258</v>
+        <v>285</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>276</v>
+        <v>286</v>
       </c>
       <c r="J24" s="2" t="s">
-        <v>277</v>
+        <v>287</v>
       </c>
       <c r="K24" s="2" t="s">
         <v>76</v>
       </c>
       <c r="L24" s="2" t="s">
-        <v>278</v>
+        <v>288</v>
       </c>
       <c r="M24" s="2" t="s">
-        <v>262</v>
+        <v>238</v>
       </c>
       <c r="N24" s="2" t="s">
-        <v>279</v>
+        <v>289</v>
       </c>
       <c r="O24" s="2" t="s">
-        <v>280</v>
+        <v>290</v>
       </c>
     </row>
     <row r="25" spans="1:15">
       <c r="A25" s="2" t="s">
-        <v>281</v>
+        <v>291</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>46</v>
+        <v>292</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>254</v>
+        <v>217</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>282</v>
+        <v>293</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>283</v>
+        <v>294</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>284</v>
+        <v>295</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>86</v>
+        <v>221</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>258</v>
+        <v>296</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>285</v>
+        <v>297</v>
       </c>
       <c r="J25" s="2" t="s">
-        <v>286</v>
+        <v>298</v>
       </c>
       <c r="K25" s="2" t="s">
-        <v>55</v>
+        <v>126</v>
       </c>
       <c r="L25" s="2" t="s">
-        <v>287</v>
+        <v>299</v>
       </c>
       <c r="M25" s="2" t="s">
-        <v>262</v>
+        <v>238</v>
       </c>
       <c r="N25" s="2" t="s">
-        <v>288</v>
+        <v>300</v>
       </c>
       <c r="O25" s="2" t="s">
-        <v>289</v>
+        <v>301</v>
       </c>
     </row>
     <row r="26" spans="1:15">
       <c r="A26" s="2" t="s">
-        <v>290</v>
+        <v>302</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>46</v>
+        <v>303</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>254</v>
+        <v>304</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>291</v>
+        <v>305</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>292</v>
+        <v>306</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>257</v>
+        <v>307</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>258</v>
+        <v>308</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>293</v>
+        <v>309</v>
       </c>
       <c r="J26" s="2" t="s">
-        <v>294</v>
+        <v>310</v>
       </c>
       <c r="K26" s="2" t="s">
-        <v>76</v>
+        <v>40</v>
       </c>
       <c r="L26" s="2" t="s">
-        <v>295</v>
+        <v>311</v>
       </c>
       <c r="M26" s="2" t="s">
-        <v>262</v>
+        <v>312</v>
       </c>
       <c r="N26" s="2" t="s">
-        <v>296</v>
+        <v>313</v>
       </c>
       <c r="O26" s="2" t="s">
-        <v>297</v>
+        <v>314</v>
       </c>
     </row>
     <row r="27" spans="1:15">
       <c r="A27" s="2" t="s">
-        <v>298</v>
+        <v>315</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>81</v>
+        <v>316</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>254</v>
+        <v>317</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>299</v>
+        <v>318</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>300</v>
+        <v>319</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>257</v>
+        <v>320</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>21</v>
+        <v>321</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>258</v>
+        <v>322</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>301</v>
+        <v>323</v>
       </c>
       <c r="J27" s="2" t="s">
-        <v>302</v>
+        <v>324</v>
       </c>
       <c r="K27" s="2" t="s">
-        <v>76</v>
+        <v>325</v>
       </c>
       <c r="L27" s="2" t="s">
-        <v>303</v>
+        <v>326</v>
       </c>
       <c r="M27" s="2" t="s">
-        <v>262</v>
+        <v>327</v>
       </c>
       <c r="N27" s="2" t="s">
-        <v>304</v>
+        <v>328</v>
       </c>
       <c r="O27" s="2" t="s">
-        <v>305</v>
+        <v>170</v>
       </c>
     </row>
     <row r="28" spans="1:15">
       <c r="A28" s="2" t="s">
-        <v>306</v>
+        <v>329</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>81</v>
+        <v>330</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>254</v>
+        <v>331</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>307</v>
+        <v>332</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>308</v>
+        <v>333</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>257</v>
+        <v>334</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>21</v>
+        <v>335</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>258</v>
+        <v>336</v>
       </c>
       <c r="I28" s="2" t="s">
-        <v>309</v>
+        <v>337</v>
       </c>
       <c r="J28" s="2" t="s">
-        <v>310</v>
+        <v>338</v>
       </c>
       <c r="K28" s="2" t="s">
-        <v>90</v>
+        <v>55</v>
       </c>
       <c r="L28" s="2" t="s">
-        <v>311</v>
+        <v>339</v>
       </c>
       <c r="M28" s="2" t="s">
-        <v>262</v>
+        <v>340</v>
       </c>
       <c r="N28" s="2" t="s">
-        <v>312</v>
+        <v>341</v>
       </c>
       <c r="O28" s="2" t="s">
-        <v>313</v>
+        <v>342</v>
       </c>
     </row>
     <row r="29" spans="1:15">
       <c r="A29" s="2" t="s">
-        <v>314</v>
+        <v>343</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>81</v>
+        <v>16</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>254</v>
+        <v>344</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>315</v>
+        <v>345</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>316</v>
+        <v>346</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>257</v>
+        <v>347</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>21</v>
+        <v>335</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>258</v>
+        <v>348</v>
       </c>
       <c r="I29" s="2" t="s">
-        <v>317</v>
+        <v>349</v>
       </c>
       <c r="J29" s="2" t="s">
-        <v>318</v>
+        <v>350</v>
       </c>
       <c r="K29" s="2" t="s">
-        <v>76</v>
+        <v>40</v>
       </c>
       <c r="L29" s="2" t="s">
-        <v>319</v>
+        <v>351</v>
       </c>
       <c r="M29" s="2" t="s">
-        <v>262</v>
+        <v>352</v>
       </c>
       <c r="N29" s="2" t="s">
-        <v>320</v>
+        <v>353</v>
       </c>
       <c r="O29" s="2" t="s">
-        <v>321</v>
+        <v>342</v>
       </c>
     </row>
     <row r="30" spans="1:15">
       <c r="A30" s="2" t="s">
-        <v>322</v>
+        <v>354</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>81</v>
+        <v>16</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>254</v>
+        <v>355</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>323</v>
+        <v>356</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>324</v>
+        <v>357</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>257</v>
+        <v>188</v>
       </c>
       <c r="G30" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>258</v>
+        <v>189</v>
       </c>
       <c r="I30" s="2" t="s">
-        <v>325</v>
+        <v>358</v>
       </c>
       <c r="J30" s="2" t="s">
-        <v>326</v>
+        <v>359</v>
       </c>
       <c r="K30" s="2" t="s">
-        <v>90</v>
+        <v>126</v>
       </c>
       <c r="L30" s="2" t="s">
-        <v>327</v>
+        <v>360</v>
       </c>
       <c r="M30" s="2" t="s">
-        <v>262</v>
+        <v>42</v>
       </c>
       <c r="N30" s="2" t="s">
-        <v>328</v>
+        <v>361</v>
       </c>
       <c r="O30" s="2" t="s">
-        <v>329</v>
+        <v>362</v>
       </c>
     </row>
     <row r="31" spans="1:15">
       <c r="A31" s="2" t="s">
-        <v>330</v>
+        <v>363</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>81</v>
+        <v>16</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>254</v>
+        <v>364</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>331</v>
+        <v>365</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>332</v>
+        <v>366</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>257</v>
+        <v>176</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>21</v>
+        <v>177</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>258</v>
+        <v>178</v>
       </c>
       <c r="I31" s="2" t="s">
-        <v>333</v>
+        <v>367</v>
       </c>
       <c r="J31" s="2" t="s">
-        <v>334</v>
+        <v>368</v>
       </c>
       <c r="K31" s="2" t="s">
-        <v>90</v>
+        <v>126</v>
       </c>
       <c r="L31" s="2" t="s">
-        <v>335</v>
+        <v>369</v>
       </c>
       <c r="M31" s="2" t="s">
-        <v>262</v>
+        <v>42</v>
       </c>
       <c r="N31" s="2" t="s">
-        <v>336</v>
+        <v>370</v>
       </c>
       <c r="O31" s="2" t="s">
-        <v>337</v>
+        <v>371</v>
       </c>
     </row>
     <row r="32" spans="1:15">
       <c r="A32" s="2" t="s">
-        <v>338</v>
+        <v>372</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>81</v>
+        <v>16</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>254</v>
+        <v>364</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>339</v>
+        <v>373</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>340</v>
+        <v>374</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>257</v>
+        <v>375</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>21</v>
+        <v>51</v>
       </c>
       <c r="H32" s="2" t="s">
-        <v>258</v>
+        <v>189</v>
       </c>
       <c r="I32" s="2" t="s">
-        <v>341</v>
+        <v>376</v>
       </c>
       <c r="J32" s="2" t="s">
-        <v>342</v>
+        <v>377</v>
       </c>
       <c r="K32" s="2" t="s">
         <v>76</v>
       </c>
       <c r="L32" s="2" t="s">
-        <v>343</v>
+        <v>378</v>
       </c>
       <c r="M32" s="2" t="s">
-        <v>262</v>
+        <v>42</v>
       </c>
       <c r="N32" s="2" t="s">
-        <v>344</v>
+        <v>379</v>
       </c>
       <c r="O32" s="2" t="s">
-        <v>345</v>
+        <v>380</v>
       </c>
     </row>
     <row r="33" spans="1:15">
       <c r="A33" s="2" t="s">
-        <v>346</v>
+        <v>381</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>81</v>
+        <v>16</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>254</v>
+        <v>382</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>347</v>
+        <v>383</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>348</v>
+        <v>384</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>257</v>
+        <v>385</v>
       </c>
       <c r="G33" s="2" t="s">
-        <v>21</v>
+        <v>51</v>
       </c>
       <c r="H33" s="2" t="s">
-        <v>258</v>
+        <v>386</v>
       </c>
       <c r="I33" s="2" t="s">
-        <v>349</v>
+        <v>387</v>
       </c>
       <c r="J33" s="2" t="s">
-        <v>350</v>
+        <v>388</v>
       </c>
       <c r="K33" s="2" t="s">
-        <v>90</v>
+        <v>76</v>
       </c>
       <c r="L33" s="2" t="s">
-        <v>335</v>
+        <v>389</v>
       </c>
       <c r="M33" s="2" t="s">
-        <v>262</v>
+        <v>390</v>
       </c>
       <c r="N33" s="2" t="s">
-        <v>351</v>
+        <v>391</v>
       </c>
       <c r="O33" s="2" t="s">
-        <v>352</v>
+        <v>392</v>
       </c>
     </row>
     <row r="34" spans="1:15">
       <c r="A34" s="2" t="s">
-        <v>353</v>
+        <v>393</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>81</v>
+        <v>16</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>254</v>
+        <v>394</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>354</v>
+        <v>395</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>355</v>
+        <v>396</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>257</v>
+        <v>397</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>258</v>
+        <v>398</v>
       </c>
       <c r="I34" s="2" t="s">
-        <v>356</v>
+        <v>399</v>
       </c>
       <c r="J34" s="2" t="s">
-        <v>357</v>
+        <v>400</v>
       </c>
       <c r="K34" s="2" t="s">
-        <v>90</v>
+        <v>126</v>
       </c>
       <c r="L34" s="2" t="s">
-        <v>358</v>
+        <v>401</v>
       </c>
       <c r="M34" s="2" t="s">
-        <v>262</v>
+        <v>238</v>
       </c>
       <c r="N34" s="2" t="s">
-        <v>359</v>
+        <v>402</v>
       </c>
       <c r="O34" s="2" t="s">
-        <v>360</v>
+        <v>403</v>
       </c>
     </row>
     <row r="35" spans="1:15">
       <c r="A35" s="2" t="s">
-        <v>361</v>
+        <v>404</v>
       </c>
       <c r="B35" s="2" t="s">
         <v>81</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>254</v>
+        <v>405</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>362</v>
+        <v>406</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>363</v>
+        <v>407</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>257</v>
+        <v>408</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>21</v>
+        <v>409</v>
       </c>
       <c r="H35" s="2" t="s">
-        <v>258</v>
+        <v>322</v>
       </c>
       <c r="I35" s="2" t="s">
-        <v>364</v>
+        <v>410</v>
       </c>
       <c r="J35" s="2" t="s">
-        <v>365</v>
+        <v>411</v>
       </c>
       <c r="K35" s="2" t="s">
-        <v>76</v>
+        <v>325</v>
       </c>
       <c r="L35" s="2" t="s">
-        <v>366</v>
+        <v>326</v>
       </c>
       <c r="M35" s="2" t="s">
-        <v>262</v>
+        <v>412</v>
       </c>
       <c r="N35" s="2" t="s">
-        <v>367</v>
+        <v>413</v>
       </c>
       <c r="O35" s="2" t="s">
-        <v>368</v>
+        <v>170</v>
       </c>
     </row>
     <row r="36" spans="1:15">
       <c r="A36" s="2" t="s">
-        <v>369</v>
+        <v>414</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>81</v>
+        <v>46</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>254</v>
+        <v>415</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>370</v>
+        <v>416</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>371</v>
+        <v>417</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>257</v>
+        <v>418</v>
       </c>
       <c r="G36" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H36" s="2" t="s">
-        <v>258</v>
+        <v>419</v>
       </c>
       <c r="I36" s="2" t="s">
-        <v>372</v>
+        <v>420</v>
       </c>
       <c r="J36" s="2" t="s">
-        <v>373</v>
+        <v>421</v>
       </c>
       <c r="K36" s="2" t="s">
-        <v>90</v>
+        <v>76</v>
       </c>
       <c r="L36" s="2" t="s">
-        <v>335</v>
+        <v>422</v>
       </c>
       <c r="M36" s="2" t="s">
-        <v>262</v>
+        <v>423</v>
       </c>
       <c r="N36" s="2" t="s">
-        <v>374</v>
+        <v>424</v>
       </c>
       <c r="O36" s="2" t="s">
-        <v>375</v>
+        <v>425</v>
       </c>
     </row>
     <row r="37" spans="1:15">
       <c r="A37" s="2" t="s">
-        <v>376</v>
+        <v>426</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>81</v>
+        <v>46</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>254</v>
+        <v>415</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>377</v>
+        <v>427</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>378</v>
+        <v>428</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>257</v>
+        <v>418</v>
       </c>
       <c r="G37" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H37" s="2" t="s">
-        <v>258</v>
+        <v>419</v>
       </c>
       <c r="I37" s="2" t="s">
-        <v>379</v>
+        <v>429</v>
       </c>
       <c r="J37" s="2" t="s">
-        <v>380</v>
+        <v>430</v>
       </c>
       <c r="K37" s="2" t="s">
-        <v>76</v>
+        <v>126</v>
       </c>
       <c r="L37" s="2" t="s">
-        <v>381</v>
+        <v>431</v>
       </c>
       <c r="M37" s="2" t="s">
-        <v>262</v>
+        <v>423</v>
       </c>
       <c r="N37" s="2" t="s">
-        <v>382</v>
+        <v>432</v>
       </c>
       <c r="O37" s="2" t="s">
-        <v>383</v>
+        <v>433</v>
       </c>
     </row>
     <row r="38" spans="1:15">
       <c r="A38" s="2" t="s">
-        <v>384</v>
+        <v>434</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>81</v>
+        <v>46</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>254</v>
+        <v>415</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>385</v>
+        <v>435</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>386</v>
+        <v>436</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>257</v>
+        <v>418</v>
       </c>
       <c r="G38" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H38" s="2" t="s">
-        <v>258</v>
+        <v>419</v>
       </c>
       <c r="I38" s="2" t="s">
-        <v>387</v>
+        <v>437</v>
       </c>
       <c r="J38" s="2" t="s">
-        <v>388</v>
+        <v>438</v>
       </c>
       <c r="K38" s="2" t="s">
-        <v>90</v>
+        <v>76</v>
       </c>
       <c r="L38" s="2" t="s">
-        <v>389</v>
+        <v>439</v>
       </c>
       <c r="M38" s="2" t="s">
-        <v>262</v>
+        <v>423</v>
       </c>
       <c r="N38" s="2" t="s">
-        <v>390</v>
+        <v>440</v>
       </c>
       <c r="O38" s="2" t="s">
-        <v>391</v>
+        <v>441</v>
       </c>
     </row>
     <row r="39" spans="1:15">
       <c r="A39" s="2" t="s">
-        <v>392</v>
+        <v>442</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>393</v>
+        <v>46</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>254</v>
+        <v>415</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>394</v>
+        <v>443</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>395</v>
+        <v>444</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>257</v>
+        <v>445</v>
       </c>
       <c r="G39" s="2" t="s">
-        <v>21</v>
+        <v>177</v>
       </c>
       <c r="H39" s="2" t="s">
-        <v>258</v>
+        <v>419</v>
       </c>
       <c r="I39" s="2" t="s">
-        <v>396</v>
+        <v>446</v>
       </c>
       <c r="J39" s="2" t="s">
-        <v>397</v>
+        <v>447</v>
       </c>
       <c r="K39" s="2" t="s">
-        <v>90</v>
+        <v>55</v>
       </c>
       <c r="L39" s="2" t="s">
-        <v>398</v>
+        <v>448</v>
       </c>
       <c r="M39" s="2" t="s">
-        <v>262</v>
+        <v>423</v>
       </c>
       <c r="N39" s="2" t="s">
-        <v>399</v>
+        <v>449</v>
       </c>
       <c r="O39" s="2" t="s">
-        <v>400</v>
+        <v>450</v>
       </c>
     </row>
     <row r="40" spans="1:15">
       <c r="A40" s="2" t="s">
-        <v>401</v>
+        <v>451</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>402</v>
+        <v>46</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>254</v>
+        <v>415</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>403</v>
+        <v>452</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>404</v>
+        <v>453</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>257</v>
+        <v>418</v>
       </c>
       <c r="G40" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H40" s="2" t="s">
-        <v>258</v>
+        <v>419</v>
       </c>
       <c r="I40" s="2" t="s">
-        <v>405</v>
+        <v>454</v>
       </c>
       <c r="J40" s="2" t="s">
-        <v>406</v>
+        <v>455</v>
       </c>
       <c r="K40" s="2" t="s">
         <v>76</v>
       </c>
       <c r="L40" s="2" t="s">
-        <v>407</v>
+        <v>456</v>
       </c>
       <c r="M40" s="2" t="s">
-        <v>262</v>
+        <v>423</v>
       </c>
       <c r="N40" s="2" t="s">
-        <v>408</v>
+        <v>457</v>
       </c>
       <c r="O40" s="2" t="s">
-        <v>409</v>
+        <v>458</v>
       </c>
     </row>
     <row r="41" spans="1:15">
       <c r="A41" s="2" t="s">
-        <v>410</v>
+        <v>459</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>81</v>
+        <v>172</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>254</v>
+        <v>415</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>411</v>
+        <v>460</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>412</v>
+        <v>461</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>257</v>
+        <v>418</v>
       </c>
       <c r="G41" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H41" s="2" t="s">
-        <v>258</v>
+        <v>419</v>
       </c>
       <c r="I41" s="2" t="s">
-        <v>413</v>
+        <v>462</v>
       </c>
       <c r="J41" s="2" t="s">
-        <v>414</v>
+        <v>463</v>
       </c>
       <c r="K41" s="2" t="s">
-        <v>90</v>
+        <v>76</v>
       </c>
       <c r="L41" s="2" t="s">
-        <v>415</v>
+        <v>464</v>
       </c>
       <c r="M41" s="2" t="s">
-        <v>262</v>
+        <v>423</v>
       </c>
       <c r="N41" s="2" t="s">
-        <v>416</v>
+        <v>465</v>
       </c>
       <c r="O41" s="2" t="s">
-        <v>417</v>
+        <v>466</v>
       </c>
     </row>
     <row r="42" spans="1:15">
       <c r="A42" s="2" t="s">
+        <v>467</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>468</v>
+      </c>
+      <c r="E42" s="3" t="s">
+        <v>469</v>
+      </c>
+      <c r="F42" s="2" t="s">
         <v>418</v>
       </c>
-      <c r="B42" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="C42" s="2" t="s">
-        <v>254</v>
-      </c>
-      <c r="D42" s="2" t="s">
+      <c r="G42" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H42" s="2" t="s">
         <v>419</v>
       </c>
-      <c r="E42" s="3" t="s">
-        <v>420</v>
-      </c>
-      <c r="F42" s="2" t="s">
-        <v>284</v>
-      </c>
-      <c r="G42" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="H42" s="2" t="s">
-        <v>258</v>
-      </c>
       <c r="I42" s="2" t="s">
-        <v>421</v>
+        <v>470</v>
       </c>
       <c r="J42" s="2" t="s">
-        <v>422</v>
+        <v>471</v>
       </c>
       <c r="K42" s="2" t="s">
-        <v>90</v>
+        <v>126</v>
       </c>
       <c r="L42" s="2" t="s">
-        <v>91</v>
+        <v>472</v>
       </c>
       <c r="M42" s="2" t="s">
-        <v>262</v>
+        <v>423</v>
       </c>
       <c r="N42" s="2" t="s">
-        <v>423</v>
+        <v>473</v>
       </c>
       <c r="O42" s="2" t="s">
-        <v>424</v>
+        <v>474</v>
       </c>
     </row>
     <row r="43" spans="1:15">
       <c r="A43" s="2" t="s">
-        <v>425</v>
+        <v>475</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>81</v>
+        <v>172</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>254</v>
+        <v>415</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>426</v>
+        <v>476</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>427</v>
+        <v>477</v>
       </c>
       <c r="F43" s="2" t="s">
-        <v>257</v>
+        <v>418</v>
       </c>
       <c r="G43" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H43" s="2" t="s">
-        <v>258</v>
+        <v>419</v>
       </c>
       <c r="I43" s="2" t="s">
-        <v>428</v>
+        <v>478</v>
       </c>
       <c r="J43" s="2" t="s">
-        <v>429</v>
+        <v>479</v>
       </c>
       <c r="K43" s="2" t="s">
-        <v>90</v>
+        <v>76</v>
       </c>
       <c r="L43" s="2" t="s">
-        <v>430</v>
+        <v>480</v>
       </c>
       <c r="M43" s="2" t="s">
-        <v>262</v>
+        <v>423</v>
       </c>
       <c r="N43" s="2" t="s">
-        <v>431</v>
+        <v>481</v>
       </c>
       <c r="O43" s="2" t="s">
-        <v>432</v>
+        <v>482</v>
       </c>
     </row>
     <row r="44" spans="1:15">
       <c r="A44" s="2" t="s">
-        <v>433</v>
+        <v>483</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>393</v>
+        <v>172</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>254</v>
+        <v>415</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>434</v>
+        <v>484</v>
       </c>
       <c r="E44" s="3" t="s">
-        <v>435</v>
+        <v>485</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>257</v>
+        <v>418</v>
       </c>
       <c r="G44" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H44" s="2" t="s">
-        <v>258</v>
+        <v>419</v>
       </c>
       <c r="I44" s="2" t="s">
-        <v>436</v>
+        <v>486</v>
       </c>
       <c r="J44" s="2" t="s">
-        <v>437</v>
+        <v>487</v>
       </c>
       <c r="K44" s="2" t="s">
-        <v>90</v>
+        <v>126</v>
       </c>
       <c r="L44" s="2" t="s">
-        <v>438</v>
+        <v>488</v>
       </c>
       <c r="M44" s="2" t="s">
-        <v>262</v>
+        <v>423</v>
       </c>
       <c r="N44" s="2" t="s">
-        <v>439</v>
+        <v>489</v>
       </c>
       <c r="O44" s="2" t="s">
-        <v>440</v>
+        <v>490</v>
       </c>
     </row>
     <row r="45" spans="1:15">
       <c r="A45" s="2" t="s">
-        <v>441</v>
+        <v>491</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>402</v>
+        <v>172</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>254</v>
+        <v>415</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>442</v>
+        <v>492</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>443</v>
+        <v>493</v>
       </c>
       <c r="F45" s="2" t="s">
-        <v>257</v>
+        <v>418</v>
       </c>
       <c r="G45" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H45" s="2" t="s">
-        <v>258</v>
+        <v>419</v>
       </c>
       <c r="I45" s="2" t="s">
-        <v>444</v>
+        <v>494</v>
       </c>
       <c r="J45" s="2" t="s">
-        <v>445</v>
+        <v>495</v>
       </c>
       <c r="K45" s="2" t="s">
-        <v>76</v>
+        <v>126</v>
       </c>
       <c r="L45" s="2" t="s">
-        <v>446</v>
+        <v>496</v>
       </c>
       <c r="M45" s="2" t="s">
-        <v>262</v>
+        <v>423</v>
       </c>
       <c r="N45" s="2" t="s">
-        <v>447</v>
+        <v>497</v>
       </c>
       <c r="O45" s="2" t="s">
-        <v>448</v>
+        <v>498</v>
       </c>
     </row>
     <row r="46" spans="1:15">
       <c r="A46" s="2" t="s">
-        <v>449</v>
+        <v>499</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>402</v>
+        <v>172</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>254</v>
+        <v>415</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>450</v>
+        <v>500</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>451</v>
+        <v>501</v>
       </c>
       <c r="F46" s="2" t="s">
-        <v>257</v>
+        <v>418</v>
       </c>
       <c r="G46" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H46" s="2" t="s">
-        <v>258</v>
+        <v>419</v>
       </c>
       <c r="I46" s="2" t="s">
-        <v>452</v>
+        <v>502</v>
       </c>
       <c r="J46" s="2" t="s">
-        <v>453</v>
+        <v>503</v>
       </c>
       <c r="K46" s="2" t="s">
-        <v>90</v>
+        <v>76</v>
       </c>
       <c r="L46" s="2" t="s">
-        <v>335</v>
+        <v>504</v>
       </c>
       <c r="M46" s="2" t="s">
-        <v>262</v>
+        <v>423</v>
       </c>
       <c r="N46" s="2" t="s">
-        <v>454</v>
+        <v>505</v>
       </c>
       <c r="O46" s="2" t="s">
-        <v>455</v>
+        <v>506</v>
+      </c>
+    </row>
+    <row r="47" spans="1:15">
+      <c r="A47" s="2" t="s">
+        <v>507</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>508</v>
+      </c>
+      <c r="E47" s="3" t="s">
+        <v>509</v>
+      </c>
+      <c r="F47" s="2" t="s">
+        <v>418</v>
+      </c>
+      <c r="G47" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H47" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="I47" s="2" t="s">
+        <v>510</v>
+      </c>
+      <c r="J47" s="2" t="s">
+        <v>511</v>
+      </c>
+      <c r="K47" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="L47" s="2" t="s">
+        <v>496</v>
+      </c>
+      <c r="M47" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="N47" s="2" t="s">
+        <v>512</v>
+      </c>
+      <c r="O47" s="2" t="s">
+        <v>513</v>
+      </c>
+    </row>
+    <row r="48" spans="1:15">
+      <c r="A48" s="2" t="s">
+        <v>514</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>515</v>
+      </c>
+      <c r="E48" s="3" t="s">
+        <v>516</v>
+      </c>
+      <c r="F48" s="2" t="s">
+        <v>418</v>
+      </c>
+      <c r="G48" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H48" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="I48" s="2" t="s">
+        <v>517</v>
+      </c>
+      <c r="J48" s="2" t="s">
+        <v>518</v>
+      </c>
+      <c r="K48" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="L48" s="2" t="s">
+        <v>519</v>
+      </c>
+      <c r="M48" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="N48" s="2" t="s">
+        <v>520</v>
+      </c>
+      <c r="O48" s="2" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="49" spans="1:15">
+      <c r="A49" s="2" t="s">
+        <v>522</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>523</v>
+      </c>
+      <c r="E49" s="3" t="s">
+        <v>524</v>
+      </c>
+      <c r="F49" s="2" t="s">
+        <v>418</v>
+      </c>
+      <c r="G49" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H49" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="I49" s="2" t="s">
+        <v>525</v>
+      </c>
+      <c r="J49" s="2" t="s">
+        <v>526</v>
+      </c>
+      <c r="K49" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="L49" s="2" t="s">
+        <v>527</v>
+      </c>
+      <c r="M49" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="N49" s="2" t="s">
+        <v>528</v>
+      </c>
+      <c r="O49" s="2" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="50" spans="1:15">
+      <c r="A50" s="2" t="s">
+        <v>530</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>531</v>
+      </c>
+      <c r="E50" s="3" t="s">
+        <v>532</v>
+      </c>
+      <c r="F50" s="2" t="s">
+        <v>418</v>
+      </c>
+      <c r="G50" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H50" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="I50" s="2" t="s">
+        <v>533</v>
+      </c>
+      <c r="J50" s="2" t="s">
+        <v>534</v>
+      </c>
+      <c r="K50" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="L50" s="2" t="s">
+        <v>496</v>
+      </c>
+      <c r="M50" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="N50" s="2" t="s">
+        <v>535</v>
+      </c>
+      <c r="O50" s="2" t="s">
+        <v>536</v>
+      </c>
+    </row>
+    <row r="51" spans="1:15">
+      <c r="A51" s="2" t="s">
+        <v>537</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="D51" s="2" t="s">
+        <v>538</v>
+      </c>
+      <c r="E51" s="3" t="s">
+        <v>539</v>
+      </c>
+      <c r="F51" s="2" t="s">
+        <v>418</v>
+      </c>
+      <c r="G51" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H51" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="I51" s="2" t="s">
+        <v>540</v>
+      </c>
+      <c r="J51" s="2" t="s">
+        <v>541</v>
+      </c>
+      <c r="K51" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="L51" s="2" t="s">
+        <v>542</v>
+      </c>
+      <c r="M51" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="N51" s="2" t="s">
+        <v>543</v>
+      </c>
+      <c r="O51" s="2" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="52" spans="1:15">
+      <c r="A52" s="2" t="s">
+        <v>545</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="D52" s="2" t="s">
+        <v>546</v>
+      </c>
+      <c r="E52" s="3" t="s">
+        <v>547</v>
+      </c>
+      <c r="F52" s="2" t="s">
+        <v>418</v>
+      </c>
+      <c r="G52" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H52" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="I52" s="2" t="s">
+        <v>548</v>
+      </c>
+      <c r="J52" s="2" t="s">
+        <v>549</v>
+      </c>
+      <c r="K52" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="L52" s="2" t="s">
+        <v>550</v>
+      </c>
+      <c r="M52" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="N52" s="2" t="s">
+        <v>551</v>
+      </c>
+      <c r="O52" s="2" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="53" spans="1:15">
+      <c r="A53" s="2" t="s">
+        <v>553</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="C53" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="D53" s="2" t="s">
+        <v>554</v>
+      </c>
+      <c r="E53" s="3" t="s">
+        <v>555</v>
+      </c>
+      <c r="F53" s="2" t="s">
+        <v>418</v>
+      </c>
+      <c r="G53" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H53" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="I53" s="2" t="s">
+        <v>556</v>
+      </c>
+      <c r="J53" s="2" t="s">
+        <v>557</v>
+      </c>
+      <c r="K53" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="L53" s="2" t="s">
+        <v>558</v>
+      </c>
+      <c r="M53" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="N53" s="2" t="s">
+        <v>559</v>
+      </c>
+      <c r="O53" s="2" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="54" spans="1:15">
+      <c r="A54" s="2" t="s">
+        <v>561</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>562</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="D54" s="2" t="s">
+        <v>563</v>
+      </c>
+      <c r="E54" s="3" t="s">
+        <v>564</v>
+      </c>
+      <c r="F54" s="2" t="s">
+        <v>418</v>
+      </c>
+      <c r="G54" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H54" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="I54" s="2" t="s">
+        <v>565</v>
+      </c>
+      <c r="J54" s="2" t="s">
+        <v>566</v>
+      </c>
+      <c r="K54" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="L54" s="2" t="s">
+        <v>567</v>
+      </c>
+      <c r="M54" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="N54" s="2" t="s">
+        <v>568</v>
+      </c>
+      <c r="O54" s="2" t="s">
+        <v>569</v>
+      </c>
+    </row>
+    <row r="55" spans="1:15">
+      <c r="A55" s="2" t="s">
+        <v>570</v>
+      </c>
+      <c r="B55" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="C55" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="D55" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="E55" s="3" t="s">
+        <v>572</v>
+      </c>
+      <c r="F55" s="2" t="s">
+        <v>418</v>
+      </c>
+      <c r="G55" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H55" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="I55" s="2" t="s">
+        <v>573</v>
+      </c>
+      <c r="J55" s="2" t="s">
+        <v>574</v>
+      </c>
+      <c r="K55" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="L55" s="2" t="s">
+        <v>575</v>
+      </c>
+      <c r="M55" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="N55" s="2" t="s">
+        <v>576</v>
+      </c>
+      <c r="O55" s="2" t="s">
+        <v>577</v>
+      </c>
+    </row>
+    <row r="56" spans="1:15">
+      <c r="A56" s="2" t="s">
+        <v>578</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="C56" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="D56" s="2" t="s">
+        <v>579</v>
+      </c>
+      <c r="E56" s="3" t="s">
+        <v>580</v>
+      </c>
+      <c r="F56" s="2" t="s">
+        <v>445</v>
+      </c>
+      <c r="G56" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="H56" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="I56" s="2" t="s">
+        <v>581</v>
+      </c>
+      <c r="J56" s="2" t="s">
+        <v>582</v>
+      </c>
+      <c r="K56" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="L56" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="M56" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="N56" s="2" t="s">
+        <v>583</v>
+      </c>
+      <c r="O56" s="2" t="s">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="57" spans="1:15">
+      <c r="A57" s="2" t="s">
+        <v>585</v>
+      </c>
+      <c r="B57" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="C57" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="D57" s="2" t="s">
+        <v>586</v>
+      </c>
+      <c r="E57" s="3" t="s">
+        <v>587</v>
+      </c>
+      <c r="F57" s="2" t="s">
+        <v>418</v>
+      </c>
+      <c r="G57" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H57" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="I57" s="2" t="s">
+        <v>588</v>
+      </c>
+      <c r="J57" s="2" t="s">
+        <v>589</v>
+      </c>
+      <c r="K57" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="L57" s="2" t="s">
+        <v>590</v>
+      </c>
+      <c r="M57" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="N57" s="2" t="s">
+        <v>591</v>
+      </c>
+      <c r="O57" s="2" t="s">
+        <v>592</v>
+      </c>
+    </row>
+    <row r="58" spans="1:15">
+      <c r="A58" s="2" t="s">
+        <v>593</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="C58" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="D58" s="2" t="s">
+        <v>594</v>
+      </c>
+      <c r="E58" s="3" t="s">
+        <v>595</v>
+      </c>
+      <c r="F58" s="2" t="s">
+        <v>418</v>
+      </c>
+      <c r="G58" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H58" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="I58" s="2" t="s">
+        <v>596</v>
+      </c>
+      <c r="J58" s="2" t="s">
+        <v>597</v>
+      </c>
+      <c r="K58" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="L58" s="2" t="s">
+        <v>598</v>
+      </c>
+      <c r="M58" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="N58" s="2" t="s">
+        <v>599</v>
+      </c>
+      <c r="O58" s="2" t="s">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="59" spans="1:15">
+      <c r="A59" s="2" t="s">
+        <v>601</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>562</v>
+      </c>
+      <c r="C59" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="D59" s="2" t="s">
+        <v>602</v>
+      </c>
+      <c r="E59" s="3" t="s">
+        <v>603</v>
+      </c>
+      <c r="F59" s="2" t="s">
+        <v>418</v>
+      </c>
+      <c r="G59" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H59" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="I59" s="2" t="s">
+        <v>604</v>
+      </c>
+      <c r="J59" s="2" t="s">
+        <v>605</v>
+      </c>
+      <c r="K59" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="L59" s="2" t="s">
+        <v>606</v>
+      </c>
+      <c r="M59" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="N59" s="2" t="s">
+        <v>607</v>
+      </c>
+      <c r="O59" s="2" t="s">
+        <v>608</v>
+      </c>
+    </row>
+    <row r="60" spans="1:15">
+      <c r="A60" s="2" t="s">
+        <v>609</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>562</v>
+      </c>
+      <c r="C60" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="D60" s="2" t="s">
+        <v>610</v>
+      </c>
+      <c r="E60" s="3" t="s">
+        <v>611</v>
+      </c>
+      <c r="F60" s="2" t="s">
+        <v>418</v>
+      </c>
+      <c r="G60" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H60" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="I60" s="2" t="s">
+        <v>612</v>
+      </c>
+      <c r="J60" s="2" t="s">
+        <v>613</v>
+      </c>
+      <c r="K60" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="L60" s="2" t="s">
+        <v>496</v>
+      </c>
+      <c r="M60" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="N60" s="2" t="s">
+        <v>614</v>
+      </c>
+      <c r="O60" s="2" t="s">
+        <v>615</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O46"/>
+  <autoFilter ref="A1:O60"/>
   <hyperlinks>
     <hyperlink ref="E2" r:id="rId1"/>
     <hyperlink ref="E3" r:id="rId2"/>
@@ -3991,6 +5129,20 @@
     <hyperlink ref="E44" r:id="rId43"/>
     <hyperlink ref="E45" r:id="rId44"/>
     <hyperlink ref="E46" r:id="rId45"/>
+    <hyperlink ref="E47" r:id="rId46"/>
+    <hyperlink ref="E48" r:id="rId47"/>
+    <hyperlink ref="E49" r:id="rId48"/>
+    <hyperlink ref="E50" r:id="rId49"/>
+    <hyperlink ref="E51" r:id="rId50"/>
+    <hyperlink ref="E52" r:id="rId51"/>
+    <hyperlink ref="E53" r:id="rId52"/>
+    <hyperlink ref="E54" r:id="rId53"/>
+    <hyperlink ref="E55" r:id="rId54"/>
+    <hyperlink ref="E56" r:id="rId55"/>
+    <hyperlink ref="E57" r:id="rId56"/>
+    <hyperlink ref="E58" r:id="rId57"/>
+    <hyperlink ref="E59" r:id="rId58"/>
+    <hyperlink ref="E60" r:id="rId59"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update source dossier and remove unreferenced files
</commit_message>
<xml_diff>
--- a/dossier/source_dossier.xlsx
+++ b/dossier/source_dossier.xlsx
@@ -10,14 +10,14 @@
     <sheet name="Source Dossier" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Source Dossier'!$A$1:$O$60</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Source Dossier'!$A$1:$O$63</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="900" uniqueCount="616">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="945" uniqueCount="653">
   <si>
     <t>id</t>
   </si>
@@ -925,6 +925,87 @@
     <t>{{cite web |title=Academic Credential &amp; Experiential Learning Implementation Guide |url=https://cache.nebula.phx3.secureserver.net/78bacabe0c17ff11c6ee2e735abaa371?AccessKeyId=4CF7FAE11697F99C9E6B&amp;disposition=0&amp;alloworigin=1 |website=PESC |date=November 2016 |access-date=June 8, 2026}}</t>
   </si>
   <si>
+    <t>MDB2</t>
+  </si>
+  <si>
+    <t>Hack Education</t>
+  </si>
+  <si>
+    <t>Download All Your Education Data With the Click of One Button</t>
+  </si>
+  <si>
+    <t>https://hackeducation.com/2012/04/11/download-all-your-education-data-with-the-click-of-one-button</t>
+  </si>
+  <si>
+    <t>Education-technology blog post</t>
+  </si>
+  <si>
+    <t>Partial; independent of Alderson but not about him</t>
+  </si>
+  <si>
+    <t>Medium for contemporary MyDataButton and HMH initiative context; not a source for Alderson-specific facts</t>
+  </si>
+  <si>
+    <t>Background only. Article describes the Department of Education's proposed MyData button, compares it to the VA Blue Button, discusses education-data silos and standards, and states that ETS, Pearson, Parchment, and Houghton Mifflin Harcourt were among key industry players on board. Does not mention Alderson, ConnectEDU, or PESC.</t>
+  </si>
+  <si>
+    <t>Background context for MyDataButton and Houghton Mifflin Harcourt's inclusion in the initiative; does not independently verify Alderson's involvement.</t>
+  </si>
+  <si>
+    <t>Low for Alderson; Medium for MyDataButton / HMH context</t>
+  </si>
+  <si>
+    <t>Use only as MyDataButton/HMH context; pair Alderson-specific claims with PESC2012/ERUG1 and HMH role claims with Data &amp; Society or another HMH-specific source.</t>
+  </si>
+  <si>
+    <t>Verified from downloaded HTML and extracted text</t>
+  </si>
+  <si>
+    <t>Reviewed in sources/mydata_button_sources.md; local files data/hack_education_mydata_button_2012.html and data/hack_education_mydata_button_2012.txt</t>
+  </si>
+  <si>
+    <t>{{cite web |last=Watters |first=Audrey |title=Download All Your Education Data With the Click of One Button |url=https://hackeducation.com/2012/04/11/download-all-your-education-data-with-the-click-of-one-button |website=Hack Education |date=April 11, 2012 |access-date=June 8, 2026}}</t>
+  </si>
+  <si>
+    <t>MDB1</t>
+  </si>
+  <si>
+    <t>ESP Solutions Group / ArnieDocs mirror</t>
+  </si>
+  <si>
+    <t>MyData Button: Button, Button, Who's Got the Button?</t>
+  </si>
+  <si>
+    <t>https://www.arniedocs.info/wp-content/uploads/2016/05/MyData-Button-Disappears-2016-05-03.pdf</t>
+  </si>
+  <si>
+    <t>White paper / commentary</t>
+  </si>
+  <si>
+    <t>Partial; not about Alderson</t>
+  </si>
+  <si>
+    <t>Medium for MyDataButton background; not a source for Alderson-specific facts</t>
+  </si>
+  <si>
+    <t>Background only. Paper states that in 2012 the White House, Secretary of Education, and several major companies promised students a button to download education data; describes MyDataButton as part of the Obama administration smart-disclosure/open-government effort; says the January 19 2012 Executive Office announcement said MyDataButton would appear on the U.S. Department of Education Federal Student Aid website; names Houghton Mifflin Harcourt among companies in the announcement. Does not mention Alderson, ConnectEDU, or PESC.</t>
+  </si>
+  <si>
+    <t>Background context for the White House / U.S. Department of Education MyDataButton initiative and Houghton Mifflin Harcourt's inclusion in the announcement; does not independently verify Alderson's involvement.</t>
+  </si>
+  <si>
+    <t>Low for Alderson; Medium for MyDataButton context</t>
+  </si>
+  <si>
+    <t>Use only as MyDataButton initiative background; pair Alderson-specific claims with PESC2012/ERUG1 and HMH role claims with Data &amp; Society or another HMH-specific source.</t>
+  </si>
+  <si>
+    <t>Reviewed in sources/mydata_button_sources.md; local files data/mydata_button_white_house_disappears_2016.pdf and data/mydata_button_white_house_disappears_2016.txt</t>
+  </si>
+  <si>
+    <t>{{cite web |last=Ligon |first=Glynn D. |title=MyData Button: Button, Button, Who's Got the Button? |url=https://www.arniedocs.info/wp-content/uploads/2016/05/MyData-Button-Disappears-2016-05-03.pdf |website=ArnieDocs |publisher=ESP Solutions Group |date=May 3, 2016 |access-date=June 8, 2026}}</t>
+  </si>
+  <si>
     <t>CB1</t>
   </si>
   <si>
@@ -1229,6 +1310,36 @@
   </si>
   <si>
     <t>{{cite web |title=Official Election Results - March 28, 2017 |url=https://www.natickma.gov/DocumentCenter/View/4563/Official-Election-Results---March-28-2017?bidId= |website=Town of Natick |date=April 4, 2017 |access-date=June 8, 2026}}</t>
+  </si>
+  <si>
+    <t>TN2</t>
+  </si>
+  <si>
+    <t>Hybrid Town Meeting Committee</t>
+  </si>
+  <si>
+    <t>https://www.natickma.gov/2301/Hybrid-Town-Meeting-Committee</t>
+  </si>
+  <si>
+    <t>Official committee page</t>
+  </si>
+  <si>
+    <t>Medium for official committee existence; does not name Alderson</t>
+  </si>
+  <si>
+    <t>Minor. Official Town of Natick committee page verifies the Hybrid Town Meeting Committee exists under Boards &amp; Committees and includes a public survey link.</t>
+  </si>
+  <si>
+    <t>The Hybrid Town Meeting Committee exists as an official Town of Natick committee; use only to corroborate committee existence alongside Natick Report's Alderson-specific operational coverage.</t>
+  </si>
+  <si>
+    <t>Use only to corroborate official committee existence and public-facing activity; pair with Natick Report N6 for Alderson-specific action.</t>
+  </si>
+  <si>
+    <t>Reviewed in sources/town_of_natick_sources.md; local files data/town_of_natick_hybrid_town_meeting_committee.html and data/town_of_natick_hybrid_town_meeting_committee.txt</t>
+  </si>
+  <si>
+    <t>{{cite web |title=Hybrid Town Meeting Committee |url=https://www.natickma.gov/2301/Hybrid-Town-Meeting-Committee |website=Town of Natick |access-date=June 8, 2026}}</t>
   </si>
   <si>
     <t>S11</t>
@@ -2242,7 +2353,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O60"/>
+  <dimension ref="A1:O63"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -3441,22 +3552,22 @@
         <v>302</v>
       </c>
       <c r="B26" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="C26" s="2" t="s">
         <v>303</v>
       </c>
-      <c r="C26" s="2" t="s">
+      <c r="D26" s="2" t="s">
         <v>304</v>
       </c>
-      <c r="D26" s="2" t="s">
+      <c r="E26" s="3" t="s">
         <v>305</v>
       </c>
-      <c r="E26" s="3" t="s">
+      <c r="F26" s="2" t="s">
         <v>306</v>
       </c>
-      <c r="F26" s="2" t="s">
+      <c r="G26" s="2" t="s">
         <v>307</v>
-      </c>
-      <c r="G26" s="2" t="s">
-        <v>36</v>
       </c>
       <c r="H26" s="2" t="s">
         <v>308</v>
@@ -3468,27 +3579,27 @@
         <v>310</v>
       </c>
       <c r="K26" s="2" t="s">
-        <v>40</v>
+        <v>311</v>
       </c>
       <c r="L26" s="2" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="M26" s="2" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="N26" s="2" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="O26" s="2" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
     </row>
     <row r="27" spans="1:15">
       <c r="A27" s="2" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>316</v>
+        <v>60</v>
       </c>
       <c r="C27" s="2" t="s">
         <v>317</v>
@@ -3521,13 +3632,13 @@
         <v>326</v>
       </c>
       <c r="M27" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="N27" s="2" t="s">
         <v>327</v>
       </c>
-      <c r="N27" s="2" t="s">
+      <c r="O27" s="2" t="s">
         <v>328</v>
-      </c>
-      <c r="O27" s="2" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="28" spans="1:15">
@@ -3550,39 +3661,39 @@
         <v>334</v>
       </c>
       <c r="G28" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="H28" s="2" t="s">
         <v>335</v>
       </c>
-      <c r="H28" s="2" t="s">
+      <c r="I28" s="2" t="s">
         <v>336</v>
       </c>
-      <c r="I28" s="2" t="s">
+      <c r="J28" s="2" t="s">
         <v>337</v>
       </c>
-      <c r="J28" s="2" t="s">
+      <c r="K28" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="L28" s="2" t="s">
         <v>338</v>
       </c>
-      <c r="K28" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="L28" s="2" t="s">
+      <c r="M28" s="2" t="s">
         <v>339</v>
       </c>
-      <c r="M28" s="2" t="s">
+      <c r="N28" s="2" t="s">
         <v>340</v>
       </c>
-      <c r="N28" s="2" t="s">
+      <c r="O28" s="2" t="s">
         <v>341</v>
-      </c>
-      <c r="O28" s="2" t="s">
-        <v>342</v>
       </c>
     </row>
     <row r="29" spans="1:15">
       <c r="A29" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="B29" s="2" t="s">
         <v>343</v>
-      </c>
-      <c r="B29" s="2" t="s">
-        <v>16</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>344</v>
@@ -3597,1492 +3708,1633 @@
         <v>347</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>335</v>
+        <v>348</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="I29" s="2" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="J29" s="2" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="K29" s="2" t="s">
-        <v>40</v>
+        <v>352</v>
       </c>
       <c r="L29" s="2" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="M29" s="2" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="N29" s="2" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="O29" s="2" t="s">
-        <v>342</v>
+        <v>170</v>
       </c>
     </row>
     <row r="30" spans="1:15">
       <c r="A30" s="2" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>16</v>
+        <v>357</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>188</v>
+        <v>361</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>21</v>
+        <v>362</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>189</v>
+        <v>363</v>
       </c>
       <c r="I30" s="2" t="s">
-        <v>358</v>
+        <v>364</v>
       </c>
       <c r="J30" s="2" t="s">
-        <v>359</v>
+        <v>365</v>
       </c>
       <c r="K30" s="2" t="s">
-        <v>126</v>
+        <v>55</v>
       </c>
       <c r="L30" s="2" t="s">
-        <v>360</v>
+        <v>366</v>
       </c>
       <c r="M30" s="2" t="s">
-        <v>42</v>
+        <v>367</v>
       </c>
       <c r="N30" s="2" t="s">
-        <v>361</v>
+        <v>368</v>
       </c>
       <c r="O30" s="2" t="s">
-        <v>362</v>
+        <v>369</v>
       </c>
     </row>
     <row r="31" spans="1:15">
       <c r="A31" s="2" t="s">
-        <v>363</v>
+        <v>370</v>
       </c>
       <c r="B31" s="2" t="s">
         <v>16</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>364</v>
+        <v>371</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>365</v>
+        <v>372</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>366</v>
+        <v>373</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>176</v>
+        <v>374</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>177</v>
+        <v>362</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>178</v>
+        <v>375</v>
       </c>
       <c r="I31" s="2" t="s">
-        <v>367</v>
+        <v>376</v>
       </c>
       <c r="J31" s="2" t="s">
-        <v>368</v>
+        <v>377</v>
       </c>
       <c r="K31" s="2" t="s">
-        <v>126</v>
+        <v>40</v>
       </c>
       <c r="L31" s="2" t="s">
+        <v>378</v>
+      </c>
+      <c r="M31" s="2" t="s">
+        <v>379</v>
+      </c>
+      <c r="N31" s="2" t="s">
+        <v>380</v>
+      </c>
+      <c r="O31" s="2" t="s">
         <v>369</v>
-      </c>
-      <c r="M31" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="N31" s="2" t="s">
-        <v>370</v>
-      </c>
-      <c r="O31" s="2" t="s">
-        <v>371</v>
       </c>
     </row>
     <row r="32" spans="1:15">
       <c r="A32" s="2" t="s">
-        <v>372</v>
+        <v>381</v>
       </c>
       <c r="B32" s="2" t="s">
         <v>16</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>364</v>
+        <v>382</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>373</v>
+        <v>383</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>374</v>
+        <v>384</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>375</v>
+        <v>188</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>51</v>
+        <v>21</v>
       </c>
       <c r="H32" s="2" t="s">
         <v>189</v>
       </c>
       <c r="I32" s="2" t="s">
-        <v>376</v>
+        <v>385</v>
       </c>
       <c r="J32" s="2" t="s">
-        <v>377</v>
+        <v>386</v>
       </c>
       <c r="K32" s="2" t="s">
-        <v>76</v>
+        <v>126</v>
       </c>
       <c r="L32" s="2" t="s">
-        <v>378</v>
+        <v>387</v>
       </c>
       <c r="M32" s="2" t="s">
         <v>42</v>
       </c>
       <c r="N32" s="2" t="s">
-        <v>379</v>
+        <v>388</v>
       </c>
       <c r="O32" s="2" t="s">
-        <v>380</v>
+        <v>389</v>
       </c>
     </row>
     <row r="33" spans="1:15">
       <c r="A33" s="2" t="s">
-        <v>381</v>
+        <v>390</v>
       </c>
       <c r="B33" s="2" t="s">
         <v>16</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>382</v>
+        <v>391</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>383</v>
+        <v>392</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>384</v>
+        <v>393</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>385</v>
+        <v>176</v>
       </c>
       <c r="G33" s="2" t="s">
-        <v>51</v>
+        <v>177</v>
       </c>
       <c r="H33" s="2" t="s">
-        <v>386</v>
+        <v>178</v>
       </c>
       <c r="I33" s="2" t="s">
-        <v>387</v>
+        <v>394</v>
       </c>
       <c r="J33" s="2" t="s">
-        <v>388</v>
+        <v>395</v>
       </c>
       <c r="K33" s="2" t="s">
-        <v>76</v>
+        <v>126</v>
       </c>
       <c r="L33" s="2" t="s">
-        <v>389</v>
+        <v>396</v>
       </c>
       <c r="M33" s="2" t="s">
-        <v>390</v>
+        <v>42</v>
       </c>
       <c r="N33" s="2" t="s">
-        <v>391</v>
+        <v>397</v>
       </c>
       <c r="O33" s="2" t="s">
-        <v>392</v>
+        <v>398</v>
       </c>
     </row>
     <row r="34" spans="1:15">
       <c r="A34" s="2" t="s">
-        <v>393</v>
+        <v>399</v>
       </c>
       <c r="B34" s="2" t="s">
         <v>16</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>394</v>
+        <v>391</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>395</v>
+        <v>400</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>396</v>
+        <v>401</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>397</v>
+        <v>402</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>36</v>
+        <v>51</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>398</v>
+        <v>189</v>
       </c>
       <c r="I34" s="2" t="s">
-        <v>399</v>
+        <v>403</v>
       </c>
       <c r="J34" s="2" t="s">
-        <v>400</v>
+        <v>404</v>
       </c>
       <c r="K34" s="2" t="s">
-        <v>126</v>
+        <v>76</v>
       </c>
       <c r="L34" s="2" t="s">
-        <v>401</v>
+        <v>405</v>
       </c>
       <c r="M34" s="2" t="s">
-        <v>238</v>
+        <v>42</v>
       </c>
       <c r="N34" s="2" t="s">
-        <v>402</v>
+        <v>406</v>
       </c>
       <c r="O34" s="2" t="s">
-        <v>403</v>
+        <v>407</v>
       </c>
     </row>
     <row r="35" spans="1:15">
       <c r="A35" s="2" t="s">
-        <v>404</v>
+        <v>408</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>81</v>
+        <v>16</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>405</v>
+        <v>409</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>406</v>
+        <v>410</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>407</v>
+        <v>411</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>408</v>
+        <v>412</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>409</v>
+        <v>51</v>
       </c>
       <c r="H35" s="2" t="s">
-        <v>322</v>
+        <v>413</v>
       </c>
       <c r="I35" s="2" t="s">
-        <v>410</v>
+        <v>414</v>
       </c>
       <c r="J35" s="2" t="s">
-        <v>411</v>
+        <v>415</v>
       </c>
       <c r="K35" s="2" t="s">
-        <v>325</v>
+        <v>76</v>
       </c>
       <c r="L35" s="2" t="s">
-        <v>326</v>
+        <v>416</v>
       </c>
       <c r="M35" s="2" t="s">
-        <v>412</v>
+        <v>417</v>
       </c>
       <c r="N35" s="2" t="s">
-        <v>413</v>
+        <v>418</v>
       </c>
       <c r="O35" s="2" t="s">
-        <v>170</v>
+        <v>419</v>
       </c>
     </row>
     <row r="36" spans="1:15">
       <c r="A36" s="2" t="s">
-        <v>414</v>
+        <v>420</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>46</v>
+        <v>16</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>415</v>
+        <v>421</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>416</v>
+        <v>422</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>417</v>
+        <v>423</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>418</v>
+        <v>424</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="H36" s="2" t="s">
-        <v>419</v>
+        <v>425</v>
       </c>
       <c r="I36" s="2" t="s">
-        <v>420</v>
+        <v>426</v>
       </c>
       <c r="J36" s="2" t="s">
-        <v>421</v>
+        <v>427</v>
       </c>
       <c r="K36" s="2" t="s">
-        <v>76</v>
+        <v>126</v>
       </c>
       <c r="L36" s="2" t="s">
-        <v>422</v>
+        <v>428</v>
       </c>
       <c r="M36" s="2" t="s">
-        <v>423</v>
+        <v>238</v>
       </c>
       <c r="N36" s="2" t="s">
-        <v>424</v>
+        <v>429</v>
       </c>
       <c r="O36" s="2" t="s">
-        <v>425</v>
+        <v>430</v>
       </c>
     </row>
     <row r="37" spans="1:15">
       <c r="A37" s="2" t="s">
-        <v>426</v>
+        <v>431</v>
       </c>
       <c r="B37" s="2" t="s">
         <v>46</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>415</v>
+        <v>421</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>427</v>
+        <v>432</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>428</v>
+        <v>433</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>418</v>
+        <v>434</v>
       </c>
       <c r="G37" s="2" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="H37" s="2" t="s">
-        <v>419</v>
+        <v>435</v>
       </c>
       <c r="I37" s="2" t="s">
-        <v>429</v>
+        <v>436</v>
       </c>
       <c r="J37" s="2" t="s">
-        <v>430</v>
+        <v>437</v>
       </c>
       <c r="K37" s="2" t="s">
         <v>126</v>
       </c>
       <c r="L37" s="2" t="s">
-        <v>431</v>
+        <v>438</v>
       </c>
       <c r="M37" s="2" t="s">
-        <v>423</v>
+        <v>313</v>
       </c>
       <c r="N37" s="2" t="s">
-        <v>432</v>
+        <v>439</v>
       </c>
       <c r="O37" s="2" t="s">
-        <v>433</v>
+        <v>440</v>
       </c>
     </row>
     <row r="38" spans="1:15">
       <c r="A38" s="2" t="s">
-        <v>434</v>
+        <v>441</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>46</v>
+        <v>81</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>415</v>
+        <v>442</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>435</v>
+        <v>443</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>436</v>
+        <v>444</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>418</v>
+        <v>445</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>21</v>
+        <v>446</v>
       </c>
       <c r="H38" s="2" t="s">
-        <v>419</v>
+        <v>349</v>
       </c>
       <c r="I38" s="2" t="s">
-        <v>437</v>
+        <v>447</v>
       </c>
       <c r="J38" s="2" t="s">
-        <v>438</v>
+        <v>448</v>
       </c>
       <c r="K38" s="2" t="s">
-        <v>76</v>
+        <v>352</v>
       </c>
       <c r="L38" s="2" t="s">
-        <v>439</v>
+        <v>353</v>
       </c>
       <c r="M38" s="2" t="s">
-        <v>423</v>
+        <v>449</v>
       </c>
       <c r="N38" s="2" t="s">
-        <v>440</v>
+        <v>450</v>
       </c>
       <c r="O38" s="2" t="s">
-        <v>441</v>
+        <v>170</v>
       </c>
     </row>
     <row r="39" spans="1:15">
       <c r="A39" s="2" t="s">
-        <v>442</v>
+        <v>451</v>
       </c>
       <c r="B39" s="2" t="s">
         <v>46</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>415</v>
+        <v>452</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>443</v>
+        <v>453</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>444</v>
+        <v>454</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>445</v>
+        <v>455</v>
       </c>
       <c r="G39" s="2" t="s">
-        <v>177</v>
+        <v>21</v>
       </c>
       <c r="H39" s="2" t="s">
-        <v>419</v>
+        <v>456</v>
       </c>
       <c r="I39" s="2" t="s">
-        <v>446</v>
+        <v>457</v>
       </c>
       <c r="J39" s="2" t="s">
-        <v>447</v>
+        <v>458</v>
       </c>
       <c r="K39" s="2" t="s">
-        <v>55</v>
+        <v>76</v>
       </c>
       <c r="L39" s="2" t="s">
-        <v>448</v>
+        <v>459</v>
       </c>
       <c r="M39" s="2" t="s">
-        <v>423</v>
+        <v>460</v>
       </c>
       <c r="N39" s="2" t="s">
-        <v>449</v>
+        <v>461</v>
       </c>
       <c r="O39" s="2" t="s">
-        <v>450</v>
+        <v>462</v>
       </c>
     </row>
     <row r="40" spans="1:15">
       <c r="A40" s="2" t="s">
-        <v>451</v>
+        <v>463</v>
       </c>
       <c r="B40" s="2" t="s">
         <v>46</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>415</v>
+        <v>452</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>452</v>
+        <v>464</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>453</v>
+        <v>465</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>418</v>
+        <v>455</v>
       </c>
       <c r="G40" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H40" s="2" t="s">
-        <v>419</v>
+        <v>456</v>
       </c>
       <c r="I40" s="2" t="s">
-        <v>454</v>
+        <v>466</v>
       </c>
       <c r="J40" s="2" t="s">
-        <v>455</v>
+        <v>467</v>
       </c>
       <c r="K40" s="2" t="s">
-        <v>76</v>
+        <v>126</v>
       </c>
       <c r="L40" s="2" t="s">
-        <v>456</v>
+        <v>468</v>
       </c>
       <c r="M40" s="2" t="s">
-        <v>423</v>
+        <v>460</v>
       </c>
       <c r="N40" s="2" t="s">
-        <v>457</v>
+        <v>469</v>
       </c>
       <c r="O40" s="2" t="s">
-        <v>458</v>
+        <v>470</v>
       </c>
     </row>
     <row r="41" spans="1:15">
       <c r="A41" s="2" t="s">
-        <v>459</v>
+        <v>471</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>172</v>
+        <v>46</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>415</v>
+        <v>452</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>460</v>
+        <v>472</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>461</v>
+        <v>473</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>418</v>
+        <v>455</v>
       </c>
       <c r="G41" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H41" s="2" t="s">
-        <v>419</v>
+        <v>456</v>
       </c>
       <c r="I41" s="2" t="s">
-        <v>462</v>
+        <v>474</v>
       </c>
       <c r="J41" s="2" t="s">
-        <v>463</v>
+        <v>475</v>
       </c>
       <c r="K41" s="2" t="s">
         <v>76</v>
       </c>
       <c r="L41" s="2" t="s">
-        <v>464</v>
+        <v>476</v>
       </c>
       <c r="M41" s="2" t="s">
-        <v>423</v>
+        <v>460</v>
       </c>
       <c r="N41" s="2" t="s">
-        <v>465</v>
+        <v>477</v>
       </c>
       <c r="O41" s="2" t="s">
-        <v>466</v>
+        <v>478</v>
       </c>
     </row>
     <row r="42" spans="1:15">
       <c r="A42" s="2" t="s">
-        <v>467</v>
+        <v>479</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>172</v>
+        <v>46</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>415</v>
+        <v>452</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>468</v>
+        <v>480</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>469</v>
+        <v>481</v>
       </c>
       <c r="F42" s="2" t="s">
-        <v>418</v>
+        <v>482</v>
       </c>
       <c r="G42" s="2" t="s">
-        <v>21</v>
+        <v>177</v>
       </c>
       <c r="H42" s="2" t="s">
-        <v>419</v>
+        <v>456</v>
       </c>
       <c r="I42" s="2" t="s">
-        <v>470</v>
+        <v>483</v>
       </c>
       <c r="J42" s="2" t="s">
-        <v>471</v>
+        <v>484</v>
       </c>
       <c r="K42" s="2" t="s">
-        <v>126</v>
+        <v>55</v>
       </c>
       <c r="L42" s="2" t="s">
-        <v>472</v>
+        <v>485</v>
       </c>
       <c r="M42" s="2" t="s">
-        <v>423</v>
+        <v>460</v>
       </c>
       <c r="N42" s="2" t="s">
-        <v>473</v>
+        <v>486</v>
       </c>
       <c r="O42" s="2" t="s">
-        <v>474</v>
+        <v>487</v>
       </c>
     </row>
     <row r="43" spans="1:15">
       <c r="A43" s="2" t="s">
-        <v>475</v>
+        <v>488</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>172</v>
+        <v>46</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>415</v>
+        <v>452</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>476</v>
+        <v>489</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>477</v>
+        <v>490</v>
       </c>
       <c r="F43" s="2" t="s">
-        <v>418</v>
+        <v>455</v>
       </c>
       <c r="G43" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H43" s="2" t="s">
-        <v>419</v>
+        <v>456</v>
       </c>
       <c r="I43" s="2" t="s">
-        <v>478</v>
+        <v>491</v>
       </c>
       <c r="J43" s="2" t="s">
-        <v>479</v>
+        <v>492</v>
       </c>
       <c r="K43" s="2" t="s">
         <v>76</v>
       </c>
       <c r="L43" s="2" t="s">
-        <v>480</v>
+        <v>493</v>
       </c>
       <c r="M43" s="2" t="s">
-        <v>423</v>
+        <v>460</v>
       </c>
       <c r="N43" s="2" t="s">
-        <v>481</v>
+        <v>494</v>
       </c>
       <c r="O43" s="2" t="s">
-        <v>482</v>
+        <v>495</v>
       </c>
     </row>
     <row r="44" spans="1:15">
       <c r="A44" s="2" t="s">
-        <v>483</v>
+        <v>496</v>
       </c>
       <c r="B44" s="2" t="s">
         <v>172</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>415</v>
+        <v>452</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>484</v>
+        <v>497</v>
       </c>
       <c r="E44" s="3" t="s">
-        <v>485</v>
+        <v>498</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>418</v>
+        <v>455</v>
       </c>
       <c r="G44" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H44" s="2" t="s">
-        <v>419</v>
+        <v>456</v>
       </c>
       <c r="I44" s="2" t="s">
-        <v>486</v>
+        <v>499</v>
       </c>
       <c r="J44" s="2" t="s">
-        <v>487</v>
+        <v>500</v>
       </c>
       <c r="K44" s="2" t="s">
-        <v>126</v>
+        <v>76</v>
       </c>
       <c r="L44" s="2" t="s">
-        <v>488</v>
+        <v>501</v>
       </c>
       <c r="M44" s="2" t="s">
-        <v>423</v>
+        <v>460</v>
       </c>
       <c r="N44" s="2" t="s">
-        <v>489</v>
+        <v>502</v>
       </c>
       <c r="O44" s="2" t="s">
-        <v>490</v>
+        <v>503</v>
       </c>
     </row>
     <row r="45" spans="1:15">
       <c r="A45" s="2" t="s">
-        <v>491</v>
+        <v>504</v>
       </c>
       <c r="B45" s="2" t="s">
         <v>172</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>415</v>
+        <v>452</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>492</v>
+        <v>505</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>493</v>
+        <v>506</v>
       </c>
       <c r="F45" s="2" t="s">
-        <v>418</v>
+        <v>455</v>
       </c>
       <c r="G45" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H45" s="2" t="s">
-        <v>419</v>
+        <v>456</v>
       </c>
       <c r="I45" s="2" t="s">
-        <v>494</v>
+        <v>507</v>
       </c>
       <c r="J45" s="2" t="s">
-        <v>495</v>
+        <v>508</v>
       </c>
       <c r="K45" s="2" t="s">
         <v>126</v>
       </c>
       <c r="L45" s="2" t="s">
-        <v>496</v>
+        <v>509</v>
       </c>
       <c r="M45" s="2" t="s">
-        <v>423</v>
+        <v>460</v>
       </c>
       <c r="N45" s="2" t="s">
-        <v>497</v>
+        <v>510</v>
       </c>
       <c r="O45" s="2" t="s">
-        <v>498</v>
+        <v>511</v>
       </c>
     </row>
     <row r="46" spans="1:15">
       <c r="A46" s="2" t="s">
-        <v>499</v>
+        <v>512</v>
       </c>
       <c r="B46" s="2" t="s">
         <v>172</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>415</v>
+        <v>452</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>500</v>
+        <v>513</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>501</v>
+        <v>514</v>
       </c>
       <c r="F46" s="2" t="s">
-        <v>418</v>
+        <v>455</v>
       </c>
       <c r="G46" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H46" s="2" t="s">
-        <v>419</v>
+        <v>456</v>
       </c>
       <c r="I46" s="2" t="s">
-        <v>502</v>
+        <v>515</v>
       </c>
       <c r="J46" s="2" t="s">
-        <v>503</v>
+        <v>516</v>
       </c>
       <c r="K46" s="2" t="s">
         <v>76</v>
       </c>
       <c r="L46" s="2" t="s">
-        <v>504</v>
+        <v>517</v>
       </c>
       <c r="M46" s="2" t="s">
-        <v>423</v>
+        <v>460</v>
       </c>
       <c r="N46" s="2" t="s">
-        <v>505</v>
+        <v>518</v>
       </c>
       <c r="O46" s="2" t="s">
-        <v>506</v>
+        <v>519</v>
       </c>
     </row>
     <row r="47" spans="1:15">
       <c r="A47" s="2" t="s">
-        <v>507</v>
+        <v>520</v>
       </c>
       <c r="B47" s="2" t="s">
         <v>172</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>415</v>
+        <v>452</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>508</v>
+        <v>521</v>
       </c>
       <c r="E47" s="3" t="s">
-        <v>509</v>
+        <v>522</v>
       </c>
       <c r="F47" s="2" t="s">
-        <v>418</v>
+        <v>455</v>
       </c>
       <c r="G47" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H47" s="2" t="s">
-        <v>419</v>
+        <v>456</v>
       </c>
       <c r="I47" s="2" t="s">
-        <v>510</v>
+        <v>523</v>
       </c>
       <c r="J47" s="2" t="s">
-        <v>511</v>
+        <v>524</v>
       </c>
       <c r="K47" s="2" t="s">
         <v>126</v>
       </c>
       <c r="L47" s="2" t="s">
-        <v>496</v>
+        <v>525</v>
       </c>
       <c r="M47" s="2" t="s">
-        <v>423</v>
+        <v>460</v>
       </c>
       <c r="N47" s="2" t="s">
-        <v>512</v>
+        <v>526</v>
       </c>
       <c r="O47" s="2" t="s">
-        <v>513</v>
+        <v>527</v>
       </c>
     </row>
     <row r="48" spans="1:15">
       <c r="A48" s="2" t="s">
-        <v>514</v>
+        <v>528</v>
       </c>
       <c r="B48" s="2" t="s">
         <v>172</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>415</v>
+        <v>452</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>515</v>
+        <v>529</v>
       </c>
       <c r="E48" s="3" t="s">
-        <v>516</v>
+        <v>530</v>
       </c>
       <c r="F48" s="2" t="s">
-        <v>418</v>
+        <v>455</v>
       </c>
       <c r="G48" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H48" s="2" t="s">
-        <v>419</v>
+        <v>456</v>
       </c>
       <c r="I48" s="2" t="s">
-        <v>517</v>
+        <v>531</v>
       </c>
       <c r="J48" s="2" t="s">
-        <v>518</v>
+        <v>532</v>
       </c>
       <c r="K48" s="2" t="s">
         <v>126</v>
       </c>
       <c r="L48" s="2" t="s">
-        <v>519</v>
+        <v>533</v>
       </c>
       <c r="M48" s="2" t="s">
-        <v>423</v>
+        <v>460</v>
       </c>
       <c r="N48" s="2" t="s">
-        <v>520</v>
+        <v>534</v>
       </c>
       <c r="O48" s="2" t="s">
-        <v>521</v>
+        <v>535</v>
       </c>
     </row>
     <row r="49" spans="1:15">
       <c r="A49" s="2" t="s">
-        <v>522</v>
+        <v>536</v>
       </c>
       <c r="B49" s="2" t="s">
         <v>172</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>415</v>
+        <v>452</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>523</v>
+        <v>537</v>
       </c>
       <c r="E49" s="3" t="s">
-        <v>524</v>
+        <v>538</v>
       </c>
       <c r="F49" s="2" t="s">
-        <v>418</v>
+        <v>455</v>
       </c>
       <c r="G49" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H49" s="2" t="s">
-        <v>419</v>
+        <v>456</v>
       </c>
       <c r="I49" s="2" t="s">
-        <v>525</v>
+        <v>539</v>
       </c>
       <c r="J49" s="2" t="s">
-        <v>526</v>
+        <v>540</v>
       </c>
       <c r="K49" s="2" t="s">
         <v>76</v>
       </c>
       <c r="L49" s="2" t="s">
-        <v>527</v>
+        <v>541</v>
       </c>
       <c r="M49" s="2" t="s">
-        <v>423</v>
+        <v>460</v>
       </c>
       <c r="N49" s="2" t="s">
-        <v>528</v>
+        <v>542</v>
       </c>
       <c r="O49" s="2" t="s">
-        <v>529</v>
+        <v>543</v>
       </c>
     </row>
     <row r="50" spans="1:15">
       <c r="A50" s="2" t="s">
-        <v>530</v>
+        <v>544</v>
       </c>
       <c r="B50" s="2" t="s">
         <v>172</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>415</v>
+        <v>452</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>531</v>
+        <v>545</v>
       </c>
       <c r="E50" s="3" t="s">
-        <v>532</v>
+        <v>546</v>
       </c>
       <c r="F50" s="2" t="s">
-        <v>418</v>
+        <v>455</v>
       </c>
       <c r="G50" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H50" s="2" t="s">
-        <v>419</v>
+        <v>456</v>
       </c>
       <c r="I50" s="2" t="s">
-        <v>533</v>
+        <v>547</v>
       </c>
       <c r="J50" s="2" t="s">
-        <v>534</v>
+        <v>548</v>
       </c>
       <c r="K50" s="2" t="s">
         <v>126</v>
       </c>
       <c r="L50" s="2" t="s">
-        <v>496</v>
+        <v>533</v>
       </c>
       <c r="M50" s="2" t="s">
-        <v>423</v>
+        <v>460</v>
       </c>
       <c r="N50" s="2" t="s">
-        <v>535</v>
+        <v>549</v>
       </c>
       <c r="O50" s="2" t="s">
-        <v>536</v>
+        <v>550</v>
       </c>
     </row>
     <row r="51" spans="1:15">
       <c r="A51" s="2" t="s">
-        <v>537</v>
+        <v>551</v>
       </c>
       <c r="B51" s="2" t="s">
         <v>172</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>415</v>
+        <v>452</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>538</v>
+        <v>552</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>539</v>
+        <v>553</v>
       </c>
       <c r="F51" s="2" t="s">
-        <v>418</v>
+        <v>455</v>
       </c>
       <c r="G51" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H51" s="2" t="s">
-        <v>419</v>
+        <v>456</v>
       </c>
       <c r="I51" s="2" t="s">
-        <v>540</v>
+        <v>554</v>
       </c>
       <c r="J51" s="2" t="s">
-        <v>541</v>
+        <v>555</v>
       </c>
       <c r="K51" s="2" t="s">
-        <v>76</v>
+        <v>126</v>
       </c>
       <c r="L51" s="2" t="s">
-        <v>542</v>
+        <v>556</v>
       </c>
       <c r="M51" s="2" t="s">
-        <v>423</v>
+        <v>460</v>
       </c>
       <c r="N51" s="2" t="s">
-        <v>543</v>
+        <v>557</v>
       </c>
       <c r="O51" s="2" t="s">
-        <v>544</v>
+        <v>558</v>
       </c>
     </row>
     <row r="52" spans="1:15">
       <c r="A52" s="2" t="s">
-        <v>545</v>
+        <v>559</v>
       </c>
       <c r="B52" s="2" t="s">
         <v>172</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>415</v>
+        <v>452</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>546</v>
+        <v>560</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>547</v>
+        <v>561</v>
       </c>
       <c r="F52" s="2" t="s">
-        <v>418</v>
+        <v>455</v>
       </c>
       <c r="G52" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H52" s="2" t="s">
-        <v>419</v>
+        <v>456</v>
       </c>
       <c r="I52" s="2" t="s">
-        <v>548</v>
+        <v>562</v>
       </c>
       <c r="J52" s="2" t="s">
-        <v>549</v>
+        <v>563</v>
       </c>
       <c r="K52" s="2" t="s">
-        <v>126</v>
+        <v>76</v>
       </c>
       <c r="L52" s="2" t="s">
-        <v>550</v>
+        <v>564</v>
       </c>
       <c r="M52" s="2" t="s">
-        <v>423</v>
+        <v>460</v>
       </c>
       <c r="N52" s="2" t="s">
-        <v>551</v>
+        <v>565</v>
       </c>
       <c r="O52" s="2" t="s">
-        <v>552</v>
+        <v>566</v>
       </c>
     </row>
     <row r="53" spans="1:15">
       <c r="A53" s="2" t="s">
-        <v>553</v>
+        <v>567</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>117</v>
+        <v>172</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>415</v>
+        <v>452</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>554</v>
+        <v>568</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>555</v>
+        <v>569</v>
       </c>
       <c r="F53" s="2" t="s">
-        <v>418</v>
+        <v>455</v>
       </c>
       <c r="G53" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H53" s="2" t="s">
-        <v>419</v>
+        <v>456</v>
       </c>
       <c r="I53" s="2" t="s">
-        <v>556</v>
+        <v>570</v>
       </c>
       <c r="J53" s="2" t="s">
-        <v>557</v>
+        <v>571</v>
       </c>
       <c r="K53" s="2" t="s">
         <v>126</v>
       </c>
       <c r="L53" s="2" t="s">
-        <v>558</v>
+        <v>533</v>
       </c>
       <c r="M53" s="2" t="s">
-        <v>423</v>
+        <v>460</v>
       </c>
       <c r="N53" s="2" t="s">
-        <v>559</v>
+        <v>572</v>
       </c>
       <c r="O53" s="2" t="s">
-        <v>560</v>
+        <v>573</v>
       </c>
     </row>
     <row r="54" spans="1:15">
       <c r="A54" s="2" t="s">
-        <v>561</v>
+        <v>574</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>562</v>
+        <v>172</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>415</v>
+        <v>452</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>563</v>
+        <v>575</v>
       </c>
       <c r="E54" s="3" t="s">
-        <v>564</v>
+        <v>576</v>
       </c>
       <c r="F54" s="2" t="s">
-        <v>418</v>
+        <v>455</v>
       </c>
       <c r="G54" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H54" s="2" t="s">
-        <v>419</v>
+        <v>456</v>
       </c>
       <c r="I54" s="2" t="s">
-        <v>565</v>
+        <v>577</v>
       </c>
       <c r="J54" s="2" t="s">
-        <v>566</v>
+        <v>578</v>
       </c>
       <c r="K54" s="2" t="s">
         <v>76</v>
       </c>
       <c r="L54" s="2" t="s">
-        <v>567</v>
+        <v>579</v>
       </c>
       <c r="M54" s="2" t="s">
-        <v>423</v>
+        <v>460</v>
       </c>
       <c r="N54" s="2" t="s">
-        <v>568</v>
+        <v>580</v>
       </c>
       <c r="O54" s="2" t="s">
-        <v>569</v>
+        <v>581</v>
       </c>
     </row>
     <row r="55" spans="1:15">
       <c r="A55" s="2" t="s">
-        <v>570</v>
+        <v>582</v>
       </c>
       <c r="B55" s="2" t="s">
         <v>172</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>415</v>
+        <v>452</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>571</v>
+        <v>583</v>
       </c>
       <c r="E55" s="3" t="s">
-        <v>572</v>
+        <v>584</v>
       </c>
       <c r="F55" s="2" t="s">
-        <v>418</v>
+        <v>455</v>
       </c>
       <c r="G55" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H55" s="2" t="s">
-        <v>419</v>
+        <v>456</v>
       </c>
       <c r="I55" s="2" t="s">
-        <v>573</v>
+        <v>585</v>
       </c>
       <c r="J55" s="2" t="s">
-        <v>574</v>
+        <v>586</v>
       </c>
       <c r="K55" s="2" t="s">
         <v>126</v>
       </c>
       <c r="L55" s="2" t="s">
-        <v>575</v>
+        <v>587</v>
       </c>
       <c r="M55" s="2" t="s">
-        <v>423</v>
+        <v>460</v>
       </c>
       <c r="N55" s="2" t="s">
-        <v>576</v>
+        <v>588</v>
       </c>
       <c r="O55" s="2" t="s">
-        <v>577</v>
+        <v>589</v>
       </c>
     </row>
     <row r="56" spans="1:15">
       <c r="A56" s="2" t="s">
-        <v>578</v>
+        <v>590</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>172</v>
+        <v>117</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>415</v>
+        <v>452</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>579</v>
+        <v>591</v>
       </c>
       <c r="E56" s="3" t="s">
-        <v>580</v>
+        <v>592</v>
       </c>
       <c r="F56" s="2" t="s">
-        <v>445</v>
+        <v>455</v>
       </c>
       <c r="G56" s="2" t="s">
-        <v>177</v>
+        <v>21</v>
       </c>
       <c r="H56" s="2" t="s">
-        <v>419</v>
+        <v>456</v>
       </c>
       <c r="I56" s="2" t="s">
-        <v>581</v>
+        <v>593</v>
       </c>
       <c r="J56" s="2" t="s">
-        <v>582</v>
+        <v>594</v>
       </c>
       <c r="K56" s="2" t="s">
         <v>126</v>
       </c>
       <c r="L56" s="2" t="s">
-        <v>181</v>
+        <v>595</v>
       </c>
       <c r="M56" s="2" t="s">
-        <v>423</v>
+        <v>460</v>
       </c>
       <c r="N56" s="2" t="s">
-        <v>583</v>
+        <v>596</v>
       </c>
       <c r="O56" s="2" t="s">
-        <v>584</v>
+        <v>597</v>
       </c>
     </row>
     <row r="57" spans="1:15">
       <c r="A57" s="2" t="s">
-        <v>585</v>
+        <v>598</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>172</v>
+        <v>599</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>415</v>
+        <v>452</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>586</v>
+        <v>600</v>
       </c>
       <c r="E57" s="3" t="s">
-        <v>587</v>
+        <v>601</v>
       </c>
       <c r="F57" s="2" t="s">
-        <v>418</v>
+        <v>455</v>
       </c>
       <c r="G57" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H57" s="2" t="s">
-        <v>419</v>
+        <v>456</v>
       </c>
       <c r="I57" s="2" t="s">
-        <v>588</v>
+        <v>602</v>
       </c>
       <c r="J57" s="2" t="s">
-        <v>589</v>
+        <v>603</v>
       </c>
       <c r="K57" s="2" t="s">
-        <v>126</v>
+        <v>76</v>
       </c>
       <c r="L57" s="2" t="s">
-        <v>590</v>
+        <v>604</v>
       </c>
       <c r="M57" s="2" t="s">
-        <v>423</v>
+        <v>460</v>
       </c>
       <c r="N57" s="2" t="s">
-        <v>591</v>
+        <v>605</v>
       </c>
       <c r="O57" s="2" t="s">
-        <v>592</v>
+        <v>606</v>
       </c>
     </row>
     <row r="58" spans="1:15">
       <c r="A58" s="2" t="s">
-        <v>593</v>
+        <v>607</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>117</v>
+        <v>172</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>415</v>
+        <v>452</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>594</v>
+        <v>608</v>
       </c>
       <c r="E58" s="3" t="s">
-        <v>595</v>
+        <v>609</v>
       </c>
       <c r="F58" s="2" t="s">
-        <v>418</v>
+        <v>455</v>
       </c>
       <c r="G58" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H58" s="2" t="s">
-        <v>419</v>
+        <v>456</v>
       </c>
       <c r="I58" s="2" t="s">
-        <v>596</v>
+        <v>610</v>
       </c>
       <c r="J58" s="2" t="s">
-        <v>597</v>
+        <v>611</v>
       </c>
       <c r="K58" s="2" t="s">
         <v>126</v>
       </c>
       <c r="L58" s="2" t="s">
-        <v>598</v>
+        <v>612</v>
       </c>
       <c r="M58" s="2" t="s">
-        <v>423</v>
+        <v>460</v>
       </c>
       <c r="N58" s="2" t="s">
-        <v>599</v>
+        <v>613</v>
       </c>
       <c r="O58" s="2" t="s">
-        <v>600</v>
+        <v>614</v>
       </c>
     </row>
     <row r="59" spans="1:15">
       <c r="A59" s="2" t="s">
-        <v>601</v>
+        <v>615</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>562</v>
+        <v>172</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>415</v>
+        <v>452</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>602</v>
+        <v>616</v>
       </c>
       <c r="E59" s="3" t="s">
-        <v>603</v>
+        <v>617</v>
       </c>
       <c r="F59" s="2" t="s">
-        <v>418</v>
+        <v>482</v>
       </c>
       <c r="G59" s="2" t="s">
-        <v>21</v>
+        <v>177</v>
       </c>
       <c r="H59" s="2" t="s">
-        <v>419</v>
+        <v>456</v>
       </c>
       <c r="I59" s="2" t="s">
-        <v>604</v>
+        <v>618</v>
       </c>
       <c r="J59" s="2" t="s">
-        <v>605</v>
+        <v>619</v>
       </c>
       <c r="K59" s="2" t="s">
-        <v>76</v>
+        <v>126</v>
       </c>
       <c r="L59" s="2" t="s">
-        <v>606</v>
+        <v>181</v>
       </c>
       <c r="M59" s="2" t="s">
-        <v>423</v>
+        <v>460</v>
       </c>
       <c r="N59" s="2" t="s">
-        <v>607</v>
+        <v>620</v>
       </c>
       <c r="O59" s="2" t="s">
-        <v>608</v>
+        <v>621</v>
       </c>
     </row>
     <row r="60" spans="1:15">
       <c r="A60" s="2" t="s">
-        <v>609</v>
+        <v>622</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>562</v>
+        <v>172</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>415</v>
+        <v>452</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>610</v>
+        <v>623</v>
       </c>
       <c r="E60" s="3" t="s">
-        <v>611</v>
+        <v>624</v>
       </c>
       <c r="F60" s="2" t="s">
-        <v>418</v>
+        <v>455</v>
       </c>
       <c r="G60" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H60" s="2" t="s">
-        <v>419</v>
+        <v>456</v>
       </c>
       <c r="I60" s="2" t="s">
-        <v>612</v>
+        <v>625</v>
       </c>
       <c r="J60" s="2" t="s">
-        <v>613</v>
+        <v>626</v>
       </c>
       <c r="K60" s="2" t="s">
         <v>126</v>
       </c>
       <c r="L60" s="2" t="s">
-        <v>496</v>
+        <v>627</v>
       </c>
       <c r="M60" s="2" t="s">
-        <v>423</v>
+        <v>460</v>
       </c>
       <c r="N60" s="2" t="s">
-        <v>614</v>
+        <v>628</v>
       </c>
       <c r="O60" s="2" t="s">
-        <v>615</v>
+        <v>629</v>
+      </c>
+    </row>
+    <row r="61" spans="1:15">
+      <c r="A61" s="2" t="s">
+        <v>630</v>
+      </c>
+      <c r="B61" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="C61" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="D61" s="2" t="s">
+        <v>631</v>
+      </c>
+      <c r="E61" s="3" t="s">
+        <v>632</v>
+      </c>
+      <c r="F61" s="2" t="s">
+        <v>455</v>
+      </c>
+      <c r="G61" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H61" s="2" t="s">
+        <v>456</v>
+      </c>
+      <c r="I61" s="2" t="s">
+        <v>633</v>
+      </c>
+      <c r="J61" s="2" t="s">
+        <v>634</v>
+      </c>
+      <c r="K61" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="L61" s="2" t="s">
+        <v>635</v>
+      </c>
+      <c r="M61" s="2" t="s">
+        <v>460</v>
+      </c>
+      <c r="N61" s="2" t="s">
+        <v>636</v>
+      </c>
+      <c r="O61" s="2" t="s">
+        <v>637</v>
+      </c>
+    </row>
+    <row r="62" spans="1:15">
+      <c r="A62" s="2" t="s">
+        <v>638</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>599</v>
+      </c>
+      <c r="C62" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="D62" s="2" t="s">
+        <v>639</v>
+      </c>
+      <c r="E62" s="3" t="s">
+        <v>640</v>
+      </c>
+      <c r="F62" s="2" t="s">
+        <v>455</v>
+      </c>
+      <c r="G62" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H62" s="2" t="s">
+        <v>456</v>
+      </c>
+      <c r="I62" s="2" t="s">
+        <v>641</v>
+      </c>
+      <c r="J62" s="2" t="s">
+        <v>642</v>
+      </c>
+      <c r="K62" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="L62" s="2" t="s">
+        <v>643</v>
+      </c>
+      <c r="M62" s="2" t="s">
+        <v>460</v>
+      </c>
+      <c r="N62" s="2" t="s">
+        <v>644</v>
+      </c>
+      <c r="O62" s="2" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="63" spans="1:15">
+      <c r="A63" s="2" t="s">
+        <v>646</v>
+      </c>
+      <c r="B63" s="2" t="s">
+        <v>599</v>
+      </c>
+      <c r="C63" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="D63" s="2" t="s">
+        <v>647</v>
+      </c>
+      <c r="E63" s="3" t="s">
+        <v>648</v>
+      </c>
+      <c r="F63" s="2" t="s">
+        <v>455</v>
+      </c>
+      <c r="G63" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H63" s="2" t="s">
+        <v>456</v>
+      </c>
+      <c r="I63" s="2" t="s">
+        <v>649</v>
+      </c>
+      <c r="J63" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="K63" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="L63" s="2" t="s">
+        <v>533</v>
+      </c>
+      <c r="M63" s="2" t="s">
+        <v>460</v>
+      </c>
+      <c r="N63" s="2" t="s">
+        <v>651</v>
+      </c>
+      <c r="O63" s="2" t="s">
+        <v>652</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O60"/>
+  <autoFilter ref="A1:O63"/>
   <hyperlinks>
     <hyperlink ref="E2" r:id="rId1"/>
     <hyperlink ref="E3" r:id="rId2"/>
@@ -5143,6 +5395,9 @@
     <hyperlink ref="E58" r:id="rId57"/>
     <hyperlink ref="E59" r:id="rId58"/>
     <hyperlink ref="E60" r:id="rId59"/>
+    <hyperlink ref="E61" r:id="rId60"/>
+    <hyperlink ref="E62" r:id="rId61"/>
+    <hyperlink ref="E63" r:id="rId62"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Improve AfC draft and source context
</commit_message>
<xml_diff>
--- a/dossier/source_dossier.xlsx
+++ b/dossier/source_dossier.xlsx
@@ -10,14 +10,14 @@
     <sheet name="Source Dossier" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Source Dossier'!$A$1:$O$63</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Source Dossier'!$A$1:$O$68</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="945" uniqueCount="653">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1020" uniqueCount="716">
   <si>
     <t>id</t>
   </si>
@@ -109,12 +109,135 @@
     <t>{{cite report |last1=Bulger |first1=Monica |last2=McCormick |first2=Patrick |last3=Pitcan |first3=Mikaela |title=The Legacy of inBloom |publisher=Data &amp; Society Research Institute |date=February 2, 2017 |url=https://datasociety.net/pubs/ecl/InBloom_feb_2017.pdf |access-date=June 8, 2026}}</t>
   </si>
   <si>
+    <t>SXSW1</t>
+  </si>
+  <si>
+    <t>2020</t>
+  </si>
+  <si>
+    <t>SXSW EDU</t>
+  </si>
+  <si>
+    <t>10 Things You Probably Don't Know About SXSW EDU</t>
+  </si>
+  <si>
+    <t>https://sxswedu.com/news/2020/10-things-you-probably-dont-know-about-sxsw-edu/</t>
+  </si>
+  <si>
+    <t>Event retrospective / organizational article</t>
+  </si>
+  <si>
+    <t>Partial; official event source</t>
+  </si>
+  <si>
+    <t>Medium for SXSW EDU launch-context facts; does not name Alderson</t>
+  </si>
+  <si>
+    <t>Minor for Alderson; useful for inBloom context. SXSW EDU founder Ron Reed says the Shared Learning Collaborative was rebranded to launch InBloom at SXSW EDU in 2013, calling it one of the first and most elaborate education initiatives launched at SXSW EDU and noting that discussion shifted toward student-data security and privacy.</t>
+  </si>
+  <si>
+    <t>InBloom launched at SXSW EDU in 2013 through the rebranding of the Shared Learning Collaborative; the launch prompted discussion of student-data security and privacy. Does not verify Alderson's speaker role.</t>
+  </si>
+  <si>
+    <t>Low for Alderson; Medium for inBloom context</t>
+  </si>
+  <si>
+    <t>Use only as context for inBloom's SXSW EDU launch and privacy/security discussion; pair Alderson-specific inBloom role claims with Data &amp; Society.</t>
+  </si>
+  <si>
+    <t>Verified from downloaded HTML and extracted text</t>
+  </si>
+  <si>
+    <t>Reviewed in sources/data_society_inbloom_sources.md; local files data/sxswedu_10_things_2020_inbloom.html and data/sxswedu_10_things_2020_inbloom.txt</t>
+  </si>
+  <si>
+    <t>{{cite web |last=Reed |first=Ron |title=10 Things You Probably Don't Know About SXSW EDU |url=https://sxswedu.com/news/2020/10-things-you-probably-dont-know-about-sxsw-edu/ |website=SXSW EDU |date=January 28, 2020 |access-date=June 8, 2026}}</t>
+  </si>
+  <si>
+    <t>ESN1</t>
+  </si>
+  <si>
+    <t>2013</t>
+  </si>
+  <si>
+    <t>eSchool News / Reuters</t>
+  </si>
+  <si>
+    <t>K-12 student database jazzes tech startups, spooks parents</t>
+  </si>
+  <si>
+    <t>https://www.eschoolnews.com/district-management/2013/03/04/k-12-student-database-jazzes-tech-startups-spooks-parents/</t>
+  </si>
+  <si>
+    <t>Reuters-syndicated news article</t>
+  </si>
+  <si>
+    <t>Yes for Reuters reporting; syndicated page</t>
+  </si>
+  <si>
+    <t>Medium to High for inBloom launch/privacy context; does not name Alderson</t>
+  </si>
+  <si>
+    <t>Context only. eSchool News reprint says Reuters reported an Austin education-technology conference where startups would show products and highlights a $100 million K-12 student database holding files on millions of children. It describes privacy objections from parents and civil-liberties groups. Direct Reuters URL was blocked locally by a JS/ad-blocker page.</t>
+  </si>
+  <si>
+    <t>Contemporary news coverage of the inBloom/student-data controversy around an Austin education-technology conference; supports broader significance and privacy concerns, not Alderson-specific facts.</t>
+  </si>
+  <si>
+    <t>Use only as inBloom context if needed; do not cite for Alderson-specific facts.</t>
+  </si>
+  <si>
+    <t>Verified from downloaded syndicated HTML and extracted text; direct Reuters page locally blocked</t>
+  </si>
+  <si>
+    <t>Reviewed in sources/data_society_inbloom_sources.md; local files data/eschoolnews_reuters_2013_inbloom_database.html and data/eschoolnews_reuters_2013_inbloom_database.txt; blocked direct file data/reuters_2013_inbloom_database_sxswedu.html</t>
+  </si>
+  <si>
+    <t>{{cite web |title=K-12 student database jazzes tech startups, spooks parents |url=https://www.eschoolnews.com/district-management/2013/03/04/k-12-student-database-jazzes-tech-startups-spooks-parents/ |website=eSchool News |date=March 4, 2013 |access-date=June 8, 2026}}</t>
+  </si>
+  <si>
+    <t>EW1</t>
+  </si>
+  <si>
+    <t>2014</t>
+  </si>
+  <si>
+    <t>Education Week</t>
+  </si>
+  <si>
+    <t>InBloom Sputters Amid Concerns About Privacy of Student Data</t>
+  </si>
+  <si>
+    <t>https://www.edweek.org/technology/inbloom-sputters-amid-concerns-about-privacy-of-student-data/2014/01</t>
+  </si>
+  <si>
+    <t>Education journalism</t>
+  </si>
+  <si>
+    <t>High for education-policy reporting; does not name Alderson</t>
+  </si>
+  <si>
+    <t>Context only. Article says inBloom emerged backed by $100 million in Gates Foundation and Carnegie Corporation grants, formed partnerships with nine states serving more than 11 million students, and then lost support as privacy and third-party vendor concerns grew.</t>
+  </si>
+  <si>
+    <t>Independent education-journalism context for inBloom's scale, controversy, privacy concerns, and state/district withdrawals; not Alderson-specific.</t>
+  </si>
+  <si>
+    <t>Low for Alderson; Medium to High for inBloom context</t>
+  </si>
+  <si>
+    <t>Use as inBloom context if needed; pair Alderson-specific role claims with Data &amp; Society.</t>
+  </si>
+  <si>
+    <t>Reviewed in sources/data_society_inbloom_sources.md; local files data/edweek_2014_inbloom_sputters_privacy.html and data/edweek_2014_inbloom_sputters_privacy.txt</t>
+  </si>
+  <si>
+    <t>{{cite web |last=Kamisar |first=Ben |title=InBloom Sputters Amid Concerns About Privacy of Student Data |url=https://www.edweek.org/technology/inbloom-sputters-amid-concerns-about-privacy-of-student-data/2014/01 |website=Education Week |date=January 7, 2014 |access-date=June 8, 2026}}</t>
+  </si>
+  <si>
     <t>GF1</t>
   </si>
   <si>
-    <t>2013</t>
-  </si>
-  <si>
     <t>Gates Foundation</t>
   </si>
   <si>
@@ -259,6 +382,81 @@
     <t>{{cite web |last=Raths |first=David |title=Laying the Groundwork for Big Data |url=https://campustechnology.com/articles/2016/02/25/laying-the-groundwork-for-big-data.aspx?Page=3&amp;p=1 |website=Campus Technology |date=February 25, 2016 |access-date=June 8, 2026}}</t>
   </si>
   <si>
+    <t>PF1</t>
+  </si>
+  <si>
+    <t>ProctorFree</t>
+  </si>
+  <si>
+    <t>Ensure Student Success with ProctorFree at Eduventures Summit 2016</t>
+  </si>
+  <si>
+    <t>https://www.proctorfree.com/news/rethink-student-lifecycle-online-proctoring-eduventures-summit-2016</t>
+  </si>
+  <si>
+    <t>Vendor blog post / event coverage</t>
+  </si>
+  <si>
+    <t>Partial; third-party vendor with promotional interest</t>
+  </si>
+  <si>
+    <t>Medium for event and quote facts; limited for notability</t>
+  </si>
+  <si>
+    <t>Minor to moderate. ProctorFree says Alderson, Principal Analyst at Eduventures, would give the keynote presentation `Technology that Should be on Every Higher Education Leader's Radar` at Eduventures Summit 2016 on October 24, 2016, and references Alderson's recent comments about ProctorFree's auditing of automated exam sessions.</t>
+  </si>
+  <si>
+    <t>Alderson was listed as a keynote presenter at Eduventures Summit 2016 and was identified as Principal Analyst at Eduventures; the post also corroborates his public commentary on online proctoring.</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>Use only for Eduventures Summit / online-proctoring professional context; not a notability anchor because the source is a vendor promotional blog.</t>
+  </si>
+  <si>
+    <t>Reviewed in sources/encoura_eduventures_sources.md; local files data/proctorfree_eduventures_summit_2016.html and data/proctorfree_eduventures_summit_2016.txt</t>
+  </si>
+  <si>
+    <t>{{cite web |title=Ensure Student Success with ProctorFree at Eduventures Summit 2016 |url=https://www.proctorfree.com/news/rethink-student-lifecycle-online-proctoring-eduventures-summit-2016 |website=ProctorFree |date=October 21, 2016 |access-date=June 8, 2026}}</t>
+  </si>
+  <si>
+    <t>SS1</t>
+  </si>
+  <si>
+    <t>SlideShare / Eduventures</t>
+  </si>
+  <si>
+    <t>EduVentures: Tapping the Social Funnel for Development_June 2016_Simmons College</t>
+  </si>
+  <si>
+    <t>https://www.slideshare.net/slideshow/eduventures-tapping-the-social-funnel-for-developmentjune-2016simmons-college/63257710</t>
+  </si>
+  <si>
+    <t>Slide deck / platform-hosted presentation</t>
+  </si>
+  <si>
+    <t>No or partial; platform-hosted and likely self/affiliated</t>
+  </si>
+  <si>
+    <t>Medium for deck text and presentation metadata; weak for notability</t>
+  </si>
+  <si>
+    <t>Minor to moderate for professional-context facts. SlideShare metadata identifies a 27-slide deck uploaded by `JeffTe`, created June 20 2016 UTC, with an AI-enhanced description naming Jeffrey Alderson. Extracted slide text names `Jeffrey Alderson | Principal Analyst, Eduventures` and `Principal Analyst, Enterprise Software`; the title identifies June 2016 Simmons College.</t>
+  </si>
+  <si>
+    <t>Alderson presented or authored an Eduventures deck titled `Tapping the Social Funnel for Development` for a June 2016 Simmons College event; the deck identifies him as Principal Analyst / Principal Analyst, Enterprise Software at Eduventures and includes a short professional bio.</t>
+  </si>
+  <si>
+    <t>Use only for narrow presentation/publication-history and professional-context facts; not a notability anchor because the deck is platform-hosted and likely self/affiliated.</t>
+  </si>
+  <si>
+    <t>Reviewed in sources/encoura_eduventures_sources.md; local files data/slideshare_eduventures_social_funnel_simmons_2016.html and data/slideshare_eduventures_social_funnel_simmons_2016.txt</t>
+  </si>
+  <si>
+    <t>{{cite web |last=Alderson |first=Jeffrey |title=EduVentures: Tapping the Social Funnel for Development_June 2016_Simmons College |url=https://www.slideshare.net/slideshow/eduventures-tapping-the-social-funnel-for-developmentjune-2016simmons-college/63257710 |website=SlideShare |date=June 20, 2016 |access-date=June 8, 2026}}</t>
+  </si>
+  <si>
     <t>MOL1</t>
   </si>
   <si>
@@ -397,9 +595,6 @@
     <t>Recorded IN4OBE webinar title and publisher; supporting trail for Alderson's speaker role when paired with IN4OBE/LinkedIn metadata.</t>
   </si>
   <si>
-    <t>Low</t>
-  </si>
-  <si>
     <t>Use only as supporting evidence for the recorded webinar, paired with clearer event metadata.</t>
   </si>
   <si>
@@ -958,9 +1153,6 @@
     <t>Use only as MyDataButton/HMH context; pair Alderson-specific claims with PESC2012/ERUG1 and HMH role claims with Data &amp; Society or another HMH-specific source.</t>
   </si>
   <si>
-    <t>Verified from downloaded HTML and extracted text</t>
-  </si>
-  <si>
     <t>Reviewed in sources/mydata_button_sources.md; local files data/hack_education_mydata_button_2012.html and data/hack_education_mydata_button_2012.txt</t>
   </si>
   <si>
@@ -1007,9 +1199,6 @@
   </si>
   <si>
     <t>CB1</t>
-  </si>
-  <si>
-    <t>2014</t>
   </si>
   <si>
     <t>PACERMonitor / U.S. Bankruptcy Court filing copy</t>
@@ -2353,7 +2542,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O63"/>
+  <dimension ref="A1:O68"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -2545,13 +2734,13 @@
         <v>54</v>
       </c>
       <c r="K4" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="L4" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="L4" s="2" t="s">
+      <c r="M4" s="2" t="s">
         <v>56</v>
-      </c>
-      <c r="M4" s="2" t="s">
-        <v>42</v>
       </c>
       <c r="N4" s="2" t="s">
         <v>57</v>
@@ -2583,351 +2772,351 @@
         <v>21</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>25</v>
+        <v>65</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="M5" s="2" t="s">
         <v>42</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="O5" s="2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="6" spans="1:15">
       <c r="A6" s="2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>61</v>
+        <v>73</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>64</v>
+        <v>76</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>21</v>
+        <v>77</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>25</v>
+        <v>78</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>42</v>
+        <v>83</v>
       </c>
       <c r="N6" s="2" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="O6" s="2" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
     </row>
     <row r="7" spans="1:15">
       <c r="A7" s="2" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="D7" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="K7" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="L7" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="M7" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="E7" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="H7" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="I7" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="J7" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="K7" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="L7" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="M7" s="2" t="s">
-        <v>42</v>
-      </c>
       <c r="N7" s="2" t="s">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="O7" s="2" t="s">
-        <v>91</v>
+        <v>99</v>
       </c>
     </row>
     <row r="8" spans="1:15">
       <c r="A8" s="2" t="s">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>93</v>
+        <v>101</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>95</v>
+        <v>103</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>96</v>
+        <v>104</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>51</v>
+        <v>21</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>98</v>
+        <v>25</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>100</v>
+        <v>107</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>76</v>
+        <v>108</v>
       </c>
       <c r="L8" s="2" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>42</v>
+        <v>83</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="O8" s="2" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
     </row>
     <row r="9" spans="1:15">
       <c r="A9" s="2" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="B9" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="F9" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="C9" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>108</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>109</v>
-      </c>
       <c r="G9" s="2" t="s">
-        <v>51</v>
+        <v>21</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>110</v>
+        <v>25</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>76</v>
+        <v>117</v>
       </c>
       <c r="L9" s="2" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>42</v>
+        <v>83</v>
       </c>
       <c r="N9" s="2" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="O9" s="2" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
     </row>
     <row r="10" spans="1:15">
       <c r="A10" s="2" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>117</v>
+        <v>101</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="L10" s="2" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>128</v>
+        <v>42</v>
       </c>
       <c r="N10" s="2" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="O10" s="2" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
     </row>
     <row r="11" spans="1:15">
       <c r="A11" s="2" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>132</v>
+        <v>101</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>55</v>
+        <v>130</v>
       </c>
       <c r="L11" s="2" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="M11" s="2" t="s">
-        <v>142</v>
+        <v>42</v>
       </c>
       <c r="N11" s="2" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="O11" s="2" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="12" spans="1:15">
       <c r="A12" s="2" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>132</v>
+        <v>147</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>150</v>
+        <v>92</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>55</v>
+        <v>117</v>
       </c>
       <c r="L12" s="2" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="M12" s="2" t="s">
-        <v>155</v>
+        <v>83</v>
       </c>
       <c r="N12" s="2" t="s">
         <v>156</v>
@@ -2941,22 +3130,22 @@
         <v>158</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>132</v>
+        <v>159</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>163</v>
+        <v>92</v>
       </c>
       <c r="H13" s="2" t="s">
         <v>164</v>
@@ -2968,89 +3157,89 @@
         <v>166</v>
       </c>
       <c r="K13" s="2" t="s">
-        <v>40</v>
+        <v>117</v>
       </c>
       <c r="L13" s="2" t="s">
         <v>167</v>
       </c>
       <c r="M13" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="N13" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="N13" s="2" t="s">
+      <c r="O13" s="2" t="s">
         <v>169</v>
-      </c>
-      <c r="O13" s="2" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="14" spans="1:15">
       <c r="A14" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="B14" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="C14" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="D14" s="2" t="s">
         <v>173</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="E14" s="3" t="s">
         <v>174</v>
       </c>
-      <c r="E14" s="3" t="s">
+      <c r="F14" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="F14" s="2" t="s">
+      <c r="G14" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="H14" s="2" t="s">
         <v>176</v>
       </c>
-      <c r="G14" s="2" t="s">
+      <c r="I14" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="H14" s="2" t="s">
+      <c r="J14" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="I14" s="2" t="s">
+      <c r="K14" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="L14" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="J14" s="2" t="s">
+      <c r="M14" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="N14" s="2" t="s">
         <v>180</v>
       </c>
-      <c r="K14" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="L14" s="2" t="s">
+      <c r="O14" s="2" t="s">
         <v>181</v>
-      </c>
-      <c r="M14" s="2" t="s">
-        <v>182</v>
-      </c>
-      <c r="N14" s="2" t="s">
-        <v>183</v>
-      </c>
-      <c r="O14" s="2" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="15" spans="1:15">
       <c r="A15" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="D15" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="B15" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="D15" s="2" t="s">
+      <c r="E15" s="3" t="s">
         <v>186</v>
       </c>
-      <c r="E15" s="3" t="s">
+      <c r="F15" s="2" t="s">
         <v>187</v>
       </c>
-      <c r="F15" s="2" t="s">
+      <c r="G15" s="2" t="s">
         <v>188</v>
-      </c>
-      <c r="G15" s="2" t="s">
-        <v>21</v>
       </c>
       <c r="H15" s="2" t="s">
         <v>189</v>
@@ -3062,7 +3251,7 @@
         <v>191</v>
       </c>
       <c r="K15" s="2" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="L15" s="2" t="s">
         <v>192</v>
@@ -3082,657 +3271,657 @@
         <v>196</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>172</v>
+        <v>197</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>173</v>
+        <v>198</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>188</v>
+        <v>201</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>21</v>
+        <v>202</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>189</v>
+        <v>203</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>199</v>
+        <v>204</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>76</v>
+        <v>96</v>
       </c>
       <c r="L16" s="2" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
       <c r="M16" s="2" t="s">
-        <v>193</v>
+        <v>207</v>
       </c>
       <c r="N16" s="2" t="s">
-        <v>202</v>
+        <v>208</v>
       </c>
       <c r="O16" s="2" t="s">
-        <v>203</v>
+        <v>209</v>
       </c>
     </row>
     <row r="17" spans="1:15">
       <c r="A17" s="2" t="s">
-        <v>204</v>
+        <v>210</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>46</v>
+        <v>197</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>205</v>
+        <v>211</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>207</v>
+        <v>213</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>51</v>
+        <v>215</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>209</v>
+        <v>216</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>210</v>
+        <v>217</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>211</v>
+        <v>218</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>76</v>
+        <v>96</v>
       </c>
       <c r="L17" s="2" t="s">
-        <v>212</v>
+        <v>219</v>
       </c>
       <c r="M17" s="2" t="s">
-        <v>42</v>
+        <v>220</v>
       </c>
       <c r="N17" s="2" t="s">
-        <v>213</v>
+        <v>221</v>
       </c>
       <c r="O17" s="2" t="s">
-        <v>214</v>
+        <v>222</v>
       </c>
     </row>
     <row r="18" spans="1:15">
       <c r="A18" s="2" t="s">
-        <v>215</v>
+        <v>223</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>216</v>
+        <v>197</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>217</v>
+        <v>224</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>218</v>
+        <v>225</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>219</v>
+        <v>226</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>220</v>
+        <v>227</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>221</v>
+        <v>228</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>222</v>
+        <v>229</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>223</v>
+        <v>230</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>224</v>
+        <v>231</v>
       </c>
       <c r="K18" s="2" t="s">
-        <v>126</v>
+        <v>81</v>
       </c>
       <c r="L18" s="2" t="s">
-        <v>225</v>
+        <v>232</v>
       </c>
       <c r="M18" s="2" t="s">
-        <v>42</v>
+        <v>233</v>
       </c>
       <c r="N18" s="2" t="s">
-        <v>226</v>
+        <v>234</v>
       </c>
       <c r="O18" s="2" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
     </row>
     <row r="19" spans="1:15">
       <c r="A19" s="2" t="s">
-        <v>228</v>
+        <v>236</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>229</v>
+        <v>237</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>230</v>
+        <v>238</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>231</v>
+        <v>239</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>232</v>
+        <v>240</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>233</v>
+        <v>241</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>221</v>
+        <v>242</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>234</v>
+        <v>243</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>235</v>
+        <v>244</v>
       </c>
       <c r="J19" s="2" t="s">
-        <v>236</v>
+        <v>245</v>
       </c>
       <c r="K19" s="2" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="L19" s="2" t="s">
-        <v>237</v>
+        <v>246</v>
       </c>
       <c r="M19" s="2" t="s">
-        <v>238</v>
+        <v>247</v>
       </c>
       <c r="N19" s="2" t="s">
-        <v>239</v>
+        <v>248</v>
       </c>
       <c r="O19" s="2" t="s">
-        <v>240</v>
+        <v>249</v>
       </c>
     </row>
     <row r="20" spans="1:15">
       <c r="A20" s="2" t="s">
-        <v>241</v>
+        <v>250</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>229</v>
+        <v>237</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>217</v>
+        <v>238</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>242</v>
+        <v>251</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>243</v>
+        <v>252</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>244</v>
+        <v>253</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>221</v>
+        <v>21</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>245</v>
+        <v>254</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>246</v>
+        <v>255</v>
       </c>
       <c r="J20" s="2" t="s">
-        <v>247</v>
+        <v>256</v>
       </c>
       <c r="K20" s="2" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="L20" s="2" t="s">
-        <v>248</v>
+        <v>257</v>
       </c>
       <c r="M20" s="2" t="s">
-        <v>238</v>
+        <v>258</v>
       </c>
       <c r="N20" s="2" t="s">
-        <v>249</v>
+        <v>259</v>
       </c>
       <c r="O20" s="2" t="s">
-        <v>250</v>
+        <v>260</v>
       </c>
     </row>
     <row r="21" spans="1:15">
       <c r="A21" s="2" t="s">
-        <v>251</v>
+        <v>261</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>229</v>
+        <v>237</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>252</v>
+        <v>238</v>
       </c>
       <c r="D21" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="F21" s="2" t="s">
         <v>253</v>
       </c>
-      <c r="E21" s="3" t="s">
+      <c r="G21" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H21" s="2" t="s">
         <v>254</v>
       </c>
-      <c r="F21" s="2" t="s">
-        <v>255</v>
-      </c>
-      <c r="G21" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="H21" s="2" t="s">
-        <v>256</v>
-      </c>
       <c r="I21" s="2" t="s">
-        <v>257</v>
+        <v>264</v>
       </c>
       <c r="J21" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="K21" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="L21" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="M21" s="2" t="s">
         <v>258</v>
       </c>
-      <c r="K21" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="L21" s="2" t="s">
-        <v>259</v>
-      </c>
-      <c r="M21" s="2" t="s">
-        <v>238</v>
-      </c>
       <c r="N21" s="2" t="s">
-        <v>260</v>
+        <v>267</v>
       </c>
       <c r="O21" s="2" t="s">
-        <v>261</v>
+        <v>268</v>
       </c>
     </row>
     <row r="22" spans="1:15">
       <c r="A22" s="2" t="s">
-        <v>262</v>
+        <v>269</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>263</v>
+        <v>87</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>217</v>
+        <v>270</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>264</v>
+        <v>271</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>265</v>
+        <v>272</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>244</v>
+        <v>273</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>221</v>
+        <v>92</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>245</v>
+        <v>274</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>266</v>
+        <v>275</v>
       </c>
       <c r="J22" s="2" t="s">
-        <v>267</v>
+        <v>276</v>
       </c>
       <c r="K22" s="2" t="s">
-        <v>76</v>
+        <v>117</v>
       </c>
       <c r="L22" s="2" t="s">
-        <v>268</v>
+        <v>277</v>
       </c>
       <c r="M22" s="2" t="s">
-        <v>238</v>
+        <v>83</v>
       </c>
       <c r="N22" s="2" t="s">
-        <v>269</v>
+        <v>278</v>
       </c>
       <c r="O22" s="2" t="s">
-        <v>270</v>
+        <v>279</v>
       </c>
     </row>
     <row r="23" spans="1:15">
       <c r="A23" s="2" t="s">
-        <v>271</v>
+        <v>280</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>263</v>
+        <v>281</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>272</v>
+        <v>282</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>273</v>
+        <v>283</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>274</v>
+        <v>284</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>275</v>
+        <v>285</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>221</v>
+        <v>286</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>276</v>
+        <v>287</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>277</v>
+        <v>288</v>
       </c>
       <c r="J23" s="2" t="s">
-        <v>278</v>
+        <v>289</v>
       </c>
       <c r="K23" s="2" t="s">
-        <v>76</v>
+        <v>130</v>
       </c>
       <c r="L23" s="2" t="s">
-        <v>279</v>
+        <v>290</v>
       </c>
       <c r="M23" s="2" t="s">
-        <v>238</v>
+        <v>83</v>
       </c>
       <c r="N23" s="2" t="s">
-        <v>280</v>
+        <v>291</v>
       </c>
       <c r="O23" s="2" t="s">
-        <v>281</v>
+        <v>292</v>
       </c>
     </row>
     <row r="24" spans="1:15">
       <c r="A24" s="2" t="s">
-        <v>282</v>
+        <v>293</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>60</v>
+        <v>294</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>217</v>
+        <v>295</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>283</v>
+        <v>296</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>284</v>
+        <v>297</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>244</v>
+        <v>298</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>221</v>
+        <v>286</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>285</v>
+        <v>299</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>286</v>
+        <v>300</v>
       </c>
       <c r="J24" s="2" t="s">
-        <v>287</v>
+        <v>301</v>
       </c>
       <c r="K24" s="2" t="s">
-        <v>76</v>
+        <v>130</v>
       </c>
       <c r="L24" s="2" t="s">
-        <v>288</v>
+        <v>302</v>
       </c>
       <c r="M24" s="2" t="s">
-        <v>238</v>
+        <v>303</v>
       </c>
       <c r="N24" s="2" t="s">
-        <v>289</v>
+        <v>304</v>
       </c>
       <c r="O24" s="2" t="s">
-        <v>290</v>
+        <v>305</v>
       </c>
     </row>
     <row r="25" spans="1:15">
       <c r="A25" s="2" t="s">
-        <v>291</v>
+        <v>306</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>217</v>
+        <v>282</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>293</v>
+        <v>307</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>294</v>
+        <v>308</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>295</v>
+        <v>309</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>221</v>
+        <v>286</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>296</v>
+        <v>310</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>297</v>
+        <v>311</v>
       </c>
       <c r="J25" s="2" t="s">
-        <v>298</v>
+        <v>312</v>
       </c>
       <c r="K25" s="2" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="L25" s="2" t="s">
-        <v>299</v>
+        <v>313</v>
       </c>
       <c r="M25" s="2" t="s">
-        <v>238</v>
+        <v>303</v>
       </c>
       <c r="N25" s="2" t="s">
-        <v>300</v>
+        <v>314</v>
       </c>
       <c r="O25" s="2" t="s">
-        <v>301</v>
+        <v>315</v>
       </c>
     </row>
     <row r="26" spans="1:15">
       <c r="A26" s="2" t="s">
-        <v>302</v>
+        <v>316</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>263</v>
+        <v>294</v>
       </c>
       <c r="C26" s="2" t="s">
+        <v>317</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="E26" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="H26" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="I26" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="J26" s="2" t="s">
+        <v>323</v>
+      </c>
+      <c r="K26" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="L26" s="2" t="s">
+        <v>324</v>
+      </c>
+      <c r="M26" s="2" t="s">
         <v>303</v>
       </c>
-      <c r="D26" s="2" t="s">
-        <v>304</v>
-      </c>
-      <c r="E26" s="3" t="s">
-        <v>305</v>
-      </c>
-      <c r="F26" s="2" t="s">
-        <v>306</v>
-      </c>
-      <c r="G26" s="2" t="s">
-        <v>307</v>
-      </c>
-      <c r="H26" s="2" t="s">
-        <v>308</v>
-      </c>
-      <c r="I26" s="2" t="s">
-        <v>309</v>
-      </c>
-      <c r="J26" s="2" t="s">
-        <v>310</v>
-      </c>
-      <c r="K26" s="2" t="s">
-        <v>311</v>
-      </c>
-      <c r="L26" s="2" t="s">
-        <v>312</v>
-      </c>
-      <c r="M26" s="2" t="s">
-        <v>313</v>
-      </c>
       <c r="N26" s="2" t="s">
-        <v>314</v>
+        <v>325</v>
       </c>
       <c r="O26" s="2" t="s">
-        <v>315</v>
+        <v>326</v>
       </c>
     </row>
     <row r="27" spans="1:15">
       <c r="A27" s="2" t="s">
-        <v>316</v>
+        <v>327</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>60</v>
+        <v>328</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>317</v>
+        <v>282</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>318</v>
+        <v>329</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>319</v>
+        <v>330</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>320</v>
+        <v>309</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>321</v>
+        <v>286</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>322</v>
+        <v>310</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>323</v>
+        <v>331</v>
       </c>
       <c r="J27" s="2" t="s">
-        <v>324</v>
+        <v>332</v>
       </c>
       <c r="K27" s="2" t="s">
-        <v>325</v>
+        <v>117</v>
       </c>
       <c r="L27" s="2" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
       <c r="M27" s="2" t="s">
-        <v>238</v>
+        <v>303</v>
       </c>
       <c r="N27" s="2" t="s">
-        <v>327</v>
+        <v>334</v>
       </c>
       <c r="O27" s="2" t="s">
-        <v>328</v>
+        <v>335</v>
       </c>
     </row>
     <row r="28" spans="1:15">
       <c r="A28" s="2" t="s">
-        <v>329</v>
+        <v>336</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>331</v>
+        <v>337</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>332</v>
+        <v>338</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>333</v>
+        <v>339</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>334</v>
+        <v>340</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>36</v>
+        <v>286</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>335</v>
+        <v>341</v>
       </c>
       <c r="I28" s="2" t="s">
-        <v>336</v>
+        <v>342</v>
       </c>
       <c r="J28" s="2" t="s">
-        <v>337</v>
+        <v>343</v>
       </c>
       <c r="K28" s="2" t="s">
-        <v>40</v>
+        <v>117</v>
       </c>
       <c r="L28" s="2" t="s">
-        <v>338</v>
+        <v>344</v>
       </c>
       <c r="M28" s="2" t="s">
-        <v>339</v>
+        <v>303</v>
       </c>
       <c r="N28" s="2" t="s">
-        <v>340</v>
+        <v>345</v>
       </c>
       <c r="O28" s="2" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
     </row>
     <row r="29" spans="1:15">
       <c r="A29" s="2" t="s">
-        <v>342</v>
+        <v>347</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>343</v>
+        <v>101</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>344</v>
+        <v>282</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>347</v>
+        <v>309</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>348</v>
+        <v>286</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="I29" s="2" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="J29" s="2" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="K29" s="2" t="s">
-        <v>352</v>
+        <v>117</v>
       </c>
       <c r="L29" s="2" t="s">
         <v>353</v>
       </c>
       <c r="M29" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="N29" s="2" t="s">
         <v>354</v>
       </c>
-      <c r="N29" s="2" t="s">
+      <c r="O29" s="2" t="s">
         <v>355</v>
-      </c>
-      <c r="O29" s="2" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="30" spans="1:15">
@@ -3743,1598 +3932,1833 @@
         <v>357</v>
       </c>
       <c r="C30" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="D30" s="2" t="s">
         <v>358</v>
       </c>
-      <c r="D30" s="2" t="s">
+      <c r="E30" s="3" t="s">
         <v>359</v>
       </c>
-      <c r="E30" s="3" t="s">
+      <c r="F30" s="2" t="s">
         <v>360</v>
       </c>
-      <c r="F30" s="2" t="s">
+      <c r="G30" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="H30" s="2" t="s">
         <v>361</v>
       </c>
-      <c r="G30" s="2" t="s">
+      <c r="I30" s="2" t="s">
         <v>362</v>
       </c>
-      <c r="H30" s="2" t="s">
+      <c r="J30" s="2" t="s">
         <v>363</v>
       </c>
-      <c r="I30" s="2" t="s">
+      <c r="K30" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="L30" s="2" t="s">
         <v>364</v>
       </c>
-      <c r="J30" s="2" t="s">
+      <c r="M30" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="N30" s="2" t="s">
         <v>365</v>
       </c>
-      <c r="K30" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="L30" s="2" t="s">
+      <c r="O30" s="2" t="s">
         <v>366</v>
-      </c>
-      <c r="M30" s="2" t="s">
-        <v>367</v>
-      </c>
-      <c r="N30" s="2" t="s">
-        <v>368</v>
-      </c>
-      <c r="O30" s="2" t="s">
-        <v>369</v>
       </c>
     </row>
     <row r="31" spans="1:15">
       <c r="A31" s="2" t="s">
+        <v>367</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>368</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>369</v>
+      </c>
+      <c r="E31" s="3" t="s">
         <v>370</v>
       </c>
-      <c r="B31" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C31" s="2" t="s">
+      <c r="F31" s="2" t="s">
         <v>371</v>
       </c>
-      <c r="D31" s="2" t="s">
+      <c r="G31" s="2" t="s">
         <v>372</v>
       </c>
-      <c r="E31" s="3" t="s">
+      <c r="H31" s="2" t="s">
         <v>373</v>
       </c>
-      <c r="F31" s="2" t="s">
+      <c r="I31" s="2" t="s">
         <v>374</v>
       </c>
-      <c r="G31" s="2" t="s">
-        <v>362</v>
-      </c>
-      <c r="H31" s="2" t="s">
+      <c r="J31" s="2" t="s">
         <v>375</v>
       </c>
-      <c r="I31" s="2" t="s">
+      <c r="K31" s="2" t="s">
         <v>376</v>
       </c>
-      <c r="J31" s="2" t="s">
+      <c r="L31" s="2" t="s">
         <v>377</v>
       </c>
-      <c r="K31" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="L31" s="2" t="s">
+      <c r="M31" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="N31" s="2" t="s">
         <v>378</v>
       </c>
-      <c r="M31" s="2" t="s">
+      <c r="O31" s="2" t="s">
         <v>379</v>
-      </c>
-      <c r="N31" s="2" t="s">
-        <v>380</v>
-      </c>
-      <c r="O31" s="2" t="s">
-        <v>369</v>
       </c>
     </row>
     <row r="32" spans="1:15">
       <c r="A32" s="2" t="s">
+        <v>380</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="C32" s="2" t="s">
         <v>381</v>
       </c>
-      <c r="B32" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C32" s="2" t="s">
+      <c r="D32" s="2" t="s">
         <v>382</v>
       </c>
-      <c r="D32" s="2" t="s">
+      <c r="E32" s="3" t="s">
         <v>383</v>
       </c>
-      <c r="E32" s="3" t="s">
+      <c r="F32" s="2" t="s">
         <v>384</v>
       </c>
-      <c r="F32" s="2" t="s">
-        <v>188</v>
-      </c>
       <c r="G32" s="2" t="s">
-        <v>21</v>
+        <v>385</v>
       </c>
       <c r="H32" s="2" t="s">
-        <v>189</v>
+        <v>386</v>
       </c>
       <c r="I32" s="2" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="J32" s="2" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="K32" s="2" t="s">
-        <v>126</v>
+        <v>389</v>
       </c>
       <c r="L32" s="2" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="M32" s="2" t="s">
-        <v>42</v>
+        <v>303</v>
       </c>
       <c r="N32" s="2" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
       <c r="O32" s="2" t="s">
-        <v>389</v>
+        <v>392</v>
       </c>
     </row>
     <row r="33" spans="1:15">
       <c r="A33" s="2" t="s">
-        <v>390</v>
+        <v>393</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>16</v>
+        <v>60</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>393</v>
+        <v>396</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>176</v>
+        <v>397</v>
       </c>
       <c r="G33" s="2" t="s">
-        <v>177</v>
+        <v>77</v>
       </c>
       <c r="H33" s="2" t="s">
-        <v>178</v>
+        <v>398</v>
       </c>
       <c r="I33" s="2" t="s">
-        <v>394</v>
+        <v>399</v>
       </c>
       <c r="J33" s="2" t="s">
-        <v>395</v>
+        <v>400</v>
       </c>
       <c r="K33" s="2" t="s">
-        <v>126</v>
+        <v>81</v>
       </c>
       <c r="L33" s="2" t="s">
-        <v>396</v>
+        <v>401</v>
       </c>
       <c r="M33" s="2" t="s">
-        <v>42</v>
+        <v>402</v>
       </c>
       <c r="N33" s="2" t="s">
-        <v>397</v>
+        <v>403</v>
       </c>
       <c r="O33" s="2" t="s">
-        <v>398</v>
+        <v>404</v>
       </c>
     </row>
     <row r="34" spans="1:15">
       <c r="A34" s="2" t="s">
-        <v>399</v>
+        <v>405</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>16</v>
+        <v>406</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>391</v>
+        <v>407</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>400</v>
+        <v>408</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>401</v>
+        <v>409</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>402</v>
+        <v>410</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>51</v>
+        <v>411</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>189</v>
+        <v>412</v>
       </c>
       <c r="I34" s="2" t="s">
-        <v>403</v>
+        <v>413</v>
       </c>
       <c r="J34" s="2" t="s">
-        <v>404</v>
+        <v>414</v>
       </c>
       <c r="K34" s="2" t="s">
-        <v>76</v>
+        <v>415</v>
       </c>
       <c r="L34" s="2" t="s">
-        <v>405</v>
+        <v>416</v>
       </c>
       <c r="M34" s="2" t="s">
-        <v>42</v>
+        <v>417</v>
       </c>
       <c r="N34" s="2" t="s">
-        <v>406</v>
+        <v>418</v>
       </c>
       <c r="O34" s="2" t="s">
-        <v>407</v>
+        <v>235</v>
       </c>
     </row>
     <row r="35" spans="1:15">
       <c r="A35" s="2" t="s">
-        <v>408</v>
+        <v>419</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>16</v>
+        <v>420</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>409</v>
+        <v>421</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>410</v>
+        <v>422</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>411</v>
+        <v>423</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>412</v>
+        <v>424</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>51</v>
+        <v>425</v>
       </c>
       <c r="H35" s="2" t="s">
-        <v>413</v>
+        <v>426</v>
       </c>
       <c r="I35" s="2" t="s">
-        <v>414</v>
+        <v>427</v>
       </c>
       <c r="J35" s="2" t="s">
-        <v>415</v>
+        <v>428</v>
       </c>
       <c r="K35" s="2" t="s">
-        <v>76</v>
+        <v>96</v>
       </c>
       <c r="L35" s="2" t="s">
-        <v>416</v>
+        <v>429</v>
       </c>
       <c r="M35" s="2" t="s">
-        <v>417</v>
+        <v>430</v>
       </c>
       <c r="N35" s="2" t="s">
-        <v>418</v>
+        <v>431</v>
       </c>
       <c r="O35" s="2" t="s">
-        <v>419</v>
+        <v>432</v>
       </c>
     </row>
     <row r="36" spans="1:15">
       <c r="A36" s="2" t="s">
-        <v>420</v>
+        <v>433</v>
       </c>
       <c r="B36" s="2" t="s">
         <v>16</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>421</v>
+        <v>434</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>422</v>
+        <v>435</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>423</v>
+        <v>436</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>424</v>
+        <v>437</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>36</v>
+        <v>425</v>
       </c>
       <c r="H36" s="2" t="s">
-        <v>425</v>
+        <v>438</v>
       </c>
       <c r="I36" s="2" t="s">
-        <v>426</v>
+        <v>439</v>
       </c>
       <c r="J36" s="2" t="s">
-        <v>427</v>
+        <v>440</v>
       </c>
       <c r="K36" s="2" t="s">
-        <v>126</v>
+        <v>81</v>
       </c>
       <c r="L36" s="2" t="s">
-        <v>428</v>
+        <v>441</v>
       </c>
       <c r="M36" s="2" t="s">
-        <v>238</v>
+        <v>442</v>
       </c>
       <c r="N36" s="2" t="s">
-        <v>429</v>
+        <v>443</v>
       </c>
       <c r="O36" s="2" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
     </row>
     <row r="37" spans="1:15">
       <c r="A37" s="2" t="s">
-        <v>431</v>
+        <v>444</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>46</v>
+        <v>16</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>421</v>
+        <v>445</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>432</v>
+        <v>446</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>433</v>
+        <v>447</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>434</v>
+        <v>253</v>
       </c>
       <c r="G37" s="2" t="s">
-        <v>36</v>
+        <v>21</v>
       </c>
       <c r="H37" s="2" t="s">
-        <v>435</v>
+        <v>254</v>
       </c>
       <c r="I37" s="2" t="s">
-        <v>436</v>
+        <v>448</v>
       </c>
       <c r="J37" s="2" t="s">
-        <v>437</v>
+        <v>449</v>
       </c>
       <c r="K37" s="2" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="L37" s="2" t="s">
-        <v>438</v>
+        <v>450</v>
       </c>
       <c r="M37" s="2" t="s">
-        <v>313</v>
+        <v>83</v>
       </c>
       <c r="N37" s="2" t="s">
-        <v>439</v>
+        <v>451</v>
       </c>
       <c r="O37" s="2" t="s">
-        <v>440</v>
+        <v>452</v>
       </c>
     </row>
     <row r="38" spans="1:15">
       <c r="A38" s="2" t="s">
-        <v>441</v>
+        <v>453</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>81</v>
+        <v>16</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>442</v>
+        <v>454</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>443</v>
+        <v>455</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>444</v>
+        <v>456</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>445</v>
+        <v>241</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>446</v>
+        <v>242</v>
       </c>
       <c r="H38" s="2" t="s">
-        <v>349</v>
+        <v>243</v>
       </c>
       <c r="I38" s="2" t="s">
-        <v>447</v>
+        <v>457</v>
       </c>
       <c r="J38" s="2" t="s">
-        <v>448</v>
+        <v>458</v>
       </c>
       <c r="K38" s="2" t="s">
-        <v>352</v>
+        <v>130</v>
       </c>
       <c r="L38" s="2" t="s">
-        <v>353</v>
+        <v>459</v>
       </c>
       <c r="M38" s="2" t="s">
-        <v>449</v>
+        <v>83</v>
       </c>
       <c r="N38" s="2" t="s">
-        <v>450</v>
+        <v>460</v>
       </c>
       <c r="O38" s="2" t="s">
-        <v>170</v>
+        <v>461</v>
       </c>
     </row>
     <row r="39" spans="1:15">
       <c r="A39" s="2" t="s">
-        <v>451</v>
+        <v>462</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>46</v>
+        <v>16</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>453</v>
+        <v>463</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>454</v>
+        <v>464</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>455</v>
+        <v>465</v>
       </c>
       <c r="G39" s="2" t="s">
-        <v>21</v>
+        <v>92</v>
       </c>
       <c r="H39" s="2" t="s">
-        <v>456</v>
+        <v>254</v>
       </c>
       <c r="I39" s="2" t="s">
-        <v>457</v>
+        <v>466</v>
       </c>
       <c r="J39" s="2" t="s">
-        <v>458</v>
+        <v>467</v>
       </c>
       <c r="K39" s="2" t="s">
-        <v>76</v>
+        <v>117</v>
       </c>
       <c r="L39" s="2" t="s">
-        <v>459</v>
+        <v>468</v>
       </c>
       <c r="M39" s="2" t="s">
-        <v>460</v>
+        <v>83</v>
       </c>
       <c r="N39" s="2" t="s">
-        <v>461</v>
+        <v>469</v>
       </c>
       <c r="O39" s="2" t="s">
-        <v>462</v>
+        <v>470</v>
       </c>
     </row>
     <row r="40" spans="1:15">
       <c r="A40" s="2" t="s">
-        <v>463</v>
+        <v>471</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>46</v>
+        <v>16</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>452</v>
+        <v>472</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>464</v>
+        <v>473</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>465</v>
+        <v>474</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>455</v>
+        <v>475</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>21</v>
+        <v>92</v>
       </c>
       <c r="H40" s="2" t="s">
-        <v>456</v>
+        <v>476</v>
       </c>
       <c r="I40" s="2" t="s">
-        <v>466</v>
+        <v>477</v>
       </c>
       <c r="J40" s="2" t="s">
-        <v>467</v>
+        <v>478</v>
       </c>
       <c r="K40" s="2" t="s">
-        <v>126</v>
+        <v>117</v>
       </c>
       <c r="L40" s="2" t="s">
-        <v>468</v>
+        <v>479</v>
       </c>
       <c r="M40" s="2" t="s">
-        <v>460</v>
+        <v>480</v>
       </c>
       <c r="N40" s="2" t="s">
-        <v>469</v>
+        <v>481</v>
       </c>
       <c r="O40" s="2" t="s">
-        <v>470</v>
+        <v>482</v>
       </c>
     </row>
     <row r="41" spans="1:15">
       <c r="A41" s="2" t="s">
-        <v>471</v>
+        <v>483</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>46</v>
+        <v>16</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>452</v>
+        <v>484</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>472</v>
+        <v>485</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>473</v>
+        <v>486</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>455</v>
+        <v>487</v>
       </c>
       <c r="G41" s="2" t="s">
-        <v>21</v>
+        <v>77</v>
       </c>
       <c r="H41" s="2" t="s">
-        <v>456</v>
+        <v>488</v>
       </c>
       <c r="I41" s="2" t="s">
-        <v>474</v>
+        <v>489</v>
       </c>
       <c r="J41" s="2" t="s">
-        <v>475</v>
+        <v>490</v>
       </c>
       <c r="K41" s="2" t="s">
-        <v>76</v>
+        <v>130</v>
       </c>
       <c r="L41" s="2" t="s">
-        <v>476</v>
+        <v>491</v>
       </c>
       <c r="M41" s="2" t="s">
-        <v>460</v>
+        <v>303</v>
       </c>
       <c r="N41" s="2" t="s">
-        <v>477</v>
+        <v>492</v>
       </c>
       <c r="O41" s="2" t="s">
-        <v>478</v>
+        <v>493</v>
       </c>
     </row>
     <row r="42" spans="1:15">
       <c r="A42" s="2" t="s">
-        <v>479</v>
+        <v>494</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>46</v>
+        <v>87</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>452</v>
+        <v>484</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>480</v>
+        <v>495</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>481</v>
+        <v>496</v>
       </c>
       <c r="F42" s="2" t="s">
-        <v>482</v>
+        <v>497</v>
       </c>
       <c r="G42" s="2" t="s">
-        <v>177</v>
+        <v>77</v>
       </c>
       <c r="H42" s="2" t="s">
-        <v>456</v>
+        <v>498</v>
       </c>
       <c r="I42" s="2" t="s">
-        <v>483</v>
+        <v>499</v>
       </c>
       <c r="J42" s="2" t="s">
-        <v>484</v>
+        <v>500</v>
       </c>
       <c r="K42" s="2" t="s">
-        <v>55</v>
+        <v>130</v>
       </c>
       <c r="L42" s="2" t="s">
-        <v>485</v>
+        <v>501</v>
       </c>
       <c r="M42" s="2" t="s">
-        <v>460</v>
+        <v>42</v>
       </c>
       <c r="N42" s="2" t="s">
-        <v>486</v>
+        <v>502</v>
       </c>
       <c r="O42" s="2" t="s">
-        <v>487</v>
+        <v>503</v>
       </c>
     </row>
     <row r="43" spans="1:15">
       <c r="A43" s="2" t="s">
-        <v>488</v>
+        <v>504</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>46</v>
+        <v>147</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>452</v>
+        <v>505</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>489</v>
+        <v>506</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>490</v>
+        <v>507</v>
       </c>
       <c r="F43" s="2" t="s">
-        <v>455</v>
+        <v>508</v>
       </c>
       <c r="G43" s="2" t="s">
-        <v>21</v>
+        <v>509</v>
       </c>
       <c r="H43" s="2" t="s">
-        <v>456</v>
+        <v>412</v>
       </c>
       <c r="I43" s="2" t="s">
-        <v>491</v>
+        <v>510</v>
       </c>
       <c r="J43" s="2" t="s">
-        <v>492</v>
+        <v>511</v>
       </c>
       <c r="K43" s="2" t="s">
-        <v>76</v>
+        <v>415</v>
       </c>
       <c r="L43" s="2" t="s">
-        <v>493</v>
+        <v>416</v>
       </c>
       <c r="M43" s="2" t="s">
-        <v>460</v>
+        <v>512</v>
       </c>
       <c r="N43" s="2" t="s">
-        <v>494</v>
+        <v>513</v>
       </c>
       <c r="O43" s="2" t="s">
-        <v>495</v>
+        <v>235</v>
       </c>
     </row>
     <row r="44" spans="1:15">
       <c r="A44" s="2" t="s">
-        <v>496</v>
+        <v>514</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>172</v>
+        <v>87</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>452</v>
+        <v>515</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>497</v>
+        <v>516</v>
       </c>
       <c r="E44" s="3" t="s">
-        <v>498</v>
+        <v>517</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>455</v>
+        <v>518</v>
       </c>
       <c r="G44" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H44" s="2" t="s">
-        <v>456</v>
+        <v>519</v>
       </c>
       <c r="I44" s="2" t="s">
-        <v>499</v>
+        <v>520</v>
       </c>
       <c r="J44" s="2" t="s">
-        <v>500</v>
+        <v>521</v>
       </c>
       <c r="K44" s="2" t="s">
-        <v>76</v>
+        <v>117</v>
       </c>
       <c r="L44" s="2" t="s">
-        <v>501</v>
+        <v>522</v>
       </c>
       <c r="M44" s="2" t="s">
-        <v>460</v>
+        <v>523</v>
       </c>
       <c r="N44" s="2" t="s">
-        <v>502</v>
+        <v>524</v>
       </c>
       <c r="O44" s="2" t="s">
-        <v>503</v>
+        <v>525</v>
       </c>
     </row>
     <row r="45" spans="1:15">
       <c r="A45" s="2" t="s">
-        <v>504</v>
+        <v>526</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>172</v>
+        <v>87</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>452</v>
+        <v>515</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>505</v>
+        <v>527</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>506</v>
+        <v>528</v>
       </c>
       <c r="F45" s="2" t="s">
-        <v>455</v>
+        <v>518</v>
       </c>
       <c r="G45" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H45" s="2" t="s">
-        <v>456</v>
+        <v>519</v>
       </c>
       <c r="I45" s="2" t="s">
-        <v>507</v>
+        <v>529</v>
       </c>
       <c r="J45" s="2" t="s">
-        <v>508</v>
+        <v>530</v>
       </c>
       <c r="K45" s="2" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="L45" s="2" t="s">
-        <v>509</v>
+        <v>531</v>
       </c>
       <c r="M45" s="2" t="s">
-        <v>460</v>
+        <v>523</v>
       </c>
       <c r="N45" s="2" t="s">
-        <v>510</v>
+        <v>532</v>
       </c>
       <c r="O45" s="2" t="s">
-        <v>511</v>
+        <v>533</v>
       </c>
     </row>
     <row r="46" spans="1:15">
       <c r="A46" s="2" t="s">
-        <v>512</v>
+        <v>534</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>172</v>
+        <v>87</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>452</v>
+        <v>515</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>513</v>
+        <v>535</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>514</v>
+        <v>536</v>
       </c>
       <c r="F46" s="2" t="s">
-        <v>455</v>
+        <v>518</v>
       </c>
       <c r="G46" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H46" s="2" t="s">
-        <v>456</v>
+        <v>519</v>
       </c>
       <c r="I46" s="2" t="s">
-        <v>515</v>
+        <v>537</v>
       </c>
       <c r="J46" s="2" t="s">
-        <v>516</v>
+        <v>538</v>
       </c>
       <c r="K46" s="2" t="s">
-        <v>76</v>
+        <v>117</v>
       </c>
       <c r="L46" s="2" t="s">
-        <v>517</v>
+        <v>539</v>
       </c>
       <c r="M46" s="2" t="s">
-        <v>460</v>
+        <v>523</v>
       </c>
       <c r="N46" s="2" t="s">
-        <v>518</v>
+        <v>540</v>
       </c>
       <c r="O46" s="2" t="s">
-        <v>519</v>
+        <v>541</v>
       </c>
     </row>
     <row r="47" spans="1:15">
       <c r="A47" s="2" t="s">
-        <v>520</v>
+        <v>542</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>172</v>
+        <v>87</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>452</v>
+        <v>515</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>521</v>
+        <v>543</v>
       </c>
       <c r="E47" s="3" t="s">
-        <v>522</v>
+        <v>544</v>
       </c>
       <c r="F47" s="2" t="s">
-        <v>455</v>
+        <v>545</v>
       </c>
       <c r="G47" s="2" t="s">
-        <v>21</v>
+        <v>242</v>
       </c>
       <c r="H47" s="2" t="s">
-        <v>456</v>
+        <v>519</v>
       </c>
       <c r="I47" s="2" t="s">
+        <v>546</v>
+      </c>
+      <c r="J47" s="2" t="s">
+        <v>547</v>
+      </c>
+      <c r="K47" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="L47" s="2" t="s">
+        <v>548</v>
+      </c>
+      <c r="M47" s="2" t="s">
         <v>523</v>
       </c>
-      <c r="J47" s="2" t="s">
-        <v>524</v>
-      </c>
-      <c r="K47" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="L47" s="2" t="s">
-        <v>525</v>
-      </c>
-      <c r="M47" s="2" t="s">
-        <v>460</v>
-      </c>
       <c r="N47" s="2" t="s">
-        <v>526</v>
+        <v>549</v>
       </c>
       <c r="O47" s="2" t="s">
-        <v>527</v>
+        <v>550</v>
       </c>
     </row>
     <row r="48" spans="1:15">
       <c r="A48" s="2" t="s">
-        <v>528</v>
+        <v>551</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>172</v>
+        <v>87</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>452</v>
+        <v>515</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>529</v>
+        <v>552</v>
       </c>
       <c r="E48" s="3" t="s">
-        <v>530</v>
+        <v>553</v>
       </c>
       <c r="F48" s="2" t="s">
-        <v>455</v>
+        <v>518</v>
       </c>
       <c r="G48" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H48" s="2" t="s">
-        <v>456</v>
+        <v>519</v>
       </c>
       <c r="I48" s="2" t="s">
-        <v>531</v>
+        <v>554</v>
       </c>
       <c r="J48" s="2" t="s">
-        <v>532</v>
+        <v>555</v>
       </c>
       <c r="K48" s="2" t="s">
-        <v>126</v>
+        <v>117</v>
       </c>
       <c r="L48" s="2" t="s">
-        <v>533</v>
+        <v>556</v>
       </c>
       <c r="M48" s="2" t="s">
-        <v>460</v>
+        <v>523</v>
       </c>
       <c r="N48" s="2" t="s">
-        <v>534</v>
+        <v>557</v>
       </c>
       <c r="O48" s="2" t="s">
-        <v>535</v>
+        <v>558</v>
       </c>
     </row>
     <row r="49" spans="1:15">
       <c r="A49" s="2" t="s">
-        <v>536</v>
+        <v>559</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>172</v>
+        <v>237</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>452</v>
+        <v>515</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>537</v>
+        <v>560</v>
       </c>
       <c r="E49" s="3" t="s">
-        <v>538</v>
+        <v>561</v>
       </c>
       <c r="F49" s="2" t="s">
-        <v>455</v>
+        <v>518</v>
       </c>
       <c r="G49" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H49" s="2" t="s">
-        <v>456</v>
+        <v>519</v>
       </c>
       <c r="I49" s="2" t="s">
-        <v>539</v>
+        <v>562</v>
       </c>
       <c r="J49" s="2" t="s">
-        <v>540</v>
+        <v>563</v>
       </c>
       <c r="K49" s="2" t="s">
-        <v>76</v>
+        <v>117</v>
       </c>
       <c r="L49" s="2" t="s">
-        <v>541</v>
+        <v>564</v>
       </c>
       <c r="M49" s="2" t="s">
-        <v>460</v>
+        <v>523</v>
       </c>
       <c r="N49" s="2" t="s">
-        <v>542</v>
+        <v>565</v>
       </c>
       <c r="O49" s="2" t="s">
-        <v>543</v>
+        <v>566</v>
       </c>
     </row>
     <row r="50" spans="1:15">
       <c r="A50" s="2" t="s">
-        <v>544</v>
+        <v>567</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>172</v>
+        <v>237</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>452</v>
+        <v>515</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>545</v>
+        <v>568</v>
       </c>
       <c r="E50" s="3" t="s">
-        <v>546</v>
+        <v>569</v>
       </c>
       <c r="F50" s="2" t="s">
-        <v>455</v>
+        <v>518</v>
       </c>
       <c r="G50" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H50" s="2" t="s">
-        <v>456</v>
+        <v>519</v>
       </c>
       <c r="I50" s="2" t="s">
-        <v>547</v>
+        <v>570</v>
       </c>
       <c r="J50" s="2" t="s">
-        <v>548</v>
+        <v>571</v>
       </c>
       <c r="K50" s="2" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="L50" s="2" t="s">
-        <v>533</v>
+        <v>572</v>
       </c>
       <c r="M50" s="2" t="s">
-        <v>460</v>
+        <v>523</v>
       </c>
       <c r="N50" s="2" t="s">
-        <v>549</v>
+        <v>573</v>
       </c>
       <c r="O50" s="2" t="s">
-        <v>550</v>
+        <v>574</v>
       </c>
     </row>
     <row r="51" spans="1:15">
       <c r="A51" s="2" t="s">
-        <v>551</v>
+        <v>575</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>172</v>
+        <v>237</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>452</v>
+        <v>515</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>552</v>
+        <v>576</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>553</v>
+        <v>577</v>
       </c>
       <c r="F51" s="2" t="s">
-        <v>455</v>
+        <v>518</v>
       </c>
       <c r="G51" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H51" s="2" t="s">
-        <v>456</v>
+        <v>519</v>
       </c>
       <c r="I51" s="2" t="s">
-        <v>554</v>
+        <v>578</v>
       </c>
       <c r="J51" s="2" t="s">
-        <v>555</v>
+        <v>579</v>
       </c>
       <c r="K51" s="2" t="s">
-        <v>126</v>
+        <v>117</v>
       </c>
       <c r="L51" s="2" t="s">
-        <v>556</v>
+        <v>580</v>
       </c>
       <c r="M51" s="2" t="s">
-        <v>460</v>
+        <v>523</v>
       </c>
       <c r="N51" s="2" t="s">
-        <v>557</v>
+        <v>581</v>
       </c>
       <c r="O51" s="2" t="s">
-        <v>558</v>
+        <v>582</v>
       </c>
     </row>
     <row r="52" spans="1:15">
       <c r="A52" s="2" t="s">
-        <v>559</v>
+        <v>583</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>172</v>
+        <v>237</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>452</v>
+        <v>515</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>560</v>
+        <v>584</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>561</v>
+        <v>585</v>
       </c>
       <c r="F52" s="2" t="s">
-        <v>455</v>
+        <v>518</v>
       </c>
       <c r="G52" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H52" s="2" t="s">
-        <v>456</v>
+        <v>519</v>
       </c>
       <c r="I52" s="2" t="s">
-        <v>562</v>
+        <v>586</v>
       </c>
       <c r="J52" s="2" t="s">
-        <v>563</v>
+        <v>587</v>
       </c>
       <c r="K52" s="2" t="s">
-        <v>76</v>
+        <v>130</v>
       </c>
       <c r="L52" s="2" t="s">
-        <v>564</v>
+        <v>588</v>
       </c>
       <c r="M52" s="2" t="s">
-        <v>460</v>
+        <v>523</v>
       </c>
       <c r="N52" s="2" t="s">
-        <v>565</v>
+        <v>589</v>
       </c>
       <c r="O52" s="2" t="s">
-        <v>566</v>
+        <v>590</v>
       </c>
     </row>
     <row r="53" spans="1:15">
       <c r="A53" s="2" t="s">
-        <v>567</v>
+        <v>591</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>172</v>
+        <v>237</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>452</v>
+        <v>515</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>568</v>
+        <v>592</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>569</v>
+        <v>593</v>
       </c>
       <c r="F53" s="2" t="s">
-        <v>455</v>
+        <v>518</v>
       </c>
       <c r="G53" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H53" s="2" t="s">
-        <v>456</v>
+        <v>519</v>
       </c>
       <c r="I53" s="2" t="s">
-        <v>570</v>
+        <v>594</v>
       </c>
       <c r="J53" s="2" t="s">
-        <v>571</v>
+        <v>595</v>
       </c>
       <c r="K53" s="2" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="L53" s="2" t="s">
-        <v>533</v>
+        <v>596</v>
       </c>
       <c r="M53" s="2" t="s">
-        <v>460</v>
+        <v>523</v>
       </c>
       <c r="N53" s="2" t="s">
-        <v>572</v>
+        <v>597</v>
       </c>
       <c r="O53" s="2" t="s">
-        <v>573</v>
+        <v>598</v>
       </c>
     </row>
     <row r="54" spans="1:15">
       <c r="A54" s="2" t="s">
-        <v>574</v>
+        <v>599</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>172</v>
+        <v>237</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>452</v>
+        <v>515</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>575</v>
+        <v>600</v>
       </c>
       <c r="E54" s="3" t="s">
-        <v>576</v>
+        <v>601</v>
       </c>
       <c r="F54" s="2" t="s">
-        <v>455</v>
+        <v>518</v>
       </c>
       <c r="G54" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H54" s="2" t="s">
-        <v>456</v>
+        <v>519</v>
       </c>
       <c r="I54" s="2" t="s">
-        <v>577</v>
+        <v>602</v>
       </c>
       <c r="J54" s="2" t="s">
-        <v>578</v>
+        <v>603</v>
       </c>
       <c r="K54" s="2" t="s">
-        <v>76</v>
+        <v>117</v>
       </c>
       <c r="L54" s="2" t="s">
-        <v>579</v>
+        <v>604</v>
       </c>
       <c r="M54" s="2" t="s">
-        <v>460</v>
+        <v>523</v>
       </c>
       <c r="N54" s="2" t="s">
-        <v>580</v>
+        <v>605</v>
       </c>
       <c r="O54" s="2" t="s">
-        <v>581</v>
+        <v>606</v>
       </c>
     </row>
     <row r="55" spans="1:15">
       <c r="A55" s="2" t="s">
-        <v>582</v>
+        <v>607</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>172</v>
+        <v>237</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>452</v>
+        <v>515</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>583</v>
+        <v>608</v>
       </c>
       <c r="E55" s="3" t="s">
-        <v>584</v>
+        <v>609</v>
       </c>
       <c r="F55" s="2" t="s">
-        <v>455</v>
+        <v>518</v>
       </c>
       <c r="G55" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H55" s="2" t="s">
-        <v>456</v>
+        <v>519</v>
       </c>
       <c r="I55" s="2" t="s">
-        <v>585</v>
+        <v>610</v>
       </c>
       <c r="J55" s="2" t="s">
-        <v>586</v>
+        <v>611</v>
       </c>
       <c r="K55" s="2" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="L55" s="2" t="s">
-        <v>587</v>
+        <v>596</v>
       </c>
       <c r="M55" s="2" t="s">
-        <v>460</v>
+        <v>523</v>
       </c>
       <c r="N55" s="2" t="s">
-        <v>588</v>
+        <v>612</v>
       </c>
       <c r="O55" s="2" t="s">
-        <v>589</v>
+        <v>613</v>
       </c>
     </row>
     <row r="56" spans="1:15">
       <c r="A56" s="2" t="s">
-        <v>590</v>
+        <v>614</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>117</v>
+        <v>237</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>452</v>
+        <v>515</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>591</v>
+        <v>615</v>
       </c>
       <c r="E56" s="3" t="s">
-        <v>592</v>
+        <v>616</v>
       </c>
       <c r="F56" s="2" t="s">
-        <v>455</v>
+        <v>518</v>
       </c>
       <c r="G56" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H56" s="2" t="s">
-        <v>456</v>
+        <v>519</v>
       </c>
       <c r="I56" s="2" t="s">
-        <v>593</v>
+        <v>617</v>
       </c>
       <c r="J56" s="2" t="s">
-        <v>594</v>
+        <v>618</v>
       </c>
       <c r="K56" s="2" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="L56" s="2" t="s">
-        <v>595</v>
+        <v>619</v>
       </c>
       <c r="M56" s="2" t="s">
-        <v>460</v>
+        <v>523</v>
       </c>
       <c r="N56" s="2" t="s">
-        <v>596</v>
+        <v>620</v>
       </c>
       <c r="O56" s="2" t="s">
-        <v>597</v>
+        <v>621</v>
       </c>
     </row>
     <row r="57" spans="1:15">
       <c r="A57" s="2" t="s">
-        <v>598</v>
+        <v>622</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>599</v>
+        <v>237</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>452</v>
+        <v>515</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>600</v>
+        <v>623</v>
       </c>
       <c r="E57" s="3" t="s">
-        <v>601</v>
+        <v>624</v>
       </c>
       <c r="F57" s="2" t="s">
-        <v>455</v>
+        <v>518</v>
       </c>
       <c r="G57" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H57" s="2" t="s">
-        <v>456</v>
+        <v>519</v>
       </c>
       <c r="I57" s="2" t="s">
-        <v>602</v>
+        <v>625</v>
       </c>
       <c r="J57" s="2" t="s">
-        <v>603</v>
+        <v>626</v>
       </c>
       <c r="K57" s="2" t="s">
-        <v>76</v>
+        <v>117</v>
       </c>
       <c r="L57" s="2" t="s">
-        <v>604</v>
+        <v>627</v>
       </c>
       <c r="M57" s="2" t="s">
-        <v>460</v>
+        <v>523</v>
       </c>
       <c r="N57" s="2" t="s">
-        <v>605</v>
+        <v>628</v>
       </c>
       <c r="O57" s="2" t="s">
-        <v>606</v>
+        <v>629</v>
       </c>
     </row>
     <row r="58" spans="1:15">
       <c r="A58" s="2" t="s">
-        <v>607</v>
+        <v>630</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>172</v>
+        <v>237</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>452</v>
+        <v>515</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>608</v>
+        <v>631</v>
       </c>
       <c r="E58" s="3" t="s">
-        <v>609</v>
+        <v>632</v>
       </c>
       <c r="F58" s="2" t="s">
-        <v>455</v>
+        <v>518</v>
       </c>
       <c r="G58" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H58" s="2" t="s">
-        <v>456</v>
+        <v>519</v>
       </c>
       <c r="I58" s="2" t="s">
-        <v>610</v>
+        <v>633</v>
       </c>
       <c r="J58" s="2" t="s">
-        <v>611</v>
+        <v>634</v>
       </c>
       <c r="K58" s="2" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="L58" s="2" t="s">
-        <v>612</v>
+        <v>596</v>
       </c>
       <c r="M58" s="2" t="s">
-        <v>460</v>
+        <v>523</v>
       </c>
       <c r="N58" s="2" t="s">
-        <v>613</v>
+        <v>635</v>
       </c>
       <c r="O58" s="2" t="s">
-        <v>614</v>
+        <v>636</v>
       </c>
     </row>
     <row r="59" spans="1:15">
       <c r="A59" s="2" t="s">
-        <v>615</v>
+        <v>637</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>172</v>
+        <v>237</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>452</v>
+        <v>515</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>616</v>
+        <v>638</v>
       </c>
       <c r="E59" s="3" t="s">
-        <v>617</v>
+        <v>639</v>
       </c>
       <c r="F59" s="2" t="s">
-        <v>482</v>
+        <v>518</v>
       </c>
       <c r="G59" s="2" t="s">
-        <v>177</v>
+        <v>21</v>
       </c>
       <c r="H59" s="2" t="s">
-        <v>456</v>
+        <v>519</v>
       </c>
       <c r="I59" s="2" t="s">
-        <v>618</v>
+        <v>640</v>
       </c>
       <c r="J59" s="2" t="s">
-        <v>619</v>
+        <v>641</v>
       </c>
       <c r="K59" s="2" t="s">
-        <v>126</v>
+        <v>117</v>
       </c>
       <c r="L59" s="2" t="s">
-        <v>181</v>
+        <v>642</v>
       </c>
       <c r="M59" s="2" t="s">
-        <v>460</v>
+        <v>523</v>
       </c>
       <c r="N59" s="2" t="s">
-        <v>620</v>
+        <v>643</v>
       </c>
       <c r="O59" s="2" t="s">
-        <v>621</v>
+        <v>644</v>
       </c>
     </row>
     <row r="60" spans="1:15">
       <c r="A60" s="2" t="s">
-        <v>622</v>
+        <v>645</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>172</v>
+        <v>237</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>452</v>
+        <v>515</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>623</v>
+        <v>646</v>
       </c>
       <c r="E60" s="3" t="s">
-        <v>624</v>
+        <v>647</v>
       </c>
       <c r="F60" s="2" t="s">
-        <v>455</v>
+        <v>518</v>
       </c>
       <c r="G60" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H60" s="2" t="s">
-        <v>456</v>
+        <v>519</v>
       </c>
       <c r="I60" s="2" t="s">
-        <v>625</v>
+        <v>648</v>
       </c>
       <c r="J60" s="2" t="s">
-        <v>626</v>
+        <v>649</v>
       </c>
       <c r="K60" s="2" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="L60" s="2" t="s">
-        <v>627</v>
+        <v>650</v>
       </c>
       <c r="M60" s="2" t="s">
-        <v>460</v>
+        <v>523</v>
       </c>
       <c r="N60" s="2" t="s">
-        <v>628</v>
+        <v>651</v>
       </c>
       <c r="O60" s="2" t="s">
-        <v>629</v>
+        <v>652</v>
       </c>
     </row>
     <row r="61" spans="1:15">
       <c r="A61" s="2" t="s">
-        <v>630</v>
+        <v>653</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>117</v>
+        <v>183</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>452</v>
+        <v>515</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>631</v>
+        <v>654</v>
       </c>
       <c r="E61" s="3" t="s">
-        <v>632</v>
+        <v>655</v>
       </c>
       <c r="F61" s="2" t="s">
-        <v>455</v>
+        <v>518</v>
       </c>
       <c r="G61" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H61" s="2" t="s">
-        <v>456</v>
+        <v>519</v>
       </c>
       <c r="I61" s="2" t="s">
-        <v>633</v>
+        <v>656</v>
       </c>
       <c r="J61" s="2" t="s">
-        <v>634</v>
+        <v>657</v>
       </c>
       <c r="K61" s="2" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="L61" s="2" t="s">
-        <v>635</v>
+        <v>658</v>
       </c>
       <c r="M61" s="2" t="s">
-        <v>460</v>
+        <v>523</v>
       </c>
       <c r="N61" s="2" t="s">
-        <v>636</v>
+        <v>659</v>
       </c>
       <c r="O61" s="2" t="s">
-        <v>637</v>
+        <v>660</v>
       </c>
     </row>
     <row r="62" spans="1:15">
       <c r="A62" s="2" t="s">
-        <v>638</v>
+        <v>661</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>599</v>
+        <v>662</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>452</v>
+        <v>515</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>639</v>
+        <v>663</v>
       </c>
       <c r="E62" s="3" t="s">
-        <v>640</v>
+        <v>664</v>
       </c>
       <c r="F62" s="2" t="s">
-        <v>455</v>
+        <v>518</v>
       </c>
       <c r="G62" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H62" s="2" t="s">
-        <v>456</v>
+        <v>519</v>
       </c>
       <c r="I62" s="2" t="s">
-        <v>641</v>
+        <v>665</v>
       </c>
       <c r="J62" s="2" t="s">
-        <v>642</v>
+        <v>666</v>
       </c>
       <c r="K62" s="2" t="s">
-        <v>76</v>
+        <v>117</v>
       </c>
       <c r="L62" s="2" t="s">
-        <v>643</v>
+        <v>667</v>
       </c>
       <c r="M62" s="2" t="s">
-        <v>460</v>
+        <v>523</v>
       </c>
       <c r="N62" s="2" t="s">
-        <v>644</v>
+        <v>668</v>
       </c>
       <c r="O62" s="2" t="s">
-        <v>645</v>
+        <v>669</v>
       </c>
     </row>
     <row r="63" spans="1:15">
       <c r="A63" s="2" t="s">
-        <v>646</v>
+        <v>670</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>599</v>
+        <v>237</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>452</v>
+        <v>515</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>647</v>
+        <v>671</v>
       </c>
       <c r="E63" s="3" t="s">
-        <v>648</v>
+        <v>672</v>
       </c>
       <c r="F63" s="2" t="s">
-        <v>455</v>
+        <v>518</v>
       </c>
       <c r="G63" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H63" s="2" t="s">
-        <v>456</v>
+        <v>519</v>
       </c>
       <c r="I63" s="2" t="s">
-        <v>649</v>
+        <v>673</v>
       </c>
       <c r="J63" s="2" t="s">
-        <v>650</v>
+        <v>674</v>
       </c>
       <c r="K63" s="2" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="L63" s="2" t="s">
-        <v>533</v>
+        <v>675</v>
       </c>
       <c r="M63" s="2" t="s">
-        <v>460</v>
+        <v>523</v>
       </c>
       <c r="N63" s="2" t="s">
-        <v>651</v>
+        <v>676</v>
       </c>
       <c r="O63" s="2" t="s">
-        <v>652</v>
+        <v>677</v>
+      </c>
+    </row>
+    <row r="64" spans="1:15">
+      <c r="A64" s="2" t="s">
+        <v>678</v>
+      </c>
+      <c r="B64" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="C64" s="2" t="s">
+        <v>515</v>
+      </c>
+      <c r="D64" s="2" t="s">
+        <v>679</v>
+      </c>
+      <c r="E64" s="3" t="s">
+        <v>680</v>
+      </c>
+      <c r="F64" s="2" t="s">
+        <v>545</v>
+      </c>
+      <c r="G64" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="H64" s="2" t="s">
+        <v>519</v>
+      </c>
+      <c r="I64" s="2" t="s">
+        <v>681</v>
+      </c>
+      <c r="J64" s="2" t="s">
+        <v>682</v>
+      </c>
+      <c r="K64" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="L64" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="M64" s="2" t="s">
+        <v>523</v>
+      </c>
+      <c r="N64" s="2" t="s">
+        <v>683</v>
+      </c>
+      <c r="O64" s="2" t="s">
+        <v>684</v>
+      </c>
+    </row>
+    <row r="65" spans="1:15">
+      <c r="A65" s="2" t="s">
+        <v>685</v>
+      </c>
+      <c r="B65" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="C65" s="2" t="s">
+        <v>515</v>
+      </c>
+      <c r="D65" s="2" t="s">
+        <v>686</v>
+      </c>
+      <c r="E65" s="3" t="s">
+        <v>687</v>
+      </c>
+      <c r="F65" s="2" t="s">
+        <v>518</v>
+      </c>
+      <c r="G65" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H65" s="2" t="s">
+        <v>519</v>
+      </c>
+      <c r="I65" s="2" t="s">
+        <v>688</v>
+      </c>
+      <c r="J65" s="2" t="s">
+        <v>689</v>
+      </c>
+      <c r="K65" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="L65" s="2" t="s">
+        <v>690</v>
+      </c>
+      <c r="M65" s="2" t="s">
+        <v>523</v>
+      </c>
+      <c r="N65" s="2" t="s">
+        <v>691</v>
+      </c>
+      <c r="O65" s="2" t="s">
+        <v>692</v>
+      </c>
+    </row>
+    <row r="66" spans="1:15">
+      <c r="A66" s="2" t="s">
+        <v>693</v>
+      </c>
+      <c r="B66" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="C66" s="2" t="s">
+        <v>515</v>
+      </c>
+      <c r="D66" s="2" t="s">
+        <v>694</v>
+      </c>
+      <c r="E66" s="3" t="s">
+        <v>695</v>
+      </c>
+      <c r="F66" s="2" t="s">
+        <v>518</v>
+      </c>
+      <c r="G66" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H66" s="2" t="s">
+        <v>519</v>
+      </c>
+      <c r="I66" s="2" t="s">
+        <v>696</v>
+      </c>
+      <c r="J66" s="2" t="s">
+        <v>697</v>
+      </c>
+      <c r="K66" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="L66" s="2" t="s">
+        <v>698</v>
+      </c>
+      <c r="M66" s="2" t="s">
+        <v>523</v>
+      </c>
+      <c r="N66" s="2" t="s">
+        <v>699</v>
+      </c>
+      <c r="O66" s="2" t="s">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="67" spans="1:15">
+      <c r="A67" s="2" t="s">
+        <v>701</v>
+      </c>
+      <c r="B67" s="2" t="s">
+        <v>662</v>
+      </c>
+      <c r="C67" s="2" t="s">
+        <v>515</v>
+      </c>
+      <c r="D67" s="2" t="s">
+        <v>702</v>
+      </c>
+      <c r="E67" s="3" t="s">
+        <v>703</v>
+      </c>
+      <c r="F67" s="2" t="s">
+        <v>518</v>
+      </c>
+      <c r="G67" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H67" s="2" t="s">
+        <v>519</v>
+      </c>
+      <c r="I67" s="2" t="s">
+        <v>704</v>
+      </c>
+      <c r="J67" s="2" t="s">
+        <v>705</v>
+      </c>
+      <c r="K67" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="L67" s="2" t="s">
+        <v>706</v>
+      </c>
+      <c r="M67" s="2" t="s">
+        <v>523</v>
+      </c>
+      <c r="N67" s="2" t="s">
+        <v>707</v>
+      </c>
+      <c r="O67" s="2" t="s">
+        <v>708</v>
+      </c>
+    </row>
+    <row r="68" spans="1:15">
+      <c r="A68" s="2" t="s">
+        <v>709</v>
+      </c>
+      <c r="B68" s="2" t="s">
+        <v>662</v>
+      </c>
+      <c r="C68" s="2" t="s">
+        <v>515</v>
+      </c>
+      <c r="D68" s="2" t="s">
+        <v>710</v>
+      </c>
+      <c r="E68" s="3" t="s">
+        <v>711</v>
+      </c>
+      <c r="F68" s="2" t="s">
+        <v>518</v>
+      </c>
+      <c r="G68" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H68" s="2" t="s">
+        <v>519</v>
+      </c>
+      <c r="I68" s="2" t="s">
+        <v>712</v>
+      </c>
+      <c r="J68" s="2" t="s">
+        <v>713</v>
+      </c>
+      <c r="K68" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="L68" s="2" t="s">
+        <v>596</v>
+      </c>
+      <c r="M68" s="2" t="s">
+        <v>523</v>
+      </c>
+      <c r="N68" s="2" t="s">
+        <v>714</v>
+      </c>
+      <c r="O68" s="2" t="s">
+        <v>715</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O63"/>
+  <autoFilter ref="A1:O68"/>
   <hyperlinks>
     <hyperlink ref="E2" r:id="rId1"/>
     <hyperlink ref="E3" r:id="rId2"/>
@@ -5398,6 +5822,11 @@
     <hyperlink ref="E61" r:id="rId60"/>
     <hyperlink ref="E62" r:id="rId61"/>
     <hyperlink ref="E63" r:id="rId62"/>
+    <hyperlink ref="E64" r:id="rId63"/>
+    <hyperlink ref="E65" r:id="rId64"/>
+    <hyperlink ref="E66" r:id="rId65"/>
+    <hyperlink ref="E67" r:id="rId66"/>
+    <hyperlink ref="E68" r:id="rId67"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Prepare AfC package for education update
</commit_message>
<xml_diff>
--- a/dossier/source_dossier.xlsx
+++ b/dossier/source_dossier.xlsx
@@ -10,14 +10,14 @@
     <sheet name="Source Dossier" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Source Dossier'!$A$1:$O$68</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Source Dossier'!$A$1:$O$70</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1020" uniqueCount="716">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1050" uniqueCount="738">
   <si>
     <t>id</t>
   </si>
@@ -686,6 +686,72 @@
   </si>
   <si>
     <t>Do not cite until exact video pages are verified</t>
+  </si>
+  <si>
+    <t>MWV1</t>
+  </si>
+  <si>
+    <t>Enhancing Teaching and Learning with MATLAB Copilot and Simulink Copilot</t>
+  </si>
+  <si>
+    <t>https://www.mathworks.com/videos/enhancing-teaching-and-learning-with-generative-ai-and-matlab-1758823408469.html</t>
+  </si>
+  <si>
+    <t>Affiliated video page / speaker bio</t>
+  </si>
+  <si>
+    <t>High for MathWorks page metadata and speaker-bio text; limited as biographical source</t>
+  </si>
+  <si>
+    <t>Minor to moderate. MathWorks video page includes a speaker bio for Jeff Alderson, identifies him as Education Product Manager at MathWorks, and states that he received a B.S. from WPI and an M.Ed. in Education Policy, Organization &amp; Leadership from the University of Illinois at Urbana-Champaign.</t>
+  </si>
+  <si>
+    <t>Alderson earned a Master of Education in education policy, organization, and leadership from the University of Illinois Urbana-Champaign; he was Education Product Manager at MathWorks and led marketing efforts for MATLAB Grader and MATLAB Course Designer.</t>
+  </si>
+  <si>
+    <t>Use for the narrow education item and MathWorks professional-context facts; do not use as notability support.</t>
+  </si>
+  <si>
+    <t>Reviewed in sources/mathworks_matlab_grader_sources.md; local file data/mathworks_video_enhancing_teaching_learning_generative_ai_matlab.html</t>
+  </si>
+  <si>
+    <t>{{cite web |title=Enhancing Teaching and Learning with MATLAB Copilot and Simulink Copilot |url=https://www.mathworks.com/videos/enhancing-teaching-and-learning-with-generative-ai-and-matlab-1758823408469.html |website=MathWorks |date=May 28, 2026 |access-date=June 8, 2026}}</t>
+  </si>
+  <si>
+    <t>UIUC1</t>
+  </si>
+  <si>
+    <t>University of Illinois at Urbana-Champaign / Digication</t>
+  </si>
+  <si>
+    <t>Jeff Alderson Instructional Design</t>
+  </si>
+  <si>
+    <t>https://illinois.digication.com/jeff-alderson-instructional-design/welcome</t>
+  </si>
+  <si>
+    <t>Institution-hosted portfolio</t>
+  </si>
+  <si>
+    <t>Partial / subject-created portfolio on institutional platform</t>
+  </si>
+  <si>
+    <t>Medium for platform metadata; limited for biographical facts</t>
+  </si>
+  <si>
+    <t>Minor. UIUC Digication page metadata identifies the system as University of Illinois at Urbana-Champaign, the published portfolio title as `Jeff Alderson Instructional Design`, and the welcome page as published. A related course page is titled `EPOL 483 Learning Technologies`.</t>
+  </si>
+  <si>
+    <t>Alderson had a published instructional-design portfolio hosted in the University of Illinois at Urbana-Champaign Digication system during graduate classwork context; the page does not itself verify the completed degree.</t>
+  </si>
+  <si>
+    <t>Retain as supporting education/portfolio context only; do not use as notability support or as the primary degree citation.</t>
+  </si>
+  <si>
+    <t>Reviewed in sources/education_sources.md; local files data/uiuc_digication_jeff_alderson_instructional_design_welcome.html and data/uiuc_digication_jeff_alderson_epol_483_learning_technologies.html</t>
+  </si>
+  <si>
+    <t>{{cite web |title=Jeff Alderson Instructional Design |url=https://illinois.digication.com/jeff-alderson-instructional-design/welcome |website=University of Illinois at Urbana-Champaign Digication |access-date=June 8, 2026}}</t>
   </si>
   <si>
     <t>RG1</t>
@@ -2542,7 +2608,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O68"/>
+  <dimension ref="A1:O70"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -3365,383 +3431,383 @@
         <v>223</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>197</v>
+        <v>87</v>
       </c>
       <c r="C18" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="D18" s="2" t="s">
         <v>224</v>
       </c>
-      <c r="D18" s="2" t="s">
+      <c r="E18" s="3" t="s">
         <v>225</v>
       </c>
-      <c r="E18" s="3" t="s">
+      <c r="F18" s="2" t="s">
         <v>226</v>
       </c>
-      <c r="F18" s="2" t="s">
+      <c r="G18" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="H18" s="2" t="s">
         <v>227</v>
       </c>
-      <c r="G18" s="2" t="s">
+      <c r="I18" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="H18" s="2" t="s">
+      <c r="J18" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="I18" s="2" t="s">
+      <c r="K18" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="L18" s="2" t="s">
         <v>230</v>
       </c>
-      <c r="J18" s="2" t="s">
+      <c r="M18" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="N18" s="2" t="s">
         <v>231</v>
       </c>
-      <c r="K18" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="L18" s="2" t="s">
+      <c r="O18" s="2" t="s">
         <v>232</v>
-      </c>
-      <c r="M18" s="2" t="s">
-        <v>233</v>
-      </c>
-      <c r="N18" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="O18" s="2" t="s">
-        <v>235</v>
       </c>
     </row>
     <row r="19" spans="1:15">
       <c r="A19" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="E19" s="3" t="s">
         <v>236</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="F19" s="2" t="s">
         <v>237</v>
       </c>
-      <c r="C19" s="2" t="s">
+      <c r="G19" s="2" t="s">
         <v>238</v>
       </c>
-      <c r="D19" s="2" t="s">
+      <c r="H19" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="E19" s="3" t="s">
+      <c r="I19" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="F19" s="2" t="s">
+      <c r="J19" s="2" t="s">
         <v>241</v>
       </c>
-      <c r="G19" s="2" t="s">
+      <c r="K19" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="L19" s="2" t="s">
         <v>242</v>
       </c>
-      <c r="H19" s="2" t="s">
+      <c r="M19" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="N19" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="I19" s="2" t="s">
+      <c r="O19" s="2" t="s">
         <v>244</v>
-      </c>
-      <c r="J19" s="2" t="s">
-        <v>245</v>
-      </c>
-      <c r="K19" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="L19" s="2" t="s">
-        <v>246</v>
-      </c>
-      <c r="M19" s="2" t="s">
-        <v>247</v>
-      </c>
-      <c r="N19" s="2" t="s">
-        <v>248</v>
-      </c>
-      <c r="O19" s="2" t="s">
-        <v>249</v>
       </c>
     </row>
     <row r="20" spans="1:15">
       <c r="A20" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="G20" s="2" t="s">
         <v>250</v>
       </c>
-      <c r="B20" s="2" t="s">
-        <v>237</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>238</v>
-      </c>
-      <c r="D20" s="2" t="s">
+      <c r="H20" s="2" t="s">
         <v>251</v>
       </c>
-      <c r="E20" s="3" t="s">
+      <c r="I20" s="2" t="s">
         <v>252</v>
       </c>
-      <c r="F20" s="2" t="s">
+      <c r="J20" s="2" t="s">
         <v>253</v>
       </c>
-      <c r="G20" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H20" s="2" t="s">
+      <c r="K20" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="L20" s="2" t="s">
         <v>254</v>
       </c>
-      <c r="I20" s="2" t="s">
+      <c r="M20" s="2" t="s">
         <v>255</v>
       </c>
-      <c r="J20" s="2" t="s">
+      <c r="N20" s="2" t="s">
         <v>256</v>
       </c>
-      <c r="K20" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="L20" s="2" t="s">
+      <c r="O20" s="2" t="s">
         <v>257</v>
-      </c>
-      <c r="M20" s="2" t="s">
-        <v>258</v>
-      </c>
-      <c r="N20" s="2" t="s">
-        <v>259</v>
-      </c>
-      <c r="O20" s="2" t="s">
-        <v>260</v>
       </c>
     </row>
     <row r="21" spans="1:15">
       <c r="A21" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="D21" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="B21" s="2" t="s">
-        <v>237</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>238</v>
-      </c>
-      <c r="D21" s="2" t="s">
+      <c r="E21" s="3" t="s">
         <v>262</v>
       </c>
-      <c r="E21" s="3" t="s">
+      <c r="F21" s="2" t="s">
         <v>263</v>
       </c>
-      <c r="F21" s="2" t="s">
-        <v>253</v>
-      </c>
       <c r="G21" s="2" t="s">
-        <v>21</v>
+        <v>264</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>254</v>
+        <v>265</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="J21" s="2" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="K21" s="2" t="s">
-        <v>117</v>
+        <v>130</v>
       </c>
       <c r="L21" s="2" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="M21" s="2" t="s">
-        <v>258</v>
+        <v>269</v>
       </c>
       <c r="N21" s="2" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="O21" s="2" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
     </row>
     <row r="22" spans="1:15">
       <c r="A22" s="2" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>87</v>
+        <v>259</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>270</v>
+        <v>260</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>92</v>
+        <v>21</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="J22" s="2" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="K22" s="2" t="s">
-        <v>117</v>
+        <v>130</v>
       </c>
       <c r="L22" s="2" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="M22" s="2" t="s">
-        <v>83</v>
+        <v>280</v>
       </c>
       <c r="N22" s="2" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="O22" s="2" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
     </row>
     <row r="23" spans="1:15">
       <c r="A23" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>285</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H23" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="I23" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="J23" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="K23" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="L23" s="2" t="s">
+        <v>288</v>
+      </c>
+      <c r="M23" s="2" t="s">
         <v>280</v>
       </c>
-      <c r="B23" s="2" t="s">
-        <v>281</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>282</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>283</v>
-      </c>
-      <c r="E23" s="3" t="s">
-        <v>284</v>
-      </c>
-      <c r="F23" s="2" t="s">
-        <v>285</v>
-      </c>
-      <c r="G23" s="2" t="s">
-        <v>286</v>
-      </c>
-      <c r="H23" s="2" t="s">
-        <v>287</v>
-      </c>
-      <c r="I23" s="2" t="s">
-        <v>288</v>
-      </c>
-      <c r="J23" s="2" t="s">
+      <c r="N23" s="2" t="s">
         <v>289</v>
       </c>
-      <c r="K23" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="L23" s="2" t="s">
+      <c r="O23" s="2" t="s">
         <v>290</v>
-      </c>
-      <c r="M23" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="N23" s="2" t="s">
-        <v>291</v>
-      </c>
-      <c r="O23" s="2" t="s">
-        <v>292</v>
       </c>
     </row>
     <row r="24" spans="1:15">
       <c r="A24" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="D24" s="2" t="s">
         <v>293</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="E24" s="3" t="s">
         <v>294</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="F24" s="2" t="s">
         <v>295</v>
       </c>
-      <c r="D24" s="2" t="s">
+      <c r="G24" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="H24" s="2" t="s">
         <v>296</v>
       </c>
-      <c r="E24" s="3" t="s">
+      <c r="I24" s="2" t="s">
         <v>297</v>
       </c>
-      <c r="F24" s="2" t="s">
+      <c r="J24" s="2" t="s">
         <v>298</v>
       </c>
-      <c r="G24" s="2" t="s">
-        <v>286</v>
-      </c>
-      <c r="H24" s="2" t="s">
+      <c r="K24" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="L24" s="2" t="s">
         <v>299</v>
       </c>
-      <c r="I24" s="2" t="s">
+      <c r="M24" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="N24" s="2" t="s">
         <v>300</v>
       </c>
-      <c r="J24" s="2" t="s">
+      <c r="O24" s="2" t="s">
         <v>301</v>
-      </c>
-      <c r="K24" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="L24" s="2" t="s">
-        <v>302</v>
-      </c>
-      <c r="M24" s="2" t="s">
-        <v>303</v>
-      </c>
-      <c r="N24" s="2" t="s">
-        <v>304</v>
-      </c>
-      <c r="O24" s="2" t="s">
-        <v>305</v>
       </c>
     </row>
     <row r="25" spans="1:15">
       <c r="A25" s="2" t="s">
+        <v>302</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="E25" s="3" t="s">
         <v>306</v>
       </c>
-      <c r="B25" s="2" t="s">
-        <v>294</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>282</v>
-      </c>
-      <c r="D25" s="2" t="s">
+      <c r="F25" s="2" t="s">
         <v>307</v>
       </c>
-      <c r="E25" s="3" t="s">
+      <c r="G25" s="2" t="s">
         <v>308</v>
       </c>
-      <c r="F25" s="2" t="s">
+      <c r="H25" s="2" t="s">
         <v>309</v>
       </c>
-      <c r="G25" s="2" t="s">
-        <v>286</v>
-      </c>
-      <c r="H25" s="2" t="s">
+      <c r="I25" s="2" t="s">
         <v>310</v>
       </c>
-      <c r="I25" s="2" t="s">
+      <c r="J25" s="2" t="s">
         <v>311</v>
-      </c>
-      <c r="J25" s="2" t="s">
-        <v>312</v>
       </c>
       <c r="K25" s="2" t="s">
         <v>130</v>
       </c>
       <c r="L25" s="2" t="s">
+        <v>312</v>
+      </c>
+      <c r="M25" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="N25" s="2" t="s">
         <v>313</v>
       </c>
-      <c r="M25" s="2" t="s">
-        <v>303</v>
-      </c>
-      <c r="N25" s="2" t="s">
+      <c r="O25" s="2" t="s">
         <v>314</v>
-      </c>
-      <c r="O25" s="2" t="s">
-        <v>315</v>
       </c>
     </row>
     <row r="26" spans="1:15">
       <c r="A26" s="2" t="s">
+        <v>315</v>
+      </c>
+      <c r="B26" s="2" t="s">
         <v>316</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>294</v>
       </c>
       <c r="C26" s="2" t="s">
         <v>317</v>
@@ -3756,7 +3822,7 @@
         <v>320</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>92</v>
+        <v>308</v>
       </c>
       <c r="H26" s="2" t="s">
         <v>321</v>
@@ -3768,30 +3834,30 @@
         <v>323</v>
       </c>
       <c r="K26" s="2" t="s">
-        <v>117</v>
+        <v>130</v>
       </c>
       <c r="L26" s="2" t="s">
         <v>324</v>
       </c>
       <c r="M26" s="2" t="s">
-        <v>303</v>
+        <v>325</v>
       </c>
       <c r="N26" s="2" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="O26" s="2" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
     </row>
     <row r="27" spans="1:15">
       <c r="A27" s="2" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>328</v>
+        <v>316</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>282</v>
+        <v>304</v>
       </c>
       <c r="D27" s="2" t="s">
         <v>329</v>
@@ -3800,656 +3866,656 @@
         <v>330</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>309</v>
+        <v>331</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>286</v>
+        <v>308</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>310</v>
+        <v>332</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="J27" s="2" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="K27" s="2" t="s">
-        <v>117</v>
+        <v>130</v>
       </c>
       <c r="L27" s="2" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="M27" s="2" t="s">
-        <v>303</v>
+        <v>325</v>
       </c>
       <c r="N27" s="2" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="O27" s="2" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
     </row>
     <row r="28" spans="1:15">
       <c r="A28" s="2" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>328</v>
+        <v>316</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>286</v>
+        <v>92</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="I28" s="2" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="J28" s="2" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="K28" s="2" t="s">
         <v>117</v>
       </c>
       <c r="L28" s="2" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="M28" s="2" t="s">
-        <v>303</v>
+        <v>325</v>
       </c>
       <c r="N28" s="2" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="O28" s="2" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
     </row>
     <row r="29" spans="1:15">
       <c r="A29" s="2" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>101</v>
+        <v>350</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>282</v>
+        <v>304</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>309</v>
+        <v>331</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>286</v>
+        <v>308</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>350</v>
+        <v>332</v>
       </c>
       <c r="I29" s="2" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="J29" s="2" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="K29" s="2" t="s">
         <v>117</v>
       </c>
       <c r="L29" s="2" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="M29" s="2" t="s">
-        <v>303</v>
+        <v>325</v>
       </c>
       <c r="N29" s="2" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="O29" s="2" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
     </row>
     <row r="30" spans="1:15">
       <c r="A30" s="2" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>357</v>
+        <v>350</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>282</v>
+        <v>359</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>286</v>
+        <v>308</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="I30" s="2" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="J30" s="2" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="K30" s="2" t="s">
-        <v>130</v>
+        <v>117</v>
       </c>
       <c r="L30" s="2" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="M30" s="2" t="s">
-        <v>303</v>
+        <v>325</v>
       </c>
       <c r="N30" s="2" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="O30" s="2" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
     </row>
     <row r="31" spans="1:15">
       <c r="A31" s="2" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>328</v>
+        <v>101</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>368</v>
+        <v>304</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>371</v>
+        <v>331</v>
       </c>
       <c r="G31" s="2" t="s">
+        <v>308</v>
+      </c>
+      <c r="H31" s="2" t="s">
         <v>372</v>
       </c>
-      <c r="H31" s="2" t="s">
+      <c r="I31" s="2" t="s">
         <v>373</v>
       </c>
-      <c r="I31" s="2" t="s">
+      <c r="J31" s="2" t="s">
         <v>374</v>
       </c>
-      <c r="J31" s="2" t="s">
+      <c r="K31" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="L31" s="2" t="s">
         <v>375</v>
       </c>
-      <c r="K31" s="2" t="s">
+      <c r="M31" s="2" t="s">
+        <v>325</v>
+      </c>
+      <c r="N31" s="2" t="s">
         <v>376</v>
       </c>
-      <c r="L31" s="2" t="s">
+      <c r="O31" s="2" t="s">
         <v>377</v>
-      </c>
-      <c r="M31" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="N31" s="2" t="s">
-        <v>378</v>
-      </c>
-      <c r="O31" s="2" t="s">
-        <v>379</v>
       </c>
     </row>
     <row r="32" spans="1:15">
       <c r="A32" s="2" t="s">
+        <v>378</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>379</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="D32" s="2" t="s">
         <v>380</v>
       </c>
-      <c r="B32" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="C32" s="2" t="s">
+      <c r="E32" s="3" t="s">
         <v>381</v>
       </c>
-      <c r="D32" s="2" t="s">
+      <c r="F32" s="2" t="s">
         <v>382</v>
       </c>
-      <c r="E32" s="3" t="s">
+      <c r="G32" s="2" t="s">
+        <v>308</v>
+      </c>
+      <c r="H32" s="2" t="s">
         <v>383</v>
       </c>
-      <c r="F32" s="2" t="s">
+      <c r="I32" s="2" t="s">
         <v>384</v>
       </c>
-      <c r="G32" s="2" t="s">
+      <c r="J32" s="2" t="s">
         <v>385</v>
       </c>
-      <c r="H32" s="2" t="s">
+      <c r="K32" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="L32" s="2" t="s">
         <v>386</v>
       </c>
-      <c r="I32" s="2" t="s">
+      <c r="M32" s="2" t="s">
+        <v>325</v>
+      </c>
+      <c r="N32" s="2" t="s">
         <v>387</v>
       </c>
-      <c r="J32" s="2" t="s">
+      <c r="O32" s="2" t="s">
         <v>388</v>
-      </c>
-      <c r="K32" s="2" t="s">
-        <v>389</v>
-      </c>
-      <c r="L32" s="2" t="s">
-        <v>390</v>
-      </c>
-      <c r="M32" s="2" t="s">
-        <v>303</v>
-      </c>
-      <c r="N32" s="2" t="s">
-        <v>391</v>
-      </c>
-      <c r="O32" s="2" t="s">
-        <v>392</v>
       </c>
     </row>
     <row r="33" spans="1:15">
       <c r="A33" s="2" t="s">
+        <v>389</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>390</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>391</v>
+      </c>
+      <c r="E33" s="3" t="s">
+        <v>392</v>
+      </c>
+      <c r="F33" s="2" t="s">
         <v>393</v>
       </c>
-      <c r="B33" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="C33" s="2" t="s">
+      <c r="G33" s="2" t="s">
         <v>394</v>
       </c>
-      <c r="D33" s="2" t="s">
+      <c r="H33" s="2" t="s">
         <v>395</v>
       </c>
-      <c r="E33" s="3" t="s">
+      <c r="I33" s="2" t="s">
         <v>396</v>
       </c>
-      <c r="F33" s="2" t="s">
+      <c r="J33" s="2" t="s">
         <v>397</v>
       </c>
-      <c r="G33" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="H33" s="2" t="s">
+      <c r="K33" s="2" t="s">
         <v>398</v>
       </c>
-      <c r="I33" s="2" t="s">
+      <c r="L33" s="2" t="s">
         <v>399</v>
       </c>
-      <c r="J33" s="2" t="s">
+      <c r="M33" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="N33" s="2" t="s">
         <v>400</v>
       </c>
-      <c r="K33" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="L33" s="2" t="s">
+      <c r="O33" s="2" t="s">
         <v>401</v>
-      </c>
-      <c r="M33" s="2" t="s">
-        <v>402</v>
-      </c>
-      <c r="N33" s="2" t="s">
-        <v>403</v>
-      </c>
-      <c r="O33" s="2" t="s">
-        <v>404</v>
       </c>
     </row>
     <row r="34" spans="1:15">
       <c r="A34" s="2" t="s">
+        <v>402</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>403</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>404</v>
+      </c>
+      <c r="E34" s="3" t="s">
         <v>405</v>
       </c>
-      <c r="B34" s="2" t="s">
+      <c r="F34" s="2" t="s">
         <v>406</v>
       </c>
-      <c r="C34" s="2" t="s">
+      <c r="G34" s="2" t="s">
         <v>407</v>
       </c>
-      <c r="D34" s="2" t="s">
+      <c r="H34" s="2" t="s">
         <v>408</v>
       </c>
-      <c r="E34" s="3" t="s">
+      <c r="I34" s="2" t="s">
         <v>409</v>
       </c>
-      <c r="F34" s="2" t="s">
+      <c r="J34" s="2" t="s">
         <v>410</v>
       </c>
-      <c r="G34" s="2" t="s">
+      <c r="K34" s="2" t="s">
         <v>411</v>
       </c>
-      <c r="H34" s="2" t="s">
+      <c r="L34" s="2" t="s">
         <v>412</v>
       </c>
-      <c r="I34" s="2" t="s">
+      <c r="M34" s="2" t="s">
+        <v>325</v>
+      </c>
+      <c r="N34" s="2" t="s">
         <v>413</v>
       </c>
-      <c r="J34" s="2" t="s">
+      <c r="O34" s="2" t="s">
         <v>414</v>
-      </c>
-      <c r="K34" s="2" t="s">
-        <v>415</v>
-      </c>
-      <c r="L34" s="2" t="s">
-        <v>416</v>
-      </c>
-      <c r="M34" s="2" t="s">
-        <v>417</v>
-      </c>
-      <c r="N34" s="2" t="s">
-        <v>418</v>
-      </c>
-      <c r="O34" s="2" t="s">
-        <v>235</v>
       </c>
     </row>
     <row r="35" spans="1:15">
       <c r="A35" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>416</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>417</v>
+      </c>
+      <c r="E35" s="3" t="s">
+        <v>418</v>
+      </c>
+      <c r="F35" s="2" t="s">
         <v>419</v>
       </c>
-      <c r="B35" s="2" t="s">
+      <c r="G35" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="H35" s="2" t="s">
         <v>420</v>
       </c>
-      <c r="C35" s="2" t="s">
+      <c r="I35" s="2" t="s">
         <v>421</v>
       </c>
-      <c r="D35" s="2" t="s">
+      <c r="J35" s="2" t="s">
         <v>422</v>
       </c>
-      <c r="E35" s="3" t="s">
+      <c r="K35" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="L35" s="2" t="s">
         <v>423</v>
       </c>
-      <c r="F35" s="2" t="s">
+      <c r="M35" s="2" t="s">
         <v>424</v>
       </c>
-      <c r="G35" s="2" t="s">
+      <c r="N35" s="2" t="s">
         <v>425</v>
       </c>
-      <c r="H35" s="2" t="s">
+      <c r="O35" s="2" t="s">
         <v>426</v>
-      </c>
-      <c r="I35" s="2" t="s">
-        <v>427</v>
-      </c>
-      <c r="J35" s="2" t="s">
-        <v>428</v>
-      </c>
-      <c r="K35" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="L35" s="2" t="s">
-        <v>429</v>
-      </c>
-      <c r="M35" s="2" t="s">
-        <v>430</v>
-      </c>
-      <c r="N35" s="2" t="s">
-        <v>431</v>
-      </c>
-      <c r="O35" s="2" t="s">
-        <v>432</v>
       </c>
     </row>
     <row r="36" spans="1:15">
       <c r="A36" s="2" t="s">
+        <v>427</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>428</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>429</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>430</v>
+      </c>
+      <c r="E36" s="3" t="s">
+        <v>431</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="G36" s="2" t="s">
         <v>433</v>
       </c>
-      <c r="B36" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C36" s="2" t="s">
+      <c r="H36" s="2" t="s">
         <v>434</v>
       </c>
-      <c r="D36" s="2" t="s">
+      <c r="I36" s="2" t="s">
         <v>435</v>
       </c>
-      <c r="E36" s="3" t="s">
+      <c r="J36" s="2" t="s">
         <v>436</v>
       </c>
-      <c r="F36" s="2" t="s">
+      <c r="K36" s="2" t="s">
         <v>437</v>
       </c>
-      <c r="G36" s="2" t="s">
-        <v>425</v>
-      </c>
-      <c r="H36" s="2" t="s">
+      <c r="L36" s="2" t="s">
         <v>438</v>
       </c>
-      <c r="I36" s="2" t="s">
+      <c r="M36" s="2" t="s">
         <v>439</v>
       </c>
-      <c r="J36" s="2" t="s">
+      <c r="N36" s="2" t="s">
         <v>440</v>
       </c>
-      <c r="K36" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="L36" s="2" t="s">
-        <v>441</v>
-      </c>
-      <c r="M36" s="2" t="s">
-        <v>442</v>
-      </c>
-      <c r="N36" s="2" t="s">
-        <v>443</v>
-      </c>
       <c r="O36" s="2" t="s">
-        <v>432</v>
+        <v>257</v>
       </c>
     </row>
     <row r="37" spans="1:15">
       <c r="A37" s="2" t="s">
+        <v>441</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>442</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>443</v>
+      </c>
+      <c r="D37" s="2" t="s">
         <v>444</v>
       </c>
-      <c r="B37" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C37" s="2" t="s">
+      <c r="E37" s="3" t="s">
         <v>445</v>
       </c>
-      <c r="D37" s="2" t="s">
+      <c r="F37" s="2" t="s">
         <v>446</v>
       </c>
-      <c r="E37" s="3" t="s">
+      <c r="G37" s="2" t="s">
         <v>447</v>
       </c>
-      <c r="F37" s="2" t="s">
-        <v>253</v>
-      </c>
-      <c r="G37" s="2" t="s">
-        <v>21</v>
-      </c>
       <c r="H37" s="2" t="s">
-        <v>254</v>
+        <v>448</v>
       </c>
       <c r="I37" s="2" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="J37" s="2" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="K37" s="2" t="s">
-        <v>130</v>
+        <v>96</v>
       </c>
       <c r="L37" s="2" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="M37" s="2" t="s">
-        <v>83</v>
+        <v>452</v>
       </c>
       <c r="N37" s="2" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="O37" s="2" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
     </row>
     <row r="38" spans="1:15">
       <c r="A38" s="2" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="B38" s="2" t="s">
         <v>16</v>
       </c>
       <c r="C38" s="2" t="s">
+        <v>456</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>457</v>
+      </c>
+      <c r="E38" s="3" t="s">
+        <v>458</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>459</v>
+      </c>
+      <c r="G38" s="2" t="s">
+        <v>447</v>
+      </c>
+      <c r="H38" s="2" t="s">
+        <v>460</v>
+      </c>
+      <c r="I38" s="2" t="s">
+        <v>461</v>
+      </c>
+      <c r="J38" s="2" t="s">
+        <v>462</v>
+      </c>
+      <c r="K38" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="L38" s="2" t="s">
+        <v>463</v>
+      </c>
+      <c r="M38" s="2" t="s">
+        <v>464</v>
+      </c>
+      <c r="N38" s="2" t="s">
+        <v>465</v>
+      </c>
+      <c r="O38" s="2" t="s">
         <v>454</v>
-      </c>
-      <c r="D38" s="2" t="s">
-        <v>455</v>
-      </c>
-      <c r="E38" s="3" t="s">
-        <v>456</v>
-      </c>
-      <c r="F38" s="2" t="s">
-        <v>241</v>
-      </c>
-      <c r="G38" s="2" t="s">
-        <v>242</v>
-      </c>
-      <c r="H38" s="2" t="s">
-        <v>243</v>
-      </c>
-      <c r="I38" s="2" t="s">
-        <v>457</v>
-      </c>
-      <c r="J38" s="2" t="s">
-        <v>458</v>
-      </c>
-      <c r="K38" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="L38" s="2" t="s">
-        <v>459</v>
-      </c>
-      <c r="M38" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="N38" s="2" t="s">
-        <v>460</v>
-      </c>
-      <c r="O38" s="2" t="s">
-        <v>461</v>
       </c>
     </row>
     <row r="39" spans="1:15">
       <c r="A39" s="2" t="s">
-        <v>462</v>
+        <v>466</v>
       </c>
       <c r="B39" s="2" t="s">
         <v>16</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>454</v>
+        <v>467</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>463</v>
+        <v>468</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>464</v>
+        <v>469</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>465</v>
+        <v>275</v>
       </c>
       <c r="G39" s="2" t="s">
-        <v>92</v>
+        <v>21</v>
       </c>
       <c r="H39" s="2" t="s">
-        <v>254</v>
+        <v>276</v>
       </c>
       <c r="I39" s="2" t="s">
-        <v>466</v>
+        <v>470</v>
       </c>
       <c r="J39" s="2" t="s">
-        <v>467</v>
+        <v>471</v>
       </c>
       <c r="K39" s="2" t="s">
-        <v>117</v>
+        <v>130</v>
       </c>
       <c r="L39" s="2" t="s">
-        <v>468</v>
+        <v>472</v>
       </c>
       <c r="M39" s="2" t="s">
         <v>83</v>
       </c>
       <c r="N39" s="2" t="s">
-        <v>469</v>
+        <v>473</v>
       </c>
       <c r="O39" s="2" t="s">
-        <v>470</v>
+        <v>474</v>
       </c>
     </row>
     <row r="40" spans="1:15">
       <c r="A40" s="2" t="s">
-        <v>471</v>
+        <v>475</v>
       </c>
       <c r="B40" s="2" t="s">
         <v>16</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>472</v>
+        <v>476</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>474</v>
+        <v>478</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>475</v>
+        <v>263</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>92</v>
+        <v>264</v>
       </c>
       <c r="H40" s="2" t="s">
-        <v>476</v>
+        <v>265</v>
       </c>
       <c r="I40" s="2" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="J40" s="2" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="K40" s="2" t="s">
-        <v>117</v>
+        <v>130</v>
       </c>
       <c r="L40" s="2" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="M40" s="2" t="s">
-        <v>480</v>
+        <v>83</v>
       </c>
       <c r="N40" s="2" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="O40" s="2" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
     </row>
     <row r="41" spans="1:15">
       <c r="A41" s="2" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="B41" s="2" t="s">
         <v>16</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>484</v>
+        <v>476</v>
       </c>
       <c r="D41" s="2" t="s">
         <v>485</v>
@@ -4461,42 +4527,42 @@
         <v>487</v>
       </c>
       <c r="G41" s="2" t="s">
-        <v>77</v>
+        <v>92</v>
       </c>
       <c r="H41" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="I41" s="2" t="s">
         <v>488</v>
       </c>
-      <c r="I41" s="2" t="s">
+      <c r="J41" s="2" t="s">
         <v>489</v>
       </c>
-      <c r="J41" s="2" t="s">
+      <c r="K41" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="L41" s="2" t="s">
         <v>490</v>
       </c>
-      <c r="K41" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="L41" s="2" t="s">
+      <c r="M41" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="N41" s="2" t="s">
         <v>491</v>
       </c>
-      <c r="M41" s="2" t="s">
-        <v>303</v>
-      </c>
-      <c r="N41" s="2" t="s">
+      <c r="O41" s="2" t="s">
         <v>492</v>
-      </c>
-      <c r="O41" s="2" t="s">
-        <v>493</v>
       </c>
     </row>
     <row r="42" spans="1:15">
       <c r="A42" s="2" t="s">
+        <v>493</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C42" s="2" t="s">
         <v>494</v>
-      </c>
-      <c r="B42" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="C42" s="2" t="s">
-        <v>484</v>
       </c>
       <c r="D42" s="2" t="s">
         <v>495</v>
@@ -4508,7 +4574,7 @@
         <v>497</v>
       </c>
       <c r="G42" s="2" t="s">
-        <v>77</v>
+        <v>92</v>
       </c>
       <c r="H42" s="2" t="s">
         <v>498</v>
@@ -4520,107 +4586,107 @@
         <v>500</v>
       </c>
       <c r="K42" s="2" t="s">
-        <v>130</v>
+        <v>117</v>
       </c>
       <c r="L42" s="2" t="s">
         <v>501</v>
       </c>
       <c r="M42" s="2" t="s">
-        <v>42</v>
+        <v>502</v>
       </c>
       <c r="N42" s="2" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="O42" s="2" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
     </row>
     <row r="43" spans="1:15">
       <c r="A43" s="2" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>147</v>
+        <v>16</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="F43" s="2" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="G43" s="2" t="s">
-        <v>509</v>
+        <v>77</v>
       </c>
       <c r="H43" s="2" t="s">
-        <v>412</v>
+        <v>510</v>
       </c>
       <c r="I43" s="2" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="J43" s="2" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="K43" s="2" t="s">
-        <v>415</v>
+        <v>130</v>
       </c>
       <c r="L43" s="2" t="s">
-        <v>416</v>
+        <v>513</v>
       </c>
       <c r="M43" s="2" t="s">
-        <v>512</v>
+        <v>325</v>
       </c>
       <c r="N43" s="2" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="O43" s="2" t="s">
-        <v>235</v>
+        <v>515</v>
       </c>
     </row>
     <row r="44" spans="1:15">
       <c r="A44" s="2" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="B44" s="2" t="s">
         <v>87</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>515</v>
+        <v>506</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="E44" s="3" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="G44" s="2" t="s">
-        <v>21</v>
+        <v>77</v>
       </c>
       <c r="H44" s="2" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="I44" s="2" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="J44" s="2" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="K44" s="2" t="s">
-        <v>117</v>
+        <v>130</v>
       </c>
       <c r="L44" s="2" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="M44" s="2" t="s">
-        <v>523</v>
+        <v>42</v>
       </c>
       <c r="N44" s="2" t="s">
         <v>524</v>
@@ -4634,1131 +4700,1225 @@
         <v>526</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>87</v>
+        <v>147</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>515</v>
+        <v>527</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="F45" s="2" t="s">
-        <v>518</v>
+        <v>530</v>
       </c>
       <c r="G45" s="2" t="s">
-        <v>21</v>
+        <v>531</v>
       </c>
       <c r="H45" s="2" t="s">
-        <v>519</v>
+        <v>434</v>
       </c>
       <c r="I45" s="2" t="s">
-        <v>529</v>
+        <v>532</v>
       </c>
       <c r="J45" s="2" t="s">
-        <v>530</v>
+        <v>533</v>
       </c>
       <c r="K45" s="2" t="s">
-        <v>130</v>
+        <v>437</v>
       </c>
       <c r="L45" s="2" t="s">
-        <v>531</v>
+        <v>438</v>
       </c>
       <c r="M45" s="2" t="s">
-        <v>523</v>
+        <v>534</v>
       </c>
       <c r="N45" s="2" t="s">
-        <v>532</v>
+        <v>535</v>
       </c>
       <c r="O45" s="2" t="s">
-        <v>533</v>
+        <v>257</v>
       </c>
     </row>
     <row r="46" spans="1:15">
       <c r="A46" s="2" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
       <c r="B46" s="2" t="s">
         <v>87</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>515</v>
+        <v>537</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>535</v>
+        <v>538</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>536</v>
+        <v>539</v>
       </c>
       <c r="F46" s="2" t="s">
-        <v>518</v>
+        <v>540</v>
       </c>
       <c r="G46" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H46" s="2" t="s">
-        <v>519</v>
+        <v>541</v>
       </c>
       <c r="I46" s="2" t="s">
-        <v>537</v>
+        <v>542</v>
       </c>
       <c r="J46" s="2" t="s">
-        <v>538</v>
+        <v>543</v>
       </c>
       <c r="K46" s="2" t="s">
         <v>117</v>
       </c>
       <c r="L46" s="2" t="s">
-        <v>539</v>
+        <v>544</v>
       </c>
       <c r="M46" s="2" t="s">
-        <v>523</v>
+        <v>545</v>
       </c>
       <c r="N46" s="2" t="s">
-        <v>540</v>
+        <v>546</v>
       </c>
       <c r="O46" s="2" t="s">
-        <v>541</v>
+        <v>547</v>
       </c>
     </row>
     <row r="47" spans="1:15">
       <c r="A47" s="2" t="s">
-        <v>542</v>
+        <v>548</v>
       </c>
       <c r="B47" s="2" t="s">
         <v>87</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>515</v>
+        <v>537</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>543</v>
+        <v>549</v>
       </c>
       <c r="E47" s="3" t="s">
-        <v>544</v>
+        <v>550</v>
       </c>
       <c r="F47" s="2" t="s">
+        <v>540</v>
+      </c>
+      <c r="G47" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H47" s="2" t="s">
+        <v>541</v>
+      </c>
+      <c r="I47" s="2" t="s">
+        <v>551</v>
+      </c>
+      <c r="J47" s="2" t="s">
+        <v>552</v>
+      </c>
+      <c r="K47" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="L47" s="2" t="s">
+        <v>553</v>
+      </c>
+      <c r="M47" s="2" t="s">
         <v>545</v>
       </c>
-      <c r="G47" s="2" t="s">
-        <v>242</v>
-      </c>
-      <c r="H47" s="2" t="s">
-        <v>519</v>
-      </c>
-      <c r="I47" s="2" t="s">
-        <v>546</v>
-      </c>
-      <c r="J47" s="2" t="s">
-        <v>547</v>
-      </c>
-      <c r="K47" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="L47" s="2" t="s">
-        <v>548</v>
-      </c>
-      <c r="M47" s="2" t="s">
-        <v>523</v>
-      </c>
       <c r="N47" s="2" t="s">
-        <v>549</v>
+        <v>554</v>
       </c>
       <c r="O47" s="2" t="s">
-        <v>550</v>
+        <v>555</v>
       </c>
     </row>
     <row r="48" spans="1:15">
       <c r="A48" s="2" t="s">
-        <v>551</v>
+        <v>556</v>
       </c>
       <c r="B48" s="2" t="s">
         <v>87</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>515</v>
+        <v>537</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>552</v>
+        <v>557</v>
       </c>
       <c r="E48" s="3" t="s">
-        <v>553</v>
+        <v>558</v>
       </c>
       <c r="F48" s="2" t="s">
-        <v>518</v>
+        <v>540</v>
       </c>
       <c r="G48" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H48" s="2" t="s">
-        <v>519</v>
+        <v>541</v>
       </c>
       <c r="I48" s="2" t="s">
-        <v>554</v>
+        <v>559</v>
       </c>
       <c r="J48" s="2" t="s">
-        <v>555</v>
+        <v>560</v>
       </c>
       <c r="K48" s="2" t="s">
         <v>117</v>
       </c>
       <c r="L48" s="2" t="s">
-        <v>556</v>
+        <v>561</v>
       </c>
       <c r="M48" s="2" t="s">
-        <v>523</v>
+        <v>545</v>
       </c>
       <c r="N48" s="2" t="s">
-        <v>557</v>
+        <v>562</v>
       </c>
       <c r="O48" s="2" t="s">
-        <v>558</v>
+        <v>563</v>
       </c>
     </row>
     <row r="49" spans="1:15">
       <c r="A49" s="2" t="s">
-        <v>559</v>
+        <v>564</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>237</v>
+        <v>87</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>515</v>
+        <v>537</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>560</v>
+        <v>565</v>
       </c>
       <c r="E49" s="3" t="s">
-        <v>561</v>
+        <v>566</v>
       </c>
       <c r="F49" s="2" t="s">
-        <v>518</v>
+        <v>567</v>
       </c>
       <c r="G49" s="2" t="s">
-        <v>21</v>
+        <v>264</v>
       </c>
       <c r="H49" s="2" t="s">
-        <v>519</v>
+        <v>541</v>
       </c>
       <c r="I49" s="2" t="s">
-        <v>562</v>
+        <v>568</v>
       </c>
       <c r="J49" s="2" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
       <c r="K49" s="2" t="s">
-        <v>117</v>
+        <v>96</v>
       </c>
       <c r="L49" s="2" t="s">
-        <v>564</v>
+        <v>570</v>
       </c>
       <c r="M49" s="2" t="s">
-        <v>523</v>
+        <v>545</v>
       </c>
       <c r="N49" s="2" t="s">
-        <v>565</v>
+        <v>571</v>
       </c>
       <c r="O49" s="2" t="s">
-        <v>566</v>
+        <v>572</v>
       </c>
     </row>
     <row r="50" spans="1:15">
       <c r="A50" s="2" t="s">
-        <v>567</v>
+        <v>573</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>237</v>
+        <v>87</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>515</v>
+        <v>537</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>568</v>
+        <v>574</v>
       </c>
       <c r="E50" s="3" t="s">
-        <v>569</v>
+        <v>575</v>
       </c>
       <c r="F50" s="2" t="s">
-        <v>518</v>
+        <v>540</v>
       </c>
       <c r="G50" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H50" s="2" t="s">
-        <v>519</v>
+        <v>541</v>
       </c>
       <c r="I50" s="2" t="s">
-        <v>570</v>
+        <v>576</v>
       </c>
       <c r="J50" s="2" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="K50" s="2" t="s">
-        <v>130</v>
+        <v>117</v>
       </c>
       <c r="L50" s="2" t="s">
-        <v>572</v>
+        <v>578</v>
       </c>
       <c r="M50" s="2" t="s">
-        <v>523</v>
+        <v>545</v>
       </c>
       <c r="N50" s="2" t="s">
-        <v>573</v>
+        <v>579</v>
       </c>
       <c r="O50" s="2" t="s">
-        <v>574</v>
+        <v>580</v>
       </c>
     </row>
     <row r="51" spans="1:15">
       <c r="A51" s="2" t="s">
-        <v>575</v>
+        <v>581</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>237</v>
+        <v>259</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>515</v>
+        <v>537</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>576</v>
+        <v>582</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>577</v>
+        <v>583</v>
       </c>
       <c r="F51" s="2" t="s">
-        <v>518</v>
+        <v>540</v>
       </c>
       <c r="G51" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H51" s="2" t="s">
-        <v>519</v>
+        <v>541</v>
       </c>
       <c r="I51" s="2" t="s">
-        <v>578</v>
+        <v>584</v>
       </c>
       <c r="J51" s="2" t="s">
-        <v>579</v>
+        <v>585</v>
       </c>
       <c r="K51" s="2" t="s">
         <v>117</v>
       </c>
       <c r="L51" s="2" t="s">
-        <v>580</v>
+        <v>586</v>
       </c>
       <c r="M51" s="2" t="s">
-        <v>523</v>
+        <v>545</v>
       </c>
       <c r="N51" s="2" t="s">
-        <v>581</v>
+        <v>587</v>
       </c>
       <c r="O51" s="2" t="s">
-        <v>582</v>
+        <v>588</v>
       </c>
     </row>
     <row r="52" spans="1:15">
       <c r="A52" s="2" t="s">
-        <v>583</v>
+        <v>589</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>237</v>
+        <v>259</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>515</v>
+        <v>537</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>584</v>
+        <v>590</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>585</v>
+        <v>591</v>
       </c>
       <c r="F52" s="2" t="s">
-        <v>518</v>
+        <v>540</v>
       </c>
       <c r="G52" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H52" s="2" t="s">
-        <v>519</v>
+        <v>541</v>
       </c>
       <c r="I52" s="2" t="s">
-        <v>586</v>
+        <v>592</v>
       </c>
       <c r="J52" s="2" t="s">
-        <v>587</v>
+        <v>593</v>
       </c>
       <c r="K52" s="2" t="s">
         <v>130</v>
       </c>
       <c r="L52" s="2" t="s">
-        <v>588</v>
+        <v>594</v>
       </c>
       <c r="M52" s="2" t="s">
-        <v>523</v>
+        <v>545</v>
       </c>
       <c r="N52" s="2" t="s">
-        <v>589</v>
+        <v>595</v>
       </c>
       <c r="O52" s="2" t="s">
-        <v>590</v>
+        <v>596</v>
       </c>
     </row>
     <row r="53" spans="1:15">
       <c r="A53" s="2" t="s">
-        <v>591</v>
+        <v>597</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>237</v>
+        <v>259</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>515</v>
+        <v>537</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>592</v>
+        <v>598</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>593</v>
+        <v>599</v>
       </c>
       <c r="F53" s="2" t="s">
-        <v>518</v>
+        <v>540</v>
       </c>
       <c r="G53" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H53" s="2" t="s">
-        <v>519</v>
+        <v>541</v>
       </c>
       <c r="I53" s="2" t="s">
-        <v>594</v>
+        <v>600</v>
       </c>
       <c r="J53" s="2" t="s">
-        <v>595</v>
+        <v>601</v>
       </c>
       <c r="K53" s="2" t="s">
-        <v>130</v>
+        <v>117</v>
       </c>
       <c r="L53" s="2" t="s">
-        <v>596</v>
+        <v>602</v>
       </c>
       <c r="M53" s="2" t="s">
-        <v>523</v>
+        <v>545</v>
       </c>
       <c r="N53" s="2" t="s">
-        <v>597</v>
+        <v>603</v>
       </c>
       <c r="O53" s="2" t="s">
-        <v>598</v>
+        <v>604</v>
       </c>
     </row>
     <row r="54" spans="1:15">
       <c r="A54" s="2" t="s">
-        <v>599</v>
+        <v>605</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>237</v>
+        <v>259</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>515</v>
+        <v>537</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>600</v>
+        <v>606</v>
       </c>
       <c r="E54" s="3" t="s">
-        <v>601</v>
+        <v>607</v>
       </c>
       <c r="F54" s="2" t="s">
-        <v>518</v>
+        <v>540</v>
       </c>
       <c r="G54" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H54" s="2" t="s">
-        <v>519</v>
+        <v>541</v>
       </c>
       <c r="I54" s="2" t="s">
-        <v>602</v>
+        <v>608</v>
       </c>
       <c r="J54" s="2" t="s">
-        <v>603</v>
+        <v>609</v>
       </c>
       <c r="K54" s="2" t="s">
-        <v>117</v>
+        <v>130</v>
       </c>
       <c r="L54" s="2" t="s">
-        <v>604</v>
+        <v>610</v>
       </c>
       <c r="M54" s="2" t="s">
-        <v>523</v>
+        <v>545</v>
       </c>
       <c r="N54" s="2" t="s">
-        <v>605</v>
+        <v>611</v>
       </c>
       <c r="O54" s="2" t="s">
-        <v>606</v>
+        <v>612</v>
       </c>
     </row>
     <row r="55" spans="1:15">
       <c r="A55" s="2" t="s">
-        <v>607</v>
+        <v>613</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>237</v>
+        <v>259</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>515</v>
+        <v>537</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>608</v>
+        <v>614</v>
       </c>
       <c r="E55" s="3" t="s">
-        <v>609</v>
+        <v>615</v>
       </c>
       <c r="F55" s="2" t="s">
-        <v>518</v>
+        <v>540</v>
       </c>
       <c r="G55" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H55" s="2" t="s">
-        <v>519</v>
+        <v>541</v>
       </c>
       <c r="I55" s="2" t="s">
-        <v>610</v>
+        <v>616</v>
       </c>
       <c r="J55" s="2" t="s">
-        <v>611</v>
+        <v>617</v>
       </c>
       <c r="K55" s="2" t="s">
         <v>130</v>
       </c>
       <c r="L55" s="2" t="s">
-        <v>596</v>
+        <v>618</v>
       </c>
       <c r="M55" s="2" t="s">
-        <v>523</v>
+        <v>545</v>
       </c>
       <c r="N55" s="2" t="s">
-        <v>612</v>
+        <v>619</v>
       </c>
       <c r="O55" s="2" t="s">
-        <v>613</v>
+        <v>620</v>
       </c>
     </row>
     <row r="56" spans="1:15">
       <c r="A56" s="2" t="s">
-        <v>614</v>
+        <v>621</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>237</v>
+        <v>259</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>515</v>
+        <v>537</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>615</v>
+        <v>622</v>
       </c>
       <c r="E56" s="3" t="s">
-        <v>616</v>
+        <v>623</v>
       </c>
       <c r="F56" s="2" t="s">
-        <v>518</v>
+        <v>540</v>
       </c>
       <c r="G56" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H56" s="2" t="s">
-        <v>519</v>
+        <v>541</v>
       </c>
       <c r="I56" s="2" t="s">
-        <v>617</v>
+        <v>624</v>
       </c>
       <c r="J56" s="2" t="s">
-        <v>618</v>
+        <v>625</v>
       </c>
       <c r="K56" s="2" t="s">
-        <v>130</v>
+        <v>117</v>
       </c>
       <c r="L56" s="2" t="s">
-        <v>619</v>
+        <v>626</v>
       </c>
       <c r="M56" s="2" t="s">
-        <v>523</v>
+        <v>545</v>
       </c>
       <c r="N56" s="2" t="s">
-        <v>620</v>
+        <v>627</v>
       </c>
       <c r="O56" s="2" t="s">
-        <v>621</v>
+        <v>628</v>
       </c>
     </row>
     <row r="57" spans="1:15">
       <c r="A57" s="2" t="s">
-        <v>622</v>
+        <v>629</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>237</v>
+        <v>259</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>515</v>
+        <v>537</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>623</v>
+        <v>630</v>
       </c>
       <c r="E57" s="3" t="s">
-        <v>624</v>
+        <v>631</v>
       </c>
       <c r="F57" s="2" t="s">
-        <v>518</v>
+        <v>540</v>
       </c>
       <c r="G57" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H57" s="2" t="s">
-        <v>519</v>
+        <v>541</v>
       </c>
       <c r="I57" s="2" t="s">
-        <v>625</v>
+        <v>632</v>
       </c>
       <c r="J57" s="2" t="s">
-        <v>626</v>
+        <v>633</v>
       </c>
       <c r="K57" s="2" t="s">
-        <v>117</v>
+        <v>130</v>
       </c>
       <c r="L57" s="2" t="s">
-        <v>627</v>
+        <v>618</v>
       </c>
       <c r="M57" s="2" t="s">
-        <v>523</v>
+        <v>545</v>
       </c>
       <c r="N57" s="2" t="s">
-        <v>628</v>
+        <v>634</v>
       </c>
       <c r="O57" s="2" t="s">
-        <v>629</v>
+        <v>635</v>
       </c>
     </row>
     <row r="58" spans="1:15">
       <c r="A58" s="2" t="s">
-        <v>630</v>
+        <v>636</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>237</v>
+        <v>259</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>515</v>
+        <v>537</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>631</v>
+        <v>637</v>
       </c>
       <c r="E58" s="3" t="s">
-        <v>632</v>
+        <v>638</v>
       </c>
       <c r="F58" s="2" t="s">
-        <v>518</v>
+        <v>540</v>
       </c>
       <c r="G58" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H58" s="2" t="s">
-        <v>519</v>
+        <v>541</v>
       </c>
       <c r="I58" s="2" t="s">
-        <v>633</v>
+        <v>639</v>
       </c>
       <c r="J58" s="2" t="s">
-        <v>634</v>
+        <v>640</v>
       </c>
       <c r="K58" s="2" t="s">
         <v>130</v>
       </c>
       <c r="L58" s="2" t="s">
-        <v>596</v>
+        <v>641</v>
       </c>
       <c r="M58" s="2" t="s">
-        <v>523</v>
+        <v>545</v>
       </c>
       <c r="N58" s="2" t="s">
-        <v>635</v>
+        <v>642</v>
       </c>
       <c r="O58" s="2" t="s">
-        <v>636</v>
+        <v>643</v>
       </c>
     </row>
     <row r="59" spans="1:15">
       <c r="A59" s="2" t="s">
-        <v>637</v>
+        <v>644</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>237</v>
+        <v>259</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>515</v>
+        <v>537</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>638</v>
+        <v>645</v>
       </c>
       <c r="E59" s="3" t="s">
-        <v>639</v>
+        <v>646</v>
       </c>
       <c r="F59" s="2" t="s">
-        <v>518</v>
+        <v>540</v>
       </c>
       <c r="G59" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H59" s="2" t="s">
-        <v>519</v>
+        <v>541</v>
       </c>
       <c r="I59" s="2" t="s">
-        <v>640</v>
+        <v>647</v>
       </c>
       <c r="J59" s="2" t="s">
-        <v>641</v>
+        <v>648</v>
       </c>
       <c r="K59" s="2" t="s">
         <v>117</v>
       </c>
       <c r="L59" s="2" t="s">
-        <v>642</v>
+        <v>649</v>
       </c>
       <c r="M59" s="2" t="s">
-        <v>523</v>
+        <v>545</v>
       </c>
       <c r="N59" s="2" t="s">
-        <v>643</v>
+        <v>650</v>
       </c>
       <c r="O59" s="2" t="s">
-        <v>644</v>
+        <v>651</v>
       </c>
     </row>
     <row r="60" spans="1:15">
       <c r="A60" s="2" t="s">
-        <v>645</v>
+        <v>652</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>237</v>
+        <v>259</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>515</v>
+        <v>537</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>646</v>
+        <v>653</v>
       </c>
       <c r="E60" s="3" t="s">
-        <v>647</v>
+        <v>654</v>
       </c>
       <c r="F60" s="2" t="s">
-        <v>518</v>
+        <v>540</v>
       </c>
       <c r="G60" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H60" s="2" t="s">
-        <v>519</v>
+        <v>541</v>
       </c>
       <c r="I60" s="2" t="s">
-        <v>648</v>
+        <v>655</v>
       </c>
       <c r="J60" s="2" t="s">
-        <v>649</v>
+        <v>656</v>
       </c>
       <c r="K60" s="2" t="s">
         <v>130</v>
       </c>
       <c r="L60" s="2" t="s">
-        <v>650</v>
+        <v>618</v>
       </c>
       <c r="M60" s="2" t="s">
-        <v>523</v>
+        <v>545</v>
       </c>
       <c r="N60" s="2" t="s">
-        <v>651</v>
+        <v>657</v>
       </c>
       <c r="O60" s="2" t="s">
-        <v>652</v>
+        <v>658</v>
       </c>
     </row>
     <row r="61" spans="1:15">
       <c r="A61" s="2" t="s">
-        <v>653</v>
+        <v>659</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>183</v>
+        <v>259</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>515</v>
+        <v>537</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>654</v>
+        <v>660</v>
       </c>
       <c r="E61" s="3" t="s">
-        <v>655</v>
+        <v>661</v>
       </c>
       <c r="F61" s="2" t="s">
-        <v>518</v>
+        <v>540</v>
       </c>
       <c r="G61" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H61" s="2" t="s">
-        <v>519</v>
+        <v>541</v>
       </c>
       <c r="I61" s="2" t="s">
-        <v>656</v>
+        <v>662</v>
       </c>
       <c r="J61" s="2" t="s">
-        <v>657</v>
+        <v>663</v>
       </c>
       <c r="K61" s="2" t="s">
-        <v>130</v>
+        <v>117</v>
       </c>
       <c r="L61" s="2" t="s">
-        <v>658</v>
+        <v>664</v>
       </c>
       <c r="M61" s="2" t="s">
-        <v>523</v>
+        <v>545</v>
       </c>
       <c r="N61" s="2" t="s">
-        <v>659</v>
+        <v>665</v>
       </c>
       <c r="O61" s="2" t="s">
-        <v>660</v>
+        <v>666</v>
       </c>
     </row>
     <row r="62" spans="1:15">
       <c r="A62" s="2" t="s">
-        <v>661</v>
+        <v>667</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>662</v>
+        <v>259</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>515</v>
+        <v>537</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>663</v>
+        <v>668</v>
       </c>
       <c r="E62" s="3" t="s">
-        <v>664</v>
+        <v>669</v>
       </c>
       <c r="F62" s="2" t="s">
-        <v>518</v>
+        <v>540</v>
       </c>
       <c r="G62" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H62" s="2" t="s">
-        <v>519</v>
+        <v>541</v>
       </c>
       <c r="I62" s="2" t="s">
-        <v>665</v>
+        <v>670</v>
       </c>
       <c r="J62" s="2" t="s">
-        <v>666</v>
+        <v>671</v>
       </c>
       <c r="K62" s="2" t="s">
-        <v>117</v>
+        <v>130</v>
       </c>
       <c r="L62" s="2" t="s">
-        <v>667</v>
+        <v>672</v>
       </c>
       <c r="M62" s="2" t="s">
-        <v>523</v>
+        <v>545</v>
       </c>
       <c r="N62" s="2" t="s">
-        <v>668</v>
+        <v>673</v>
       </c>
       <c r="O62" s="2" t="s">
-        <v>669</v>
+        <v>674</v>
       </c>
     </row>
     <row r="63" spans="1:15">
       <c r="A63" s="2" t="s">
-        <v>670</v>
+        <v>675</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>237</v>
+        <v>183</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>515</v>
+        <v>537</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>671</v>
+        <v>676</v>
       </c>
       <c r="E63" s="3" t="s">
-        <v>672</v>
+        <v>677</v>
       </c>
       <c r="F63" s="2" t="s">
-        <v>518</v>
+        <v>540</v>
       </c>
       <c r="G63" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H63" s="2" t="s">
-        <v>519</v>
+        <v>541</v>
       </c>
       <c r="I63" s="2" t="s">
-        <v>673</v>
+        <v>678</v>
       </c>
       <c r="J63" s="2" t="s">
-        <v>674</v>
+        <v>679</v>
       </c>
       <c r="K63" s="2" t="s">
         <v>130</v>
       </c>
       <c r="L63" s="2" t="s">
-        <v>675</v>
+        <v>680</v>
       </c>
       <c r="M63" s="2" t="s">
-        <v>523</v>
+        <v>545</v>
       </c>
       <c r="N63" s="2" t="s">
-        <v>676</v>
+        <v>681</v>
       </c>
       <c r="O63" s="2" t="s">
-        <v>677</v>
+        <v>682</v>
       </c>
     </row>
     <row r="64" spans="1:15">
       <c r="A64" s="2" t="s">
-        <v>678</v>
+        <v>683</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>237</v>
+        <v>684</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>515</v>
+        <v>537</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>679</v>
+        <v>685</v>
       </c>
       <c r="E64" s="3" t="s">
-        <v>680</v>
+        <v>686</v>
       </c>
       <c r="F64" s="2" t="s">
+        <v>540</v>
+      </c>
+      <c r="G64" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H64" s="2" t="s">
+        <v>541</v>
+      </c>
+      <c r="I64" s="2" t="s">
+        <v>687</v>
+      </c>
+      <c r="J64" s="2" t="s">
+        <v>688</v>
+      </c>
+      <c r="K64" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="L64" s="2" t="s">
+        <v>689</v>
+      </c>
+      <c r="M64" s="2" t="s">
         <v>545</v>
       </c>
-      <c r="G64" s="2" t="s">
-        <v>242</v>
-      </c>
-      <c r="H64" s="2" t="s">
-        <v>519</v>
-      </c>
-      <c r="I64" s="2" t="s">
-        <v>681</v>
-      </c>
-      <c r="J64" s="2" t="s">
-        <v>682</v>
-      </c>
-      <c r="K64" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="L64" s="2" t="s">
-        <v>246</v>
-      </c>
-      <c r="M64" s="2" t="s">
-        <v>523</v>
-      </c>
       <c r="N64" s="2" t="s">
-        <v>683</v>
+        <v>690</v>
       </c>
       <c r="O64" s="2" t="s">
-        <v>684</v>
+        <v>691</v>
       </c>
     </row>
     <row r="65" spans="1:15">
       <c r="A65" s="2" t="s">
-        <v>685</v>
+        <v>692</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>237</v>
+        <v>259</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>515</v>
+        <v>537</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>686</v>
+        <v>693</v>
       </c>
       <c r="E65" s="3" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
       <c r="F65" s="2" t="s">
-        <v>518</v>
+        <v>540</v>
       </c>
       <c r="G65" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H65" s="2" t="s">
-        <v>519</v>
+        <v>541</v>
       </c>
       <c r="I65" s="2" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
       <c r="J65" s="2" t="s">
-        <v>689</v>
+        <v>696</v>
       </c>
       <c r="K65" s="2" t="s">
         <v>130</v>
       </c>
       <c r="L65" s="2" t="s">
-        <v>690</v>
+        <v>697</v>
       </c>
       <c r="M65" s="2" t="s">
-        <v>523</v>
+        <v>545</v>
       </c>
       <c r="N65" s="2" t="s">
-        <v>691</v>
+        <v>698</v>
       </c>
       <c r="O65" s="2" t="s">
-        <v>692</v>
+        <v>699</v>
       </c>
     </row>
     <row r="66" spans="1:15">
       <c r="A66" s="2" t="s">
-        <v>693</v>
+        <v>700</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>183</v>
+        <v>259</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>515</v>
+        <v>537</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>694</v>
+        <v>701</v>
       </c>
       <c r="E66" s="3" t="s">
-        <v>695</v>
+        <v>702</v>
       </c>
       <c r="F66" s="2" t="s">
-        <v>518</v>
+        <v>567</v>
       </c>
       <c r="G66" s="2" t="s">
-        <v>21</v>
+        <v>264</v>
       </c>
       <c r="H66" s="2" t="s">
-        <v>519</v>
+        <v>541</v>
       </c>
       <c r="I66" s="2" t="s">
-        <v>696</v>
+        <v>703</v>
       </c>
       <c r="J66" s="2" t="s">
-        <v>697</v>
+        <v>704</v>
       </c>
       <c r="K66" s="2" t="s">
         <v>130</v>
       </c>
       <c r="L66" s="2" t="s">
-        <v>698</v>
+        <v>268</v>
       </c>
       <c r="M66" s="2" t="s">
-        <v>523</v>
+        <v>545</v>
       </c>
       <c r="N66" s="2" t="s">
-        <v>699</v>
+        <v>705</v>
       </c>
       <c r="O66" s="2" t="s">
-        <v>700</v>
+        <v>706</v>
       </c>
     </row>
     <row r="67" spans="1:15">
       <c r="A67" s="2" t="s">
-        <v>701</v>
+        <v>707</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>662</v>
+        <v>259</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>515</v>
+        <v>537</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>702</v>
+        <v>708</v>
       </c>
       <c r="E67" s="3" t="s">
-        <v>703</v>
+        <v>709</v>
       </c>
       <c r="F67" s="2" t="s">
-        <v>518</v>
+        <v>540</v>
       </c>
       <c r="G67" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H67" s="2" t="s">
-        <v>519</v>
+        <v>541</v>
       </c>
       <c r="I67" s="2" t="s">
-        <v>704</v>
+        <v>710</v>
       </c>
       <c r="J67" s="2" t="s">
-        <v>705</v>
+        <v>711</v>
       </c>
       <c r="K67" s="2" t="s">
-        <v>117</v>
+        <v>130</v>
       </c>
       <c r="L67" s="2" t="s">
-        <v>706</v>
+        <v>712</v>
       </c>
       <c r="M67" s="2" t="s">
-        <v>523</v>
+        <v>545</v>
       </c>
       <c r="N67" s="2" t="s">
-        <v>707</v>
+        <v>713</v>
       </c>
       <c r="O67" s="2" t="s">
-        <v>708</v>
+        <v>714</v>
       </c>
     </row>
     <row r="68" spans="1:15">
       <c r="A68" s="2" t="s">
-        <v>709</v>
+        <v>715</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>662</v>
+        <v>183</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>515</v>
+        <v>537</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>710</v>
+        <v>716</v>
       </c>
       <c r="E68" s="3" t="s">
-        <v>711</v>
+        <v>717</v>
       </c>
       <c r="F68" s="2" t="s">
-        <v>518</v>
+        <v>540</v>
       </c>
       <c r="G68" s="2" t="s">
         <v>21</v>
       </c>
       <c r="H68" s="2" t="s">
-        <v>519</v>
+        <v>541</v>
       </c>
       <c r="I68" s="2" t="s">
-        <v>712</v>
+        <v>718</v>
       </c>
       <c r="J68" s="2" t="s">
-        <v>713</v>
+        <v>719</v>
       </c>
       <c r="K68" s="2" t="s">
         <v>130</v>
       </c>
       <c r="L68" s="2" t="s">
-        <v>596</v>
+        <v>720</v>
       </c>
       <c r="M68" s="2" t="s">
-        <v>523</v>
+        <v>545</v>
       </c>
       <c r="N68" s="2" t="s">
-        <v>714</v>
+        <v>721</v>
       </c>
       <c r="O68" s="2" t="s">
-        <v>715</v>
+        <v>722</v>
+      </c>
+    </row>
+    <row r="69" spans="1:15">
+      <c r="A69" s="2" t="s">
+        <v>723</v>
+      </c>
+      <c r="B69" s="2" t="s">
+        <v>684</v>
+      </c>
+      <c r="C69" s="2" t="s">
+        <v>537</v>
+      </c>
+      <c r="D69" s="2" t="s">
+        <v>724</v>
+      </c>
+      <c r="E69" s="3" t="s">
+        <v>725</v>
+      </c>
+      <c r="F69" s="2" t="s">
+        <v>540</v>
+      </c>
+      <c r="G69" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H69" s="2" t="s">
+        <v>541</v>
+      </c>
+      <c r="I69" s="2" t="s">
+        <v>726</v>
+      </c>
+      <c r="J69" s="2" t="s">
+        <v>727</v>
+      </c>
+      <c r="K69" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="L69" s="2" t="s">
+        <v>728</v>
+      </c>
+      <c r="M69" s="2" t="s">
+        <v>545</v>
+      </c>
+      <c r="N69" s="2" t="s">
+        <v>729</v>
+      </c>
+      <c r="O69" s="2" t="s">
+        <v>730</v>
+      </c>
+    </row>
+    <row r="70" spans="1:15">
+      <c r="A70" s="2" t="s">
+        <v>731</v>
+      </c>
+      <c r="B70" s="2" t="s">
+        <v>684</v>
+      </c>
+      <c r="C70" s="2" t="s">
+        <v>537</v>
+      </c>
+      <c r="D70" s="2" t="s">
+        <v>732</v>
+      </c>
+      <c r="E70" s="3" t="s">
+        <v>733</v>
+      </c>
+      <c r="F70" s="2" t="s">
+        <v>540</v>
+      </c>
+      <c r="G70" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H70" s="2" t="s">
+        <v>541</v>
+      </c>
+      <c r="I70" s="2" t="s">
+        <v>734</v>
+      </c>
+      <c r="J70" s="2" t="s">
+        <v>735</v>
+      </c>
+      <c r="K70" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="L70" s="2" t="s">
+        <v>618</v>
+      </c>
+      <c r="M70" s="2" t="s">
+        <v>545</v>
+      </c>
+      <c r="N70" s="2" t="s">
+        <v>736</v>
+      </c>
+      <c r="O70" s="2" t="s">
+        <v>737</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O68"/>
+  <autoFilter ref="A1:O70"/>
   <hyperlinks>
     <hyperlink ref="E2" r:id="rId1"/>
     <hyperlink ref="E3" r:id="rId2"/>
@@ -5827,6 +5987,8 @@
     <hyperlink ref="E66" r:id="rId65"/>
     <hyperlink ref="E67" r:id="rId66"/>
     <hyperlink ref="E68" r:id="rId67"/>
+    <hyperlink ref="E69" r:id="rId68"/>
+    <hyperlink ref="E70" r:id="rId69"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Archive education transcripts and fix dossier formatting
</commit_message>
<xml_diff>
--- a/dossier/source_dossier.xlsx
+++ b/dossier/source_dossier.xlsx
@@ -9,15 +9,12 @@
   <sheets>
     <sheet name="Source Dossier" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Source Dossier'!$A$1:$O$70</definedName>
-  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1050" uniqueCount="738">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1065" uniqueCount="738">
   <si>
     <t>id</t>
   </si>
@@ -2237,16 +2234,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="3">
+  <fonts count="2">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -2262,18 +2251,12 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFD9EAF7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -2303,15 +2286,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2321,6 +2301,30 @@
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:O70" totalsRowShown="0">
+  <autoFilter ref="A1:O70"/>
+  <tableColumns count="15">
+    <tableColumn id="1" name="id"/>
+    <tableColumn id="2" name="year"/>
+    <tableColumn id="3" name="source"/>
+    <tableColumn id="4" name="title"/>
+    <tableColumn id="5" name="url"/>
+    <tableColumn id="6" name="publication_type"/>
+    <tableColumn id="7" name="independent"/>
+    <tableColumn id="8" name="reliability"/>
+    <tableColumn id="9" name="coverage_of_subject"/>
+    <tableColumn id="10" name="facts_supported"/>
+    <tableColumn id="11" name="notability_weight"/>
+    <tableColumn id="12" name="article_use"/>
+    <tableColumn id="13" name="status"/>
+    <tableColumn id="14" name="notes"/>
+    <tableColumn id="15" name="citation_wikitext"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2608,3388 +2612,3323 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:O70"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="12.7109375" customWidth="1"/>
-    <col min="2" max="2" width="10.7109375" customWidth="1"/>
-    <col min="3" max="3" width="28.7109375" customWidth="1"/>
-    <col min="4" max="4" width="45.7109375" customWidth="1"/>
-    <col min="5" max="5" width="55.7109375" customWidth="1"/>
-    <col min="6" max="6" width="28.7109375" customWidth="1"/>
-    <col min="7" max="7" width="18.7109375" customWidth="1"/>
-    <col min="8" max="8" width="32.7109375" customWidth="1"/>
-    <col min="9" max="10" width="55.7109375" customWidth="1"/>
+    <col min="1" max="1" width="13.7109375" customWidth="1"/>
+    <col min="2" max="2" width="14.7109375" customWidth="1"/>
+    <col min="3" max="3" width="30.7109375" customWidth="1"/>
+    <col min="4" max="4" width="46.7109375" customWidth="1"/>
+    <col min="5" max="5" width="58.7109375" customWidth="1"/>
+    <col min="6" max="6" width="30.7109375" customWidth="1"/>
+    <col min="7" max="7" width="22.7109375" customWidth="1"/>
+    <col min="8" max="8" width="36.7109375" customWidth="1"/>
+    <col min="9" max="10" width="64.7109375" customWidth="1"/>
     <col min="11" max="11" width="20.7109375" customWidth="1"/>
-    <col min="12" max="12" width="45.7109375" customWidth="1"/>
-    <col min="13" max="13" width="35.7109375" customWidth="1"/>
-    <col min="14" max="14" width="55.7109375" customWidth="1"/>
-    <col min="15" max="15" width="65.7109375" customWidth="1"/>
+    <col min="12" max="12" width="54.7109375" customWidth="1"/>
+    <col min="13" max="13" width="34.7109375" customWidth="1"/>
+    <col min="14" max="14" width="60.7109375" customWidth="1"/>
+    <col min="15" max="15" width="72.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:15" ht="42" customHeight="1">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:15">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:15" ht="84" customHeight="1">
+      <c r="A2" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="H2" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="I2" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="J2" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="K2" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="L2" s="2" t="s">
+      <c r="L2" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="M2" s="2" t="s">
+      <c r="M2" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="N2" s="2" t="s">
+      <c r="N2" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="O2" s="2" t="s">
+      <c r="O2" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="3" spans="1:15">
-      <c r="A3" s="2" t="s">
+    <row r="3" spans="1:15" ht="84" customHeight="1">
+      <c r="A3" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F3" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="G3" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="H3" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="I3" s="2" t="s">
+      <c r="I3" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="J3" s="2" t="s">
+      <c r="J3" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="K3" s="2" t="s">
+      <c r="K3" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="L3" s="2" t="s">
+      <c r="L3" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="M3" s="2" t="s">
+      <c r="M3" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="N3" s="2" t="s">
+      <c r="N3" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="O3" s="2" t="s">
+      <c r="O3" s="1" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="4" spans="1:15">
-      <c r="A4" s="2" t="s">
+    <row r="4" spans="1:15" ht="84" customHeight="1">
+      <c r="A4" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="F4" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="G4" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="H4" s="2" t="s">
+      <c r="H4" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="I4" s="2" t="s">
+      <c r="I4" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="J4" s="2" t="s">
+      <c r="J4" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="K4" s="2" t="s">
+      <c r="K4" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="L4" s="2" t="s">
+      <c r="L4" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="M4" s="2" t="s">
+      <c r="M4" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="N4" s="2" t="s">
+      <c r="N4" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="O4" s="2" t="s">
+      <c r="O4" s="1" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="5" spans="1:15">
-      <c r="A5" s="2" t="s">
+    <row r="5" spans="1:15" ht="84" customHeight="1">
+      <c r="A5" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="F5" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="G5" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="H5" s="2" t="s">
+      <c r="H5" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="I5" s="2" t="s">
+      <c r="I5" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="J5" s="2" t="s">
+      <c r="J5" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="K5" s="2" t="s">
+      <c r="K5" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="L5" s="2" t="s">
+      <c r="L5" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="M5" s="2" t="s">
+      <c r="M5" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="N5" s="2" t="s">
+      <c r="N5" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="O5" s="2" t="s">
+      <c r="O5" s="1" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="6" spans="1:15">
-      <c r="A6" s="2" t="s">
+    <row r="6" spans="1:15" ht="84" customHeight="1">
+      <c r="A6" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D6" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="E6" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="F6" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="G6" s="2" t="s">
+      <c r="G6" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="H6" s="2" t="s">
+      <c r="H6" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="I6" s="2" t="s">
+      <c r="I6" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="J6" s="2" t="s">
+      <c r="J6" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="K6" s="2" t="s">
+      <c r="K6" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="L6" s="2" t="s">
+      <c r="L6" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="M6" s="2" t="s">
+      <c r="M6" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="N6" s="2" t="s">
+      <c r="N6" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="O6" s="2" t="s">
+      <c r="O6" s="1" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="7" spans="1:15">
-      <c r="A7" s="2" t="s">
+    <row r="7" spans="1:15" ht="84" customHeight="1">
+      <c r="A7" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D7" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="E7" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="F7" s="2" t="s">
+      <c r="F7" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="G7" s="2" t="s">
+      <c r="G7" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="H7" s="2" t="s">
+      <c r="H7" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="I7" s="2" t="s">
+      <c r="I7" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="J7" s="2" t="s">
+      <c r="J7" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="K7" s="2" t="s">
+      <c r="K7" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="L7" s="2" t="s">
+      <c r="L7" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="M7" s="2" t="s">
+      <c r="M7" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="N7" s="2" t="s">
+      <c r="N7" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="O7" s="2" t="s">
+      <c r="O7" s="1" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="8" spans="1:15">
-      <c r="A8" s="2" t="s">
+    <row r="8" spans="1:15" ht="84" customHeight="1">
+      <c r="A8" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D8" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="E8" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="F8" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="G8" s="2" t="s">
+      <c r="G8" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="H8" s="2" t="s">
+      <c r="H8" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="I8" s="2" t="s">
+      <c r="I8" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="J8" s="2" t="s">
+      <c r="J8" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="K8" s="2" t="s">
+      <c r="K8" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="L8" s="2" t="s">
+      <c r="L8" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="M8" s="2" t="s">
+      <c r="M8" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="N8" s="2" t="s">
+      <c r="N8" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="O8" s="2" t="s">
+      <c r="O8" s="1" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="9" spans="1:15">
-      <c r="A9" s="2" t="s">
+    <row r="9" spans="1:15" ht="84" customHeight="1">
+      <c r="A9" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="D9" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="E9" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="F9" s="2" t="s">
+      <c r="F9" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="G9" s="2" t="s">
+      <c r="G9" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="H9" s="2" t="s">
+      <c r="H9" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="I9" s="2" t="s">
+      <c r="I9" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="J9" s="2" t="s">
+      <c r="J9" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="K9" s="2" t="s">
+      <c r="K9" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="L9" s="2" t="s">
+      <c r="L9" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="M9" s="2" t="s">
+      <c r="M9" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="N9" s="2" t="s">
+      <c r="N9" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="O9" s="2" t="s">
+      <c r="O9" s="1" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="10" spans="1:15">
-      <c r="A10" s="2" t="s">
+    <row r="10" spans="1:15" ht="84" customHeight="1">
+      <c r="A10" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D10" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="E10" s="3" t="s">
+      <c r="E10" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="F10" s="2" t="s">
+      <c r="F10" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="G10" s="2" t="s">
+      <c r="G10" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="H10" s="2" t="s">
+      <c r="H10" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="I10" s="2" t="s">
+      <c r="I10" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="J10" s="2" t="s">
+      <c r="J10" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="K10" s="2" t="s">
+      <c r="K10" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="L10" s="2" t="s">
+      <c r="L10" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="M10" s="2" t="s">
+      <c r="M10" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="N10" s="2" t="s">
+      <c r="N10" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="O10" s="2" t="s">
+      <c r="O10" s="1" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="11" spans="1:15">
-      <c r="A11" s="2" t="s">
+    <row r="11" spans="1:15" ht="84" customHeight="1">
+      <c r="A11" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C11" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="D11" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="E11" s="3" t="s">
+      <c r="E11" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="F11" s="2" t="s">
+      <c r="F11" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="G11" s="2" t="s">
+      <c r="G11" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="H11" s="2" t="s">
+      <c r="H11" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="I11" s="2" t="s">
+      <c r="I11" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="J11" s="2" t="s">
+      <c r="J11" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="K11" s="2" t="s">
+      <c r="K11" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="L11" s="2" t="s">
+      <c r="L11" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="M11" s="2" t="s">
+      <c r="M11" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="N11" s="2" t="s">
+      <c r="N11" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="O11" s="2" t="s">
+      <c r="O11" s="1" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="12" spans="1:15">
-      <c r="A12" s="2" t="s">
+    <row r="12" spans="1:15" ht="84" customHeight="1">
+      <c r="A12" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C12" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="D12" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="E12" s="3" t="s">
+      <c r="E12" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="F12" s="2" t="s">
+      <c r="F12" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="G12" s="2" t="s">
+      <c r="G12" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="H12" s="2" t="s">
+      <c r="H12" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="I12" s="2" t="s">
+      <c r="I12" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="J12" s="2" t="s">
+      <c r="J12" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="K12" s="2" t="s">
+      <c r="K12" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="L12" s="2" t="s">
+      <c r="L12" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="M12" s="2" t="s">
+      <c r="M12" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="N12" s="2" t="s">
+      <c r="N12" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="O12" s="2" t="s">
+      <c r="O12" s="1" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="13" spans="1:15">
-      <c r="A13" s="2" t="s">
+    <row r="13" spans="1:15" ht="84" customHeight="1">
+      <c r="A13" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="C13" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="D13" s="2" t="s">
+      <c r="D13" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="E13" s="3" t="s">
+      <c r="E13" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="F13" s="2" t="s">
+      <c r="F13" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="G13" s="2" t="s">
+      <c r="G13" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="H13" s="2" t="s">
+      <c r="H13" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="I13" s="2" t="s">
+      <c r="I13" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="J13" s="2" t="s">
+      <c r="J13" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="K13" s="2" t="s">
+      <c r="K13" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="L13" s="2" t="s">
+      <c r="L13" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="M13" s="2" t="s">
+      <c r="M13" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="N13" s="2" t="s">
+      <c r="N13" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="O13" s="2" t="s">
+      <c r="O13" s="1" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="14" spans="1:15">
-      <c r="A14" s="2" t="s">
+    <row r="14" spans="1:15" ht="84" customHeight="1">
+      <c r="A14" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="C14" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="D14" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="E14" s="3" t="s">
+      <c r="E14" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="F14" s="2" t="s">
+      <c r="F14" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="G14" s="2" t="s">
+      <c r="G14" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="H14" s="2" t="s">
+      <c r="H14" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="I14" s="2" t="s">
+      <c r="I14" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="J14" s="2" t="s">
+      <c r="J14" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="K14" s="2" t="s">
+      <c r="K14" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="L14" s="2" t="s">
+      <c r="L14" s="1" t="s">
         <v>179</v>
       </c>
-      <c r="M14" s="2" t="s">
+      <c r="M14" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="N14" s="2" t="s">
+      <c r="N14" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="O14" s="2" t="s">
+      <c r="O14" s="1" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="15" spans="1:15">
-      <c r="A15" s="2" t="s">
+    <row r="15" spans="1:15" ht="84" customHeight="1">
+      <c r="A15" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B15" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="C15" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="D15" s="2" t="s">
+      <c r="D15" s="1" t="s">
         <v>185</v>
       </c>
-      <c r="E15" s="3" t="s">
+      <c r="E15" s="2" t="s">
         <v>186</v>
       </c>
-      <c r="F15" s="2" t="s">
+      <c r="F15" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="G15" s="2" t="s">
+      <c r="G15" s="1" t="s">
         <v>188</v>
       </c>
-      <c r="H15" s="2" t="s">
+      <c r="H15" s="1" t="s">
         <v>189</v>
       </c>
-      <c r="I15" s="2" t="s">
+      <c r="I15" s="1" t="s">
         <v>190</v>
       </c>
-      <c r="J15" s="2" t="s">
+      <c r="J15" s="1" t="s">
         <v>191</v>
       </c>
-      <c r="K15" s="2" t="s">
+      <c r="K15" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="L15" s="2" t="s">
+      <c r="L15" s="1" t="s">
         <v>192</v>
       </c>
-      <c r="M15" s="2" t="s">
+      <c r="M15" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="N15" s="2" t="s">
+      <c r="N15" s="1" t="s">
         <v>194</v>
       </c>
-      <c r="O15" s="2" t="s">
+      <c r="O15" s="1" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="16" spans="1:15">
-      <c r="A16" s="2" t="s">
+    <row r="16" spans="1:15" ht="84" customHeight="1">
+      <c r="A16" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" s="1" t="s">
         <v>197</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="C16" s="1" t="s">
         <v>198</v>
       </c>
-      <c r="D16" s="2" t="s">
+      <c r="D16" s="1" t="s">
         <v>199</v>
       </c>
-      <c r="E16" s="3" t="s">
+      <c r="E16" s="2" t="s">
         <v>200</v>
       </c>
-      <c r="F16" s="2" t="s">
+      <c r="F16" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="G16" s="2" t="s">
+      <c r="G16" s="1" t="s">
         <v>202</v>
       </c>
-      <c r="H16" s="2" t="s">
+      <c r="H16" s="1" t="s">
         <v>203</v>
       </c>
-      <c r="I16" s="2" t="s">
+      <c r="I16" s="1" t="s">
         <v>204</v>
       </c>
-      <c r="J16" s="2" t="s">
+      <c r="J16" s="1" t="s">
         <v>205</v>
       </c>
-      <c r="K16" s="2" t="s">
+      <c r="K16" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="L16" s="2" t="s">
+      <c r="L16" s="1" t="s">
         <v>206</v>
       </c>
-      <c r="M16" s="2" t="s">
+      <c r="M16" s="1" t="s">
         <v>207</v>
       </c>
-      <c r="N16" s="2" t="s">
+      <c r="N16" s="1" t="s">
         <v>208</v>
       </c>
-      <c r="O16" s="2" t="s">
+      <c r="O16" s="1" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="17" spans="1:15">
-      <c r="A17" s="2" t="s">
+    <row r="17" spans="1:15" ht="84" customHeight="1">
+      <c r="A17" s="1" t="s">
         <v>210</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="B17" s="1" t="s">
         <v>197</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="C17" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="D17" s="2" t="s">
+      <c r="D17" s="1" t="s">
         <v>212</v>
       </c>
-      <c r="E17" s="3" t="s">
+      <c r="E17" s="2" t="s">
         <v>213</v>
       </c>
-      <c r="F17" s="2" t="s">
+      <c r="F17" s="1" t="s">
         <v>214</v>
       </c>
-      <c r="G17" s="2" t="s">
+      <c r="G17" s="1" t="s">
         <v>215</v>
       </c>
-      <c r="H17" s="2" t="s">
+      <c r="H17" s="1" t="s">
         <v>216</v>
       </c>
-      <c r="I17" s="2" t="s">
+      <c r="I17" s="1" t="s">
         <v>217</v>
       </c>
-      <c r="J17" s="2" t="s">
+      <c r="J17" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="K17" s="2" t="s">
+      <c r="K17" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="L17" s="2" t="s">
+      <c r="L17" s="1" t="s">
         <v>219</v>
       </c>
-      <c r="M17" s="2" t="s">
+      <c r="M17" s="1" t="s">
         <v>220</v>
       </c>
-      <c r="N17" s="2" t="s">
+      <c r="N17" s="1" t="s">
         <v>221</v>
       </c>
-      <c r="O17" s="2" t="s">
+      <c r="O17" s="1" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="18" spans="1:15">
-      <c r="A18" s="2" t="s">
+    <row r="18" spans="1:15" ht="84" customHeight="1">
+      <c r="A18" s="1" t="s">
         <v>223</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="B18" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="C18" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="D18" s="2" t="s">
+      <c r="D18" s="1" t="s">
         <v>224</v>
       </c>
-      <c r="E18" s="3" t="s">
+      <c r="E18" s="2" t="s">
         <v>225</v>
       </c>
-      <c r="F18" s="2" t="s">
+      <c r="F18" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="G18" s="2" t="s">
+      <c r="G18" s="1" t="s">
         <v>215</v>
       </c>
-      <c r="H18" s="2" t="s">
+      <c r="H18" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="I18" s="2" t="s">
+      <c r="I18" s="1" t="s">
         <v>228</v>
       </c>
-      <c r="J18" s="2" t="s">
+      <c r="J18" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="K18" s="2" t="s">
+      <c r="K18" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="L18" s="2" t="s">
+      <c r="L18" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="M18" s="2" t="s">
+      <c r="M18" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="N18" s="2" t="s">
+      <c r="N18" s="1" t="s">
         <v>231</v>
       </c>
-      <c r="O18" s="2" t="s">
+      <c r="O18" s="1" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="19" spans="1:15">
-      <c r="A19" s="2" t="s">
+    <row r="19" spans="1:15" ht="84" customHeight="1">
+      <c r="A19" s="1" t="s">
         <v>233</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B19" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C19" s="2" t="s">
+      <c r="C19" s="1" t="s">
         <v>234</v>
       </c>
-      <c r="D19" s="2" t="s">
+      <c r="D19" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="E19" s="3" t="s">
+      <c r="E19" s="2" t="s">
         <v>236</v>
       </c>
-      <c r="F19" s="2" t="s">
+      <c r="F19" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="G19" s="2" t="s">
+      <c r="G19" s="1" t="s">
         <v>238</v>
       </c>
-      <c r="H19" s="2" t="s">
+      <c r="H19" s="1" t="s">
         <v>239</v>
       </c>
-      <c r="I19" s="2" t="s">
+      <c r="I19" s="1" t="s">
         <v>240</v>
       </c>
-      <c r="J19" s="2" t="s">
+      <c r="J19" s="1" t="s">
         <v>241</v>
       </c>
-      <c r="K19" s="2" t="s">
+      <c r="K19" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="L19" s="2" t="s">
+      <c r="L19" s="1" t="s">
         <v>242</v>
       </c>
-      <c r="M19" s="2" t="s">
+      <c r="M19" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="N19" s="2" t="s">
+      <c r="N19" s="1" t="s">
         <v>243</v>
       </c>
-      <c r="O19" s="2" t="s">
+      <c r="O19" s="1" t="s">
         <v>244</v>
       </c>
     </row>
-    <row r="20" spans="1:15">
-      <c r="A20" s="2" t="s">
+    <row r="20" spans="1:15" ht="84" customHeight="1">
+      <c r="A20" s="1" t="s">
         <v>245</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="B20" s="1" t="s">
         <v>197</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="C20" s="1" t="s">
         <v>246</v>
       </c>
-      <c r="D20" s="2" t="s">
+      <c r="D20" s="1" t="s">
         <v>247</v>
       </c>
-      <c r="E20" s="3" t="s">
+      <c r="E20" s="2" t="s">
         <v>248</v>
       </c>
-      <c r="F20" s="2" t="s">
+      <c r="F20" s="1" t="s">
         <v>249</v>
       </c>
-      <c r="G20" s="2" t="s">
+      <c r="G20" s="1" t="s">
         <v>250</v>
       </c>
-      <c r="H20" s="2" t="s">
+      <c r="H20" s="1" t="s">
         <v>251</v>
       </c>
-      <c r="I20" s="2" t="s">
+      <c r="I20" s="1" t="s">
         <v>252</v>
       </c>
-      <c r="J20" s="2" t="s">
+      <c r="J20" s="1" t="s">
         <v>253</v>
       </c>
-      <c r="K20" s="2" t="s">
+      <c r="K20" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="L20" s="2" t="s">
+      <c r="L20" s="1" t="s">
         <v>254</v>
       </c>
-      <c r="M20" s="2" t="s">
+      <c r="M20" s="1" t="s">
         <v>255</v>
       </c>
-      <c r="N20" s="2" t="s">
+      <c r="N20" s="1" t="s">
         <v>256</v>
       </c>
-      <c r="O20" s="2" t="s">
+      <c r="O20" s="1" t="s">
         <v>257</v>
       </c>
     </row>
-    <row r="21" spans="1:15">
-      <c r="A21" s="2" t="s">
+    <row r="21" spans="1:15" ht="84" customHeight="1">
+      <c r="A21" s="1" t="s">
         <v>258</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="B21" s="1" t="s">
         <v>259</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="C21" s="1" t="s">
         <v>260</v>
       </c>
-      <c r="D21" s="2" t="s">
+      <c r="D21" s="1" t="s">
         <v>261</v>
       </c>
-      <c r="E21" s="3" t="s">
+      <c r="E21" s="2" t="s">
         <v>262</v>
       </c>
-      <c r="F21" s="2" t="s">
+      <c r="F21" s="1" t="s">
         <v>263</v>
       </c>
-      <c r="G21" s="2" t="s">
+      <c r="G21" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="H21" s="2" t="s">
+      <c r="H21" s="1" t="s">
         <v>265</v>
       </c>
-      <c r="I21" s="2" t="s">
+      <c r="I21" s="1" t="s">
         <v>266</v>
       </c>
-      <c r="J21" s="2" t="s">
+      <c r="J21" s="1" t="s">
         <v>267</v>
       </c>
-      <c r="K21" s="2" t="s">
+      <c r="K21" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="L21" s="2" t="s">
+      <c r="L21" s="1" t="s">
         <v>268</v>
       </c>
-      <c r="M21" s="2" t="s">
+      <c r="M21" s="1" t="s">
         <v>269</v>
       </c>
-      <c r="N21" s="2" t="s">
+      <c r="N21" s="1" t="s">
         <v>270</v>
       </c>
-      <c r="O21" s="2" t="s">
+      <c r="O21" s="1" t="s">
         <v>271</v>
       </c>
     </row>
-    <row r="22" spans="1:15">
-      <c r="A22" s="2" t="s">
+    <row r="22" spans="1:15" ht="84" customHeight="1">
+      <c r="A22" s="1" t="s">
         <v>272</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="B22" s="1" t="s">
         <v>259</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="C22" s="1" t="s">
         <v>260</v>
       </c>
-      <c r="D22" s="2" t="s">
+      <c r="D22" s="1" t="s">
         <v>273</v>
       </c>
-      <c r="E22" s="3" t="s">
+      <c r="E22" s="2" t="s">
         <v>274</v>
       </c>
-      <c r="F22" s="2" t="s">
+      <c r="F22" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="G22" s="2" t="s">
+      <c r="G22" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="H22" s="2" t="s">
+      <c r="H22" s="1" t="s">
         <v>276</v>
       </c>
-      <c r="I22" s="2" t="s">
+      <c r="I22" s="1" t="s">
         <v>277</v>
       </c>
-      <c r="J22" s="2" t="s">
+      <c r="J22" s="1" t="s">
         <v>278</v>
       </c>
-      <c r="K22" s="2" t="s">
+      <c r="K22" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="L22" s="2" t="s">
+      <c r="L22" s="1" t="s">
         <v>279</v>
       </c>
-      <c r="M22" s="2" t="s">
+      <c r="M22" s="1" t="s">
         <v>280</v>
       </c>
-      <c r="N22" s="2" t="s">
+      <c r="N22" s="1" t="s">
         <v>281</v>
       </c>
-      <c r="O22" s="2" t="s">
+      <c r="O22" s="1" t="s">
         <v>282</v>
       </c>
     </row>
-    <row r="23" spans="1:15">
-      <c r="A23" s="2" t="s">
+    <row r="23" spans="1:15" ht="84" customHeight="1">
+      <c r="A23" s="1" t="s">
         <v>283</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="B23" s="1" t="s">
         <v>259</v>
       </c>
-      <c r="C23" s="2" t="s">
+      <c r="C23" s="1" t="s">
         <v>260</v>
       </c>
-      <c r="D23" s="2" t="s">
+      <c r="D23" s="1" t="s">
         <v>284</v>
       </c>
-      <c r="E23" s="3" t="s">
+      <c r="E23" s="2" t="s">
         <v>285</v>
       </c>
-      <c r="F23" s="2" t="s">
+      <c r="F23" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="G23" s="2" t="s">
+      <c r="G23" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="H23" s="2" t="s">
+      <c r="H23" s="1" t="s">
         <v>276</v>
       </c>
-      <c r="I23" s="2" t="s">
+      <c r="I23" s="1" t="s">
         <v>286</v>
       </c>
-      <c r="J23" s="2" t="s">
+      <c r="J23" s="1" t="s">
         <v>287</v>
       </c>
-      <c r="K23" s="2" t="s">
+      <c r="K23" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="L23" s="2" t="s">
+      <c r="L23" s="1" t="s">
         <v>288</v>
       </c>
-      <c r="M23" s="2" t="s">
+      <c r="M23" s="1" t="s">
         <v>280</v>
       </c>
-      <c r="N23" s="2" t="s">
+      <c r="N23" s="1" t="s">
         <v>289</v>
       </c>
-      <c r="O23" s="2" t="s">
+      <c r="O23" s="1" t="s">
         <v>290</v>
       </c>
     </row>
-    <row r="24" spans="1:15">
-      <c r="A24" s="2" t="s">
+    <row r="24" spans="1:15" ht="84" customHeight="1">
+      <c r="A24" s="1" t="s">
         <v>291</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="B24" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="C24" s="1" t="s">
         <v>292</v>
       </c>
-      <c r="D24" s="2" t="s">
+      <c r="D24" s="1" t="s">
         <v>293</v>
       </c>
-      <c r="E24" s="3" t="s">
+      <c r="E24" s="2" t="s">
         <v>294</v>
       </c>
-      <c r="F24" s="2" t="s">
+      <c r="F24" s="1" t="s">
         <v>295</v>
       </c>
-      <c r="G24" s="2" t="s">
+      <c r="G24" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="H24" s="2" t="s">
+      <c r="H24" s="1" t="s">
         <v>296</v>
       </c>
-      <c r="I24" s="2" t="s">
+      <c r="I24" s="1" t="s">
         <v>297</v>
       </c>
-      <c r="J24" s="2" t="s">
+      <c r="J24" s="1" t="s">
         <v>298</v>
       </c>
-      <c r="K24" s="2" t="s">
+      <c r="K24" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="L24" s="2" t="s">
+      <c r="L24" s="1" t="s">
         <v>299</v>
       </c>
-      <c r="M24" s="2" t="s">
+      <c r="M24" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="N24" s="2" t="s">
+      <c r="N24" s="1" t="s">
         <v>300</v>
       </c>
-      <c r="O24" s="2" t="s">
+      <c r="O24" s="1" t="s">
         <v>301</v>
       </c>
     </row>
-    <row r="25" spans="1:15">
-      <c r="A25" s="2" t="s">
+    <row r="25" spans="1:15" ht="84" customHeight="1">
+      <c r="A25" s="1" t="s">
         <v>302</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="B25" s="1" t="s">
         <v>303</v>
       </c>
-      <c r="C25" s="2" t="s">
+      <c r="C25" s="1" t="s">
         <v>304</v>
       </c>
-      <c r="D25" s="2" t="s">
+      <c r="D25" s="1" t="s">
         <v>305</v>
       </c>
-      <c r="E25" s="3" t="s">
+      <c r="E25" s="2" t="s">
         <v>306</v>
       </c>
-      <c r="F25" s="2" t="s">
+      <c r="F25" s="1" t="s">
         <v>307</v>
       </c>
-      <c r="G25" s="2" t="s">
+      <c r="G25" s="1" t="s">
         <v>308</v>
       </c>
-      <c r="H25" s="2" t="s">
+      <c r="H25" s="1" t="s">
         <v>309</v>
       </c>
-      <c r="I25" s="2" t="s">
+      <c r="I25" s="1" t="s">
         <v>310</v>
       </c>
-      <c r="J25" s="2" t="s">
+      <c r="J25" s="1" t="s">
         <v>311</v>
       </c>
-      <c r="K25" s="2" t="s">
+      <c r="K25" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="L25" s="2" t="s">
+      <c r="L25" s="1" t="s">
         <v>312</v>
       </c>
-      <c r="M25" s="2" t="s">
+      <c r="M25" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="N25" s="2" t="s">
+      <c r="N25" s="1" t="s">
         <v>313</v>
       </c>
-      <c r="O25" s="2" t="s">
+      <c r="O25" s="1" t="s">
         <v>314</v>
       </c>
     </row>
-    <row r="26" spans="1:15">
-      <c r="A26" s="2" t="s">
+    <row r="26" spans="1:15" ht="84" customHeight="1">
+      <c r="A26" s="1" t="s">
         <v>315</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="B26" s="1" t="s">
         <v>316</v>
       </c>
-      <c r="C26" s="2" t="s">
+      <c r="C26" s="1" t="s">
         <v>317</v>
       </c>
-      <c r="D26" s="2" t="s">
+      <c r="D26" s="1" t="s">
         <v>318</v>
       </c>
-      <c r="E26" s="3" t="s">
+      <c r="E26" s="2" t="s">
         <v>319</v>
       </c>
-      <c r="F26" s="2" t="s">
+      <c r="F26" s="1" t="s">
         <v>320</v>
       </c>
-      <c r="G26" s="2" t="s">
+      <c r="G26" s="1" t="s">
         <v>308</v>
       </c>
-      <c r="H26" s="2" t="s">
+      <c r="H26" s="1" t="s">
         <v>321</v>
       </c>
-      <c r="I26" s="2" t="s">
+      <c r="I26" s="1" t="s">
         <v>322</v>
       </c>
-      <c r="J26" s="2" t="s">
+      <c r="J26" s="1" t="s">
         <v>323</v>
       </c>
-      <c r="K26" s="2" t="s">
+      <c r="K26" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="L26" s="2" t="s">
+      <c r="L26" s="1" t="s">
         <v>324</v>
       </c>
-      <c r="M26" s="2" t="s">
+      <c r="M26" s="1" t="s">
         <v>325</v>
       </c>
-      <c r="N26" s="2" t="s">
+      <c r="N26" s="1" t="s">
         <v>326</v>
       </c>
-      <c r="O26" s="2" t="s">
+      <c r="O26" s="1" t="s">
         <v>327</v>
       </c>
     </row>
-    <row r="27" spans="1:15">
-      <c r="A27" s="2" t="s">
+    <row r="27" spans="1:15" ht="84" customHeight="1">
+      <c r="A27" s="1" t="s">
         <v>328</v>
       </c>
-      <c r="B27" s="2" t="s">
+      <c r="B27" s="1" t="s">
         <v>316</v>
       </c>
-      <c r="C27" s="2" t="s">
+      <c r="C27" s="1" t="s">
         <v>304</v>
       </c>
-      <c r="D27" s="2" t="s">
+      <c r="D27" s="1" t="s">
         <v>329</v>
       </c>
-      <c r="E27" s="3" t="s">
+      <c r="E27" s="2" t="s">
         <v>330</v>
       </c>
-      <c r="F27" s="2" t="s">
+      <c r="F27" s="1" t="s">
         <v>331</v>
       </c>
-      <c r="G27" s="2" t="s">
+      <c r="G27" s="1" t="s">
         <v>308</v>
       </c>
-      <c r="H27" s="2" t="s">
+      <c r="H27" s="1" t="s">
         <v>332</v>
       </c>
-      <c r="I27" s="2" t="s">
+      <c r="I27" s="1" t="s">
         <v>333</v>
       </c>
-      <c r="J27" s="2" t="s">
+      <c r="J27" s="1" t="s">
         <v>334</v>
       </c>
-      <c r="K27" s="2" t="s">
+      <c r="K27" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="L27" s="2" t="s">
+      <c r="L27" s="1" t="s">
         <v>335</v>
       </c>
-      <c r="M27" s="2" t="s">
+      <c r="M27" s="1" t="s">
         <v>325</v>
       </c>
-      <c r="N27" s="2" t="s">
+      <c r="N27" s="1" t="s">
         <v>336</v>
       </c>
-      <c r="O27" s="2" t="s">
+      <c r="O27" s="1" t="s">
         <v>337</v>
       </c>
     </row>
-    <row r="28" spans="1:15">
-      <c r="A28" s="2" t="s">
+    <row r="28" spans="1:15" ht="84" customHeight="1">
+      <c r="A28" s="1" t="s">
         <v>338</v>
       </c>
-      <c r="B28" s="2" t="s">
+      <c r="B28" s="1" t="s">
         <v>316</v>
       </c>
-      <c r="C28" s="2" t="s">
+      <c r="C28" s="1" t="s">
         <v>339</v>
       </c>
-      <c r="D28" s="2" t="s">
+      <c r="D28" s="1" t="s">
         <v>340</v>
       </c>
-      <c r="E28" s="3" t="s">
+      <c r="E28" s="2" t="s">
         <v>341</v>
       </c>
-      <c r="F28" s="2" t="s">
+      <c r="F28" s="1" t="s">
         <v>342</v>
       </c>
-      <c r="G28" s="2" t="s">
+      <c r="G28" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="H28" s="2" t="s">
+      <c r="H28" s="1" t="s">
         <v>343</v>
       </c>
-      <c r="I28" s="2" t="s">
+      <c r="I28" s="1" t="s">
         <v>344</v>
       </c>
-      <c r="J28" s="2" t="s">
+      <c r="J28" s="1" t="s">
         <v>345</v>
       </c>
-      <c r="K28" s="2" t="s">
+      <c r="K28" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="L28" s="2" t="s">
+      <c r="L28" s="1" t="s">
         <v>346</v>
       </c>
-      <c r="M28" s="2" t="s">
+      <c r="M28" s="1" t="s">
         <v>325</v>
       </c>
-      <c r="N28" s="2" t="s">
+      <c r="N28" s="1" t="s">
         <v>347</v>
       </c>
-      <c r="O28" s="2" t="s">
+      <c r="O28" s="1" t="s">
         <v>348</v>
       </c>
     </row>
-    <row r="29" spans="1:15">
-      <c r="A29" s="2" t="s">
+    <row r="29" spans="1:15" ht="84" customHeight="1">
+      <c r="A29" s="1" t="s">
         <v>349</v>
       </c>
-      <c r="B29" s="2" t="s">
+      <c r="B29" s="1" t="s">
         <v>350</v>
       </c>
-      <c r="C29" s="2" t="s">
+      <c r="C29" s="1" t="s">
         <v>304</v>
       </c>
-      <c r="D29" s="2" t="s">
+      <c r="D29" s="1" t="s">
         <v>351</v>
       </c>
-      <c r="E29" s="3" t="s">
+      <c r="E29" s="2" t="s">
         <v>352</v>
       </c>
-      <c r="F29" s="2" t="s">
+      <c r="F29" s="1" t="s">
         <v>331</v>
       </c>
-      <c r="G29" s="2" t="s">
+      <c r="G29" s="1" t="s">
         <v>308</v>
       </c>
-      <c r="H29" s="2" t="s">
+      <c r="H29" s="1" t="s">
         <v>332</v>
       </c>
-      <c r="I29" s="2" t="s">
+      <c r="I29" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="J29" s="2" t="s">
+      <c r="J29" s="1" t="s">
         <v>354</v>
       </c>
-      <c r="K29" s="2" t="s">
+      <c r="K29" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="L29" s="2" t="s">
+      <c r="L29" s="1" t="s">
         <v>355</v>
       </c>
-      <c r="M29" s="2" t="s">
+      <c r="M29" s="1" t="s">
         <v>325</v>
       </c>
-      <c r="N29" s="2" t="s">
+      <c r="N29" s="1" t="s">
         <v>356</v>
       </c>
-      <c r="O29" s="2" t="s">
+      <c r="O29" s="1" t="s">
         <v>357</v>
       </c>
     </row>
-    <row r="30" spans="1:15">
-      <c r="A30" s="2" t="s">
+    <row r="30" spans="1:15" ht="84" customHeight="1">
+      <c r="A30" s="1" t="s">
         <v>358</v>
       </c>
-      <c r="B30" s="2" t="s">
+      <c r="B30" s="1" t="s">
         <v>350</v>
       </c>
-      <c r="C30" s="2" t="s">
+      <c r="C30" s="1" t="s">
         <v>359</v>
       </c>
-      <c r="D30" s="2" t="s">
+      <c r="D30" s="1" t="s">
         <v>360</v>
       </c>
-      <c r="E30" s="3" t="s">
+      <c r="E30" s="2" t="s">
         <v>361</v>
       </c>
-      <c r="F30" s="2" t="s">
+      <c r="F30" s="1" t="s">
         <v>362</v>
       </c>
-      <c r="G30" s="2" t="s">
+      <c r="G30" s="1" t="s">
         <v>308</v>
       </c>
-      <c r="H30" s="2" t="s">
+      <c r="H30" s="1" t="s">
         <v>363</v>
       </c>
-      <c r="I30" s="2" t="s">
+      <c r="I30" s="1" t="s">
         <v>364</v>
       </c>
-      <c r="J30" s="2" t="s">
+      <c r="J30" s="1" t="s">
         <v>365</v>
       </c>
-      <c r="K30" s="2" t="s">
+      <c r="K30" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="L30" s="2" t="s">
+      <c r="L30" s="1" t="s">
         <v>366</v>
       </c>
-      <c r="M30" s="2" t="s">
+      <c r="M30" s="1" t="s">
         <v>325</v>
       </c>
-      <c r="N30" s="2" t="s">
+      <c r="N30" s="1" t="s">
         <v>367</v>
       </c>
-      <c r="O30" s="2" t="s">
+      <c r="O30" s="1" t="s">
         <v>368</v>
       </c>
     </row>
-    <row r="31" spans="1:15">
-      <c r="A31" s="2" t="s">
+    <row r="31" spans="1:15" ht="84" customHeight="1">
+      <c r="A31" s="1" t="s">
         <v>369</v>
       </c>
-      <c r="B31" s="2" t="s">
+      <c r="B31" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="C31" s="2" t="s">
+      <c r="C31" s="1" t="s">
         <v>304</v>
       </c>
-      <c r="D31" s="2" t="s">
+      <c r="D31" s="1" t="s">
         <v>370</v>
       </c>
-      <c r="E31" s="3" t="s">
+      <c r="E31" s="2" t="s">
         <v>371</v>
       </c>
-      <c r="F31" s="2" t="s">
+      <c r="F31" s="1" t="s">
         <v>331</v>
       </c>
-      <c r="G31" s="2" t="s">
+      <c r="G31" s="1" t="s">
         <v>308</v>
       </c>
-      <c r="H31" s="2" t="s">
+      <c r="H31" s="1" t="s">
         <v>372</v>
       </c>
-      <c r="I31" s="2" t="s">
+      <c r="I31" s="1" t="s">
         <v>373</v>
       </c>
-      <c r="J31" s="2" t="s">
+      <c r="J31" s="1" t="s">
         <v>374</v>
       </c>
-      <c r="K31" s="2" t="s">
+      <c r="K31" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="L31" s="2" t="s">
+      <c r="L31" s="1" t="s">
         <v>375</v>
       </c>
-      <c r="M31" s="2" t="s">
+      <c r="M31" s="1" t="s">
         <v>325</v>
       </c>
-      <c r="N31" s="2" t="s">
+      <c r="N31" s="1" t="s">
         <v>376</v>
       </c>
-      <c r="O31" s="2" t="s">
+      <c r="O31" s="1" t="s">
         <v>377</v>
       </c>
     </row>
-    <row r="32" spans="1:15">
-      <c r="A32" s="2" t="s">
+    <row r="32" spans="1:15" ht="84" customHeight="1">
+      <c r="A32" s="1" t="s">
         <v>378</v>
       </c>
-      <c r="B32" s="2" t="s">
+      <c r="B32" s="1" t="s">
         <v>379</v>
       </c>
-      <c r="C32" s="2" t="s">
+      <c r="C32" s="1" t="s">
         <v>304</v>
       </c>
-      <c r="D32" s="2" t="s">
+      <c r="D32" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="E32" s="3" t="s">
+      <c r="E32" s="2" t="s">
         <v>381</v>
       </c>
-      <c r="F32" s="2" t="s">
+      <c r="F32" s="1" t="s">
         <v>382</v>
       </c>
-      <c r="G32" s="2" t="s">
+      <c r="G32" s="1" t="s">
         <v>308</v>
       </c>
-      <c r="H32" s="2" t="s">
+      <c r="H32" s="1" t="s">
         <v>383</v>
       </c>
-      <c r="I32" s="2" t="s">
+      <c r="I32" s="1" t="s">
         <v>384</v>
       </c>
-      <c r="J32" s="2" t="s">
+      <c r="J32" s="1" t="s">
         <v>385</v>
       </c>
-      <c r="K32" s="2" t="s">
+      <c r="K32" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="L32" s="2" t="s">
+      <c r="L32" s="1" t="s">
         <v>386</v>
       </c>
-      <c r="M32" s="2" t="s">
+      <c r="M32" s="1" t="s">
         <v>325</v>
       </c>
-      <c r="N32" s="2" t="s">
+      <c r="N32" s="1" t="s">
         <v>387</v>
       </c>
-      <c r="O32" s="2" t="s">
+      <c r="O32" s="1" t="s">
         <v>388</v>
       </c>
     </row>
-    <row r="33" spans="1:15">
-      <c r="A33" s="2" t="s">
+    <row r="33" spans="1:15" ht="84" customHeight="1">
+      <c r="A33" s="1" t="s">
         <v>389</v>
       </c>
-      <c r="B33" s="2" t="s">
+      <c r="B33" s="1" t="s">
         <v>350</v>
       </c>
-      <c r="C33" s="2" t="s">
+      <c r="C33" s="1" t="s">
         <v>390</v>
       </c>
-      <c r="D33" s="2" t="s">
+      <c r="D33" s="1" t="s">
         <v>391</v>
       </c>
-      <c r="E33" s="3" t="s">
+      <c r="E33" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="F33" s="2" t="s">
+      <c r="F33" s="1" t="s">
         <v>393</v>
       </c>
-      <c r="G33" s="2" t="s">
+      <c r="G33" s="1" t="s">
         <v>394</v>
       </c>
-      <c r="H33" s="2" t="s">
+      <c r="H33" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="I33" s="2" t="s">
+      <c r="I33" s="1" t="s">
         <v>396</v>
       </c>
-      <c r="J33" s="2" t="s">
+      <c r="J33" s="1" t="s">
         <v>397</v>
       </c>
-      <c r="K33" s="2" t="s">
+      <c r="K33" s="1" t="s">
         <v>398</v>
       </c>
-      <c r="L33" s="2" t="s">
+      <c r="L33" s="1" t="s">
         <v>399</v>
       </c>
-      <c r="M33" s="2" t="s">
+      <c r="M33" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="N33" s="2" t="s">
+      <c r="N33" s="1" t="s">
         <v>400</v>
       </c>
-      <c r="O33" s="2" t="s">
+      <c r="O33" s="1" t="s">
         <v>401</v>
       </c>
     </row>
-    <row r="34" spans="1:15">
-      <c r="A34" s="2" t="s">
+    <row r="34" spans="1:15" ht="84" customHeight="1">
+      <c r="A34" s="1" t="s">
         <v>402</v>
       </c>
-      <c r="B34" s="2" t="s">
+      <c r="B34" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="C34" s="2" t="s">
+      <c r="C34" s="1" t="s">
         <v>403</v>
       </c>
-      <c r="D34" s="2" t="s">
+      <c r="D34" s="1" t="s">
         <v>404</v>
       </c>
-      <c r="E34" s="3" t="s">
+      <c r="E34" s="2" t="s">
         <v>405</v>
       </c>
-      <c r="F34" s="2" t="s">
+      <c r="F34" s="1" t="s">
         <v>406</v>
       </c>
-      <c r="G34" s="2" t="s">
+      <c r="G34" s="1" t="s">
         <v>407</v>
       </c>
-      <c r="H34" s="2" t="s">
+      <c r="H34" s="1" t="s">
         <v>408</v>
       </c>
-      <c r="I34" s="2" t="s">
+      <c r="I34" s="1" t="s">
         <v>409</v>
       </c>
-      <c r="J34" s="2" t="s">
+      <c r="J34" s="1" t="s">
         <v>410</v>
       </c>
-      <c r="K34" s="2" t="s">
+      <c r="K34" s="1" t="s">
         <v>411</v>
       </c>
-      <c r="L34" s="2" t="s">
+      <c r="L34" s="1" t="s">
         <v>412</v>
       </c>
-      <c r="M34" s="2" t="s">
+      <c r="M34" s="1" t="s">
         <v>325</v>
       </c>
-      <c r="N34" s="2" t="s">
+      <c r="N34" s="1" t="s">
         <v>413</v>
       </c>
-      <c r="O34" s="2" t="s">
+      <c r="O34" s="1" t="s">
         <v>414</v>
       </c>
     </row>
-    <row r="35" spans="1:15">
-      <c r="A35" s="2" t="s">
+    <row r="35" spans="1:15" ht="84" customHeight="1">
+      <c r="A35" s="1" t="s">
         <v>415</v>
       </c>
-      <c r="B35" s="2" t="s">
+      <c r="B35" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="C35" s="2" t="s">
+      <c r="C35" s="1" t="s">
         <v>416</v>
       </c>
-      <c r="D35" s="2" t="s">
+      <c r="D35" s="1" t="s">
         <v>417</v>
       </c>
-      <c r="E35" s="3" t="s">
+      <c r="E35" s="2" t="s">
         <v>418</v>
       </c>
-      <c r="F35" s="2" t="s">
+      <c r="F35" s="1" t="s">
         <v>419</v>
       </c>
-      <c r="G35" s="2" t="s">
+      <c r="G35" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="H35" s="2" t="s">
+      <c r="H35" s="1" t="s">
         <v>420</v>
       </c>
-      <c r="I35" s="2" t="s">
+      <c r="I35" s="1" t="s">
         <v>421</v>
       </c>
-      <c r="J35" s="2" t="s">
+      <c r="J35" s="1" t="s">
         <v>422</v>
       </c>
-      <c r="K35" s="2" t="s">
+      <c r="K35" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="L35" s="2" t="s">
+      <c r="L35" s="1" t="s">
         <v>423</v>
       </c>
-      <c r="M35" s="2" t="s">
+      <c r="M35" s="1" t="s">
         <v>424</v>
       </c>
-      <c r="N35" s="2" t="s">
+      <c r="N35" s="1" t="s">
         <v>425</v>
       </c>
-      <c r="O35" s="2" t="s">
+      <c r="O35" s="1" t="s">
         <v>426</v>
       </c>
     </row>
-    <row r="36" spans="1:15">
-      <c r="A36" s="2" t="s">
+    <row r="36" spans="1:15" ht="84" customHeight="1">
+      <c r="A36" s="1" t="s">
         <v>427</v>
       </c>
-      <c r="B36" s="2" t="s">
+      <c r="B36" s="1" t="s">
         <v>428</v>
       </c>
-      <c r="C36" s="2" t="s">
+      <c r="C36" s="1" t="s">
         <v>429</v>
       </c>
-      <c r="D36" s="2" t="s">
+      <c r="D36" s="1" t="s">
         <v>430</v>
       </c>
-      <c r="E36" s="3" t="s">
+      <c r="E36" s="2" t="s">
         <v>431</v>
       </c>
-      <c r="F36" s="2" t="s">
+      <c r="F36" s="1" t="s">
         <v>432</v>
       </c>
-      <c r="G36" s="2" t="s">
+      <c r="G36" s="1" t="s">
         <v>433</v>
       </c>
-      <c r="H36" s="2" t="s">
+      <c r="H36" s="1" t="s">
         <v>434</v>
       </c>
-      <c r="I36" s="2" t="s">
+      <c r="I36" s="1" t="s">
         <v>435</v>
       </c>
-      <c r="J36" s="2" t="s">
+      <c r="J36" s="1" t="s">
         <v>436</v>
       </c>
-      <c r="K36" s="2" t="s">
+      <c r="K36" s="1" t="s">
         <v>437</v>
       </c>
-      <c r="L36" s="2" t="s">
+      <c r="L36" s="1" t="s">
         <v>438</v>
       </c>
-      <c r="M36" s="2" t="s">
+      <c r="M36" s="1" t="s">
         <v>439</v>
       </c>
-      <c r="N36" s="2" t="s">
+      <c r="N36" s="1" t="s">
         <v>440</v>
       </c>
-      <c r="O36" s="2" t="s">
+      <c r="O36" s="1" t="s">
         <v>257</v>
       </c>
     </row>
-    <row r="37" spans="1:15">
-      <c r="A37" s="2" t="s">
+    <row r="37" spans="1:15" ht="84" customHeight="1">
+      <c r="A37" s="1" t="s">
         <v>441</v>
       </c>
-      <c r="B37" s="2" t="s">
+      <c r="B37" s="1" t="s">
         <v>442</v>
       </c>
-      <c r="C37" s="2" t="s">
+      <c r="C37" s="1" t="s">
         <v>443</v>
       </c>
-      <c r="D37" s="2" t="s">
+      <c r="D37" s="1" t="s">
         <v>444</v>
       </c>
-      <c r="E37" s="3" t="s">
+      <c r="E37" s="2" t="s">
         <v>445</v>
       </c>
-      <c r="F37" s="2" t="s">
+      <c r="F37" s="1" t="s">
         <v>446</v>
       </c>
-      <c r="G37" s="2" t="s">
+      <c r="G37" s="1" t="s">
         <v>447</v>
       </c>
-      <c r="H37" s="2" t="s">
+      <c r="H37" s="1" t="s">
         <v>448</v>
       </c>
-      <c r="I37" s="2" t="s">
+      <c r="I37" s="1" t="s">
         <v>449</v>
       </c>
-      <c r="J37" s="2" t="s">
+      <c r="J37" s="1" t="s">
         <v>450</v>
       </c>
-      <c r="K37" s="2" t="s">
+      <c r="K37" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="L37" s="2" t="s">
+      <c r="L37" s="1" t="s">
         <v>451</v>
       </c>
-      <c r="M37" s="2" t="s">
+      <c r="M37" s="1" t="s">
         <v>452</v>
       </c>
-      <c r="N37" s="2" t="s">
+      <c r="N37" s="1" t="s">
         <v>453</v>
       </c>
-      <c r="O37" s="2" t="s">
+      <c r="O37" s="1" t="s">
         <v>454</v>
       </c>
     </row>
-    <row r="38" spans="1:15">
-      <c r="A38" s="2" t="s">
+    <row r="38" spans="1:15" ht="84" customHeight="1">
+      <c r="A38" s="1" t="s">
         <v>455</v>
       </c>
-      <c r="B38" s="2" t="s">
+      <c r="B38" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C38" s="2" t="s">
+      <c r="C38" s="1" t="s">
         <v>456</v>
       </c>
-      <c r="D38" s="2" t="s">
+      <c r="D38" s="1" t="s">
         <v>457</v>
       </c>
-      <c r="E38" s="3" t="s">
+      <c r="E38" s="2" t="s">
         <v>458</v>
       </c>
-      <c r="F38" s="2" t="s">
+      <c r="F38" s="1" t="s">
         <v>459</v>
       </c>
-      <c r="G38" s="2" t="s">
+      <c r="G38" s="1" t="s">
         <v>447</v>
       </c>
-      <c r="H38" s="2" t="s">
+      <c r="H38" s="1" t="s">
         <v>460</v>
       </c>
-      <c r="I38" s="2" t="s">
+      <c r="I38" s="1" t="s">
         <v>461</v>
       </c>
-      <c r="J38" s="2" t="s">
+      <c r="J38" s="1" t="s">
         <v>462</v>
       </c>
-      <c r="K38" s="2" t="s">
+      <c r="K38" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="L38" s="2" t="s">
+      <c r="L38" s="1" t="s">
         <v>463</v>
       </c>
-      <c r="M38" s="2" t="s">
+      <c r="M38" s="1" t="s">
         <v>464</v>
       </c>
-      <c r="N38" s="2" t="s">
+      <c r="N38" s="1" t="s">
         <v>465</v>
       </c>
-      <c r="O38" s="2" t="s">
+      <c r="O38" s="1" t="s">
         <v>454</v>
       </c>
     </row>
-    <row r="39" spans="1:15">
-      <c r="A39" s="2" t="s">
+    <row r="39" spans="1:15" ht="84" customHeight="1">
+      <c r="A39" s="1" t="s">
         <v>466</v>
       </c>
-      <c r="B39" s="2" t="s">
+      <c r="B39" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C39" s="2" t="s">
+      <c r="C39" s="1" t="s">
         <v>467</v>
       </c>
-      <c r="D39" s="2" t="s">
+      <c r="D39" s="1" t="s">
         <v>468</v>
       </c>
-      <c r="E39" s="3" t="s">
+      <c r="E39" s="2" t="s">
         <v>469</v>
       </c>
-      <c r="F39" s="2" t="s">
+      <c r="F39" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="G39" s="2" t="s">
+      <c r="G39" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="H39" s="2" t="s">
+      <c r="H39" s="1" t="s">
         <v>276</v>
       </c>
-      <c r="I39" s="2" t="s">
+      <c r="I39" s="1" t="s">
         <v>470</v>
       </c>
-      <c r="J39" s="2" t="s">
+      <c r="J39" s="1" t="s">
         <v>471</v>
       </c>
-      <c r="K39" s="2" t="s">
+      <c r="K39" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="L39" s="2" t="s">
+      <c r="L39" s="1" t="s">
         <v>472</v>
       </c>
-      <c r="M39" s="2" t="s">
+      <c r="M39" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="N39" s="2" t="s">
+      <c r="N39" s="1" t="s">
         <v>473</v>
       </c>
-      <c r="O39" s="2" t="s">
+      <c r="O39" s="1" t="s">
         <v>474</v>
       </c>
     </row>
-    <row r="40" spans="1:15">
-      <c r="A40" s="2" t="s">
+    <row r="40" spans="1:15" ht="84" customHeight="1">
+      <c r="A40" s="1" t="s">
         <v>475</v>
       </c>
-      <c r="B40" s="2" t="s">
+      <c r="B40" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C40" s="2" t="s">
+      <c r="C40" s="1" t="s">
         <v>476</v>
       </c>
-      <c r="D40" s="2" t="s">
+      <c r="D40" s="1" t="s">
         <v>477</v>
       </c>
-      <c r="E40" s="3" t="s">
+      <c r="E40" s="2" t="s">
         <v>478</v>
       </c>
-      <c r="F40" s="2" t="s">
+      <c r="F40" s="1" t="s">
         <v>263</v>
       </c>
-      <c r="G40" s="2" t="s">
+      <c r="G40" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="H40" s="2" t="s">
+      <c r="H40" s="1" t="s">
         <v>265</v>
       </c>
-      <c r="I40" s="2" t="s">
+      <c r="I40" s="1" t="s">
         <v>479</v>
       </c>
-      <c r="J40" s="2" t="s">
+      <c r="J40" s="1" t="s">
         <v>480</v>
       </c>
-      <c r="K40" s="2" t="s">
+      <c r="K40" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="L40" s="2" t="s">
+      <c r="L40" s="1" t="s">
         <v>481</v>
       </c>
-      <c r="M40" s="2" t="s">
+      <c r="M40" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="N40" s="2" t="s">
+      <c r="N40" s="1" t="s">
         <v>482</v>
       </c>
-      <c r="O40" s="2" t="s">
+      <c r="O40" s="1" t="s">
         <v>483</v>
       </c>
     </row>
-    <row r="41" spans="1:15">
-      <c r="A41" s="2" t="s">
+    <row r="41" spans="1:15" ht="84" customHeight="1">
+      <c r="A41" s="1" t="s">
         <v>484</v>
       </c>
-      <c r="B41" s="2" t="s">
+      <c r="B41" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C41" s="2" t="s">
+      <c r="C41" s="1" t="s">
         <v>476</v>
       </c>
-      <c r="D41" s="2" t="s">
+      <c r="D41" s="1" t="s">
         <v>485</v>
       </c>
-      <c r="E41" s="3" t="s">
+      <c r="E41" s="2" t="s">
         <v>486</v>
       </c>
-      <c r="F41" s="2" t="s">
+      <c r="F41" s="1" t="s">
         <v>487</v>
       </c>
-      <c r="G41" s="2" t="s">
+      <c r="G41" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="H41" s="2" t="s">
+      <c r="H41" s="1" t="s">
         <v>276</v>
       </c>
-      <c r="I41" s="2" t="s">
+      <c r="I41" s="1" t="s">
         <v>488</v>
       </c>
-      <c r="J41" s="2" t="s">
+      <c r="J41" s="1" t="s">
         <v>489</v>
       </c>
-      <c r="K41" s="2" t="s">
+      <c r="K41" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="L41" s="2" t="s">
+      <c r="L41" s="1" t="s">
         <v>490</v>
       </c>
-      <c r="M41" s="2" t="s">
+      <c r="M41" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="N41" s="2" t="s">
+      <c r="N41" s="1" t="s">
         <v>491</v>
       </c>
-      <c r="O41" s="2" t="s">
+      <c r="O41" s="1" t="s">
         <v>492</v>
       </c>
     </row>
-    <row r="42" spans="1:15">
-      <c r="A42" s="2" t="s">
+    <row r="42" spans="1:15" ht="84" customHeight="1">
+      <c r="A42" s="1" t="s">
         <v>493</v>
       </c>
-      <c r="B42" s="2" t="s">
+      <c r="B42" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C42" s="2" t="s">
+      <c r="C42" s="1" t="s">
         <v>494</v>
       </c>
-      <c r="D42" s="2" t="s">
+      <c r="D42" s="1" t="s">
         <v>495</v>
       </c>
-      <c r="E42" s="3" t="s">
+      <c r="E42" s="2" t="s">
         <v>496</v>
       </c>
-      <c r="F42" s="2" t="s">
+      <c r="F42" s="1" t="s">
         <v>497</v>
       </c>
-      <c r="G42" s="2" t="s">
+      <c r="G42" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="H42" s="2" t="s">
+      <c r="H42" s="1" t="s">
         <v>498</v>
       </c>
-      <c r="I42" s="2" t="s">
+      <c r="I42" s="1" t="s">
         <v>499</v>
       </c>
-      <c r="J42" s="2" t="s">
+      <c r="J42" s="1" t="s">
         <v>500</v>
       </c>
-      <c r="K42" s="2" t="s">
+      <c r="K42" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="L42" s="2" t="s">
+      <c r="L42" s="1" t="s">
         <v>501</v>
       </c>
-      <c r="M42" s="2" t="s">
+      <c r="M42" s="1" t="s">
         <v>502</v>
       </c>
-      <c r="N42" s="2" t="s">
+      <c r="N42" s="1" t="s">
         <v>503</v>
       </c>
-      <c r="O42" s="2" t="s">
+      <c r="O42" s="1" t="s">
         <v>504</v>
       </c>
     </row>
-    <row r="43" spans="1:15">
-      <c r="A43" s="2" t="s">
+    <row r="43" spans="1:15" ht="84" customHeight="1">
+      <c r="A43" s="1" t="s">
         <v>505</v>
       </c>
-      <c r="B43" s="2" t="s">
+      <c r="B43" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C43" s="2" t="s">
+      <c r="C43" s="1" t="s">
         <v>506</v>
       </c>
-      <c r="D43" s="2" t="s">
+      <c r="D43" s="1" t="s">
         <v>507</v>
       </c>
-      <c r="E43" s="3" t="s">
+      <c r="E43" s="2" t="s">
         <v>508</v>
       </c>
-      <c r="F43" s="2" t="s">
+      <c r="F43" s="1" t="s">
         <v>509</v>
       </c>
-      <c r="G43" s="2" t="s">
+      <c r="G43" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="H43" s="2" t="s">
+      <c r="H43" s="1" t="s">
         <v>510</v>
       </c>
-      <c r="I43" s="2" t="s">
+      <c r="I43" s="1" t="s">
         <v>511</v>
       </c>
-      <c r="J43" s="2" t="s">
+      <c r="J43" s="1" t="s">
         <v>512</v>
       </c>
-      <c r="K43" s="2" t="s">
+      <c r="K43" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="L43" s="2" t="s">
+      <c r="L43" s="1" t="s">
         <v>513</v>
       </c>
-      <c r="M43" s="2" t="s">
+      <c r="M43" s="1" t="s">
         <v>325</v>
       </c>
-      <c r="N43" s="2" t="s">
+      <c r="N43" s="1" t="s">
         <v>514</v>
       </c>
-      <c r="O43" s="2" t="s">
+      <c r="O43" s="1" t="s">
         <v>515</v>
       </c>
     </row>
-    <row r="44" spans="1:15">
-      <c r="A44" s="2" t="s">
+    <row r="44" spans="1:15" ht="84" customHeight="1">
+      <c r="A44" s="1" t="s">
         <v>516</v>
       </c>
-      <c r="B44" s="2" t="s">
+      <c r="B44" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="C44" s="2" t="s">
+      <c r="C44" s="1" t="s">
         <v>506</v>
       </c>
-      <c r="D44" s="2" t="s">
+      <c r="D44" s="1" t="s">
         <v>517</v>
       </c>
-      <c r="E44" s="3" t="s">
+      <c r="E44" s="2" t="s">
         <v>518</v>
       </c>
-      <c r="F44" s="2" t="s">
+      <c r="F44" s="1" t="s">
         <v>519</v>
       </c>
-      <c r="G44" s="2" t="s">
+      <c r="G44" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="H44" s="2" t="s">
+      <c r="H44" s="1" t="s">
         <v>520</v>
       </c>
-      <c r="I44" s="2" t="s">
+      <c r="I44" s="1" t="s">
         <v>521</v>
       </c>
-      <c r="J44" s="2" t="s">
+      <c r="J44" s="1" t="s">
         <v>522</v>
       </c>
-      <c r="K44" s="2" t="s">
+      <c r="K44" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="L44" s="2" t="s">
+      <c r="L44" s="1" t="s">
         <v>523</v>
       </c>
-      <c r="M44" s="2" t="s">
+      <c r="M44" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="N44" s="2" t="s">
+      <c r="N44" s="1" t="s">
         <v>524</v>
       </c>
-      <c r="O44" s="2" t="s">
+      <c r="O44" s="1" t="s">
         <v>525</v>
       </c>
     </row>
-    <row r="45" spans="1:15">
-      <c r="A45" s="2" t="s">
+    <row r="45" spans="1:15" ht="84" customHeight="1">
+      <c r="A45" s="1" t="s">
         <v>526</v>
       </c>
-      <c r="B45" s="2" t="s">
+      <c r="B45" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="C45" s="2" t="s">
+      <c r="C45" s="1" t="s">
         <v>527</v>
       </c>
-      <c r="D45" s="2" t="s">
+      <c r="D45" s="1" t="s">
         <v>528</v>
       </c>
-      <c r="E45" s="3" t="s">
+      <c r="E45" s="2" t="s">
         <v>529</v>
       </c>
-      <c r="F45" s="2" t="s">
+      <c r="F45" s="1" t="s">
         <v>530</v>
       </c>
-      <c r="G45" s="2" t="s">
+      <c r="G45" s="1" t="s">
         <v>531</v>
       </c>
-      <c r="H45" s="2" t="s">
+      <c r="H45" s="1" t="s">
         <v>434</v>
       </c>
-      <c r="I45" s="2" t="s">
+      <c r="I45" s="1" t="s">
         <v>532</v>
       </c>
-      <c r="J45" s="2" t="s">
+      <c r="J45" s="1" t="s">
         <v>533</v>
       </c>
-      <c r="K45" s="2" t="s">
+      <c r="K45" s="1" t="s">
         <v>437</v>
       </c>
-      <c r="L45" s="2" t="s">
+      <c r="L45" s="1" t="s">
         <v>438</v>
       </c>
-      <c r="M45" s="2" t="s">
+      <c r="M45" s="1" t="s">
         <v>534</v>
       </c>
-      <c r="N45" s="2" t="s">
+      <c r="N45" s="1" t="s">
         <v>535</v>
       </c>
-      <c r="O45" s="2" t="s">
+      <c r="O45" s="1" t="s">
         <v>257</v>
       </c>
     </row>
-    <row r="46" spans="1:15">
-      <c r="A46" s="2" t="s">
+    <row r="46" spans="1:15" ht="84" customHeight="1">
+      <c r="A46" s="1" t="s">
         <v>536</v>
       </c>
-      <c r="B46" s="2" t="s">
+      <c r="B46" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="C46" s="2" t="s">
+      <c r="C46" s="1" t="s">
         <v>537</v>
       </c>
-      <c r="D46" s="2" t="s">
+      <c r="D46" s="1" t="s">
         <v>538</v>
       </c>
-      <c r="E46" s="3" t="s">
+      <c r="E46" s="2" t="s">
         <v>539</v>
       </c>
-      <c r="F46" s="2" t="s">
+      <c r="F46" s="1" t="s">
         <v>540</v>
       </c>
-      <c r="G46" s="2" t="s">
+      <c r="G46" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="H46" s="2" t="s">
+      <c r="H46" s="1" t="s">
         <v>541</v>
       </c>
-      <c r="I46" s="2" t="s">
+      <c r="I46" s="1" t="s">
         <v>542</v>
       </c>
-      <c r="J46" s="2" t="s">
+      <c r="J46" s="1" t="s">
         <v>543</v>
       </c>
-      <c r="K46" s="2" t="s">
+      <c r="K46" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="L46" s="2" t="s">
+      <c r="L46" s="1" t="s">
         <v>544</v>
       </c>
-      <c r="M46" s="2" t="s">
+      <c r="M46" s="1" t="s">
         <v>545</v>
       </c>
-      <c r="N46" s="2" t="s">
+      <c r="N46" s="1" t="s">
         <v>546</v>
       </c>
-      <c r="O46" s="2" t="s">
+      <c r="O46" s="1" t="s">
         <v>547</v>
       </c>
     </row>
-    <row r="47" spans="1:15">
-      <c r="A47" s="2" t="s">
+    <row r="47" spans="1:15" ht="84" customHeight="1">
+      <c r="A47" s="1" t="s">
         <v>548</v>
       </c>
-      <c r="B47" s="2" t="s">
+      <c r="B47" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="C47" s="2" t="s">
+      <c r="C47" s="1" t="s">
         <v>537</v>
       </c>
-      <c r="D47" s="2" t="s">
+      <c r="D47" s="1" t="s">
         <v>549</v>
       </c>
-      <c r="E47" s="3" t="s">
+      <c r="E47" s="2" t="s">
         <v>550</v>
       </c>
-      <c r="F47" s="2" t="s">
+      <c r="F47" s="1" t="s">
         <v>540</v>
       </c>
-      <c r="G47" s="2" t="s">
+      <c r="G47" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="H47" s="2" t="s">
+      <c r="H47" s="1" t="s">
         <v>541</v>
       </c>
-      <c r="I47" s="2" t="s">
+      <c r="I47" s="1" t="s">
         <v>551</v>
       </c>
-      <c r="J47" s="2" t="s">
+      <c r="J47" s="1" t="s">
         <v>552</v>
       </c>
-      <c r="K47" s="2" t="s">
+      <c r="K47" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="L47" s="2" t="s">
+      <c r="L47" s="1" t="s">
         <v>553</v>
       </c>
-      <c r="M47" s="2" t="s">
+      <c r="M47" s="1" t="s">
         <v>545</v>
       </c>
-      <c r="N47" s="2" t="s">
+      <c r="N47" s="1" t="s">
         <v>554</v>
       </c>
-      <c r="O47" s="2" t="s">
+      <c r="O47" s="1" t="s">
         <v>555</v>
       </c>
     </row>
-    <row r="48" spans="1:15">
-      <c r="A48" s="2" t="s">
+    <row r="48" spans="1:15" ht="84" customHeight="1">
+      <c r="A48" s="1" t="s">
         <v>556</v>
       </c>
-      <c r="B48" s="2" t="s">
+      <c r="B48" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="C48" s="2" t="s">
+      <c r="C48" s="1" t="s">
         <v>537</v>
       </c>
-      <c r="D48" s="2" t="s">
+      <c r="D48" s="1" t="s">
         <v>557</v>
       </c>
-      <c r="E48" s="3" t="s">
+      <c r="E48" s="2" t="s">
         <v>558</v>
       </c>
-      <c r="F48" s="2" t="s">
+      <c r="F48" s="1" t="s">
         <v>540</v>
       </c>
-      <c r="G48" s="2" t="s">
+      <c r="G48" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="H48" s="2" t="s">
+      <c r="H48" s="1" t="s">
         <v>541</v>
       </c>
-      <c r="I48" s="2" t="s">
+      <c r="I48" s="1" t="s">
         <v>559</v>
       </c>
-      <c r="J48" s="2" t="s">
+      <c r="J48" s="1" t="s">
         <v>560</v>
       </c>
-      <c r="K48" s="2" t="s">
+      <c r="K48" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="L48" s="2" t="s">
+      <c r="L48" s="1" t="s">
         <v>561</v>
       </c>
-      <c r="M48" s="2" t="s">
+      <c r="M48" s="1" t="s">
         <v>545</v>
       </c>
-      <c r="N48" s="2" t="s">
+      <c r="N48" s="1" t="s">
         <v>562</v>
       </c>
-      <c r="O48" s="2" t="s">
+      <c r="O48" s="1" t="s">
         <v>563</v>
       </c>
     </row>
-    <row r="49" spans="1:15">
-      <c r="A49" s="2" t="s">
+    <row r="49" spans="1:15" ht="84" customHeight="1">
+      <c r="A49" s="1" t="s">
         <v>564</v>
       </c>
-      <c r="B49" s="2" t="s">
+      <c r="B49" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="C49" s="2" t="s">
+      <c r="C49" s="1" t="s">
         <v>537</v>
       </c>
-      <c r="D49" s="2" t="s">
+      <c r="D49" s="1" t="s">
         <v>565</v>
       </c>
-      <c r="E49" s="3" t="s">
+      <c r="E49" s="2" t="s">
         <v>566</v>
       </c>
-      <c r="F49" s="2" t="s">
+      <c r="F49" s="1" t="s">
         <v>567</v>
       </c>
-      <c r="G49" s="2" t="s">
+      <c r="G49" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="H49" s="2" t="s">
+      <c r="H49" s="1" t="s">
         <v>541</v>
       </c>
-      <c r="I49" s="2" t="s">
+      <c r="I49" s="1" t="s">
         <v>568</v>
       </c>
-      <c r="J49" s="2" t="s">
+      <c r="J49" s="1" t="s">
         <v>569</v>
       </c>
-      <c r="K49" s="2" t="s">
+      <c r="K49" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="L49" s="2" t="s">
+      <c r="L49" s="1" t="s">
         <v>570</v>
       </c>
-      <c r="M49" s="2" t="s">
+      <c r="M49" s="1" t="s">
         <v>545</v>
       </c>
-      <c r="N49" s="2" t="s">
+      <c r="N49" s="1" t="s">
         <v>571</v>
       </c>
-      <c r="O49" s="2" t="s">
+      <c r="O49" s="1" t="s">
         <v>572</v>
       </c>
     </row>
-    <row r="50" spans="1:15">
-      <c r="A50" s="2" t="s">
+    <row r="50" spans="1:15" ht="84" customHeight="1">
+      <c r="A50" s="1" t="s">
         <v>573</v>
       </c>
-      <c r="B50" s="2" t="s">
+      <c r="B50" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="C50" s="2" t="s">
+      <c r="C50" s="1" t="s">
         <v>537</v>
       </c>
-      <c r="D50" s="2" t="s">
+      <c r="D50" s="1" t="s">
         <v>574</v>
       </c>
-      <c r="E50" s="3" t="s">
+      <c r="E50" s="2" t="s">
         <v>575</v>
       </c>
-      <c r="F50" s="2" t="s">
+      <c r="F50" s="1" t="s">
         <v>540</v>
       </c>
-      <c r="G50" s="2" t="s">
+      <c r="G50" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="H50" s="2" t="s">
+      <c r="H50" s="1" t="s">
         <v>541</v>
       </c>
-      <c r="I50" s="2" t="s">
+      <c r="I50" s="1" t="s">
         <v>576</v>
       </c>
-      <c r="J50" s="2" t="s">
+      <c r="J50" s="1" t="s">
         <v>577</v>
       </c>
-      <c r="K50" s="2" t="s">
+      <c r="K50" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="L50" s="2" t="s">
+      <c r="L50" s="1" t="s">
         <v>578</v>
       </c>
-      <c r="M50" s="2" t="s">
+      <c r="M50" s="1" t="s">
         <v>545</v>
       </c>
-      <c r="N50" s="2" t="s">
+      <c r="N50" s="1" t="s">
         <v>579</v>
       </c>
-      <c r="O50" s="2" t="s">
+      <c r="O50" s="1" t="s">
         <v>580</v>
       </c>
     </row>
-    <row r="51" spans="1:15">
-      <c r="A51" s="2" t="s">
+    <row r="51" spans="1:15" ht="84" customHeight="1">
+      <c r="A51" s="1" t="s">
         <v>581</v>
       </c>
-      <c r="B51" s="2" t="s">
+      <c r="B51" s="1" t="s">
         <v>259</v>
       </c>
-      <c r="C51" s="2" t="s">
+      <c r="C51" s="1" t="s">
         <v>537</v>
       </c>
-      <c r="D51" s="2" t="s">
+      <c r="D51" s="1" t="s">
         <v>582</v>
       </c>
-      <c r="E51" s="3" t="s">
+      <c r="E51" s="2" t="s">
         <v>583</v>
       </c>
-      <c r="F51" s="2" t="s">
+      <c r="F51" s="1" t="s">
         <v>540</v>
       </c>
-      <c r="G51" s="2" t="s">
+      <c r="G51" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="H51" s="2" t="s">
+      <c r="H51" s="1" t="s">
         <v>541</v>
       </c>
-      <c r="I51" s="2" t="s">
+      <c r="I51" s="1" t="s">
         <v>584</v>
       </c>
-      <c r="J51" s="2" t="s">
+      <c r="J51" s="1" t="s">
         <v>585</v>
       </c>
-      <c r="K51" s="2" t="s">
+      <c r="K51" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="L51" s="2" t="s">
+      <c r="L51" s="1" t="s">
         <v>586</v>
       </c>
-      <c r="M51" s="2" t="s">
+      <c r="M51" s="1" t="s">
         <v>545</v>
       </c>
-      <c r="N51" s="2" t="s">
+      <c r="N51" s="1" t="s">
         <v>587</v>
       </c>
-      <c r="O51" s="2" t="s">
+      <c r="O51" s="1" t="s">
         <v>588</v>
       </c>
     </row>
-    <row r="52" spans="1:15">
-      <c r="A52" s="2" t="s">
+    <row r="52" spans="1:15" ht="84" customHeight="1">
+      <c r="A52" s="1" t="s">
         <v>589</v>
       </c>
-      <c r="B52" s="2" t="s">
+      <c r="B52" s="1" t="s">
         <v>259</v>
       </c>
-      <c r="C52" s="2" t="s">
+      <c r="C52" s="1" t="s">
         <v>537</v>
       </c>
-      <c r="D52" s="2" t="s">
+      <c r="D52" s="1" t="s">
         <v>590</v>
       </c>
-      <c r="E52" s="3" t="s">
+      <c r="E52" s="2" t="s">
         <v>591</v>
       </c>
-      <c r="F52" s="2" t="s">
+      <c r="F52" s="1" t="s">
         <v>540</v>
       </c>
-      <c r="G52" s="2" t="s">
+      <c r="G52" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="H52" s="2" t="s">
+      <c r="H52" s="1" t="s">
         <v>541</v>
       </c>
-      <c r="I52" s="2" t="s">
+      <c r="I52" s="1" t="s">
         <v>592</v>
       </c>
-      <c r="J52" s="2" t="s">
+      <c r="J52" s="1" t="s">
         <v>593</v>
       </c>
-      <c r="K52" s="2" t="s">
+      <c r="K52" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="L52" s="2" t="s">
+      <c r="L52" s="1" t="s">
         <v>594</v>
       </c>
-      <c r="M52" s="2" t="s">
+      <c r="M52" s="1" t="s">
         <v>545</v>
       </c>
-      <c r="N52" s="2" t="s">
+      <c r="N52" s="1" t="s">
         <v>595</v>
       </c>
-      <c r="O52" s="2" t="s">
+      <c r="O52" s="1" t="s">
         <v>596</v>
       </c>
     </row>
-    <row r="53" spans="1:15">
-      <c r="A53" s="2" t="s">
+    <row r="53" spans="1:15" ht="84" customHeight="1">
+      <c r="A53" s="1" t="s">
         <v>597</v>
       </c>
-      <c r="B53" s="2" t="s">
+      <c r="B53" s="1" t="s">
         <v>259</v>
       </c>
-      <c r="C53" s="2" t="s">
+      <c r="C53" s="1" t="s">
         <v>537</v>
       </c>
-      <c r="D53" s="2" t="s">
+      <c r="D53" s="1" t="s">
         <v>598</v>
       </c>
-      <c r="E53" s="3" t="s">
+      <c r="E53" s="2" t="s">
         <v>599</v>
       </c>
-      <c r="F53" s="2" t="s">
+      <c r="F53" s="1" t="s">
         <v>540</v>
       </c>
-      <c r="G53" s="2" t="s">
+      <c r="G53" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="H53" s="2" t="s">
+      <c r="H53" s="1" t="s">
         <v>541</v>
       </c>
-      <c r="I53" s="2" t="s">
+      <c r="I53" s="1" t="s">
         <v>600</v>
       </c>
-      <c r="J53" s="2" t="s">
+      <c r="J53" s="1" t="s">
         <v>601</v>
       </c>
-      <c r="K53" s="2" t="s">
+      <c r="K53" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="L53" s="2" t="s">
+      <c r="L53" s="1" t="s">
         <v>602</v>
       </c>
-      <c r="M53" s="2" t="s">
+      <c r="M53" s="1" t="s">
         <v>545</v>
       </c>
-      <c r="N53" s="2" t="s">
+      <c r="N53" s="1" t="s">
         <v>603</v>
       </c>
-      <c r="O53" s="2" t="s">
+      <c r="O53" s="1" t="s">
         <v>604</v>
       </c>
     </row>
-    <row r="54" spans="1:15">
-      <c r="A54" s="2" t="s">
+    <row r="54" spans="1:15" ht="84" customHeight="1">
+      <c r="A54" s="1" t="s">
         <v>605</v>
       </c>
-      <c r="B54" s="2" t="s">
+      <c r="B54" s="1" t="s">
         <v>259</v>
       </c>
-      <c r="C54" s="2" t="s">
+      <c r="C54" s="1" t="s">
         <v>537</v>
       </c>
-      <c r="D54" s="2" t="s">
+      <c r="D54" s="1" t="s">
         <v>606</v>
       </c>
-      <c r="E54" s="3" t="s">
+      <c r="E54" s="2" t="s">
         <v>607</v>
       </c>
-      <c r="F54" s="2" t="s">
+      <c r="F54" s="1" t="s">
         <v>540</v>
       </c>
-      <c r="G54" s="2" t="s">
+      <c r="G54" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="H54" s="2" t="s">
+      <c r="H54" s="1" t="s">
         <v>541</v>
       </c>
-      <c r="I54" s="2" t="s">
+      <c r="I54" s="1" t="s">
         <v>608</v>
       </c>
-      <c r="J54" s="2" t="s">
+      <c r="J54" s="1" t="s">
         <v>609</v>
       </c>
-      <c r="K54" s="2" t="s">
+      <c r="K54" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="L54" s="2" t="s">
+      <c r="L54" s="1" t="s">
         <v>610</v>
       </c>
-      <c r="M54" s="2" t="s">
+      <c r="M54" s="1" t="s">
         <v>545</v>
       </c>
-      <c r="N54" s="2" t="s">
+      <c r="N54" s="1" t="s">
         <v>611</v>
       </c>
-      <c r="O54" s="2" t="s">
+      <c r="O54" s="1" t="s">
         <v>612</v>
       </c>
     </row>
-    <row r="55" spans="1:15">
-      <c r="A55" s="2" t="s">
+    <row r="55" spans="1:15" ht="84" customHeight="1">
+      <c r="A55" s="1" t="s">
         <v>613</v>
       </c>
-      <c r="B55" s="2" t="s">
+      <c r="B55" s="1" t="s">
         <v>259</v>
       </c>
-      <c r="C55" s="2" t="s">
+      <c r="C55" s="1" t="s">
         <v>537</v>
       </c>
-      <c r="D55" s="2" t="s">
+      <c r="D55" s="1" t="s">
         <v>614</v>
       </c>
-      <c r="E55" s="3" t="s">
+      <c r="E55" s="2" t="s">
         <v>615</v>
       </c>
-      <c r="F55" s="2" t="s">
+      <c r="F55" s="1" t="s">
         <v>540</v>
       </c>
-      <c r="G55" s="2" t="s">
+      <c r="G55" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="H55" s="2" t="s">
+      <c r="H55" s="1" t="s">
         <v>541</v>
       </c>
-      <c r="I55" s="2" t="s">
+      <c r="I55" s="1" t="s">
         <v>616</v>
       </c>
-      <c r="J55" s="2" t="s">
+      <c r="J55" s="1" t="s">
         <v>617</v>
       </c>
-      <c r="K55" s="2" t="s">
+      <c r="K55" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="L55" s="2" t="s">
+      <c r="L55" s="1" t="s">
         <v>618</v>
       </c>
-      <c r="M55" s="2" t="s">
+      <c r="M55" s="1" t="s">
         <v>545</v>
       </c>
-      <c r="N55" s="2" t="s">
+      <c r="N55" s="1" t="s">
         <v>619</v>
       </c>
-      <c r="O55" s="2" t="s">
+      <c r="O55" s="1" t="s">
         <v>620</v>
       </c>
     </row>
-    <row r="56" spans="1:15">
-      <c r="A56" s="2" t="s">
+    <row r="56" spans="1:15" ht="84" customHeight="1">
+      <c r="A56" s="1" t="s">
         <v>621</v>
       </c>
-      <c r="B56" s="2" t="s">
+      <c r="B56" s="1" t="s">
         <v>259</v>
       </c>
-      <c r="C56" s="2" t="s">
+      <c r="C56" s="1" t="s">
         <v>537</v>
       </c>
-      <c r="D56" s="2" t="s">
+      <c r="D56" s="1" t="s">
         <v>622</v>
       </c>
-      <c r="E56" s="3" t="s">
+      <c r="E56" s="2" t="s">
         <v>623</v>
       </c>
-      <c r="F56" s="2" t="s">
+      <c r="F56" s="1" t="s">
         <v>540</v>
       </c>
-      <c r="G56" s="2" t="s">
+      <c r="G56" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="H56" s="2" t="s">
+      <c r="H56" s="1" t="s">
         <v>541</v>
       </c>
-      <c r="I56" s="2" t="s">
+      <c r="I56" s="1" t="s">
         <v>624</v>
       </c>
-      <c r="J56" s="2" t="s">
+      <c r="J56" s="1" t="s">
         <v>625</v>
       </c>
-      <c r="K56" s="2" t="s">
+      <c r="K56" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="L56" s="2" t="s">
+      <c r="L56" s="1" t="s">
         <v>626</v>
       </c>
-      <c r="M56" s="2" t="s">
+      <c r="M56" s="1" t="s">
         <v>545</v>
       </c>
-      <c r="N56" s="2" t="s">
+      <c r="N56" s="1" t="s">
         <v>627</v>
       </c>
-      <c r="O56" s="2" t="s">
+      <c r="O56" s="1" t="s">
         <v>628</v>
       </c>
     </row>
-    <row r="57" spans="1:15">
-      <c r="A57" s="2" t="s">
+    <row r="57" spans="1:15" ht="84" customHeight="1">
+      <c r="A57" s="1" t="s">
         <v>629</v>
       </c>
-      <c r="B57" s="2" t="s">
+      <c r="B57" s="1" t="s">
         <v>259</v>
       </c>
-      <c r="C57" s="2" t="s">
+      <c r="C57" s="1" t="s">
         <v>537</v>
       </c>
-      <c r="D57" s="2" t="s">
+      <c r="D57" s="1" t="s">
         <v>630</v>
       </c>
-      <c r="E57" s="3" t="s">
+      <c r="E57" s="2" t="s">
         <v>631</v>
       </c>
-      <c r="F57" s="2" t="s">
+      <c r="F57" s="1" t="s">
         <v>540</v>
       </c>
-      <c r="G57" s="2" t="s">
+      <c r="G57" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="H57" s="2" t="s">
+      <c r="H57" s="1" t="s">
         <v>541</v>
       </c>
-      <c r="I57" s="2" t="s">
+      <c r="I57" s="1" t="s">
         <v>632</v>
       </c>
-      <c r="J57" s="2" t="s">
+      <c r="J57" s="1" t="s">
         <v>633</v>
       </c>
-      <c r="K57" s="2" t="s">
+      <c r="K57" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="L57" s="2" t="s">
+      <c r="L57" s="1" t="s">
         <v>618</v>
       </c>
-      <c r="M57" s="2" t="s">
+      <c r="M57" s="1" t="s">
         <v>545</v>
       </c>
-      <c r="N57" s="2" t="s">
+      <c r="N57" s="1" t="s">
         <v>634</v>
       </c>
-      <c r="O57" s="2" t="s">
+      <c r="O57" s="1" t="s">
         <v>635</v>
       </c>
     </row>
-    <row r="58" spans="1:15">
-      <c r="A58" s="2" t="s">
+    <row r="58" spans="1:15" ht="84" customHeight="1">
+      <c r="A58" s="1" t="s">
         <v>636</v>
       </c>
-      <c r="B58" s="2" t="s">
+      <c r="B58" s="1" t="s">
         <v>259</v>
       </c>
-      <c r="C58" s="2" t="s">
+      <c r="C58" s="1" t="s">
         <v>537</v>
       </c>
-      <c r="D58" s="2" t="s">
+      <c r="D58" s="1" t="s">
         <v>637</v>
       </c>
-      <c r="E58" s="3" t="s">
+      <c r="E58" s="2" t="s">
         <v>638</v>
       </c>
-      <c r="F58" s="2" t="s">
+      <c r="F58" s="1" t="s">
         <v>540</v>
       </c>
-      <c r="G58" s="2" t="s">
+      <c r="G58" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="H58" s="2" t="s">
+      <c r="H58" s="1" t="s">
         <v>541</v>
       </c>
-      <c r="I58" s="2" t="s">
+      <c r="I58" s="1" t="s">
         <v>639</v>
       </c>
-      <c r="J58" s="2" t="s">
+      <c r="J58" s="1" t="s">
         <v>640</v>
       </c>
-      <c r="K58" s="2" t="s">
+      <c r="K58" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="L58" s="2" t="s">
+      <c r="L58" s="1" t="s">
         <v>641</v>
       </c>
-      <c r="M58" s="2" t="s">
+      <c r="M58" s="1" t="s">
         <v>545</v>
       </c>
-      <c r="N58" s="2" t="s">
+      <c r="N58" s="1" t="s">
         <v>642</v>
       </c>
-      <c r="O58" s="2" t="s">
+      <c r="O58" s="1" t="s">
         <v>643</v>
       </c>
     </row>
-    <row r="59" spans="1:15">
-      <c r="A59" s="2" t="s">
+    <row r="59" spans="1:15" ht="84" customHeight="1">
+      <c r="A59" s="1" t="s">
         <v>644</v>
       </c>
-      <c r="B59" s="2" t="s">
+      <c r="B59" s="1" t="s">
         <v>259</v>
       </c>
-      <c r="C59" s="2" t="s">
+      <c r="C59" s="1" t="s">
         <v>537</v>
       </c>
-      <c r="D59" s="2" t="s">
+      <c r="D59" s="1" t="s">
         <v>645</v>
       </c>
-      <c r="E59" s="3" t="s">
+      <c r="E59" s="2" t="s">
         <v>646</v>
       </c>
-      <c r="F59" s="2" t="s">
+      <c r="F59" s="1" t="s">
         <v>540</v>
       </c>
-      <c r="G59" s="2" t="s">
+      <c r="G59" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="H59" s="2" t="s">
+      <c r="H59" s="1" t="s">
         <v>541</v>
       </c>
-      <c r="I59" s="2" t="s">
+      <c r="I59" s="1" t="s">
         <v>647</v>
       </c>
-      <c r="J59" s="2" t="s">
+      <c r="J59" s="1" t="s">
         <v>648</v>
       </c>
-      <c r="K59" s="2" t="s">
+      <c r="K59" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="L59" s="2" t="s">
+      <c r="L59" s="1" t="s">
         <v>649</v>
       </c>
-      <c r="M59" s="2" t="s">
+      <c r="M59" s="1" t="s">
         <v>545</v>
       </c>
-      <c r="N59" s="2" t="s">
+      <c r="N59" s="1" t="s">
         <v>650</v>
       </c>
-      <c r="O59" s="2" t="s">
+      <c r="O59" s="1" t="s">
         <v>651</v>
       </c>
     </row>
-    <row r="60" spans="1:15">
-      <c r="A60" s="2" t="s">
+    <row r="60" spans="1:15" ht="84" customHeight="1">
+      <c r="A60" s="1" t="s">
         <v>652</v>
       </c>
-      <c r="B60" s="2" t="s">
+      <c r="B60" s="1" t="s">
         <v>259</v>
       </c>
-      <c r="C60" s="2" t="s">
+      <c r="C60" s="1" t="s">
         <v>537</v>
       </c>
-      <c r="D60" s="2" t="s">
+      <c r="D60" s="1" t="s">
         <v>653</v>
       </c>
-      <c r="E60" s="3" t="s">
+      <c r="E60" s="2" t="s">
         <v>654</v>
       </c>
-      <c r="F60" s="2" t="s">
+      <c r="F60" s="1" t="s">
         <v>540</v>
       </c>
-      <c r="G60" s="2" t="s">
+      <c r="G60" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="H60" s="2" t="s">
+      <c r="H60" s="1" t="s">
         <v>541</v>
       </c>
-      <c r="I60" s="2" t="s">
+      <c r="I60" s="1" t="s">
         <v>655</v>
       </c>
-      <c r="J60" s="2" t="s">
+      <c r="J60" s="1" t="s">
         <v>656</v>
       </c>
-      <c r="K60" s="2" t="s">
+      <c r="K60" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="L60" s="2" t="s">
+      <c r="L60" s="1" t="s">
         <v>618</v>
       </c>
-      <c r="M60" s="2" t="s">
+      <c r="M60" s="1" t="s">
         <v>545</v>
       </c>
-      <c r="N60" s="2" t="s">
+      <c r="N60" s="1" t="s">
         <v>657</v>
       </c>
-      <c r="O60" s="2" t="s">
+      <c r="O60" s="1" t="s">
         <v>658</v>
       </c>
     </row>
-    <row r="61" spans="1:15">
-      <c r="A61" s="2" t="s">
+    <row r="61" spans="1:15" ht="84" customHeight="1">
+      <c r="A61" s="1" t="s">
         <v>659</v>
       </c>
-      <c r="B61" s="2" t="s">
+      <c r="B61" s="1" t="s">
         <v>259</v>
       </c>
-      <c r="C61" s="2" t="s">
+      <c r="C61" s="1" t="s">
         <v>537</v>
       </c>
-      <c r="D61" s="2" t="s">
+      <c r="D61" s="1" t="s">
         <v>660</v>
       </c>
-      <c r="E61" s="3" t="s">
+      <c r="E61" s="2" t="s">
         <v>661</v>
       </c>
-      <c r="F61" s="2" t="s">
+      <c r="F61" s="1" t="s">
         <v>540</v>
       </c>
-      <c r="G61" s="2" t="s">
+      <c r="G61" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="H61" s="2" t="s">
+      <c r="H61" s="1" t="s">
         <v>541</v>
       </c>
-      <c r="I61" s="2" t="s">
+      <c r="I61" s="1" t="s">
         <v>662</v>
       </c>
-      <c r="J61" s="2" t="s">
+      <c r="J61" s="1" t="s">
         <v>663</v>
       </c>
-      <c r="K61" s="2" t="s">
+      <c r="K61" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="L61" s="2" t="s">
+      <c r="L61" s="1" t="s">
         <v>664</v>
       </c>
-      <c r="M61" s="2" t="s">
+      <c r="M61" s="1" t="s">
         <v>545</v>
       </c>
-      <c r="N61" s="2" t="s">
+      <c r="N61" s="1" t="s">
         <v>665</v>
       </c>
-      <c r="O61" s="2" t="s">
+      <c r="O61" s="1" t="s">
         <v>666</v>
       </c>
     </row>
-    <row r="62" spans="1:15">
-      <c r="A62" s="2" t="s">
+    <row r="62" spans="1:15" ht="84" customHeight="1">
+      <c r="A62" s="1" t="s">
         <v>667</v>
       </c>
-      <c r="B62" s="2" t="s">
+      <c r="B62" s="1" t="s">
         <v>259</v>
       </c>
-      <c r="C62" s="2" t="s">
+      <c r="C62" s="1" t="s">
         <v>537</v>
       </c>
-      <c r="D62" s="2" t="s">
+      <c r="D62" s="1" t="s">
         <v>668</v>
       </c>
-      <c r="E62" s="3" t="s">
+      <c r="E62" s="2" t="s">
         <v>669</v>
       </c>
-      <c r="F62" s="2" t="s">
+      <c r="F62" s="1" t="s">
         <v>540</v>
       </c>
-      <c r="G62" s="2" t="s">
+      <c r="G62" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="H62" s="2" t="s">
+      <c r="H62" s="1" t="s">
         <v>541</v>
       </c>
-      <c r="I62" s="2" t="s">
+      <c r="I62" s="1" t="s">
         <v>670</v>
       </c>
-      <c r="J62" s="2" t="s">
+      <c r="J62" s="1" t="s">
         <v>671</v>
       </c>
-      <c r="K62" s="2" t="s">
+      <c r="K62" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="L62" s="2" t="s">
+      <c r="L62" s="1" t="s">
         <v>672</v>
       </c>
-      <c r="M62" s="2" t="s">
+      <c r="M62" s="1" t="s">
         <v>545</v>
       </c>
-      <c r="N62" s="2" t="s">
+      <c r="N62" s="1" t="s">
         <v>673</v>
       </c>
-      <c r="O62" s="2" t="s">
+      <c r="O62" s="1" t="s">
         <v>674</v>
       </c>
     </row>
-    <row r="63" spans="1:15">
-      <c r="A63" s="2" t="s">
+    <row r="63" spans="1:15" ht="84" customHeight="1">
+      <c r="A63" s="1" t="s">
         <v>675</v>
       </c>
-      <c r="B63" s="2" t="s">
+      <c r="B63" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="C63" s="2" t="s">
+      <c r="C63" s="1" t="s">
         <v>537</v>
       </c>
-      <c r="D63" s="2" t="s">
+      <c r="D63" s="1" t="s">
         <v>676</v>
       </c>
-      <c r="E63" s="3" t="s">
+      <c r="E63" s="2" t="s">
         <v>677</v>
       </c>
-      <c r="F63" s="2" t="s">
+      <c r="F63" s="1" t="s">
         <v>540</v>
       </c>
-      <c r="G63" s="2" t="s">
+      <c r="G63" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="H63" s="2" t="s">
+      <c r="H63" s="1" t="s">
         <v>541</v>
       </c>
-      <c r="I63" s="2" t="s">
+      <c r="I63" s="1" t="s">
         <v>678</v>
       </c>
-      <c r="J63" s="2" t="s">
+      <c r="J63" s="1" t="s">
         <v>679</v>
       </c>
-      <c r="K63" s="2" t="s">
+      <c r="K63" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="L63" s="2" t="s">
+      <c r="L63" s="1" t="s">
         <v>680</v>
       </c>
-      <c r="M63" s="2" t="s">
+      <c r="M63" s="1" t="s">
         <v>545</v>
       </c>
-      <c r="N63" s="2" t="s">
+      <c r="N63" s="1" t="s">
         <v>681</v>
       </c>
-      <c r="O63" s="2" t="s">
+      <c r="O63" s="1" t="s">
         <v>682</v>
       </c>
     </row>
-    <row r="64" spans="1:15">
-      <c r="A64" s="2" t="s">
+    <row r="64" spans="1:15" ht="84" customHeight="1">
+      <c r="A64" s="1" t="s">
         <v>683</v>
       </c>
-      <c r="B64" s="2" t="s">
+      <c r="B64" s="1" t="s">
         <v>684</v>
       </c>
-      <c r="C64" s="2" t="s">
+      <c r="C64" s="1" t="s">
         <v>537</v>
       </c>
-      <c r="D64" s="2" t="s">
+      <c r="D64" s="1" t="s">
         <v>685</v>
       </c>
-      <c r="E64" s="3" t="s">
+      <c r="E64" s="2" t="s">
         <v>686</v>
       </c>
-      <c r="F64" s="2" t="s">
+      <c r="F64" s="1" t="s">
         <v>540</v>
       </c>
-      <c r="G64" s="2" t="s">
+      <c r="G64" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="H64" s="2" t="s">
+      <c r="H64" s="1" t="s">
         <v>541</v>
       </c>
-      <c r="I64" s="2" t="s">
+      <c r="I64" s="1" t="s">
         <v>687</v>
       </c>
-      <c r="J64" s="2" t="s">
+      <c r="J64" s="1" t="s">
         <v>688</v>
       </c>
-      <c r="K64" s="2" t="s">
+      <c r="K64" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="L64" s="2" t="s">
+      <c r="L64" s="1" t="s">
         <v>689</v>
       </c>
-      <c r="M64" s="2" t="s">
+      <c r="M64" s="1" t="s">
         <v>545</v>
       </c>
-      <c r="N64" s="2" t="s">
+      <c r="N64" s="1" t="s">
         <v>690</v>
       </c>
-      <c r="O64" s="2" t="s">
+      <c r="O64" s="1" t="s">
         <v>691</v>
       </c>
     </row>
-    <row r="65" spans="1:15">
-      <c r="A65" s="2" t="s">
+    <row r="65" spans="1:15" ht="84" customHeight="1">
+      <c r="A65" s="1" t="s">
         <v>692</v>
       </c>
-      <c r="B65" s="2" t="s">
+      <c r="B65" s="1" t="s">
         <v>259</v>
       </c>
-      <c r="C65" s="2" t="s">
+      <c r="C65" s="1" t="s">
         <v>537</v>
       </c>
-      <c r="D65" s="2" t="s">
+      <c r="D65" s="1" t="s">
         <v>693</v>
       </c>
-      <c r="E65" s="3" t="s">
+      <c r="E65" s="2" t="s">
         <v>694</v>
       </c>
-      <c r="F65" s="2" t="s">
+      <c r="F65" s="1" t="s">
         <v>540</v>
       </c>
-      <c r="G65" s="2" t="s">
+      <c r="G65" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="H65" s="2" t="s">
+      <c r="H65" s="1" t="s">
         <v>541</v>
       </c>
-      <c r="I65" s="2" t="s">
+      <c r="I65" s="1" t="s">
         <v>695</v>
       </c>
-      <c r="J65" s="2" t="s">
+      <c r="J65" s="1" t="s">
         <v>696</v>
       </c>
-      <c r="K65" s="2" t="s">
+      <c r="K65" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="L65" s="2" t="s">
+      <c r="L65" s="1" t="s">
         <v>697</v>
       </c>
-      <c r="M65" s="2" t="s">
+      <c r="M65" s="1" t="s">
         <v>545</v>
       </c>
-      <c r="N65" s="2" t="s">
+      <c r="N65" s="1" t="s">
         <v>698</v>
       </c>
-      <c r="O65" s="2" t="s">
+      <c r="O65" s="1" t="s">
         <v>699</v>
       </c>
     </row>
-    <row r="66" spans="1:15">
-      <c r="A66" s="2" t="s">
+    <row r="66" spans="1:15" ht="84" customHeight="1">
+      <c r="A66" s="1" t="s">
         <v>700</v>
       </c>
-      <c r="B66" s="2" t="s">
+      <c r="B66" s="1" t="s">
         <v>259</v>
       </c>
-      <c r="C66" s="2" t="s">
+      <c r="C66" s="1" t="s">
         <v>537</v>
       </c>
-      <c r="D66" s="2" t="s">
+      <c r="D66" s="1" t="s">
         <v>701</v>
       </c>
-      <c r="E66" s="3" t="s">
+      <c r="E66" s="2" t="s">
         <v>702</v>
       </c>
-      <c r="F66" s="2" t="s">
+      <c r="F66" s="1" t="s">
         <v>567</v>
       </c>
-      <c r="G66" s="2" t="s">
+      <c r="G66" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="H66" s="2" t="s">
+      <c r="H66" s="1" t="s">
         <v>541</v>
       </c>
-      <c r="I66" s="2" t="s">
+      <c r="I66" s="1" t="s">
         <v>703</v>
       </c>
-      <c r="J66" s="2" t="s">
+      <c r="J66" s="1" t="s">
         <v>704</v>
       </c>
-      <c r="K66" s="2" t="s">
+      <c r="K66" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="L66" s="2" t="s">
+      <c r="L66" s="1" t="s">
         <v>268</v>
       </c>
-      <c r="M66" s="2" t="s">
+      <c r="M66" s="1" t="s">
         <v>545</v>
       </c>
-      <c r="N66" s="2" t="s">
+      <c r="N66" s="1" t="s">
         <v>705</v>
       </c>
-      <c r="O66" s="2" t="s">
+      <c r="O66" s="1" t="s">
         <v>706</v>
       </c>
     </row>
-    <row r="67" spans="1:15">
-      <c r="A67" s="2" t="s">
+    <row r="67" spans="1:15" ht="84" customHeight="1">
+      <c r="A67" s="1" t="s">
         <v>707</v>
       </c>
-      <c r="B67" s="2" t="s">
+      <c r="B67" s="1" t="s">
         <v>259</v>
       </c>
-      <c r="C67" s="2" t="s">
+      <c r="C67" s="1" t="s">
         <v>537</v>
       </c>
-      <c r="D67" s="2" t="s">
+      <c r="D67" s="1" t="s">
         <v>708</v>
       </c>
-      <c r="E67" s="3" t="s">
+      <c r="E67" s="2" t="s">
         <v>709</v>
       </c>
-      <c r="F67" s="2" t="s">
+      <c r="F67" s="1" t="s">
         <v>540</v>
       </c>
-      <c r="G67" s="2" t="s">
+      <c r="G67" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="H67" s="2" t="s">
+      <c r="H67" s="1" t="s">
         <v>541</v>
       </c>
-      <c r="I67" s="2" t="s">
+      <c r="I67" s="1" t="s">
         <v>710</v>
       </c>
-      <c r="J67" s="2" t="s">
+      <c r="J67" s="1" t="s">
         <v>711</v>
       </c>
-      <c r="K67" s="2" t="s">
+      <c r="K67" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="L67" s="2" t="s">
+      <c r="L67" s="1" t="s">
         <v>712</v>
       </c>
-      <c r="M67" s="2" t="s">
+      <c r="M67" s="1" t="s">
         <v>545</v>
       </c>
-      <c r="N67" s="2" t="s">
+      <c r="N67" s="1" t="s">
         <v>713</v>
       </c>
-      <c r="O67" s="2" t="s">
+      <c r="O67" s="1" t="s">
         <v>714</v>
       </c>
     </row>
-    <row r="68" spans="1:15">
-      <c r="A68" s="2" t="s">
+    <row r="68" spans="1:15" ht="84" customHeight="1">
+      <c r="A68" s="1" t="s">
         <v>715</v>
       </c>
-      <c r="B68" s="2" t="s">
+      <c r="B68" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="C68" s="2" t="s">
+      <c r="C68" s="1" t="s">
         <v>537</v>
       </c>
-      <c r="D68" s="2" t="s">
+      <c r="D68" s="1" t="s">
         <v>716</v>
       </c>
-      <c r="E68" s="3" t="s">
+      <c r="E68" s="2" t="s">
         <v>717</v>
       </c>
-      <c r="F68" s="2" t="s">
+      <c r="F68" s="1" t="s">
         <v>540</v>
       </c>
-      <c r="G68" s="2" t="s">
+      <c r="G68" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="H68" s="2" t="s">
+      <c r="H68" s="1" t="s">
         <v>541</v>
       </c>
-      <c r="I68" s="2" t="s">
+      <c r="I68" s="1" t="s">
         <v>718</v>
       </c>
-      <c r="J68" s="2" t="s">
+      <c r="J68" s="1" t="s">
         <v>719</v>
       </c>
-      <c r="K68" s="2" t="s">
+      <c r="K68" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="L68" s="2" t="s">
+      <c r="L68" s="1" t="s">
         <v>720</v>
       </c>
-      <c r="M68" s="2" t="s">
+      <c r="M68" s="1" t="s">
         <v>545</v>
       </c>
-      <c r="N68" s="2" t="s">
+      <c r="N68" s="1" t="s">
         <v>721</v>
       </c>
-      <c r="O68" s="2" t="s">
+      <c r="O68" s="1" t="s">
         <v>722</v>
       </c>
     </row>
-    <row r="69" spans="1:15">
-      <c r="A69" s="2" t="s">
+    <row r="69" spans="1:15" ht="84" customHeight="1">
+      <c r="A69" s="1" t="s">
         <v>723</v>
       </c>
-      <c r="B69" s="2" t="s">
+      <c r="B69" s="1" t="s">
         <v>684</v>
       </c>
-      <c r="C69" s="2" t="s">
+      <c r="C69" s="1" t="s">
         <v>537</v>
       </c>
-      <c r="D69" s="2" t="s">
+      <c r="D69" s="1" t="s">
         <v>724</v>
       </c>
-      <c r="E69" s="3" t="s">
+      <c r="E69" s="2" t="s">
         <v>725</v>
       </c>
-      <c r="F69" s="2" t="s">
+      <c r="F69" s="1" t="s">
         <v>540</v>
       </c>
-      <c r="G69" s="2" t="s">
+      <c r="G69" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="H69" s="2" t="s">
+      <c r="H69" s="1" t="s">
         <v>541</v>
       </c>
-      <c r="I69" s="2" t="s">
+      <c r="I69" s="1" t="s">
         <v>726</v>
       </c>
-      <c r="J69" s="2" t="s">
+      <c r="J69" s="1" t="s">
         <v>727</v>
       </c>
-      <c r="K69" s="2" t="s">
+      <c r="K69" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="L69" s="2" t="s">
+      <c r="L69" s="1" t="s">
         <v>728</v>
       </c>
-      <c r="M69" s="2" t="s">
+      <c r="M69" s="1" t="s">
         <v>545</v>
       </c>
-      <c r="N69" s="2" t="s">
+      <c r="N69" s="1" t="s">
         <v>729</v>
       </c>
-      <c r="O69" s="2" t="s">
+      <c r="O69" s="1" t="s">
         <v>730</v>
       </c>
     </row>
-    <row r="70" spans="1:15">
-      <c r="A70" s="2" t="s">
+    <row r="70" spans="1:15" ht="84" customHeight="1">
+      <c r="A70" s="1" t="s">
         <v>731</v>
       </c>
-      <c r="B70" s="2" t="s">
+      <c r="B70" s="1" t="s">
         <v>684</v>
       </c>
-      <c r="C70" s="2" t="s">
+      <c r="C70" s="1" t="s">
         <v>537</v>
       </c>
-      <c r="D70" s="2" t="s">
+      <c r="D70" s="1" t="s">
         <v>732</v>
       </c>
-      <c r="E70" s="3" t="s">
+      <c r="E70" s="2" t="s">
         <v>733</v>
       </c>
-      <c r="F70" s="2" t="s">
+      <c r="F70" s="1" t="s">
         <v>540</v>
       </c>
-      <c r="G70" s="2" t="s">
+      <c r="G70" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="H70" s="2" t="s">
+      <c r="H70" s="1" t="s">
         <v>541</v>
       </c>
-      <c r="I70" s="2" t="s">
+      <c r="I70" s="1" t="s">
         <v>734</v>
       </c>
-      <c r="J70" s="2" t="s">
+      <c r="J70" s="1" t="s">
         <v>735</v>
       </c>
-      <c r="K70" s="2" t="s">
+      <c r="K70" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="L70" s="2" t="s">
+      <c r="L70" s="1" t="s">
         <v>618</v>
       </c>
-      <c r="M70" s="2" t="s">
+      <c r="M70" s="1" t="s">
         <v>545</v>
       </c>
-      <c r="N70" s="2" t="s">
+      <c r="N70" s="1" t="s">
         <v>736</v>
       </c>
-      <c r="O70" s="2" t="s">
+      <c r="O70" s="1" t="s">
         <v>737</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O70"/>
-  <hyperlinks>
-    <hyperlink ref="E2" r:id="rId1"/>
-    <hyperlink ref="E3" r:id="rId2"/>
-    <hyperlink ref="E4" r:id="rId3"/>
-    <hyperlink ref="E5" r:id="rId4"/>
-    <hyperlink ref="E6" r:id="rId5"/>
-    <hyperlink ref="E7" r:id="rId6"/>
-    <hyperlink ref="E8" r:id="rId7"/>
-    <hyperlink ref="E9" r:id="rId8"/>
-    <hyperlink ref="E10" r:id="rId9"/>
-    <hyperlink ref="E11" r:id="rId10"/>
-    <hyperlink ref="E12" r:id="rId11"/>
-    <hyperlink ref="E13" r:id="rId12"/>
-    <hyperlink ref="E14" r:id="rId13"/>
-    <hyperlink ref="E15" r:id="rId14"/>
-    <hyperlink ref="E16" r:id="rId15"/>
-    <hyperlink ref="E17" r:id="rId16"/>
-    <hyperlink ref="E18" r:id="rId17"/>
-    <hyperlink ref="E19" r:id="rId18"/>
-    <hyperlink ref="E20" r:id="rId19"/>
-    <hyperlink ref="E21" r:id="rId20"/>
-    <hyperlink ref="E22" r:id="rId21"/>
-    <hyperlink ref="E23" r:id="rId22"/>
-    <hyperlink ref="E24" r:id="rId23"/>
-    <hyperlink ref="E25" r:id="rId24"/>
-    <hyperlink ref="E26" r:id="rId25"/>
-    <hyperlink ref="E27" r:id="rId26"/>
-    <hyperlink ref="E28" r:id="rId27"/>
-    <hyperlink ref="E29" r:id="rId28"/>
-    <hyperlink ref="E30" r:id="rId29"/>
-    <hyperlink ref="E31" r:id="rId30"/>
-    <hyperlink ref="E32" r:id="rId31"/>
-    <hyperlink ref="E33" r:id="rId32"/>
-    <hyperlink ref="E34" r:id="rId33"/>
-    <hyperlink ref="E35" r:id="rId34"/>
-    <hyperlink ref="E36" r:id="rId35"/>
-    <hyperlink ref="E37" r:id="rId36"/>
-    <hyperlink ref="E38" r:id="rId37"/>
-    <hyperlink ref="E39" r:id="rId38"/>
-    <hyperlink ref="E40" r:id="rId39"/>
-    <hyperlink ref="E41" r:id="rId40"/>
-    <hyperlink ref="E42" r:id="rId41"/>
-    <hyperlink ref="E43" r:id="rId42"/>
-    <hyperlink ref="E44" r:id="rId43"/>
-    <hyperlink ref="E45" r:id="rId44"/>
-    <hyperlink ref="E46" r:id="rId45"/>
-    <hyperlink ref="E47" r:id="rId46"/>
-    <hyperlink ref="E48" r:id="rId47"/>
-    <hyperlink ref="E49" r:id="rId48"/>
-    <hyperlink ref="E50" r:id="rId49"/>
-    <hyperlink ref="E51" r:id="rId50"/>
-    <hyperlink ref="E52" r:id="rId51"/>
-    <hyperlink ref="E53" r:id="rId52"/>
-    <hyperlink ref="E54" r:id="rId53"/>
-    <hyperlink ref="E55" r:id="rId54"/>
-    <hyperlink ref="E56" r:id="rId55"/>
-    <hyperlink ref="E57" r:id="rId56"/>
-    <hyperlink ref="E58" r:id="rId57"/>
-    <hyperlink ref="E59" r:id="rId58"/>
-    <hyperlink ref="E60" r:id="rId59"/>
-    <hyperlink ref="E61" r:id="rId60"/>
-    <hyperlink ref="E62" r:id="rId61"/>
-    <hyperlink ref="E63" r:id="rId62"/>
-    <hyperlink ref="E64" r:id="rId63"/>
-    <hyperlink ref="E65" r:id="rId64"/>
-    <hyperlink ref="E66" r:id="rId65"/>
-    <hyperlink ref="E67" r:id="rId66"/>
-    <hyperlink ref="E68" r:id="rId67"/>
-    <hyperlink ref="E69" r:id="rId68"/>
-    <hyperlink ref="E70" r:id="rId69"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
+  <pageSetup fitToHeight="0" orientation="landscape"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add ConnectEDU patent and MyDataButton sources
</commit_message>
<xml_diff>
--- a/dossier/source_dossier.xlsx
+++ b/dossier/source_dossier.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1065" uniqueCount="738">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1125" uniqueCount="785">
   <si>
     <t>id</t>
   </si>
@@ -316,6 +316,51 @@
     <t>{{cite web |title=ConnectEdu: Funding, Team &amp; Investors |url=https://startupintros.com/orgs/connectedu |website=Startup Intros |access-date=June 8, 2026}}</t>
   </si>
   <si>
+    <t>SSV1</t>
+  </si>
+  <si>
+    <t>2009</t>
+  </si>
+  <si>
+    <t>SlideServe / Studylib mirror</t>
+  </si>
+  <si>
+    <t>A Standards-Based Data Exchange Network</t>
+  </si>
+  <si>
+    <t>https://www.slideserve.com/licia/a-standards-based-data-exchange-network</t>
+  </si>
+  <si>
+    <t>Platform-hosted presentation / source lead</t>
+  </si>
+  <si>
+    <t>No or partial; platform-hosted and likely self/affiliated</t>
+  </si>
+  <si>
+    <t>Medium for slide-image evidence; page shell blocked but individual slide images verified</t>
+  </si>
+  <si>
+    <t>Minor. Downloaded SlideServe slide images verify a ConnectEDU-branded presentation titled `A Standards Based Data Exchange Network`. Slide 1 lists Jeff Alderson as Director of Pre-Sales Solutions, gives a ConnectEDU email address, and dates the presentation April 8, 2009.</t>
+  </si>
+  <si>
+    <t>Alderson was associated with ConnectEDU as Director of Pre-Sales Solutions in an April 8, 2009 standards-based data exchange network presentation.</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>Retain as supporting ConnectEDU-era professional-context evidence only; do not use as AfC notability support.</t>
+  </si>
+  <si>
+    <t>Verified from downloaded slide images; SlideServe page shell blocked</t>
+  </si>
+  <si>
+    <t>Reviewed in sources/connectedu_company_sources.md; local slide images in data/slideserve_standards_based_data_exchange_network_images/; blocked page file data/slideserve_standards_based_data_exchange_network.html</t>
+  </si>
+  <si>
+    <t>{{cite web |title=A Standards-Based Data Exchange Network |url=https://www.slideserve.com/licia/a-standards-based-data-exchange-network |website=SlideServe |date=April 8, 2009 |access-date=June 8, 2026}}</t>
+  </si>
+  <si>
     <t>S2</t>
   </si>
   <si>
@@ -406,9 +451,6 @@
     <t>Alderson was listed as a keynote presenter at Eduventures Summit 2016 and was identified as Principal Analyst at Eduventures; the post also corroborates his public commentary on online proctoring.</t>
   </si>
   <si>
-    <t>Low</t>
-  </si>
-  <si>
     <t>Use only for Eduventures Summit / online-proctoring professional context; not a notability anchor because the source is a vendor promotional blog.</t>
   </si>
   <si>
@@ -433,9 +475,6 @@
     <t>Slide deck / platform-hosted presentation</t>
   </si>
   <si>
-    <t>No or partial; platform-hosted and likely self/affiliated</t>
-  </si>
-  <si>
     <t>Medium for deck text and presentation metadata; weak for notability</t>
   </si>
   <si>
@@ -2228,6 +2267,108 @@
   </si>
   <si>
     <t>{{cite web |last=Brown |first=Bob |title=Natick Town Meeting recap week #3: Dissolved; Dam, Dam &amp; Dam articles; Capital concerns &amp; other business |url=https://www.natickreport.com/2023/05/natick-town-meeting-recap-week-3-dissolved-dam-dam-capital-concerns-other-business/ |website=Natick Report |date=May 12, 2023 |access-date=June 8, 2026}}</t>
+  </si>
+  <si>
+    <t>JPT1</t>
+  </si>
+  <si>
+    <t>Justia Patents</t>
+  </si>
+  <si>
+    <t>Patents Assigned to ConnectEDU, Inc.</t>
+  </si>
+  <si>
+    <t>https://patents.justia.com/assignee/connectedu-inc</t>
+  </si>
+  <si>
+    <t>Patent database / assignee listing</t>
+  </si>
+  <si>
+    <t>Partial / database listing</t>
+  </si>
+  <si>
+    <t>Medium for patent metadata; low for biographical claims</t>
+  </si>
+  <si>
+    <t>Narrow patent-metadata source. Justia indexes ConnectEDU patent applications and live search-index results show at least one ConnectEDU application listing Jeffrey Alderson among the inventors. Direct local fetch returned a Cloudflare challenge page.</t>
+  </si>
+  <si>
+    <t>ConnectEDU patent-application metadata and a narrow inventor-context lead for Alderson.</t>
+  </si>
+  <si>
+    <t>Dossier/source lead only unless browser review confirms exact patent pages. Do not use for AfC notability.</t>
+  </si>
+  <si>
+    <t>Partially verified from Justia search-index result; direct local fetch blocked by Cloudflare challenge</t>
+  </si>
+  <si>
+    <t>Reviewed in sources/patent_sources.md; local file data/justia_patents_connectedu_inc.html is a Cloudflare challenge page, not useful source content</t>
+  </si>
+  <si>
+    <t>{{cite web |title=Patents Assigned to ConnectEDU, Inc. |url=https://patents.justia.com/assignee/connectedu-inc |website=Justia Patents |access-date=June 8, 2026}}</t>
+  </si>
+  <si>
+    <t>GSC1</t>
+  </si>
+  <si>
+    <t>Google Scholar</t>
+  </si>
+  <si>
+    <t>Jeff Alderson - Google Scholar profile</t>
+  </si>
+  <si>
+    <t>https://scholar.google.com/citations?hl=en&amp;user=mhuGZ-EAAAAJ</t>
+  </si>
+  <si>
+    <t>Scholar profile / patent and publication index</t>
+  </si>
+  <si>
+    <t>No / profile-index source</t>
+  </si>
+  <si>
+    <t>Medium for profile-index metadata; low for independent biographical claims</t>
+  </si>
+  <si>
+    <t>Profile page lists Jeff Alderson as Education Product Marketing at MathWorks and includes patent-application entries for Apparatus and Methods for an Application Process and Data Analysis with C. Powell, J. Alderson, S. Mansfield, and H. Van Zile as authors/inventors.</t>
+  </si>
+  <si>
+    <t>Patent-application index entries: US Patent App. 11/406,065 (2006), US Patent App. 13/618,015 (2013), and US Patent App. 13/618,249 (2013); also lists the ASEE MATLAB Grader paper.</t>
+  </si>
+  <si>
+    <t>Useful for patent/publication discovery and corroborating patent metadata. Do not use for AfC notability; prefer underlying patent records for article claims.</t>
+  </si>
+  <si>
+    <t>Verified from downloaded Google Scholar profile HTML</t>
+  </si>
+  <si>
+    <t>Reviewed in sources/patent_sources.md; local file data/google_scholar_jeff_alderson.html</t>
+  </si>
+  <si>
+    <t>{{cite web |title=Jeff Alderson - Google Scholar |url=https://scholar.google.com/citations?hl=en&amp;user=mhuGZ-EAAAAJ |website=Google Scholar |access-date=June 8, 2026}}</t>
+  </si>
+  <si>
+    <t>NCES2013</t>
+  </si>
+  <si>
+    <t>NCES / MIS Conference</t>
+  </si>
+  <si>
+    <t>26th Annual Management Information Systems (MIS) Conference agenda</t>
+  </si>
+  <si>
+    <t>https://nces.ed.gov/whatsnew/conferences/pdf/MIS_2013_Agenda.pdf</t>
+  </si>
+  <si>
+    <t>Moderate for narrow MyDataButton involvement. Agenda lists session `IX-F MyDataButton` with Michael Sessa of PESC, Jeffrey Alderson of ConnectEDU, Inc., and Shawn Bay of eScholar LLC; session description says the White House and U.S. Department of Education teamed up on MyDataButton and that PESC representatives had participated in the initiative.</t>
+  </si>
+  <si>
+    <t>Alderson was listed as a ConnectEDU participant in an NCES MIS 2013 conference session on MyDataButton, an initiative described by the agenda as involving the White House and U.S. Department of Education.</t>
+  </si>
+  <si>
+    <t>Reviewed in sources/mydata_button_sources.md and sources/pesc_sources.md; local files data/nces_mis_2013_agenda.pdf and data/nces_mis_2013_agenda.txt</t>
+  </si>
+  <si>
+    <t>{{cite conference |title=26th Annual Management Information Systems (MIS) Conference agenda |conference=Management Information Systems Conference |publisher=National Center for Education Statistics |date=2013 |url=https://nces.ed.gov/whatsnew/conferences/pdf/MIS_2013_Agenda.pdf |access-date=June 8, 2026}}</t>
   </si>
 </sst>
 </file>
@@ -2304,8 +2445,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:O70" totalsRowShown="0">
-  <autoFilter ref="A1:O70"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SourceDossier" displayName="SourceDossier" ref="A1:O74" totalsRowShown="0">
+  <autoFilter ref="A1:O74"/>
   <tableColumns count="15">
     <tableColumn id="1" name="id"/>
     <tableColumn id="2" name="year"/>
@@ -2612,29 +2753,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <sheetPr>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="A1:O70"/>
+  <dimension ref="A1:O74"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="13.7109375" customWidth="1"/>
-    <col min="2" max="2" width="14.7109375" customWidth="1"/>
-    <col min="3" max="3" width="30.7109375" customWidth="1"/>
-    <col min="4" max="4" width="46.7109375" customWidth="1"/>
-    <col min="5" max="5" width="58.7109375" customWidth="1"/>
-    <col min="6" max="6" width="30.7109375" customWidth="1"/>
-    <col min="7" max="7" width="22.7109375" customWidth="1"/>
-    <col min="8" max="8" width="36.7109375" customWidth="1"/>
-    <col min="9" max="10" width="64.7109375" customWidth="1"/>
-    <col min="11" max="11" width="20.7109375" customWidth="1"/>
-    <col min="12" max="12" width="54.7109375" customWidth="1"/>
-    <col min="13" max="13" width="34.7109375" customWidth="1"/>
-    <col min="14" max="14" width="60.7109375" customWidth="1"/>
-    <col min="15" max="15" width="72.7109375" customWidth="1"/>
+    <col min="1" max="2" width="10.7109375" customWidth="1"/>
+    <col min="3" max="3" width="24.7109375" customWidth="1"/>
+    <col min="4" max="4" width="44.7109375" customWidth="1"/>
+    <col min="5" max="5" width="52.7109375" customWidth="1"/>
+    <col min="6" max="6" width="24.7109375" customWidth="1"/>
+    <col min="7" max="7" width="18.7109375" customWidth="1"/>
+    <col min="8" max="8" width="34.7109375" customWidth="1"/>
+    <col min="9" max="10" width="52.7109375" customWidth="1"/>
+    <col min="11" max="11" width="18.7109375" customWidth="1"/>
+    <col min="12" max="12" width="44.7109375" customWidth="1"/>
+    <col min="13" max="13" width="32.7109375" customWidth="1"/>
+    <col min="14" max="14" width="52.7109375" customWidth="1"/>
+    <col min="15" max="15" width="64.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="42" customHeight="1">
+    <row r="1" spans="1:15" ht="36" customHeight="1">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2983,51 +3120,51 @@
         <v>105</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>21</v>
+        <v>106</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>25</v>
+        <v>107</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="L8" s="1" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="M8" s="1" t="s">
-        <v>83</v>
+        <v>112</v>
       </c>
       <c r="N8" s="1" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="O8" s="1" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
     </row>
     <row r="9" spans="1:15" ht="84" customHeight="1">
       <c r="A9" s="1" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>101</v>
+        <v>116</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>105</v>
+        <v>120</v>
       </c>
       <c r="G9" s="1" t="s">
         <v>21</v>
@@ -3036,283 +3173,283 @@
         <v>25</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="L9" s="1" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="M9" s="1" t="s">
         <v>83</v>
       </c>
       <c r="N9" s="1" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="O9" s="1" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
     </row>
     <row r="10" spans="1:15" ht="84" customHeight="1">
       <c r="A10" s="1" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>101</v>
+        <v>116</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>126</v>
+        <v>21</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>127</v>
+        <v>25</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="L10" s="1" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="M10" s="1" t="s">
-        <v>42</v>
+        <v>83</v>
       </c>
       <c r="N10" s="1" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="O10" s="1" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="11" spans="1:15" ht="84" customHeight="1">
       <c r="A11" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>101</v>
+        <v>116</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="K11" s="1" t="s">
-        <v>130</v>
+        <v>110</v>
       </c>
       <c r="L11" s="1" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="M11" s="1" t="s">
         <v>42</v>
       </c>
       <c r="N11" s="1" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="O11" s="1" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="12" spans="1:15" ht="84" customHeight="1">
       <c r="A12" s="1" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>147</v>
+        <v>116</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>92</v>
+        <v>106</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="K12" s="1" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="L12" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="M12" s="1" t="s">
-        <v>83</v>
+        <v>42</v>
       </c>
       <c r="N12" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="O12" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="13" spans="1:15" ht="84" customHeight="1">
       <c r="A13" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="G13" s="1" t="s">
         <v>92</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="K13" s="1" t="s">
-        <v>117</v>
+        <v>132</v>
       </c>
       <c r="L13" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="M13" s="1" t="s">
         <v>83</v>
       </c>
       <c r="N13" s="1" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="O13" s="1" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="14" spans="1:15" ht="84" customHeight="1">
       <c r="A14" s="1" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="G14" s="1" t="s">
         <v>92</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="J14" s="1" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="K14" s="1" t="s">
-        <v>117</v>
+        <v>132</v>
       </c>
       <c r="L14" s="1" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="M14" s="1" t="s">
         <v>83</v>
       </c>
       <c r="N14" s="1" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="O14" s="1" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="15" spans="1:15" ht="84" customHeight="1">
       <c r="A15" s="1" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>188</v>
+        <v>92</v>
       </c>
       <c r="H15" s="1" t="s">
         <v>189</v>
@@ -3324,74 +3461,74 @@
         <v>191</v>
       </c>
       <c r="K15" s="1" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="L15" s="1" t="s">
         <v>192</v>
       </c>
       <c r="M15" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="N15" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="N15" s="1" t="s">
+      <c r="O15" s="1" t="s">
         <v>194</v>
-      </c>
-      <c r="O15" s="1" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="16" spans="1:15" ht="84" customHeight="1">
       <c r="A16" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="B16" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="C16" s="1" t="s">
         <v>197</v>
       </c>
-      <c r="C16" s="1" t="s">
+      <c r="D16" s="1" t="s">
         <v>198</v>
       </c>
-      <c r="D16" s="1" t="s">
+      <c r="E16" s="2" t="s">
         <v>199</v>
       </c>
-      <c r="E16" s="2" t="s">
+      <c r="F16" s="1" t="s">
         <v>200</v>
       </c>
-      <c r="F16" s="1" t="s">
+      <c r="G16" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="G16" s="1" t="s">
+      <c r="H16" s="1" t="s">
         <v>202</v>
       </c>
-      <c r="H16" s="1" t="s">
+      <c r="I16" s="1" t="s">
         <v>203</v>
       </c>
-      <c r="I16" s="1" t="s">
+      <c r="J16" s="1" t="s">
         <v>204</v>
       </c>
-      <c r="J16" s="1" t="s">
+      <c r="K16" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="L16" s="1" t="s">
         <v>205</v>
       </c>
-      <c r="K16" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="L16" s="1" t="s">
+      <c r="M16" s="1" t="s">
         <v>206</v>
       </c>
-      <c r="M16" s="1" t="s">
+      <c r="N16" s="1" t="s">
         <v>207</v>
       </c>
-      <c r="N16" s="1" t="s">
+      <c r="O16" s="1" t="s">
         <v>208</v>
-      </c>
-      <c r="O16" s="1" t="s">
-        <v>209</v>
       </c>
     </row>
     <row r="17" spans="1:15" ht="84" customHeight="1">
       <c r="A17" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="B17" s="1" t="s">
         <v>210</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>197</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>211</v>
@@ -3438,134 +3575,134 @@
         <v>223</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>87</v>
+        <v>210</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>211</v>
+        <v>224</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>215</v>
+        <v>228</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="I18" s="1" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="J18" s="1" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="K18" s="1" t="s">
-        <v>130</v>
+        <v>96</v>
       </c>
       <c r="L18" s="1" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="M18" s="1" t="s">
-        <v>83</v>
+        <v>233</v>
       </c>
       <c r="N18" s="1" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="O18" s="1" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
     </row>
     <row r="19" spans="1:15" ht="84" customHeight="1">
       <c r="A19" s="1" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>31</v>
+        <v>87</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>234</v>
+        <v>224</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>238</v>
+        <v>228</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="I19" s="1" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="J19" s="1" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="K19" s="1" t="s">
-        <v>96</v>
+        <v>110</v>
       </c>
       <c r="L19" s="1" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="M19" s="1" t="s">
         <v>83</v>
       </c>
       <c r="N19" s="1" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="O19" s="1" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="20" spans="1:15" ht="84" customHeight="1">
       <c r="A20" s="1" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>197</v>
+        <v>31</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="H20" s="1" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="I20" s="1" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="J20" s="1" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="K20" s="1" t="s">
-        <v>81</v>
+        <v>96</v>
       </c>
       <c r="L20" s="1" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="M20" s="1" t="s">
-        <v>255</v>
+        <v>83</v>
       </c>
       <c r="N20" s="1" t="s">
         <v>256</v>
@@ -3579,210 +3716,210 @@
         <v>258</v>
       </c>
       <c r="B21" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="C21" s="1" t="s">
         <v>259</v>
       </c>
-      <c r="C21" s="1" t="s">
+      <c r="D21" s="1" t="s">
         <v>260</v>
       </c>
-      <c r="D21" s="1" t="s">
+      <c r="E21" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="E21" s="2" t="s">
+      <c r="F21" s="1" t="s">
         <v>262</v>
       </c>
-      <c r="F21" s="1" t="s">
+      <c r="G21" s="1" t="s">
         <v>263</v>
       </c>
-      <c r="G21" s="1" t="s">
+      <c r="H21" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="H21" s="1" t="s">
+      <c r="I21" s="1" t="s">
         <v>265</v>
       </c>
-      <c r="I21" s="1" t="s">
+      <c r="J21" s="1" t="s">
         <v>266</v>
       </c>
-      <c r="J21" s="1" t="s">
+      <c r="K21" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="L21" s="1" t="s">
         <v>267</v>
       </c>
-      <c r="K21" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="L21" s="1" t="s">
+      <c r="M21" s="1" t="s">
         <v>268</v>
       </c>
-      <c r="M21" s="1" t="s">
+      <c r="N21" s="1" t="s">
         <v>269</v>
       </c>
-      <c r="N21" s="1" t="s">
+      <c r="O21" s="1" t="s">
         <v>270</v>
-      </c>
-      <c r="O21" s="1" t="s">
-        <v>271</v>
       </c>
     </row>
     <row r="22" spans="1:15" ht="84" customHeight="1">
       <c r="A22" s="1" t="s">
+        <v>271</v>
+      </c>
+      <c r="B22" s="1" t="s">
         <v>272</v>
       </c>
-      <c r="B22" s="1" t="s">
-        <v>259</v>
-      </c>
       <c r="C22" s="1" t="s">
-        <v>260</v>
+        <v>273</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>21</v>
+        <v>277</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="I22" s="1" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="J22" s="1" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="K22" s="1" t="s">
-        <v>130</v>
+        <v>110</v>
       </c>
       <c r="L22" s="1" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="M22" s="1" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="N22" s="1" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="O22" s="1" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
     </row>
     <row r="23" spans="1:15" ht="84" customHeight="1">
       <c r="A23" s="1" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>259</v>
+        <v>272</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>260</v>
+        <v>273</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>275</v>
+        <v>288</v>
       </c>
       <c r="G23" s="1" t="s">
         <v>21</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>276</v>
+        <v>289</v>
       </c>
       <c r="I23" s="1" t="s">
-        <v>286</v>
+        <v>290</v>
       </c>
       <c r="J23" s="1" t="s">
-        <v>287</v>
+        <v>291</v>
       </c>
       <c r="K23" s="1" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="L23" s="1" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="M23" s="1" t="s">
-        <v>280</v>
+        <v>293</v>
       </c>
       <c r="N23" s="1" t="s">
-        <v>289</v>
+        <v>294</v>
       </c>
       <c r="O23" s="1" t="s">
-        <v>290</v>
+        <v>295</v>
       </c>
     </row>
     <row r="24" spans="1:15" ht="84" customHeight="1">
       <c r="A24" s="1" t="s">
-        <v>291</v>
+        <v>296</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>87</v>
+        <v>272</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>292</v>
+        <v>273</v>
       </c>
       <c r="D24" s="1" t="s">
+        <v>297</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="F24" s="1" t="s">
+        <v>288</v>
+      </c>
+      <c r="G24" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="H24" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="I24" s="1" t="s">
+        <v>299</v>
+      </c>
+      <c r="J24" s="1" t="s">
+        <v>300</v>
+      </c>
+      <c r="K24" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="L24" s="1" t="s">
+        <v>301</v>
+      </c>
+      <c r="M24" s="1" t="s">
         <v>293</v>
       </c>
-      <c r="E24" s="2" t="s">
-        <v>294</v>
-      </c>
-      <c r="F24" s="1" t="s">
-        <v>295</v>
-      </c>
-      <c r="G24" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="H24" s="1" t="s">
-        <v>296</v>
-      </c>
-      <c r="I24" s="1" t="s">
-        <v>297</v>
-      </c>
-      <c r="J24" s="1" t="s">
-        <v>298</v>
-      </c>
-      <c r="K24" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="L24" s="1" t="s">
-        <v>299</v>
-      </c>
-      <c r="M24" s="1" t="s">
-        <v>83</v>
-      </c>
       <c r="N24" s="1" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="O24" s="1" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
     </row>
     <row r="25" spans="1:15" ht="84" customHeight="1">
       <c r="A25" s="1" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>303</v>
+        <v>87</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>308</v>
+        <v>92</v>
       </c>
       <c r="H25" s="1" t="s">
         <v>309</v>
@@ -3794,7 +3931,7 @@
         <v>311</v>
       </c>
       <c r="K25" s="1" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="L25" s="1" t="s">
         <v>312</v>
@@ -3829,25 +3966,25 @@
         <v>320</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>308</v>
+        <v>321</v>
       </c>
       <c r="H26" s="1" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="I26" s="1" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="J26" s="1" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="K26" s="1" t="s">
-        <v>130</v>
+        <v>110</v>
       </c>
       <c r="L26" s="1" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="M26" s="1" t="s">
-        <v>325</v>
+        <v>83</v>
       </c>
       <c r="N26" s="1" t="s">
         <v>326</v>
@@ -3861,322 +3998,322 @@
         <v>328</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>316</v>
+        <v>329</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>304</v>
+        <v>330</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>308</v>
+        <v>321</v>
       </c>
       <c r="H27" s="1" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="I27" s="1" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="J27" s="1" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="K27" s="1" t="s">
-        <v>130</v>
+        <v>110</v>
       </c>
       <c r="L27" s="1" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="M27" s="1" t="s">
-        <v>325</v>
+        <v>338</v>
       </c>
       <c r="N27" s="1" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="O27" s="1" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
     </row>
     <row r="28" spans="1:15" ht="84" customHeight="1">
       <c r="A28" s="1" t="s">
+        <v>341</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>317</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>342</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>343</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="G28" s="1" t="s">
+        <v>321</v>
+      </c>
+      <c r="H28" s="1" t="s">
+        <v>345</v>
+      </c>
+      <c r="I28" s="1" t="s">
+        <v>346</v>
+      </c>
+      <c r="J28" s="1" t="s">
+        <v>347</v>
+      </c>
+      <c r="K28" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="L28" s="1" t="s">
+        <v>348</v>
+      </c>
+      <c r="M28" s="1" t="s">
         <v>338</v>
       </c>
-      <c r="B28" s="1" t="s">
-        <v>316</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>339</v>
-      </c>
-      <c r="D28" s="1" t="s">
-        <v>340</v>
-      </c>
-      <c r="E28" s="2" t="s">
-        <v>341</v>
-      </c>
-      <c r="F28" s="1" t="s">
-        <v>342</v>
-      </c>
-      <c r="G28" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="H28" s="1" t="s">
-        <v>343</v>
-      </c>
-      <c r="I28" s="1" t="s">
-        <v>344</v>
-      </c>
-      <c r="J28" s="1" t="s">
-        <v>345</v>
-      </c>
-      <c r="K28" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="L28" s="1" t="s">
-        <v>346</v>
-      </c>
-      <c r="M28" s="1" t="s">
-        <v>325</v>
-      </c>
       <c r="N28" s="1" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="O28" s="1" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
     </row>
     <row r="29" spans="1:15" ht="84" customHeight="1">
       <c r="A29" s="1" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>350</v>
+        <v>329</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>304</v>
+        <v>352</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>331</v>
+        <v>355</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>308</v>
+        <v>92</v>
       </c>
       <c r="H29" s="1" t="s">
-        <v>332</v>
+        <v>356</v>
       </c>
       <c r="I29" s="1" t="s">
-        <v>353</v>
+        <v>357</v>
       </c>
       <c r="J29" s="1" t="s">
-        <v>354</v>
+        <v>358</v>
       </c>
       <c r="K29" s="1" t="s">
-        <v>117</v>
+        <v>132</v>
       </c>
       <c r="L29" s="1" t="s">
-        <v>355</v>
+        <v>359</v>
       </c>
       <c r="M29" s="1" t="s">
-        <v>325</v>
+        <v>338</v>
       </c>
       <c r="N29" s="1" t="s">
-        <v>356</v>
+        <v>360</v>
       </c>
       <c r="O29" s="1" t="s">
-        <v>357</v>
+        <v>361</v>
       </c>
     </row>
     <row r="30" spans="1:15" ht="84" customHeight="1">
       <c r="A30" s="1" t="s">
-        <v>358</v>
+        <v>362</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>350</v>
+        <v>363</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>359</v>
+        <v>317</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>360</v>
+        <v>364</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>361</v>
+        <v>365</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>362</v>
+        <v>344</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>308</v>
+        <v>321</v>
       </c>
       <c r="H30" s="1" t="s">
-        <v>363</v>
+        <v>345</v>
       </c>
       <c r="I30" s="1" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="J30" s="1" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="K30" s="1" t="s">
-        <v>117</v>
+        <v>132</v>
       </c>
       <c r="L30" s="1" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="M30" s="1" t="s">
-        <v>325</v>
+        <v>338</v>
       </c>
       <c r="N30" s="1" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="O30" s="1" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
     </row>
     <row r="31" spans="1:15" ht="84" customHeight="1">
       <c r="A31" s="1" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>101</v>
+        <v>363</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>304</v>
+        <v>372</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>331</v>
+        <v>375</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>308</v>
+        <v>321</v>
       </c>
       <c r="H31" s="1" t="s">
-        <v>372</v>
+        <v>376</v>
       </c>
       <c r="I31" s="1" t="s">
-        <v>373</v>
+        <v>377</v>
       </c>
       <c r="J31" s="1" t="s">
-        <v>374</v>
+        <v>378</v>
       </c>
       <c r="K31" s="1" t="s">
-        <v>117</v>
+        <v>132</v>
       </c>
       <c r="L31" s="1" t="s">
-        <v>375</v>
+        <v>379</v>
       </c>
       <c r="M31" s="1" t="s">
-        <v>325</v>
+        <v>338</v>
       </c>
       <c r="N31" s="1" t="s">
-        <v>376</v>
+        <v>380</v>
       </c>
       <c r="O31" s="1" t="s">
-        <v>377</v>
+        <v>381</v>
       </c>
     </row>
     <row r="32" spans="1:15" ht="84" customHeight="1">
       <c r="A32" s="1" t="s">
-        <v>378</v>
+        <v>382</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>379</v>
+        <v>116</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>304</v>
+        <v>317</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>381</v>
+        <v>384</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>382</v>
+        <v>344</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>308</v>
+        <v>321</v>
       </c>
       <c r="H32" s="1" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="I32" s="1" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="J32" s="1" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="K32" s="1" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="L32" s="1" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="M32" s="1" t="s">
-        <v>325</v>
+        <v>338</v>
       </c>
       <c r="N32" s="1" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="O32" s="1" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
     </row>
     <row r="33" spans="1:15" ht="84" customHeight="1">
       <c r="A33" s="1" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>350</v>
+        <v>392</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>390</v>
+        <v>317</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="G33" s="1" t="s">
-        <v>394</v>
+        <v>321</v>
       </c>
       <c r="H33" s="1" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="I33" s="1" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="J33" s="1" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="K33" s="1" t="s">
-        <v>398</v>
+        <v>110</v>
       </c>
       <c r="L33" s="1" t="s">
         <v>399</v>
       </c>
       <c r="M33" s="1" t="s">
-        <v>42</v>
+        <v>338</v>
       </c>
       <c r="N33" s="1" t="s">
         <v>400</v>
@@ -4190,7 +4327,7 @@
         <v>402</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>101</v>
+        <v>363</v>
       </c>
       <c r="C34" s="1" t="s">
         <v>403</v>
@@ -4223,7 +4360,7 @@
         <v>412</v>
       </c>
       <c r="M34" s="1" t="s">
-        <v>325</v>
+        <v>42</v>
       </c>
       <c r="N34" s="1" t="s">
         <v>413</v>
@@ -4237,7 +4374,7 @@
         <v>415</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>60</v>
+        <v>116</v>
       </c>
       <c r="C35" s="1" t="s">
         <v>416</v>
@@ -4252,39 +4389,39 @@
         <v>419</v>
       </c>
       <c r="G35" s="1" t="s">
-        <v>77</v>
+        <v>420</v>
       </c>
       <c r="H35" s="1" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="I35" s="1" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="J35" s="1" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="K35" s="1" t="s">
-        <v>81</v>
+        <v>424</v>
       </c>
       <c r="L35" s="1" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="M35" s="1" t="s">
-        <v>424</v>
+        <v>338</v>
       </c>
       <c r="N35" s="1" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="O35" s="1" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
     </row>
     <row r="36" spans="1:15" ht="84" customHeight="1">
       <c r="A36" s="1" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>428</v>
+        <v>60</v>
       </c>
       <c r="C36" s="1" t="s">
         <v>429</v>
@@ -4299,66 +4436,66 @@
         <v>432</v>
       </c>
       <c r="G36" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="H36" s="1" t="s">
         <v>433</v>
       </c>
-      <c r="H36" s="1" t="s">
+      <c r="I36" s="1" t="s">
         <v>434</v>
       </c>
-      <c r="I36" s="1" t="s">
+      <c r="J36" s="1" t="s">
         <v>435</v>
       </c>
-      <c r="J36" s="1" t="s">
+      <c r="K36" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="L36" s="1" t="s">
         <v>436</v>
       </c>
-      <c r="K36" s="1" t="s">
+      <c r="M36" s="1" t="s">
         <v>437</v>
       </c>
-      <c r="L36" s="1" t="s">
+      <c r="N36" s="1" t="s">
         <v>438</v>
       </c>
-      <c r="M36" s="1" t="s">
+      <c r="O36" s="1" t="s">
         <v>439</v>
-      </c>
-      <c r="N36" s="1" t="s">
-        <v>440</v>
-      </c>
-      <c r="O36" s="1" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="37" spans="1:15" ht="84" customHeight="1">
       <c r="A37" s="1" t="s">
+        <v>440</v>
+      </c>
+      <c r="B37" s="1" t="s">
         <v>441</v>
       </c>
-      <c r="B37" s="1" t="s">
+      <c r="C37" s="1" t="s">
         <v>442</v>
       </c>
-      <c r="C37" s="1" t="s">
+      <c r="D37" s="1" t="s">
         <v>443</v>
       </c>
-      <c r="D37" s="1" t="s">
+      <c r="E37" s="2" t="s">
         <v>444</v>
       </c>
-      <c r="E37" s="2" t="s">
+      <c r="F37" s="1" t="s">
         <v>445</v>
       </c>
-      <c r="F37" s="1" t="s">
+      <c r="G37" s="1" t="s">
         <v>446</v>
       </c>
-      <c r="G37" s="1" t="s">
+      <c r="H37" s="1" t="s">
         <v>447</v>
       </c>
-      <c r="H37" s="1" t="s">
+      <c r="I37" s="1" t="s">
         <v>448</v>
       </c>
-      <c r="I37" s="1" t="s">
+      <c r="J37" s="1" t="s">
         <v>449</v>
       </c>
-      <c r="J37" s="1" t="s">
+      <c r="K37" s="1" t="s">
         <v>450</v>
-      </c>
-      <c r="K37" s="1" t="s">
-        <v>96</v>
       </c>
       <c r="L37" s="1" t="s">
         <v>451</v>
@@ -4370,15 +4507,15 @@
         <v>453</v>
       </c>
       <c r="O37" s="1" t="s">
-        <v>454</v>
+        <v>270</v>
       </c>
     </row>
     <row r="38" spans="1:15" ht="84" customHeight="1">
       <c r="A38" s="1" t="s">
+        <v>454</v>
+      </c>
+      <c r="B38" s="1" t="s">
         <v>455</v>
-      </c>
-      <c r="B38" s="1" t="s">
-        <v>16</v>
       </c>
       <c r="C38" s="1" t="s">
         <v>456</v>
@@ -4393,1540 +4530,1727 @@
         <v>459</v>
       </c>
       <c r="G38" s="1" t="s">
-        <v>447</v>
+        <v>460</v>
       </c>
       <c r="H38" s="1" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="I38" s="1" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="J38" s="1" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="K38" s="1" t="s">
-        <v>81</v>
+        <v>96</v>
       </c>
       <c r="L38" s="1" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="M38" s="1" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="N38" s="1" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="O38" s="1" t="s">
-        <v>454</v>
+        <v>467</v>
       </c>
     </row>
     <row r="39" spans="1:15" ht="84" customHeight="1">
       <c r="A39" s="1" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="B39" s="1" t="s">
         <v>16</v>
       </c>
       <c r="C39" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>470</v>
+      </c>
+      <c r="E39" s="2" t="s">
+        <v>471</v>
+      </c>
+      <c r="F39" s="1" t="s">
+        <v>472</v>
+      </c>
+      <c r="G39" s="1" t="s">
+        <v>460</v>
+      </c>
+      <c r="H39" s="1" t="s">
+        <v>473</v>
+      </c>
+      <c r="I39" s="1" t="s">
+        <v>474</v>
+      </c>
+      <c r="J39" s="1" t="s">
+        <v>475</v>
+      </c>
+      <c r="K39" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="L39" s="1" t="s">
+        <v>476</v>
+      </c>
+      <c r="M39" s="1" t="s">
+        <v>477</v>
+      </c>
+      <c r="N39" s="1" t="s">
+        <v>478</v>
+      </c>
+      <c r="O39" s="1" t="s">
         <v>467</v>
-      </c>
-      <c r="D39" s="1" t="s">
-        <v>468</v>
-      </c>
-      <c r="E39" s="2" t="s">
-        <v>469</v>
-      </c>
-      <c r="F39" s="1" t="s">
-        <v>275</v>
-      </c>
-      <c r="G39" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="H39" s="1" t="s">
-        <v>276</v>
-      </c>
-      <c r="I39" s="1" t="s">
-        <v>470</v>
-      </c>
-      <c r="J39" s="1" t="s">
-        <v>471</v>
-      </c>
-      <c r="K39" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="L39" s="1" t="s">
-        <v>472</v>
-      </c>
-      <c r="M39" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="N39" s="1" t="s">
-        <v>473</v>
-      </c>
-      <c r="O39" s="1" t="s">
-        <v>474</v>
       </c>
     </row>
     <row r="40" spans="1:15" ht="84" customHeight="1">
       <c r="A40" s="1" t="s">
-        <v>475</v>
+        <v>479</v>
       </c>
       <c r="B40" s="1" t="s">
         <v>16</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>476</v>
+        <v>480</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>477</v>
+        <v>481</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>478</v>
+        <v>482</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>263</v>
+        <v>288</v>
       </c>
       <c r="G40" s="1" t="s">
-        <v>264</v>
+        <v>21</v>
       </c>
       <c r="H40" s="1" t="s">
-        <v>265</v>
+        <v>289</v>
       </c>
       <c r="I40" s="1" t="s">
-        <v>479</v>
+        <v>483</v>
       </c>
       <c r="J40" s="1" t="s">
-        <v>480</v>
+        <v>484</v>
       </c>
       <c r="K40" s="1" t="s">
-        <v>130</v>
+        <v>110</v>
       </c>
       <c r="L40" s="1" t="s">
-        <v>481</v>
+        <v>485</v>
       </c>
       <c r="M40" s="1" t="s">
         <v>83</v>
       </c>
       <c r="N40" s="1" t="s">
-        <v>482</v>
+        <v>486</v>
       </c>
       <c r="O40" s="1" t="s">
-        <v>483</v>
+        <v>487</v>
       </c>
     </row>
     <row r="41" spans="1:15" ht="84" customHeight="1">
       <c r="A41" s="1" t="s">
-        <v>484</v>
+        <v>488</v>
       </c>
       <c r="B41" s="1" t="s">
         <v>16</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>476</v>
+        <v>489</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>485</v>
+        <v>490</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>486</v>
+        <v>491</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>487</v>
+        <v>276</v>
       </c>
       <c r="G41" s="1" t="s">
-        <v>92</v>
+        <v>277</v>
       </c>
       <c r="H41" s="1" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="I41" s="1" t="s">
-        <v>488</v>
+        <v>492</v>
       </c>
       <c r="J41" s="1" t="s">
-        <v>489</v>
+        <v>493</v>
       </c>
       <c r="K41" s="1" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="L41" s="1" t="s">
-        <v>490</v>
+        <v>494</v>
       </c>
       <c r="M41" s="1" t="s">
         <v>83</v>
       </c>
       <c r="N41" s="1" t="s">
-        <v>491</v>
+        <v>495</v>
       </c>
       <c r="O41" s="1" t="s">
-        <v>492</v>
+        <v>496</v>
       </c>
     </row>
     <row r="42" spans="1:15" ht="84" customHeight="1">
       <c r="A42" s="1" t="s">
-        <v>493</v>
+        <v>497</v>
       </c>
       <c r="B42" s="1" t="s">
         <v>16</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>494</v>
+        <v>489</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>495</v>
+        <v>498</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>496</v>
+        <v>499</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>497</v>
+        <v>500</v>
       </c>
       <c r="G42" s="1" t="s">
         <v>92</v>
       </c>
       <c r="H42" s="1" t="s">
-        <v>498</v>
+        <v>289</v>
       </c>
       <c r="I42" s="1" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="J42" s="1" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="K42" s="1" t="s">
-        <v>117</v>
+        <v>132</v>
       </c>
       <c r="L42" s="1" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="M42" s="1" t="s">
-        <v>502</v>
+        <v>83</v>
       </c>
       <c r="N42" s="1" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="O42" s="1" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
     </row>
     <row r="43" spans="1:15" ht="84" customHeight="1">
       <c r="A43" s="1" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="B43" s="1" t="s">
         <v>16</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="G43" s="1" t="s">
-        <v>77</v>
+        <v>92</v>
       </c>
       <c r="H43" s="1" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="I43" s="1" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="J43" s="1" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="K43" s="1" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="L43" s="1" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="M43" s="1" t="s">
-        <v>325</v>
+        <v>515</v>
       </c>
       <c r="N43" s="1" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="O43" s="1" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
     </row>
     <row r="44" spans="1:15" ht="84" customHeight="1">
       <c r="A44" s="1" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>87</v>
+        <v>16</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>506</v>
+        <v>519</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>517</v>
+        <v>520</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>518</v>
+        <v>521</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>519</v>
+        <v>522</v>
       </c>
       <c r="G44" s="1" t="s">
         <v>77</v>
       </c>
       <c r="H44" s="1" t="s">
-        <v>520</v>
+        <v>523</v>
       </c>
       <c r="I44" s="1" t="s">
-        <v>521</v>
+        <v>524</v>
       </c>
       <c r="J44" s="1" t="s">
-        <v>522</v>
+        <v>525</v>
       </c>
       <c r="K44" s="1" t="s">
-        <v>130</v>
+        <v>110</v>
       </c>
       <c r="L44" s="1" t="s">
-        <v>523</v>
+        <v>526</v>
       </c>
       <c r="M44" s="1" t="s">
-        <v>42</v>
+        <v>338</v>
       </c>
       <c r="N44" s="1" t="s">
-        <v>524</v>
+        <v>527</v>
       </c>
       <c r="O44" s="1" t="s">
-        <v>525</v>
+        <v>528</v>
       </c>
     </row>
     <row r="45" spans="1:15" ht="84" customHeight="1">
       <c r="A45" s="1" t="s">
-        <v>526</v>
+        <v>529</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>147</v>
+        <v>87</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>527</v>
+        <v>519</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="G45" s="1" t="s">
-        <v>531</v>
+        <v>77</v>
       </c>
       <c r="H45" s="1" t="s">
-        <v>434</v>
+        <v>533</v>
       </c>
       <c r="I45" s="1" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="J45" s="1" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="K45" s="1" t="s">
-        <v>437</v>
+        <v>110</v>
       </c>
       <c r="L45" s="1" t="s">
-        <v>438</v>
+        <v>536</v>
       </c>
       <c r="M45" s="1" t="s">
-        <v>534</v>
+        <v>42</v>
       </c>
       <c r="N45" s="1" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
       <c r="O45" s="1" t="s">
-        <v>257</v>
+        <v>538</v>
       </c>
     </row>
     <row r="46" spans="1:15" ht="84" customHeight="1">
       <c r="A46" s="1" t="s">
-        <v>536</v>
+        <v>539</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>87</v>
+        <v>160</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>538</v>
+        <v>541</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>539</v>
+        <v>542</v>
       </c>
       <c r="F46" s="1" t="s">
-        <v>540</v>
+        <v>543</v>
       </c>
       <c r="G46" s="1" t="s">
-        <v>21</v>
+        <v>544</v>
       </c>
       <c r="H46" s="1" t="s">
-        <v>541</v>
+        <v>447</v>
       </c>
       <c r="I46" s="1" t="s">
-        <v>542</v>
+        <v>545</v>
       </c>
       <c r="J46" s="1" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="K46" s="1" t="s">
-        <v>117</v>
+        <v>450</v>
       </c>
       <c r="L46" s="1" t="s">
-        <v>544</v>
+        <v>451</v>
       </c>
       <c r="M46" s="1" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="N46" s="1" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="O46" s="1" t="s">
-        <v>547</v>
+        <v>270</v>
       </c>
     </row>
     <row r="47" spans="1:15" ht="84" customHeight="1">
       <c r="A47" s="1" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="B47" s="1" t="s">
         <v>87</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>537</v>
+        <v>550</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>540</v>
+        <v>553</v>
       </c>
       <c r="G47" s="1" t="s">
         <v>21</v>
       </c>
       <c r="H47" s="1" t="s">
-        <v>541</v>
+        <v>554</v>
       </c>
       <c r="I47" s="1" t="s">
-        <v>551</v>
+        <v>555</v>
       </c>
       <c r="J47" s="1" t="s">
-        <v>552</v>
+        <v>556</v>
       </c>
       <c r="K47" s="1" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="L47" s="1" t="s">
-        <v>553</v>
+        <v>557</v>
       </c>
       <c r="M47" s="1" t="s">
-        <v>545</v>
+        <v>558</v>
       </c>
       <c r="N47" s="1" t="s">
-        <v>554</v>
+        <v>559</v>
       </c>
       <c r="O47" s="1" t="s">
-        <v>555</v>
+        <v>560</v>
       </c>
     </row>
     <row r="48" spans="1:15" ht="84" customHeight="1">
       <c r="A48" s="1" t="s">
-        <v>556</v>
+        <v>561</v>
       </c>
       <c r="B48" s="1" t="s">
         <v>87</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>537</v>
+        <v>550</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>557</v>
+        <v>562</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>558</v>
+        <v>563</v>
       </c>
       <c r="F48" s="1" t="s">
-        <v>540</v>
+        <v>553</v>
       </c>
       <c r="G48" s="1" t="s">
         <v>21</v>
       </c>
       <c r="H48" s="1" t="s">
-        <v>541</v>
+        <v>554</v>
       </c>
       <c r="I48" s="1" t="s">
-        <v>559</v>
+        <v>564</v>
       </c>
       <c r="J48" s="1" t="s">
-        <v>560</v>
+        <v>565</v>
       </c>
       <c r="K48" s="1" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="L48" s="1" t="s">
-        <v>561</v>
+        <v>566</v>
       </c>
       <c r="M48" s="1" t="s">
-        <v>545</v>
+        <v>558</v>
       </c>
       <c r="N48" s="1" t="s">
-        <v>562</v>
+        <v>567</v>
       </c>
       <c r="O48" s="1" t="s">
-        <v>563</v>
+        <v>568</v>
       </c>
     </row>
     <row r="49" spans="1:15" ht="84" customHeight="1">
       <c r="A49" s="1" t="s">
-        <v>564</v>
+        <v>569</v>
       </c>
       <c r="B49" s="1" t="s">
         <v>87</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>537</v>
+        <v>550</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>565</v>
+        <v>570</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>566</v>
+        <v>571</v>
       </c>
       <c r="F49" s="1" t="s">
-        <v>567</v>
+        <v>553</v>
       </c>
       <c r="G49" s="1" t="s">
-        <v>264</v>
+        <v>21</v>
       </c>
       <c r="H49" s="1" t="s">
-        <v>541</v>
+        <v>554</v>
       </c>
       <c r="I49" s="1" t="s">
-        <v>568</v>
+        <v>572</v>
       </c>
       <c r="J49" s="1" t="s">
-        <v>569</v>
+        <v>573</v>
       </c>
       <c r="K49" s="1" t="s">
-        <v>96</v>
+        <v>132</v>
       </c>
       <c r="L49" s="1" t="s">
-        <v>570</v>
+        <v>574</v>
       </c>
       <c r="M49" s="1" t="s">
-        <v>545</v>
+        <v>558</v>
       </c>
       <c r="N49" s="1" t="s">
-        <v>571</v>
+        <v>575</v>
       </c>
       <c r="O49" s="1" t="s">
-        <v>572</v>
+        <v>576</v>
       </c>
     </row>
     <row r="50" spans="1:15" ht="84" customHeight="1">
       <c r="A50" s="1" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B50" s="1" t="s">
         <v>87</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>537</v>
+        <v>550</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="F50" s="1" t="s">
-        <v>540</v>
+        <v>580</v>
       </c>
       <c r="G50" s="1" t="s">
-        <v>21</v>
+        <v>277</v>
       </c>
       <c r="H50" s="1" t="s">
-        <v>541</v>
+        <v>554</v>
       </c>
       <c r="I50" s="1" t="s">
-        <v>576</v>
+        <v>581</v>
       </c>
       <c r="J50" s="1" t="s">
-        <v>577</v>
+        <v>582</v>
       </c>
       <c r="K50" s="1" t="s">
-        <v>117</v>
+        <v>96</v>
       </c>
       <c r="L50" s="1" t="s">
-        <v>578</v>
+        <v>583</v>
       </c>
       <c r="M50" s="1" t="s">
-        <v>545</v>
+        <v>558</v>
       </c>
       <c r="N50" s="1" t="s">
-        <v>579</v>
+        <v>584</v>
       </c>
       <c r="O50" s="1" t="s">
-        <v>580</v>
+        <v>585</v>
       </c>
     </row>
     <row r="51" spans="1:15" ht="84" customHeight="1">
       <c r="A51" s="1" t="s">
-        <v>581</v>
+        <v>586</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>259</v>
+        <v>87</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>537</v>
+        <v>550</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>582</v>
+        <v>587</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>583</v>
+        <v>588</v>
       </c>
       <c r="F51" s="1" t="s">
-        <v>540</v>
+        <v>553</v>
       </c>
       <c r="G51" s="1" t="s">
         <v>21</v>
       </c>
       <c r="H51" s="1" t="s">
-        <v>541</v>
+        <v>554</v>
       </c>
       <c r="I51" s="1" t="s">
-        <v>584</v>
+        <v>589</v>
       </c>
       <c r="J51" s="1" t="s">
-        <v>585</v>
+        <v>590</v>
       </c>
       <c r="K51" s="1" t="s">
-        <v>117</v>
+        <v>132</v>
       </c>
       <c r="L51" s="1" t="s">
-        <v>586</v>
+        <v>591</v>
       </c>
       <c r="M51" s="1" t="s">
-        <v>545</v>
+        <v>558</v>
       </c>
       <c r="N51" s="1" t="s">
-        <v>587</v>
+        <v>592</v>
       </c>
       <c r="O51" s="1" t="s">
-        <v>588</v>
+        <v>593</v>
       </c>
     </row>
     <row r="52" spans="1:15" ht="84" customHeight="1">
       <c r="A52" s="1" t="s">
-        <v>589</v>
+        <v>594</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>259</v>
+        <v>272</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>537</v>
+        <v>550</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>590</v>
+        <v>595</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>591</v>
+        <v>596</v>
       </c>
       <c r="F52" s="1" t="s">
-        <v>540</v>
+        <v>553</v>
       </c>
       <c r="G52" s="1" t="s">
         <v>21</v>
       </c>
       <c r="H52" s="1" t="s">
-        <v>541</v>
+        <v>554</v>
       </c>
       <c r="I52" s="1" t="s">
-        <v>592</v>
+        <v>597</v>
       </c>
       <c r="J52" s="1" t="s">
-        <v>593</v>
+        <v>598</v>
       </c>
       <c r="K52" s="1" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="L52" s="1" t="s">
-        <v>594</v>
+        <v>599</v>
       </c>
       <c r="M52" s="1" t="s">
-        <v>545</v>
+        <v>558</v>
       </c>
       <c r="N52" s="1" t="s">
-        <v>595</v>
+        <v>600</v>
       </c>
       <c r="O52" s="1" t="s">
-        <v>596</v>
+        <v>601</v>
       </c>
     </row>
     <row r="53" spans="1:15" ht="84" customHeight="1">
       <c r="A53" s="1" t="s">
-        <v>597</v>
+        <v>602</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>259</v>
+        <v>272</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>537</v>
+        <v>550</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>598</v>
+        <v>603</v>
       </c>
       <c r="E53" s="2" t="s">
-        <v>599</v>
+        <v>604</v>
       </c>
       <c r="F53" s="1" t="s">
-        <v>540</v>
+        <v>553</v>
       </c>
       <c r="G53" s="1" t="s">
         <v>21</v>
       </c>
       <c r="H53" s="1" t="s">
-        <v>541</v>
+        <v>554</v>
       </c>
       <c r="I53" s="1" t="s">
-        <v>600</v>
+        <v>605</v>
       </c>
       <c r="J53" s="1" t="s">
-        <v>601</v>
+        <v>606</v>
       </c>
       <c r="K53" s="1" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="L53" s="1" t="s">
-        <v>602</v>
+        <v>607</v>
       </c>
       <c r="M53" s="1" t="s">
-        <v>545</v>
+        <v>558</v>
       </c>
       <c r="N53" s="1" t="s">
-        <v>603</v>
+        <v>608</v>
       </c>
       <c r="O53" s="1" t="s">
-        <v>604</v>
+        <v>609</v>
       </c>
     </row>
     <row r="54" spans="1:15" ht="84" customHeight="1">
       <c r="A54" s="1" t="s">
-        <v>605</v>
+        <v>610</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>259</v>
+        <v>272</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>537</v>
+        <v>550</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>606</v>
+        <v>611</v>
       </c>
       <c r="E54" s="2" t="s">
-        <v>607</v>
+        <v>612</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>540</v>
+        <v>553</v>
       </c>
       <c r="G54" s="1" t="s">
         <v>21</v>
       </c>
       <c r="H54" s="1" t="s">
-        <v>541</v>
+        <v>554</v>
       </c>
       <c r="I54" s="1" t="s">
-        <v>608</v>
+        <v>613</v>
       </c>
       <c r="J54" s="1" t="s">
-        <v>609</v>
+        <v>614</v>
       </c>
       <c r="K54" s="1" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="L54" s="1" t="s">
-        <v>610</v>
+        <v>615</v>
       </c>
       <c r="M54" s="1" t="s">
-        <v>545</v>
+        <v>558</v>
       </c>
       <c r="N54" s="1" t="s">
-        <v>611</v>
+        <v>616</v>
       </c>
       <c r="O54" s="1" t="s">
-        <v>612</v>
+        <v>617</v>
       </c>
     </row>
     <row r="55" spans="1:15" ht="84" customHeight="1">
       <c r="A55" s="1" t="s">
-        <v>613</v>
+        <v>618</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>259</v>
+        <v>272</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>537</v>
+        <v>550</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>614</v>
+        <v>619</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>615</v>
+        <v>620</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>540</v>
+        <v>553</v>
       </c>
       <c r="G55" s="1" t="s">
         <v>21</v>
       </c>
       <c r="H55" s="1" t="s">
-        <v>541</v>
+        <v>554</v>
       </c>
       <c r="I55" s="1" t="s">
-        <v>616</v>
+        <v>621</v>
       </c>
       <c r="J55" s="1" t="s">
-        <v>617</v>
+        <v>622</v>
       </c>
       <c r="K55" s="1" t="s">
-        <v>130</v>
+        <v>110</v>
       </c>
       <c r="L55" s="1" t="s">
-        <v>618</v>
+        <v>623</v>
       </c>
       <c r="M55" s="1" t="s">
-        <v>545</v>
+        <v>558</v>
       </c>
       <c r="N55" s="1" t="s">
-        <v>619</v>
+        <v>624</v>
       </c>
       <c r="O55" s="1" t="s">
-        <v>620</v>
+        <v>625</v>
       </c>
     </row>
     <row r="56" spans="1:15" ht="84" customHeight="1">
       <c r="A56" s="1" t="s">
-        <v>621</v>
+        <v>626</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>259</v>
+        <v>272</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>537</v>
+        <v>550</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>622</v>
+        <v>627</v>
       </c>
       <c r="E56" s="2" t="s">
-        <v>623</v>
+        <v>628</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>540</v>
+        <v>553</v>
       </c>
       <c r="G56" s="1" t="s">
         <v>21</v>
       </c>
       <c r="H56" s="1" t="s">
-        <v>541</v>
+        <v>554</v>
       </c>
       <c r="I56" s="1" t="s">
-        <v>624</v>
+        <v>629</v>
       </c>
       <c r="J56" s="1" t="s">
-        <v>625</v>
+        <v>630</v>
       </c>
       <c r="K56" s="1" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="L56" s="1" t="s">
-        <v>626</v>
+        <v>631</v>
       </c>
       <c r="M56" s="1" t="s">
-        <v>545</v>
+        <v>558</v>
       </c>
       <c r="N56" s="1" t="s">
-        <v>627</v>
+        <v>632</v>
       </c>
       <c r="O56" s="1" t="s">
-        <v>628</v>
+        <v>633</v>
       </c>
     </row>
     <row r="57" spans="1:15" ht="84" customHeight="1">
       <c r="A57" s="1" t="s">
-        <v>629</v>
+        <v>634</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>259</v>
+        <v>272</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>537</v>
+        <v>550</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>630</v>
+        <v>635</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>631</v>
+        <v>636</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>540</v>
+        <v>553</v>
       </c>
       <c r="G57" s="1" t="s">
         <v>21</v>
       </c>
       <c r="H57" s="1" t="s">
-        <v>541</v>
+        <v>554</v>
       </c>
       <c r="I57" s="1" t="s">
-        <v>632</v>
+        <v>637</v>
       </c>
       <c r="J57" s="1" t="s">
-        <v>633</v>
+        <v>638</v>
       </c>
       <c r="K57" s="1" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="L57" s="1" t="s">
-        <v>618</v>
+        <v>639</v>
       </c>
       <c r="M57" s="1" t="s">
-        <v>545</v>
+        <v>558</v>
       </c>
       <c r="N57" s="1" t="s">
-        <v>634</v>
+        <v>640</v>
       </c>
       <c r="O57" s="1" t="s">
-        <v>635</v>
+        <v>641</v>
       </c>
     </row>
     <row r="58" spans="1:15" ht="84" customHeight="1">
       <c r="A58" s="1" t="s">
-        <v>636</v>
+        <v>642</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>259</v>
+        <v>272</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>537</v>
+        <v>550</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>637</v>
+        <v>643</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>638</v>
+        <v>644</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>540</v>
+        <v>553</v>
       </c>
       <c r="G58" s="1" t="s">
         <v>21</v>
       </c>
       <c r="H58" s="1" t="s">
-        <v>541</v>
+        <v>554</v>
       </c>
       <c r="I58" s="1" t="s">
-        <v>639</v>
+        <v>645</v>
       </c>
       <c r="J58" s="1" t="s">
-        <v>640</v>
+        <v>646</v>
       </c>
       <c r="K58" s="1" t="s">
-        <v>130</v>
+        <v>110</v>
       </c>
       <c r="L58" s="1" t="s">
-        <v>641</v>
+        <v>631</v>
       </c>
       <c r="M58" s="1" t="s">
-        <v>545</v>
+        <v>558</v>
       </c>
       <c r="N58" s="1" t="s">
-        <v>642</v>
+        <v>647</v>
       </c>
       <c r="O58" s="1" t="s">
-        <v>643</v>
+        <v>648</v>
       </c>
     </row>
     <row r="59" spans="1:15" ht="84" customHeight="1">
       <c r="A59" s="1" t="s">
-        <v>644</v>
+        <v>649</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>259</v>
+        <v>272</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>537</v>
+        <v>550</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>645</v>
+        <v>650</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>646</v>
+        <v>651</v>
       </c>
       <c r="F59" s="1" t="s">
-        <v>540</v>
+        <v>553</v>
       </c>
       <c r="G59" s="1" t="s">
         <v>21</v>
       </c>
       <c r="H59" s="1" t="s">
-        <v>541</v>
+        <v>554</v>
       </c>
       <c r="I59" s="1" t="s">
-        <v>647</v>
+        <v>652</v>
       </c>
       <c r="J59" s="1" t="s">
-        <v>648</v>
+        <v>653</v>
       </c>
       <c r="K59" s="1" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="L59" s="1" t="s">
-        <v>649</v>
+        <v>654</v>
       </c>
       <c r="M59" s="1" t="s">
-        <v>545</v>
+        <v>558</v>
       </c>
       <c r="N59" s="1" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="O59" s="1" t="s">
-        <v>651</v>
+        <v>656</v>
       </c>
     </row>
     <row r="60" spans="1:15" ht="84" customHeight="1">
       <c r="A60" s="1" t="s">
-        <v>652</v>
+        <v>657</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>259</v>
+        <v>272</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>537</v>
+        <v>550</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>653</v>
+        <v>658</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>654</v>
+        <v>659</v>
       </c>
       <c r="F60" s="1" t="s">
-        <v>540</v>
+        <v>553</v>
       </c>
       <c r="G60" s="1" t="s">
         <v>21</v>
       </c>
       <c r="H60" s="1" t="s">
-        <v>541</v>
+        <v>554</v>
       </c>
       <c r="I60" s="1" t="s">
-        <v>655</v>
+        <v>660</v>
       </c>
       <c r="J60" s="1" t="s">
-        <v>656</v>
+        <v>661</v>
       </c>
       <c r="K60" s="1" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="L60" s="1" t="s">
-        <v>618</v>
+        <v>662</v>
       </c>
       <c r="M60" s="1" t="s">
-        <v>545</v>
+        <v>558</v>
       </c>
       <c r="N60" s="1" t="s">
-        <v>657</v>
+        <v>663</v>
       </c>
       <c r="O60" s="1" t="s">
-        <v>658</v>
+        <v>664</v>
       </c>
     </row>
     <row r="61" spans="1:15" ht="84" customHeight="1">
       <c r="A61" s="1" t="s">
-        <v>659</v>
+        <v>665</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>259</v>
+        <v>272</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>537</v>
+        <v>550</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>660</v>
+        <v>666</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>661</v>
+        <v>667</v>
       </c>
       <c r="F61" s="1" t="s">
-        <v>540</v>
+        <v>553</v>
       </c>
       <c r="G61" s="1" t="s">
         <v>21</v>
       </c>
       <c r="H61" s="1" t="s">
-        <v>541</v>
+        <v>554</v>
       </c>
       <c r="I61" s="1" t="s">
-        <v>662</v>
+        <v>668</v>
       </c>
       <c r="J61" s="1" t="s">
-        <v>663</v>
+        <v>669</v>
       </c>
       <c r="K61" s="1" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="L61" s="1" t="s">
-        <v>664</v>
+        <v>631</v>
       </c>
       <c r="M61" s="1" t="s">
-        <v>545</v>
+        <v>558</v>
       </c>
       <c r="N61" s="1" t="s">
-        <v>665</v>
+        <v>670</v>
       </c>
       <c r="O61" s="1" t="s">
-        <v>666</v>
+        <v>671</v>
       </c>
     </row>
     <row r="62" spans="1:15" ht="84" customHeight="1">
       <c r="A62" s="1" t="s">
-        <v>667</v>
+        <v>672</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>259</v>
+        <v>272</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>537</v>
+        <v>550</v>
       </c>
       <c r="D62" s="1" t="s">
-        <v>668</v>
+        <v>673</v>
       </c>
       <c r="E62" s="2" t="s">
-        <v>669</v>
+        <v>674</v>
       </c>
       <c r="F62" s="1" t="s">
-        <v>540</v>
+        <v>553</v>
       </c>
       <c r="G62" s="1" t="s">
         <v>21</v>
       </c>
       <c r="H62" s="1" t="s">
-        <v>541</v>
+        <v>554</v>
       </c>
       <c r="I62" s="1" t="s">
-        <v>670</v>
+        <v>675</v>
       </c>
       <c r="J62" s="1" t="s">
-        <v>671</v>
+        <v>676</v>
       </c>
       <c r="K62" s="1" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="L62" s="1" t="s">
-        <v>672</v>
+        <v>677</v>
       </c>
       <c r="M62" s="1" t="s">
-        <v>545</v>
+        <v>558</v>
       </c>
       <c r="N62" s="1" t="s">
-        <v>673</v>
+        <v>678</v>
       </c>
       <c r="O62" s="1" t="s">
-        <v>674</v>
+        <v>679</v>
       </c>
     </row>
     <row r="63" spans="1:15" ht="84" customHeight="1">
       <c r="A63" s="1" t="s">
-        <v>675</v>
+        <v>680</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>183</v>
+        <v>272</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>537</v>
+        <v>550</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>676</v>
+        <v>681</v>
       </c>
       <c r="E63" s="2" t="s">
-        <v>677</v>
+        <v>682</v>
       </c>
       <c r="F63" s="1" t="s">
-        <v>540</v>
+        <v>553</v>
       </c>
       <c r="G63" s="1" t="s">
         <v>21</v>
       </c>
       <c r="H63" s="1" t="s">
-        <v>541</v>
+        <v>554</v>
       </c>
       <c r="I63" s="1" t="s">
-        <v>678</v>
+        <v>683</v>
       </c>
       <c r="J63" s="1" t="s">
-        <v>679</v>
+        <v>684</v>
       </c>
       <c r="K63" s="1" t="s">
-        <v>130</v>
+        <v>110</v>
       </c>
       <c r="L63" s="1" t="s">
-        <v>680</v>
+        <v>685</v>
       </c>
       <c r="M63" s="1" t="s">
-        <v>545</v>
+        <v>558</v>
       </c>
       <c r="N63" s="1" t="s">
-        <v>681</v>
+        <v>686</v>
       </c>
       <c r="O63" s="1" t="s">
-        <v>682</v>
+        <v>687</v>
       </c>
     </row>
     <row r="64" spans="1:15" ht="84" customHeight="1">
       <c r="A64" s="1" t="s">
-        <v>683</v>
+        <v>688</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>684</v>
+        <v>196</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>537</v>
+        <v>550</v>
       </c>
       <c r="D64" s="1" t="s">
-        <v>685</v>
+        <v>689</v>
       </c>
       <c r="E64" s="2" t="s">
-        <v>686</v>
+        <v>690</v>
       </c>
       <c r="F64" s="1" t="s">
-        <v>540</v>
+        <v>553</v>
       </c>
       <c r="G64" s="1" t="s">
         <v>21</v>
       </c>
       <c r="H64" s="1" t="s">
-        <v>541</v>
+        <v>554</v>
       </c>
       <c r="I64" s="1" t="s">
-        <v>687</v>
+        <v>691</v>
       </c>
       <c r="J64" s="1" t="s">
-        <v>688</v>
+        <v>692</v>
       </c>
       <c r="K64" s="1" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="L64" s="1" t="s">
-        <v>689</v>
+        <v>693</v>
       </c>
       <c r="M64" s="1" t="s">
-        <v>545</v>
+        <v>558</v>
       </c>
       <c r="N64" s="1" t="s">
-        <v>690</v>
+        <v>694</v>
       </c>
       <c r="O64" s="1" t="s">
-        <v>691</v>
+        <v>695</v>
       </c>
     </row>
     <row r="65" spans="1:15" ht="84" customHeight="1">
       <c r="A65" s="1" t="s">
-        <v>692</v>
+        <v>696</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>259</v>
+        <v>697</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>537</v>
+        <v>550</v>
       </c>
       <c r="D65" s="1" t="s">
-        <v>693</v>
+        <v>698</v>
       </c>
       <c r="E65" s="2" t="s">
-        <v>694</v>
+        <v>699</v>
       </c>
       <c r="F65" s="1" t="s">
-        <v>540</v>
+        <v>553</v>
       </c>
       <c r="G65" s="1" t="s">
         <v>21</v>
       </c>
       <c r="H65" s="1" t="s">
-        <v>541</v>
+        <v>554</v>
       </c>
       <c r="I65" s="1" t="s">
-        <v>695</v>
+        <v>700</v>
       </c>
       <c r="J65" s="1" t="s">
-        <v>696</v>
+        <v>701</v>
       </c>
       <c r="K65" s="1" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="L65" s="1" t="s">
-        <v>697</v>
+        <v>702</v>
       </c>
       <c r="M65" s="1" t="s">
-        <v>545</v>
+        <v>558</v>
       </c>
       <c r="N65" s="1" t="s">
-        <v>698</v>
+        <v>703</v>
       </c>
       <c r="O65" s="1" t="s">
-        <v>699</v>
+        <v>704</v>
       </c>
     </row>
     <row r="66" spans="1:15" ht="84" customHeight="1">
       <c r="A66" s="1" t="s">
-        <v>700</v>
+        <v>705</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>259</v>
+        <v>272</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>537</v>
+        <v>550</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>701</v>
+        <v>706</v>
       </c>
       <c r="E66" s="2" t="s">
-        <v>702</v>
+        <v>707</v>
       </c>
       <c r="F66" s="1" t="s">
-        <v>567</v>
+        <v>553</v>
       </c>
       <c r="G66" s="1" t="s">
-        <v>264</v>
+        <v>21</v>
       </c>
       <c r="H66" s="1" t="s">
-        <v>541</v>
+        <v>554</v>
       </c>
       <c r="I66" s="1" t="s">
-        <v>703</v>
+        <v>708</v>
       </c>
       <c r="J66" s="1" t="s">
-        <v>704</v>
+        <v>709</v>
       </c>
       <c r="K66" s="1" t="s">
-        <v>130</v>
+        <v>110</v>
       </c>
       <c r="L66" s="1" t="s">
-        <v>268</v>
+        <v>710</v>
       </c>
       <c r="M66" s="1" t="s">
-        <v>545</v>
+        <v>558</v>
       </c>
       <c r="N66" s="1" t="s">
-        <v>705</v>
+        <v>711</v>
       </c>
       <c r="O66" s="1" t="s">
-        <v>706</v>
+        <v>712</v>
       </c>
     </row>
     <row r="67" spans="1:15" ht="84" customHeight="1">
       <c r="A67" s="1" t="s">
-        <v>707</v>
+        <v>713</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>259</v>
+        <v>272</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>537</v>
+        <v>550</v>
       </c>
       <c r="D67" s="1" t="s">
-        <v>708</v>
+        <v>714</v>
       </c>
       <c r="E67" s="2" t="s">
-        <v>709</v>
+        <v>715</v>
       </c>
       <c r="F67" s="1" t="s">
-        <v>540</v>
+        <v>580</v>
       </c>
       <c r="G67" s="1" t="s">
-        <v>21</v>
+        <v>277</v>
       </c>
       <c r="H67" s="1" t="s">
-        <v>541</v>
+        <v>554</v>
       </c>
       <c r="I67" s="1" t="s">
-        <v>710</v>
+        <v>716</v>
       </c>
       <c r="J67" s="1" t="s">
-        <v>711</v>
+        <v>717</v>
       </c>
       <c r="K67" s="1" t="s">
-        <v>130</v>
+        <v>110</v>
       </c>
       <c r="L67" s="1" t="s">
-        <v>712</v>
+        <v>281</v>
       </c>
       <c r="M67" s="1" t="s">
-        <v>545</v>
+        <v>558</v>
       </c>
       <c r="N67" s="1" t="s">
-        <v>713</v>
+        <v>718</v>
       </c>
       <c r="O67" s="1" t="s">
-        <v>714</v>
+        <v>719</v>
       </c>
     </row>
     <row r="68" spans="1:15" ht="84" customHeight="1">
       <c r="A68" s="1" t="s">
-        <v>715</v>
+        <v>720</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>183</v>
+        <v>272</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>537</v>
+        <v>550</v>
       </c>
       <c r="D68" s="1" t="s">
-        <v>716</v>
+        <v>721</v>
       </c>
       <c r="E68" s="2" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
       <c r="F68" s="1" t="s">
-        <v>540</v>
+        <v>553</v>
       </c>
       <c r="G68" s="1" t="s">
         <v>21</v>
       </c>
       <c r="H68" s="1" t="s">
-        <v>541</v>
+        <v>554</v>
       </c>
       <c r="I68" s="1" t="s">
-        <v>718</v>
+        <v>723</v>
       </c>
       <c r="J68" s="1" t="s">
-        <v>719</v>
+        <v>724</v>
       </c>
       <c r="K68" s="1" t="s">
-        <v>130</v>
+        <v>110</v>
       </c>
       <c r="L68" s="1" t="s">
-        <v>720</v>
+        <v>725</v>
       </c>
       <c r="M68" s="1" t="s">
-        <v>545</v>
+        <v>558</v>
       </c>
       <c r="N68" s="1" t="s">
-        <v>721</v>
+        <v>726</v>
       </c>
       <c r="O68" s="1" t="s">
-        <v>722</v>
+        <v>727</v>
       </c>
     </row>
     <row r="69" spans="1:15" ht="84" customHeight="1">
       <c r="A69" s="1" t="s">
-        <v>723</v>
+        <v>728</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>684</v>
+        <v>196</v>
       </c>
       <c r="C69" s="1" t="s">
-        <v>537</v>
+        <v>550</v>
       </c>
       <c r="D69" s="1" t="s">
-        <v>724</v>
+        <v>729</v>
       </c>
       <c r="E69" s="2" t="s">
-        <v>725</v>
+        <v>730</v>
       </c>
       <c r="F69" s="1" t="s">
-        <v>540</v>
+        <v>553</v>
       </c>
       <c r="G69" s="1" t="s">
         <v>21</v>
       </c>
       <c r="H69" s="1" t="s">
-        <v>541</v>
+        <v>554</v>
       </c>
       <c r="I69" s="1" t="s">
-        <v>726</v>
+        <v>731</v>
       </c>
       <c r="J69" s="1" t="s">
-        <v>727</v>
+        <v>732</v>
       </c>
       <c r="K69" s="1" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="L69" s="1" t="s">
-        <v>728</v>
+        <v>733</v>
       </c>
       <c r="M69" s="1" t="s">
-        <v>545</v>
+        <v>558</v>
       </c>
       <c r="N69" s="1" t="s">
-        <v>729</v>
+        <v>734</v>
       </c>
       <c r="O69" s="1" t="s">
-        <v>730</v>
+        <v>735</v>
       </c>
     </row>
     <row r="70" spans="1:15" ht="84" customHeight="1">
       <c r="A70" s="1" t="s">
-        <v>731</v>
+        <v>736</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>684</v>
+        <v>697</v>
       </c>
       <c r="C70" s="1" t="s">
-        <v>537</v>
+        <v>550</v>
       </c>
       <c r="D70" s="1" t="s">
-        <v>732</v>
+        <v>737</v>
       </c>
       <c r="E70" s="2" t="s">
-        <v>733</v>
+        <v>738</v>
       </c>
       <c r="F70" s="1" t="s">
-        <v>540</v>
+        <v>553</v>
       </c>
       <c r="G70" s="1" t="s">
         <v>21</v>
       </c>
       <c r="H70" s="1" t="s">
-        <v>541</v>
+        <v>554</v>
       </c>
       <c r="I70" s="1" t="s">
-        <v>734</v>
+        <v>739</v>
       </c>
       <c r="J70" s="1" t="s">
-        <v>735</v>
+        <v>740</v>
       </c>
       <c r="K70" s="1" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="L70" s="1" t="s">
-        <v>618</v>
+        <v>741</v>
       </c>
       <c r="M70" s="1" t="s">
-        <v>545</v>
+        <v>558</v>
       </c>
       <c r="N70" s="1" t="s">
-        <v>736</v>
+        <v>742</v>
       </c>
       <c r="O70" s="1" t="s">
-        <v>737</v>
+        <v>743</v>
+      </c>
+    </row>
+    <row r="71" spans="1:15" ht="84" customHeight="1">
+      <c r="A71" s="1" t="s">
+        <v>744</v>
+      </c>
+      <c r="B71" s="1" t="s">
+        <v>697</v>
+      </c>
+      <c r="C71" s="1" t="s">
+        <v>550</v>
+      </c>
+      <c r="D71" s="1" t="s">
+        <v>745</v>
+      </c>
+      <c r="E71" s="2" t="s">
+        <v>746</v>
+      </c>
+      <c r="F71" s="1" t="s">
+        <v>553</v>
+      </c>
+      <c r="G71" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="H71" s="1" t="s">
+        <v>554</v>
+      </c>
+      <c r="I71" s="1" t="s">
+        <v>747</v>
+      </c>
+      <c r="J71" s="1" t="s">
+        <v>748</v>
+      </c>
+      <c r="K71" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="L71" s="1" t="s">
+        <v>631</v>
+      </c>
+      <c r="M71" s="1" t="s">
+        <v>558</v>
+      </c>
+      <c r="N71" s="1" t="s">
+        <v>749</v>
+      </c>
+      <c r="O71" s="1" t="s">
+        <v>750</v>
+      </c>
+    </row>
+    <row r="72" spans="1:15" ht="84" customHeight="1">
+      <c r="A72" s="1" t="s">
+        <v>751</v>
+      </c>
+      <c r="B72" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C72" s="1" t="s">
+        <v>752</v>
+      </c>
+      <c r="D72" s="1" t="s">
+        <v>753</v>
+      </c>
+      <c r="E72" s="2" t="s">
+        <v>754</v>
+      </c>
+      <c r="F72" s="1" t="s">
+        <v>755</v>
+      </c>
+      <c r="G72" s="1" t="s">
+        <v>756</v>
+      </c>
+      <c r="H72" s="1" t="s">
+        <v>757</v>
+      </c>
+      <c r="I72" s="1" t="s">
+        <v>758</v>
+      </c>
+      <c r="J72" s="1" t="s">
+        <v>759</v>
+      </c>
+      <c r="K72" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="L72" s="1" t="s">
+        <v>760</v>
+      </c>
+      <c r="M72" s="1" t="s">
+        <v>761</v>
+      </c>
+      <c r="N72" s="1" t="s">
+        <v>762</v>
+      </c>
+      <c r="O72" s="1" t="s">
+        <v>763</v>
+      </c>
+    </row>
+    <row r="73" spans="1:15" ht="84" customHeight="1">
+      <c r="A73" s="1" t="s">
+        <v>764</v>
+      </c>
+      <c r="B73" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="C73" s="1" t="s">
+        <v>765</v>
+      </c>
+      <c r="D73" s="1" t="s">
+        <v>766</v>
+      </c>
+      <c r="E73" s="2" t="s">
+        <v>767</v>
+      </c>
+      <c r="F73" s="1" t="s">
+        <v>768</v>
+      </c>
+      <c r="G73" s="1" t="s">
+        <v>769</v>
+      </c>
+      <c r="H73" s="1" t="s">
+        <v>770</v>
+      </c>
+      <c r="I73" s="1" t="s">
+        <v>771</v>
+      </c>
+      <c r="J73" s="1" t="s">
+        <v>772</v>
+      </c>
+      <c r="K73" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="L73" s="1" t="s">
+        <v>773</v>
+      </c>
+      <c r="M73" s="1" t="s">
+        <v>774</v>
+      </c>
+      <c r="N73" s="1" t="s">
+        <v>775</v>
+      </c>
+      <c r="O73" s="1" t="s">
+        <v>776</v>
+      </c>
+    </row>
+    <row r="74" spans="1:15" ht="84" customHeight="1">
+      <c r="A74" s="1" t="s">
+        <v>777</v>
+      </c>
+      <c r="B74" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C74" s="1" t="s">
+        <v>778</v>
+      </c>
+      <c r="D74" s="1" t="s">
+        <v>779</v>
+      </c>
+      <c r="E74" s="2" t="s">
+        <v>780</v>
+      </c>
+      <c r="F74" s="1" t="s">
+        <v>355</v>
+      </c>
+      <c r="G74" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="H74" s="1" t="s">
+        <v>356</v>
+      </c>
+      <c r="I74" s="1" t="s">
+        <v>781</v>
+      </c>
+      <c r="J74" s="1" t="s">
+        <v>782</v>
+      </c>
+      <c r="K74" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="L74" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="M74" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="N74" s="1" t="s">
+        <v>783</v>
+      </c>
+      <c r="O74" s="1" t="s">
+        <v>784</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
-  <pageSetup fitToHeight="0" orientation="landscape"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>

</xml_diff>

<commit_message>
Add ConnectEDU transcript exchange source
</commit_message>
<xml_diff>
--- a/dossier/source_dossier.xlsx
+++ b/dossier/source_dossier.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1125" uniqueCount="785">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1140" uniqueCount="796">
   <si>
     <t>id</t>
   </si>
@@ -2369,6 +2369,39 @@
   </si>
   <si>
     <t>{{cite conference |title=26th Annual Management Information Systems (MIS) Conference agenda |conference=Management Information Systems Conference |publisher=National Center for Education Statistics |date=2013 |url=https://nces.ed.gov/whatsnew/conferences/pdf/MIS_2013_Agenda.pdf |access-date=June 8, 2026}}</t>
+  </si>
+  <si>
+    <t>CT0</t>
+  </si>
+  <si>
+    <t>2007</t>
+  </si>
+  <si>
+    <t>Service Links Student Data to Web College Planning Platform</t>
+  </si>
+  <si>
+    <t>https://campustechnology.com/articles/2007/03/service-links-student-data-to-web-college-planning-platform.aspx</t>
+  </si>
+  <si>
+    <t>Medium to High for ConnectEDU project context; does not name Alderson</t>
+  </si>
+  <si>
+    <t>Independent trade article about ConnectEDU and Rediker Software exporting school student data into a college planning, admissions, and financial-aid platform. Describes electronic college transcripts and application materials, PESC and SIFA guideline alignment, and ConnectEDU's expected 1.3 million transcript deliveries. Does not name Alderson.</t>
+  </si>
+  <si>
+    <t>ConnectEDU transcript-exchange and college-planning platform context; PESC/SIFA interoperability context; not Alderson-specific by itself.</t>
+  </si>
+  <si>
+    <t>Low for Alderson; Medium for ConnectEDU project context</t>
+  </si>
+  <si>
+    <t>Use only as ConnectEDU/project background paired with Alderson-specific sources such as Data &amp; Society or verified PESC biography/meeting materials. Do not use alone for Alderson-specific claims.</t>
+  </si>
+  <si>
+    <t>Reviewed in sources/campus_technology_sources.md and sources/connectedu_company_sources.md; local files data/campus_technology_connectedu_student_data_platform_2007.html and data/campus_technology_connectedu_student_data_platform_2007.txt</t>
+  </si>
+  <si>
+    <t>{{cite web |last=McCloskey |first=Paul |title=Service Links Student Data to Web College Planning Platform |url=https://campustechnology.com/articles/2007/03/service-links-student-data-to-web-college-planning-platform.aspx |website=Campus Technology |date=March 26, 2007 |access-date=June 8, 2026}}</t>
   </si>
 </sst>
 </file>
@@ -2445,8 +2478,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SourceDossier" displayName="SourceDossier" ref="A1:O74" totalsRowShown="0">
-  <autoFilter ref="A1:O74"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SourceDossier" displayName="SourceDossier" ref="A1:O75" totalsRowShown="0">
+  <autoFilter ref="A1:O75"/>
   <tableColumns count="15">
     <tableColumn id="1" name="id"/>
     <tableColumn id="2" name="year"/>
@@ -2753,7 +2786,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O74"/>
+  <dimension ref="A1:O75"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="2" width="10.7109375" customWidth="1"/>
@@ -6249,6 +6282,53 @@
         <v>784</v>
       </c>
     </row>
+    <row r="75" spans="1:15" ht="84" customHeight="1">
+      <c r="A75" s="1" t="s">
+        <v>785</v>
+      </c>
+      <c r="B75" s="1" t="s">
+        <v>786</v>
+      </c>
+      <c r="C75" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="D75" s="1" t="s">
+        <v>787</v>
+      </c>
+      <c r="E75" s="2" t="s">
+        <v>788</v>
+      </c>
+      <c r="F75" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="G75" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="H75" s="1" t="s">
+        <v>789</v>
+      </c>
+      <c r="I75" s="1" t="s">
+        <v>790</v>
+      </c>
+      <c r="J75" s="1" t="s">
+        <v>791</v>
+      </c>
+      <c r="K75" s="1" t="s">
+        <v>792</v>
+      </c>
+      <c r="L75" s="1" t="s">
+        <v>793</v>
+      </c>
+      <c r="M75" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="N75" s="1" t="s">
+        <v>794</v>
+      </c>
+      <c r="O75" s="1" t="s">
+        <v>795</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Add CEDS context sources
</commit_message>
<xml_diff>
--- a/dossier/source_dossier.xlsx
+++ b/dossier/source_dossier.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1140" uniqueCount="796">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1170" uniqueCount="822">
   <si>
     <t>id</t>
   </si>
@@ -2402,6 +2402,84 @@
   </si>
   <si>
     <t>{{cite web |last=McCloskey |first=Paul |title=Service Links Student Data to Web College Planning Platform |url=https://campustechnology.com/articles/2007/03/service-links-student-data-to-web-college-planning-platform.aspx |website=Campus Technology |date=March 26, 2007 |access-date=June 8, 2026}}</t>
+  </si>
+  <si>
+    <t>QIP1</t>
+  </si>
+  <si>
+    <t>Quality Information Partners</t>
+  </si>
+  <si>
+    <t>Developing National Education Data Standards</t>
+  </si>
+  <si>
+    <t>https://www.qi-partners.com/developing-national-education-data-standards/</t>
+  </si>
+  <si>
+    <t>Organizational blog / project history</t>
+  </si>
+  <si>
+    <t>Partial; independent of Alderson but QIP was CEDS contractor</t>
+  </si>
+  <si>
+    <t>Medium for CEDS history/context; not Alderson-specific</t>
+  </si>
+  <si>
+    <t>Context source. Describes NCES contracting QIP in fall 2009 to establish a technical working group for voluntary common standards; says CEDS became a data dictionary for P-20W data; describes 2011 model and tools work; and says CEDS development was enriched through collaboration with standards initiatives including PESC. Does not mention Alderson or ConnectEDU.</t>
+  </si>
+  <si>
+    <t>CEDS history and PESC standards-organization context only; not Alderson-specific by itself.</t>
+  </si>
+  <si>
+    <t>Low for Alderson; Medium for CEDS context</t>
+  </si>
+  <si>
+    <t>Use only as CEDS/project background paired with a source that directly verifies Alderson's role. Do not use for Alderson notability.</t>
+  </si>
+  <si>
+    <t>Reviewed in sources/ceds_sources.md; local files data/qi_partners_developing_national_education_data_standards.html and data/qi_partners_developing_national_education_data_standards.txt</t>
+  </si>
+  <si>
+    <t>{{cite web |last=Goodell |first=Jim |title=Developing National Education Data Standards |url=https://www.qi-partners.com/developing-national-education-data-standards/ |website=Quality Information Partners |date=July 10, 2024 |access-date=June 8, 2026}}</t>
+  </si>
+  <si>
+    <t>IES1</t>
+  </si>
+  <si>
+    <t>2010</t>
+  </si>
+  <si>
+    <t>Institute of Education Sciences / National Forum on Education Statistics</t>
+  </si>
+  <si>
+    <t>Forum Voice Fall 2010, Volume 13, No. 2</t>
+  </si>
+  <si>
+    <t>https://ies.ed.gov/use-work/non-data-collection-program/nfes-national-forum-education-statistics/member-resources/forum-voice/forum-voice-fall-2010-volume-13-no-2</t>
+  </si>
+  <si>
+    <t>Government newsletter / project history</t>
+  </si>
+  <si>
+    <t>Partial; independent of Alderson</t>
+  </si>
+  <si>
+    <t>High for CEDS 1.0 release context; not Alderson-specific</t>
+  </si>
+  <si>
+    <t>Context source. The Forum Voice Fall 2010 issue says CEDS Version 1.0 was released in September with 161 data elements for K-12 and transition-to-postsecondary data; says standards were drawn from or synchronized with NCES Handbooks Online, SIF, PESC schema, and EDFacts; and says Technical Working Group participants included state/local education agencies, higher education organizations, and key nonprofits. Does not mention Alderson or ConnectEDU.</t>
+  </si>
+  <si>
+    <t>CEDS 1.0 release history, PESC schema context, and transcript/use-case context only; not Alderson-specific by itself.</t>
+  </si>
+  <si>
+    <t>Low for Alderson; Medium to High for CEDS context</t>
+  </si>
+  <si>
+    <t>Reviewed in sources/ceds_sources.md; local files data/ies_forum_voice_fall_2010_ceds.html and data/ies_forum_voice_fall_2010_ceds.txt</t>
+  </si>
+  <si>
+    <t>{{cite web |title=Forum Voice Fall 2010, Volume 13, No. 2 |url=https://ies.ed.gov/use-work/non-data-collection-program/nfes-national-forum-education-statistics/member-resources/forum-voice/forum-voice-fall-2010-volume-13-no-2 |website=Institute of Education Sciences |publisher=National Forum on Education Statistics |date=Fall 2010 |access-date=June 8, 2026}}</t>
   </si>
 </sst>
 </file>
@@ -2478,8 +2556,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SourceDossier" displayName="SourceDossier" ref="A1:O75" totalsRowShown="0">
-  <autoFilter ref="A1:O75"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SourceDossier" displayName="SourceDossier" ref="A1:O77" totalsRowShown="0">
+  <autoFilter ref="A1:O77"/>
   <tableColumns count="15">
     <tableColumn id="1" name="id"/>
     <tableColumn id="2" name="year"/>
@@ -2786,7 +2864,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O75"/>
+  <dimension ref="A1:O77"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="2" width="10.7109375" customWidth="1"/>
@@ -6329,6 +6407,100 @@
         <v>795</v>
       </c>
     </row>
+    <row r="76" spans="1:15" ht="84" customHeight="1">
+      <c r="A76" s="1" t="s">
+        <v>796</v>
+      </c>
+      <c r="B76" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="C76" s="1" t="s">
+        <v>797</v>
+      </c>
+      <c r="D76" s="1" t="s">
+        <v>798</v>
+      </c>
+      <c r="E76" s="2" t="s">
+        <v>799</v>
+      </c>
+      <c r="F76" s="1" t="s">
+        <v>800</v>
+      </c>
+      <c r="G76" s="1" t="s">
+        <v>801</v>
+      </c>
+      <c r="H76" s="1" t="s">
+        <v>802</v>
+      </c>
+      <c r="I76" s="1" t="s">
+        <v>803</v>
+      </c>
+      <c r="J76" s="1" t="s">
+        <v>804</v>
+      </c>
+      <c r="K76" s="1" t="s">
+        <v>805</v>
+      </c>
+      <c r="L76" s="1" t="s">
+        <v>806</v>
+      </c>
+      <c r="M76" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="N76" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="O76" s="1" t="s">
+        <v>808</v>
+      </c>
+    </row>
+    <row r="77" spans="1:15" ht="84" customHeight="1">
+      <c r="A77" s="1" t="s">
+        <v>809</v>
+      </c>
+      <c r="B77" s="1" t="s">
+        <v>810</v>
+      </c>
+      <c r="C77" s="1" t="s">
+        <v>811</v>
+      </c>
+      <c r="D77" s="1" t="s">
+        <v>812</v>
+      </c>
+      <c r="E77" s="2" t="s">
+        <v>813</v>
+      </c>
+      <c r="F77" s="1" t="s">
+        <v>814</v>
+      </c>
+      <c r="G77" s="1" t="s">
+        <v>815</v>
+      </c>
+      <c r="H77" s="1" t="s">
+        <v>816</v>
+      </c>
+      <c r="I77" s="1" t="s">
+        <v>817</v>
+      </c>
+      <c r="J77" s="1" t="s">
+        <v>818</v>
+      </c>
+      <c r="K77" s="1" t="s">
+        <v>819</v>
+      </c>
+      <c r="L77" s="1" t="s">
+        <v>806</v>
+      </c>
+      <c r="M77" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="N77" s="1" t="s">
+        <v>820</v>
+      </c>
+      <c r="O77" s="1" t="s">
+        <v>821</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Update AfC source plan and draft quality report
</commit_message>
<xml_diff>
--- a/dossier/source_dossier.xlsx
+++ b/dossier/source_dossier.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1170" uniqueCount="822">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1215" uniqueCount="861">
   <si>
     <t>id</t>
   </si>
@@ -2480,6 +2480,123 @@
   </si>
   <si>
     <t>{{cite web |title=Forum Voice Fall 2010, Volume 13, No. 2 |url=https://ies.ed.gov/use-work/non-data-collection-program/nfes-national-forum-education-statistics/member-resources/forum-voice/forum-voice-fall-2010-volume-13-no-2 |website=Institute of Education Sciences |publisher=National Forum on Education Statistics |date=Fall 2010 |access-date=June 8, 2026}}</t>
+  </si>
+  <si>
+    <t>SCH1</t>
+  </si>
+  <si>
+    <t>2008</t>
+  </si>
+  <si>
+    <t>Fortnightly Mailing / Jim Farmer guest contribution</t>
+  </si>
+  <si>
+    <t>Bologna: are European entrepreneurs now leading the US on the development of Higher Education student record software? Guest Contribution by Jim Farmer</t>
+  </si>
+  <si>
+    <t>https://schmoller.net/fm.schmoller.net/2008/06/washington-rs3g.html</t>
+  </si>
+  <si>
+    <t>Independent blog / guest contribution</t>
+  </si>
+  <si>
+    <t>Yes, independent of Alderson and ConnectEDU</t>
+  </si>
+  <si>
+    <t>Medium for brief professional-context reporting; not in-depth biographical coverage</t>
+  </si>
+  <si>
+    <t>Directly names Jeff Alderson, ConnectEdu, in coverage of a PESC-hosted Washington briefing on RS3G, Bologna Process student-record exchange, HR-XML, and U.S. supplier perspectives. Says Alderson said ConnectEDU wanted electronic exchange among servicers and later direct standards-based connections to colleges and universities.</t>
+  </si>
+  <si>
+    <t>Alderson was associated with ConnectEDU in standards-based student-record exchange discussions at a PESC-hosted briefing.</t>
+  </si>
+  <si>
+    <t>Useful for narrow ConnectEDU/PESC professional-context evidence. Do not use as a standalone AfC notability anchor.</t>
+  </si>
+  <si>
+    <t>Reviewed in sources/connectedu_company_sources.md and sources/pesc_sources.md; local files data/schmoller_washington_rs3g_2008.html and data/schmoller_washington_rs3g_2008.txt</t>
+  </si>
+  <si>
+    <t>{{cite web |last=Farmer |first=Jim |title=Bologna: are European entrepreneurs now leading the US on the development of Higher Education student record software? Guest Contribution by Jim Farmer |url=https://schmoller.net/fm.schmoller.net/2008/06/washington-rs3g.html |website=Fortnightly Mailing |date=June 15, 2008 |access-date=June 9, 2026}}</t>
+  </si>
+  <si>
+    <t>PESCNEWS2013</t>
+  </si>
+  <si>
+    <t>PESC / Yumpu</t>
+  </si>
+  <si>
+    <t>February 2013 - PESC</t>
+  </si>
+  <si>
+    <t>https://www.yumpu.com/en/document/read/38261340/february-2013-pesc/7</t>
+  </si>
+  <si>
+    <t>Organizational publication hosted on document platform</t>
+  </si>
+  <si>
+    <t>No / primary-organizational</t>
+  </si>
+  <si>
+    <t>Medium for PESC publication metadata; not independent biographical coverage</t>
+  </si>
+  <si>
+    <t>PESC publication hosted on Yumpu. Visible page 7 lists JEFFREY ALDERSON, Senior Director of Product Innovation, ConnectEDU - MyData; also lists ConnectEDU as a Diamond Sponsor and describes PESC data-summit/data-standards context.</t>
+  </si>
+  <si>
+    <t>Alderson was listed by PESC as Senior Director of Product Innovation at ConnectEDU for MyData in February 2013.</t>
+  </si>
+  <si>
+    <t>Useful for narrow Alderson/ConnectEDU/PESC/MyData context. Do not use as a notability anchor.</t>
+  </si>
+  <si>
+    <t>Verified from downloaded Yumpu HTML/JSON and page image manual review</t>
+  </si>
+  <si>
+    <t>Reviewed in sources/pesc_sources.md, sources/connectedu_company_sources.md, and sources/mydata_button_sources.md; local files data/yumpu_pesc_february_2013_page7.html, data/yumpu_pesc_february_2013.json, data/yumpu_pesc_february_2013_visible_page7.jpg, and data/yumpu_pesc_february_2013_visible_page7_review.txt</t>
+  </si>
+  <si>
+    <t>{{cite web |title=February 2013 - PESC |url=https://www.yumpu.com/en/document/read/38261340/february-2013-pesc/7 |website=Yumpu |publisher=Postsecondary Electronic Standards Council |date=February 2013 |access-date=June 9, 2026}}</t>
+  </si>
+  <si>
+    <t>FAW1</t>
+  </si>
+  <si>
+    <t>StudyLib / PESC document mirror</t>
+  </si>
+  <si>
+    <t>PESC Functional Acknowledgment Workgroup CCB Review</t>
+  </si>
+  <si>
+    <t>https://studylib.net/doc/8601923/pesc-functional-acknowledgment-workgroup-ccb-review</t>
+  </si>
+  <si>
+    <t>Document mirror / source lead</t>
+  </si>
+  <si>
+    <t>Unknown; likely PESC organizational material if verified</t>
+  </si>
+  <si>
+    <t>Unverified locally; local fetch returned Cloudflare challenge</t>
+  </si>
+  <si>
+    <t>Source lead submitted as identifying Alderson working with the PESC Functional Acknowledgment working group. Direct local capture returned a Cloudflare challenge page, so the underlying document text was not verified locally.</t>
+  </si>
+  <si>
+    <t>Potential narrow PESC Functional Acknowledgment workgroup participation fact if verified.</t>
+  </si>
+  <si>
+    <t>Do not cite until browser/manual review confirms the underlying document. Retain as source lead only.</t>
+  </si>
+  <si>
+    <t>Blocked/source lead only; not verified for article use</t>
+  </si>
+  <si>
+    <t>Listed in sources/pesc_sources.md and sources/unverified_publication_leads.md; local files data/studylib_pesc_functional_acknowledgment_workgroup_ccb_review.html, data/studylib_pesc_functional_acknowledgment_workgroup_ccb_review.txt, and data/studylib_pesc_functional_acknowledgment_workgroup_ccb_review_note.txt</t>
+  </si>
+  <si>
+    <t>{{cite web |title=PESC Functional Acknowledgment Workgroup CCB Review |url=https://studylib.net/doc/8601923/pesc-functional-acknowledgment-workgroup-ccb-review |website=StudyLib |access-date=June 9, 2026}}</t>
   </si>
 </sst>
 </file>
@@ -2556,8 +2673,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SourceDossier" displayName="SourceDossier" ref="A1:O77" totalsRowShown="0">
-  <autoFilter ref="A1:O77"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SourceDossier" displayName="SourceDossier" ref="A1:O80" totalsRowShown="0">
+  <autoFilter ref="A1:O80"/>
   <tableColumns count="15">
     <tableColumn id="1" name="id"/>
     <tableColumn id="2" name="year"/>
@@ -2864,7 +2981,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O77"/>
+  <dimension ref="A1:O80"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="2" width="10.7109375" customWidth="1"/>
@@ -6501,6 +6618,147 @@
         <v>821</v>
       </c>
     </row>
+    <row r="78" spans="1:15" ht="84" customHeight="1">
+      <c r="A78" s="1" t="s">
+        <v>822</v>
+      </c>
+      <c r="B78" s="1" t="s">
+        <v>823</v>
+      </c>
+      <c r="C78" s="1" t="s">
+        <v>824</v>
+      </c>
+      <c r="D78" s="1" t="s">
+        <v>825</v>
+      </c>
+      <c r="E78" s="2" t="s">
+        <v>826</v>
+      </c>
+      <c r="F78" s="1" t="s">
+        <v>827</v>
+      </c>
+      <c r="G78" s="1" t="s">
+        <v>828</v>
+      </c>
+      <c r="H78" s="1" t="s">
+        <v>829</v>
+      </c>
+      <c r="I78" s="1" t="s">
+        <v>830</v>
+      </c>
+      <c r="J78" s="1" t="s">
+        <v>831</v>
+      </c>
+      <c r="K78" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="L78" s="1" t="s">
+        <v>832</v>
+      </c>
+      <c r="M78" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="N78" s="1" t="s">
+        <v>833</v>
+      </c>
+      <c r="O78" s="1" t="s">
+        <v>834</v>
+      </c>
+    </row>
+    <row r="79" spans="1:15" ht="84" customHeight="1">
+      <c r="A79" s="1" t="s">
+        <v>835</v>
+      </c>
+      <c r="B79" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C79" s="1" t="s">
+        <v>836</v>
+      </c>
+      <c r="D79" s="1" t="s">
+        <v>837</v>
+      </c>
+      <c r="E79" s="2" t="s">
+        <v>838</v>
+      </c>
+      <c r="F79" s="1" t="s">
+        <v>839</v>
+      </c>
+      <c r="G79" s="1" t="s">
+        <v>840</v>
+      </c>
+      <c r="H79" s="1" t="s">
+        <v>841</v>
+      </c>
+      <c r="I79" s="1" t="s">
+        <v>842</v>
+      </c>
+      <c r="J79" s="1" t="s">
+        <v>843</v>
+      </c>
+      <c r="K79" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="L79" s="1" t="s">
+        <v>844</v>
+      </c>
+      <c r="M79" s="1" t="s">
+        <v>845</v>
+      </c>
+      <c r="N79" s="1" t="s">
+        <v>846</v>
+      </c>
+      <c r="O79" s="1" t="s">
+        <v>847</v>
+      </c>
+    </row>
+    <row r="80" spans="1:15" ht="84" customHeight="1">
+      <c r="A80" s="1" t="s">
+        <v>848</v>
+      </c>
+      <c r="B80" s="1" t="s">
+        <v>441</v>
+      </c>
+      <c r="C80" s="1" t="s">
+        <v>849</v>
+      </c>
+      <c r="D80" s="1" t="s">
+        <v>850</v>
+      </c>
+      <c r="E80" s="2" t="s">
+        <v>851</v>
+      </c>
+      <c r="F80" s="1" t="s">
+        <v>852</v>
+      </c>
+      <c r="G80" s="1" t="s">
+        <v>853</v>
+      </c>
+      <c r="H80" s="1" t="s">
+        <v>854</v>
+      </c>
+      <c r="I80" s="1" t="s">
+        <v>855</v>
+      </c>
+      <c r="J80" s="1" t="s">
+        <v>856</v>
+      </c>
+      <c r="K80" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="L80" s="1" t="s">
+        <v>857</v>
+      </c>
+      <c r="M80" s="1" t="s">
+        <v>858</v>
+      </c>
+      <c r="N80" s="1" t="s">
+        <v>859</v>
+      </c>
+      <c r="O80" s="1" t="s">
+        <v>860</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Update draft with PESC and local video sources
</commit_message>
<xml_diff>
--- a/dossier/source_dossier.xlsx
+++ b/dossier/source_dossier.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1215" uniqueCount="861">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1275" uniqueCount="905">
   <si>
     <t>id</t>
   </si>
@@ -2563,7 +2563,7 @@
     <t>FAW1</t>
   </si>
   <si>
-    <t>StudyLib / PESC document mirror</t>
+    <t>StudyLib / PESC document mirror; local PDF copy</t>
   </si>
   <si>
     <t>PESC Functional Acknowledgment Workgroup CCB Review</t>
@@ -2572,49 +2572,173 @@
     <t>https://studylib.net/doc/8601923/pesc-functional-acknowledgment-workgroup-ccb-review</t>
   </si>
   <si>
-    <t>Document mirror / source lead</t>
-  </si>
-  <si>
-    <t>Unknown; likely PESC organizational material if verified</t>
-  </si>
-  <si>
-    <t>Unverified locally; local fetch returned Cloudflare challenge</t>
-  </si>
-  <si>
-    <t>Source lead submitted as identifying Alderson working with the PESC Functional Acknowledgment working group. Direct local capture returned a Cloudflare challenge page, so the underlying document text was not verified locally.</t>
-  </si>
-  <si>
-    <t>Potential narrow PESC Functional Acknowledgment workgroup participation fact if verified.</t>
-  </si>
-  <si>
-    <t>Do not cite until browser/manual review confirms the underlying document. Retain as source lead only.</t>
-  </si>
-  <si>
-    <t>Blocked/source lead only; not verified for article use</t>
-  </si>
-  <si>
-    <t>Listed in sources/pesc_sources.md and sources/unverified_publication_leads.md; local files data/studylib_pesc_functional_acknowledgment_workgroup_ccb_review.html, data/studylib_pesc_functional_acknowledgment_workgroup_ccb_review.txt, and data/studylib_pesc_functional_acknowledgment_workgroup_ccb_review_note.txt</t>
-  </si>
-  <si>
-    <t>{{cite web |title=PESC Functional Acknowledgment Workgroup CCB Review |url=https://studylib.net/doc/8601923/pesc-functional-acknowledgment-workgroup-ccb-review |website=StudyLib |access-date=June 9, 2026}}</t>
+    <t>Document mirror / PESC meeting minutes</t>
+  </si>
+  <si>
+    <t>No / primary-organizational PESC workgroup record</t>
+  </si>
+  <si>
+    <t>Medium for narrow meeting-minutes evidence from local PDF rendering; direct URL capture remains blocked</t>
+  </si>
+  <si>
+    <t>Local PDF rendering shows PESC Functional Acknowledgment Workgroup CCB Review Meeting Minutes 3/30/09 3 pm EDT and lists Jeffrey Alderson, jalderson@ConnectEdu.net, ConnectEdu, among workgroup presenters with Rob Moore and Monterey Sims.</t>
+  </si>
+  <si>
+    <t>Alderson was listed as a ConnectEdu presenter for the PESC Functional Acknowledgment Workgroup CCB Review meeting minutes dated March 30, 2009.</t>
+  </si>
+  <si>
+    <t>Use only for narrow PESC Functional Acknowledgment workgroup participation if needed. Do not use as a notability anchor.</t>
+  </si>
+  <si>
+    <t>Verified from local PDF rendering; direct StudyLib capture remains Cloudflare-blocked</t>
+  </si>
+  <si>
+    <t>Listed in sources/pesc_sources.md; removed from unverified leads. Local files data/studylib_pesc_functional_acknowledgment_workgroup_ccb_review.pdf, data/studylib_pesc_functional_acknowledgment_workgroup_ccb_review_pdf.txt, data/studylib_pesc_functional_acknowledgment_workgroup_ccb_review.html, data/studylib_pesc_functional_acknowledgment_workgroup_ccb_review.txt, and data/studylib_pesc_functional_acknowledgment_workgroup_ccb_review_note.txt</t>
+  </si>
+  <si>
+    <t>{{cite web |title=PESC Functional Acknowledgment Workgroup CCB Review |url=https://studylib.net/doc/8601923/pesc-functional-acknowledgment-workgroup-ccb-review |website=StudyLib |date=March 30, 2009 |access-date=June 9, 2026}}</t>
+  </si>
+  <si>
+    <t>NPEG1</t>
+  </si>
+  <si>
+    <t>2025-2026</t>
+  </si>
+  <si>
+    <t>Natick Pegasus / TelVue</t>
+  </si>
+  <si>
+    <t>Town Meeting playlist and 2025 Fall Town Meeting primer videos</t>
+  </si>
+  <si>
+    <t>https://videoplayer.telvue.com/player/994DtmGEsi0VDYK3jJI2BJ72GfgNIpU2/playlists/4742/media/1020538?showtabssearch=true&amp;fullscreen=false</t>
+  </si>
+  <si>
+    <t>Local-access video playlist / civic programming</t>
+  </si>
+  <si>
+    <t>Partial; local access civic media, not independent biographical coverage</t>
+  </si>
+  <si>
+    <t>Medium for video metadata and caption-track content; low for notability</t>
+  </si>
+  <si>
+    <t>Supplied page is a Natick Pegasus Town Meeting playlist. Playlist includes Town Meeting recordings and 2025 Fall Town Meeting primer videos. Captions reviewed from primer videos identify Alderson as town moderator in several segments.</t>
+  </si>
+  <si>
+    <t>Alderson appeared in local-access Town Meeting primer video segments as Natick town moderator.</t>
+  </si>
+  <si>
+    <t>Dossier only unless a narrow moderator-video fact is needed. Do not use as notability evidence.</t>
+  </si>
+  <si>
+    <t>Verified from TelVue HTML and Pegasus caption tracks</t>
+  </si>
+  <si>
+    <t>Reviewed in sources/local_video_sources.md; local files data/natick_pegasus_telvue_1020538.html, data/natick_pegasus_telvue_979704.html, data/natick_pegasus_telvue_980168.html, data/natick_pegasus_telvue_980169.html, data/natick_pegasus_telvue_980173.html, and related *_captions.vtt files</t>
+  </si>
+  <si>
+    <t>{{cite web |title=Natick Spring Annual Town Meeting April 30, 2026 |url=https://videoplayer.telvue.com/player/994DtmGEsi0VDYK3jJI2BJ72GfgNIpU2/playlists/4742/media/1020538?showtabssearch=true&amp;fullscreen=false |website=Natick Pegasus |publisher=TelVue |date=April 30, 2026 |access-date=June 9, 2026}}</t>
+  </si>
+  <si>
+    <t>CWAP1</t>
+  </si>
+  <si>
+    <t>Coffee with a Purpose, Natick MA / YouTube</t>
+  </si>
+  <si>
+    <t>CWAP 4/14/25 - Spring Town Meeting: Jeff Alderson &amp; Todd Gillenwater</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=Z7mz7TsZSq8</t>
+  </si>
+  <si>
+    <t>Local nonprofit civic video / YouTube</t>
+  </si>
+  <si>
+    <t>Partial; local nonprofit hosted-program source</t>
+  </si>
+  <si>
+    <t>Medium for YouTube metadata and source existence; low for independent biographical claims</t>
+  </si>
+  <si>
+    <t>YouTube metadata identifies a discussion of Natick 2025 Spring Annual Town Meeting articles with Jeff Alderson, town moderator, and Todd Gillenwater of the Finance Committee.</t>
+  </si>
+  <si>
+    <t>Alderson appeared in a Coffee with a Purpose video as Natick town moderator discussing Spring 2025 Town Meeting articles.</t>
+  </si>
+  <si>
+    <t>Dossier only; useful as local civic-video evidence, not independent biographical coverage.</t>
+  </si>
+  <si>
+    <t>Verified from downloaded YouTube HTML metadata</t>
+  </si>
+  <si>
+    <t>Reviewed in sources/local_video_sources.md; local file data/cwap_youtube_Z7mz7TsZSq8.html</t>
+  </si>
+  <si>
+    <t>{{cite web |title=CWAP 4/14/25 - Spring Town Meeting: Jeff Alderson &amp; Todd Gillenwater |url=https://www.youtube.com/watch?v=Z7mz7TsZSq8 |website=YouTube |publisher=Coffee with a Purpose, Natick MA |date=April 14, 2025 |access-date=June 9, 2026}}</t>
+  </si>
+  <si>
+    <t>CWAP2</t>
+  </si>
+  <si>
+    <t>CWAP - 10/6/25 - Town Meeting Warrant walkthrough with Fincom and Moderator</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=Af-dv2k8BNc</t>
+  </si>
+  <si>
+    <t>Medium for YouTube metadata and source existence; Alderson-specific content requires manual video review</t>
+  </si>
+  <si>
+    <t>YouTube metadata identifies a Town Meeting warrant walkthrough with the Finance Committee and moderator. The captured metadata does not name Alderson directly; user supplied it as an Alderson town-moderator interview source.</t>
+  </si>
+  <si>
+    <t>Potential support for Alderson appearing in a CWAP town-moderator video if manual review confirms the video content.</t>
+  </si>
+  <si>
+    <t>Treat as source lead until manually reviewed in the video player. Do not cite in article draft for Alderson-specific facts yet.</t>
+  </si>
+  <si>
+    <t>Partially verified from downloaded YouTube HTML metadata; content not manually reviewed</t>
+  </si>
+  <si>
+    <t>Reviewed in sources/local_video_sources.md; local file data/cwap_youtube_Af-dv2k8BNc.html</t>
+  </si>
+  <si>
+    <t>{{cite web |title=CWAP - 10/6/25 - Town Meeting Warrant walkthrough with Fincom and Moderator |url=https://www.youtube.com/watch?v=Af-dv2k8BNc |website=YouTube |publisher=Coffee with a Purpose, Natick MA |date=October 6, 2025 |access-date=June 9, 2026}}</t>
+  </si>
+  <si>
+    <t>CWAP3</t>
+  </si>
+  <si>
+    <t>CWAP 5/4/26 - Spring Town Meeting Debrief</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=ClsjG0XI0_E</t>
+  </si>
+  <si>
+    <t>YouTube metadata identifies a Spring Town Meeting debrief and includes town-meeting links. The captured metadata does not name Alderson directly; user supplied it as an Alderson town-moderator interview source.</t>
+  </si>
+  <si>
+    <t>Potential support for Alderson appearing in a CWAP town-moderator debrief video if manual review confirms the video content.</t>
+  </si>
+  <si>
+    <t>Reviewed in sources/local_video_sources.md; local file data/cwap_youtube_ClsjG0XI0_E.html</t>
+  </si>
+  <si>
+    <t>{{cite web |title=CWAP 5/4/26 - Spring Town Meeting Debrief |url=https://www.youtube.com/watch?v=ClsjG0XI0_E |website=YouTube |publisher=Coffee with a Purpose, Natick MA |date=May 4, 2026 |access-date=June 9, 2026}}</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -2628,7 +2752,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -2636,31 +2760,13 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2673,8 +2779,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SourceDossier" displayName="SourceDossier" ref="A1:O80" totalsRowShown="0">
-  <autoFilter ref="A1:O80"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:O84" totalsRowShown="0">
+  <autoFilter ref="A1:O84"/>
   <tableColumns count="15">
     <tableColumn id="1" name="id"/>
     <tableColumn id="2" name="year"/>
@@ -2981,22 +3087,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O80"/>
+  <dimension ref="A1:O84"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="2" width="10.7109375" customWidth="1"/>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="2" width="10.7109375" customWidth="1"/>
     <col min="3" max="3" width="24.7109375" customWidth="1"/>
-    <col min="4" max="4" width="44.7109375" customWidth="1"/>
-    <col min="5" max="5" width="52.7109375" customWidth="1"/>
-    <col min="6" max="6" width="24.7109375" customWidth="1"/>
-    <col min="7" max="7" width="18.7109375" customWidth="1"/>
+    <col min="4" max="4" width="36.7109375" customWidth="1"/>
+    <col min="5" max="5" width="42.7109375" customWidth="1"/>
+    <col min="6" max="7" width="24.7109375" customWidth="1"/>
     <col min="8" max="8" width="34.7109375" customWidth="1"/>
-    <col min="9" max="10" width="52.7109375" customWidth="1"/>
+    <col min="9" max="10" width="50.7109375" customWidth="1"/>
     <col min="11" max="11" width="18.7109375" customWidth="1"/>
     <col min="12" max="12" width="44.7109375" customWidth="1"/>
-    <col min="13" max="13" width="32.7109375" customWidth="1"/>
-    <col min="14" max="14" width="52.7109375" customWidth="1"/>
-    <col min="15" max="15" width="64.7109375" customWidth="1"/>
+    <col min="13" max="13" width="28.7109375" customWidth="1"/>
+    <col min="14" max="14" width="50.7109375" customWidth="1"/>
+    <col min="15" max="15" width="60.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="36" customHeight="1">
@@ -3046,7 +3152,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:15" ht="84" customHeight="1">
+    <row r="2" spans="1:15">
       <c r="A2" s="1" t="s">
         <v>15</v>
       </c>
@@ -3059,7 +3165,7 @@
       <c r="D2" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="1" t="s">
         <v>19</v>
       </c>
       <c r="F2" s="1" t="s">
@@ -3093,7 +3199,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="3" spans="1:15" ht="84" customHeight="1">
+    <row r="3" spans="1:15">
       <c r="A3" s="1" t="s">
         <v>30</v>
       </c>
@@ -3106,7 +3212,7 @@
       <c r="D3" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="1" t="s">
         <v>34</v>
       </c>
       <c r="F3" s="1" t="s">
@@ -3140,7 +3246,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="4" spans="1:15" ht="84" customHeight="1">
+    <row r="4" spans="1:15">
       <c r="A4" s="1" t="s">
         <v>45</v>
       </c>
@@ -3153,7 +3259,7 @@
       <c r="D4" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="1" t="s">
         <v>49</v>
       </c>
       <c r="F4" s="1" t="s">
@@ -3187,7 +3293,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="5" spans="1:15" ht="84" customHeight="1">
+    <row r="5" spans="1:15">
       <c r="A5" s="1" t="s">
         <v>59</v>
       </c>
@@ -3200,7 +3306,7 @@
       <c r="D5" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="E5" s="1" t="s">
         <v>63</v>
       </c>
       <c r="F5" s="1" t="s">
@@ -3234,7 +3340,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="6" spans="1:15" ht="84" customHeight="1">
+    <row r="6" spans="1:15">
       <c r="A6" s="1" t="s">
         <v>72</v>
       </c>
@@ -3247,7 +3353,7 @@
       <c r="D6" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="E6" s="1" t="s">
         <v>75</v>
       </c>
       <c r="F6" s="1" t="s">
@@ -3281,7 +3387,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="7" spans="1:15" ht="84" customHeight="1">
+    <row r="7" spans="1:15">
       <c r="A7" s="1" t="s">
         <v>86</v>
       </c>
@@ -3294,7 +3400,7 @@
       <c r="D7" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="E7" s="1" t="s">
         <v>90</v>
       </c>
       <c r="F7" s="1" t="s">
@@ -3328,7 +3434,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="8" spans="1:15" ht="84" customHeight="1">
+    <row r="8" spans="1:15">
       <c r="A8" s="1" t="s">
         <v>100</v>
       </c>
@@ -3341,7 +3447,7 @@
       <c r="D8" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="E8" s="1" t="s">
         <v>104</v>
       </c>
       <c r="F8" s="1" t="s">
@@ -3375,7 +3481,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="9" spans="1:15" ht="84" customHeight="1">
+    <row r="9" spans="1:15">
       <c r="A9" s="1" t="s">
         <v>115</v>
       </c>
@@ -3388,7 +3494,7 @@
       <c r="D9" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="E9" s="1" t="s">
         <v>119</v>
       </c>
       <c r="F9" s="1" t="s">
@@ -3422,7 +3528,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="10" spans="1:15" ht="84" customHeight="1">
+    <row r="10" spans="1:15">
       <c r="A10" s="1" t="s">
         <v>127</v>
       </c>
@@ -3435,7 +3541,7 @@
       <c r="D10" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="E10" s="1" t="s">
         <v>129</v>
       </c>
       <c r="F10" s="1" t="s">
@@ -3469,7 +3575,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="11" spans="1:15" ht="84" customHeight="1">
+    <row r="11" spans="1:15">
       <c r="A11" s="1" t="s">
         <v>136</v>
       </c>
@@ -3482,7 +3588,7 @@
       <c r="D11" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="E11" s="2" t="s">
+      <c r="E11" s="1" t="s">
         <v>139</v>
       </c>
       <c r="F11" s="1" t="s">
@@ -3516,7 +3622,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="12" spans="1:15" ht="84" customHeight="1">
+    <row r="12" spans="1:15">
       <c r="A12" s="1" t="s">
         <v>148</v>
       </c>
@@ -3529,7 +3635,7 @@
       <c r="D12" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="E12" s="2" t="s">
+      <c r="E12" s="1" t="s">
         <v>151</v>
       </c>
       <c r="F12" s="1" t="s">
@@ -3563,7 +3669,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="13" spans="1:15" ht="84" customHeight="1">
+    <row r="13" spans="1:15">
       <c r="A13" s="1" t="s">
         <v>159</v>
       </c>
@@ -3576,7 +3682,7 @@
       <c r="D13" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="E13" s="2" t="s">
+      <c r="E13" s="1" t="s">
         <v>163</v>
       </c>
       <c r="F13" s="1" t="s">
@@ -3610,7 +3716,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="14" spans="1:15" ht="84" customHeight="1">
+    <row r="14" spans="1:15">
       <c r="A14" s="1" t="s">
         <v>171</v>
       </c>
@@ -3623,7 +3729,7 @@
       <c r="D14" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="E14" s="2" t="s">
+      <c r="E14" s="1" t="s">
         <v>175</v>
       </c>
       <c r="F14" s="1" t="s">
@@ -3657,7 +3763,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="15" spans="1:15" ht="84" customHeight="1">
+    <row r="15" spans="1:15">
       <c r="A15" s="1" t="s">
         <v>183</v>
       </c>
@@ -3670,7 +3776,7 @@
       <c r="D15" s="1" t="s">
         <v>186</v>
       </c>
-      <c r="E15" s="2" t="s">
+      <c r="E15" s="1" t="s">
         <v>187</v>
       </c>
       <c r="F15" s="1" t="s">
@@ -3704,7 +3810,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="16" spans="1:15" ht="84" customHeight="1">
+    <row r="16" spans="1:15">
       <c r="A16" s="1" t="s">
         <v>195</v>
       </c>
@@ -3717,7 +3823,7 @@
       <c r="D16" s="1" t="s">
         <v>198</v>
       </c>
-      <c r="E16" s="2" t="s">
+      <c r="E16" s="1" t="s">
         <v>199</v>
       </c>
       <c r="F16" s="1" t="s">
@@ -3751,7 +3857,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="17" spans="1:15" ht="84" customHeight="1">
+    <row r="17" spans="1:15">
       <c r="A17" s="1" t="s">
         <v>209</v>
       </c>
@@ -3764,7 +3870,7 @@
       <c r="D17" s="1" t="s">
         <v>212</v>
       </c>
-      <c r="E17" s="2" t="s">
+      <c r="E17" s="1" t="s">
         <v>213</v>
       </c>
       <c r="F17" s="1" t="s">
@@ -3798,7 +3904,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="18" spans="1:15" ht="84" customHeight="1">
+    <row r="18" spans="1:15">
       <c r="A18" s="1" t="s">
         <v>223</v>
       </c>
@@ -3811,7 +3917,7 @@
       <c r="D18" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="E18" s="2" t="s">
+      <c r="E18" s="1" t="s">
         <v>226</v>
       </c>
       <c r="F18" s="1" t="s">
@@ -3845,7 +3951,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="19" spans="1:15" ht="84" customHeight="1">
+    <row r="19" spans="1:15">
       <c r="A19" s="1" t="s">
         <v>236</v>
       </c>
@@ -3858,7 +3964,7 @@
       <c r="D19" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="E19" s="2" t="s">
+      <c r="E19" s="1" t="s">
         <v>238</v>
       </c>
       <c r="F19" s="1" t="s">
@@ -3892,7 +3998,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="20" spans="1:15" ht="84" customHeight="1">
+    <row r="20" spans="1:15">
       <c r="A20" s="1" t="s">
         <v>246</v>
       </c>
@@ -3905,7 +4011,7 @@
       <c r="D20" s="1" t="s">
         <v>248</v>
       </c>
-      <c r="E20" s="2" t="s">
+      <c r="E20" s="1" t="s">
         <v>249</v>
       </c>
       <c r="F20" s="1" t="s">
@@ -3939,7 +4045,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="21" spans="1:15" ht="84" customHeight="1">
+    <row r="21" spans="1:15">
       <c r="A21" s="1" t="s">
         <v>258</v>
       </c>
@@ -3952,7 +4058,7 @@
       <c r="D21" s="1" t="s">
         <v>260</v>
       </c>
-      <c r="E21" s="2" t="s">
+      <c r="E21" s="1" t="s">
         <v>261</v>
       </c>
       <c r="F21" s="1" t="s">
@@ -3986,7 +4092,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="22" spans="1:15" ht="84" customHeight="1">
+    <row r="22" spans="1:15">
       <c r="A22" s="1" t="s">
         <v>271</v>
       </c>
@@ -3999,7 +4105,7 @@
       <c r="D22" s="1" t="s">
         <v>274</v>
       </c>
-      <c r="E22" s="2" t="s">
+      <c r="E22" s="1" t="s">
         <v>275</v>
       </c>
       <c r="F22" s="1" t="s">
@@ -4033,7 +4139,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="23" spans="1:15" ht="84" customHeight="1">
+    <row r="23" spans="1:15">
       <c r="A23" s="1" t="s">
         <v>285</v>
       </c>
@@ -4046,7 +4152,7 @@
       <c r="D23" s="1" t="s">
         <v>286</v>
       </c>
-      <c r="E23" s="2" t="s">
+      <c r="E23" s="1" t="s">
         <v>287</v>
       </c>
       <c r="F23" s="1" t="s">
@@ -4080,7 +4186,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="24" spans="1:15" ht="84" customHeight="1">
+    <row r="24" spans="1:15">
       <c r="A24" s="1" t="s">
         <v>296</v>
       </c>
@@ -4093,7 +4199,7 @@
       <c r="D24" s="1" t="s">
         <v>297</v>
       </c>
-      <c r="E24" s="2" t="s">
+      <c r="E24" s="1" t="s">
         <v>298</v>
       </c>
       <c r="F24" s="1" t="s">
@@ -4127,7 +4233,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="25" spans="1:15" ht="84" customHeight="1">
+    <row r="25" spans="1:15">
       <c r="A25" s="1" t="s">
         <v>304</v>
       </c>
@@ -4140,7 +4246,7 @@
       <c r="D25" s="1" t="s">
         <v>306</v>
       </c>
-      <c r="E25" s="2" t="s">
+      <c r="E25" s="1" t="s">
         <v>307</v>
       </c>
       <c r="F25" s="1" t="s">
@@ -4174,7 +4280,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="26" spans="1:15" ht="84" customHeight="1">
+    <row r="26" spans="1:15">
       <c r="A26" s="1" t="s">
         <v>315</v>
       </c>
@@ -4187,7 +4293,7 @@
       <c r="D26" s="1" t="s">
         <v>318</v>
       </c>
-      <c r="E26" s="2" t="s">
+      <c r="E26" s="1" t="s">
         <v>319</v>
       </c>
       <c r="F26" s="1" t="s">
@@ -4221,7 +4327,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="27" spans="1:15" ht="84" customHeight="1">
+    <row r="27" spans="1:15">
       <c r="A27" s="1" t="s">
         <v>328</v>
       </c>
@@ -4234,7 +4340,7 @@
       <c r="D27" s="1" t="s">
         <v>331</v>
       </c>
-      <c r="E27" s="2" t="s">
+      <c r="E27" s="1" t="s">
         <v>332</v>
       </c>
       <c r="F27" s="1" t="s">
@@ -4268,7 +4374,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="28" spans="1:15" ht="84" customHeight="1">
+    <row r="28" spans="1:15">
       <c r="A28" s="1" t="s">
         <v>341</v>
       </c>
@@ -4281,7 +4387,7 @@
       <c r="D28" s="1" t="s">
         <v>342</v>
       </c>
-      <c r="E28" s="2" t="s">
+      <c r="E28" s="1" t="s">
         <v>343</v>
       </c>
       <c r="F28" s="1" t="s">
@@ -4315,7 +4421,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="29" spans="1:15" ht="84" customHeight="1">
+    <row r="29" spans="1:15">
       <c r="A29" s="1" t="s">
         <v>351</v>
       </c>
@@ -4328,7 +4434,7 @@
       <c r="D29" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E29" s="2" t="s">
+      <c r="E29" s="1" t="s">
         <v>354</v>
       </c>
       <c r="F29" s="1" t="s">
@@ -4362,7 +4468,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="30" spans="1:15" ht="84" customHeight="1">
+    <row r="30" spans="1:15">
       <c r="A30" s="1" t="s">
         <v>362</v>
       </c>
@@ -4375,7 +4481,7 @@
       <c r="D30" s="1" t="s">
         <v>364</v>
       </c>
-      <c r="E30" s="2" t="s">
+      <c r="E30" s="1" t="s">
         <v>365</v>
       </c>
       <c r="F30" s="1" t="s">
@@ -4409,7 +4515,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="31" spans="1:15" ht="84" customHeight="1">
+    <row r="31" spans="1:15">
       <c r="A31" s="1" t="s">
         <v>371</v>
       </c>
@@ -4422,7 +4528,7 @@
       <c r="D31" s="1" t="s">
         <v>373</v>
       </c>
-      <c r="E31" s="2" t="s">
+      <c r="E31" s="1" t="s">
         <v>374</v>
       </c>
       <c r="F31" s="1" t="s">
@@ -4456,7 +4562,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="32" spans="1:15" ht="84" customHeight="1">
+    <row r="32" spans="1:15">
       <c r="A32" s="1" t="s">
         <v>382</v>
       </c>
@@ -4469,7 +4575,7 @@
       <c r="D32" s="1" t="s">
         <v>383</v>
       </c>
-      <c r="E32" s="2" t="s">
+      <c r="E32" s="1" t="s">
         <v>384</v>
       </c>
       <c r="F32" s="1" t="s">
@@ -4503,7 +4609,7 @@
         <v>390</v>
       </c>
     </row>
-    <row r="33" spans="1:15" ht="84" customHeight="1">
+    <row r="33" spans="1:15">
       <c r="A33" s="1" t="s">
         <v>391</v>
       </c>
@@ -4516,7 +4622,7 @@
       <c r="D33" s="1" t="s">
         <v>393</v>
       </c>
-      <c r="E33" s="2" t="s">
+      <c r="E33" s="1" t="s">
         <v>394</v>
       </c>
       <c r="F33" s="1" t="s">
@@ -4550,7 +4656,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="34" spans="1:15" ht="84" customHeight="1">
+    <row r="34" spans="1:15">
       <c r="A34" s="1" t="s">
         <v>402</v>
       </c>
@@ -4563,7 +4669,7 @@
       <c r="D34" s="1" t="s">
         <v>404</v>
       </c>
-      <c r="E34" s="2" t="s">
+      <c r="E34" s="1" t="s">
         <v>405</v>
       </c>
       <c r="F34" s="1" t="s">
@@ -4597,7 +4703,7 @@
         <v>414</v>
       </c>
     </row>
-    <row r="35" spans="1:15" ht="84" customHeight="1">
+    <row r="35" spans="1:15">
       <c r="A35" s="1" t="s">
         <v>415</v>
       </c>
@@ -4610,7 +4716,7 @@
       <c r="D35" s="1" t="s">
         <v>417</v>
       </c>
-      <c r="E35" s="2" t="s">
+      <c r="E35" s="1" t="s">
         <v>418</v>
       </c>
       <c r="F35" s="1" t="s">
@@ -4644,7 +4750,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="36" spans="1:15" ht="84" customHeight="1">
+    <row r="36" spans="1:15">
       <c r="A36" s="1" t="s">
         <v>428</v>
       </c>
@@ -4657,7 +4763,7 @@
       <c r="D36" s="1" t="s">
         <v>430</v>
       </c>
-      <c r="E36" s="2" t="s">
+      <c r="E36" s="1" t="s">
         <v>431</v>
       </c>
       <c r="F36" s="1" t="s">
@@ -4691,7 +4797,7 @@
         <v>439</v>
       </c>
     </row>
-    <row r="37" spans="1:15" ht="84" customHeight="1">
+    <row r="37" spans="1:15">
       <c r="A37" s="1" t="s">
         <v>440</v>
       </c>
@@ -4704,7 +4810,7 @@
       <c r="D37" s="1" t="s">
         <v>443</v>
       </c>
-      <c r="E37" s="2" t="s">
+      <c r="E37" s="1" t="s">
         <v>444</v>
       </c>
       <c r="F37" s="1" t="s">
@@ -4738,7 +4844,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="38" spans="1:15" ht="84" customHeight="1">
+    <row r="38" spans="1:15">
       <c r="A38" s="1" t="s">
         <v>454</v>
       </c>
@@ -4751,7 +4857,7 @@
       <c r="D38" s="1" t="s">
         <v>457</v>
       </c>
-      <c r="E38" s="2" t="s">
+      <c r="E38" s="1" t="s">
         <v>458</v>
       </c>
       <c r="F38" s="1" t="s">
@@ -4785,7 +4891,7 @@
         <v>467</v>
       </c>
     </row>
-    <row r="39" spans="1:15" ht="84" customHeight="1">
+    <row r="39" spans="1:15">
       <c r="A39" s="1" t="s">
         <v>468</v>
       </c>
@@ -4798,7 +4904,7 @@
       <c r="D39" s="1" t="s">
         <v>470</v>
       </c>
-      <c r="E39" s="2" t="s">
+      <c r="E39" s="1" t="s">
         <v>471</v>
       </c>
       <c r="F39" s="1" t="s">
@@ -4832,7 +4938,7 @@
         <v>467</v>
       </c>
     </row>
-    <row r="40" spans="1:15" ht="84" customHeight="1">
+    <row r="40" spans="1:15">
       <c r="A40" s="1" t="s">
         <v>479</v>
       </c>
@@ -4845,7 +4951,7 @@
       <c r="D40" s="1" t="s">
         <v>481</v>
       </c>
-      <c r="E40" s="2" t="s">
+      <c r="E40" s="1" t="s">
         <v>482</v>
       </c>
       <c r="F40" s="1" t="s">
@@ -4879,7 +4985,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="41" spans="1:15" ht="84" customHeight="1">
+    <row r="41" spans="1:15">
       <c r="A41" s="1" t="s">
         <v>488</v>
       </c>
@@ -4892,7 +4998,7 @@
       <c r="D41" s="1" t="s">
         <v>490</v>
       </c>
-      <c r="E41" s="2" t="s">
+      <c r="E41" s="1" t="s">
         <v>491</v>
       </c>
       <c r="F41" s="1" t="s">
@@ -4926,7 +5032,7 @@
         <v>496</v>
       </c>
     </row>
-    <row r="42" spans="1:15" ht="84" customHeight="1">
+    <row r="42" spans="1:15">
       <c r="A42" s="1" t="s">
         <v>497</v>
       </c>
@@ -4939,7 +5045,7 @@
       <c r="D42" s="1" t="s">
         <v>498</v>
       </c>
-      <c r="E42" s="2" t="s">
+      <c r="E42" s="1" t="s">
         <v>499</v>
       </c>
       <c r="F42" s="1" t="s">
@@ -4973,7 +5079,7 @@
         <v>505</v>
       </c>
     </row>
-    <row r="43" spans="1:15" ht="84" customHeight="1">
+    <row r="43" spans="1:15">
       <c r="A43" s="1" t="s">
         <v>506</v>
       </c>
@@ -4986,7 +5092,7 @@
       <c r="D43" s="1" t="s">
         <v>508</v>
       </c>
-      <c r="E43" s="2" t="s">
+      <c r="E43" s="1" t="s">
         <v>509</v>
       </c>
       <c r="F43" s="1" t="s">
@@ -5020,7 +5126,7 @@
         <v>517</v>
       </c>
     </row>
-    <row r="44" spans="1:15" ht="84" customHeight="1">
+    <row r="44" spans="1:15">
       <c r="A44" s="1" t="s">
         <v>518</v>
       </c>
@@ -5033,7 +5139,7 @@
       <c r="D44" s="1" t="s">
         <v>520</v>
       </c>
-      <c r="E44" s="2" t="s">
+      <c r="E44" s="1" t="s">
         <v>521</v>
       </c>
       <c r="F44" s="1" t="s">
@@ -5067,7 +5173,7 @@
         <v>528</v>
       </c>
     </row>
-    <row r="45" spans="1:15" ht="84" customHeight="1">
+    <row r="45" spans="1:15">
       <c r="A45" s="1" t="s">
         <v>529</v>
       </c>
@@ -5080,7 +5186,7 @@
       <c r="D45" s="1" t="s">
         <v>530</v>
       </c>
-      <c r="E45" s="2" t="s">
+      <c r="E45" s="1" t="s">
         <v>531</v>
       </c>
       <c r="F45" s="1" t="s">
@@ -5114,7 +5220,7 @@
         <v>538</v>
       </c>
     </row>
-    <row r="46" spans="1:15" ht="84" customHeight="1">
+    <row r="46" spans="1:15">
       <c r="A46" s="1" t="s">
         <v>539</v>
       </c>
@@ -5127,7 +5233,7 @@
       <c r="D46" s="1" t="s">
         <v>541</v>
       </c>
-      <c r="E46" s="2" t="s">
+      <c r="E46" s="1" t="s">
         <v>542</v>
       </c>
       <c r="F46" s="1" t="s">
@@ -5161,7 +5267,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="47" spans="1:15" ht="84" customHeight="1">
+    <row r="47" spans="1:15">
       <c r="A47" s="1" t="s">
         <v>549</v>
       </c>
@@ -5174,7 +5280,7 @@
       <c r="D47" s="1" t="s">
         <v>551</v>
       </c>
-      <c r="E47" s="2" t="s">
+      <c r="E47" s="1" t="s">
         <v>552</v>
       </c>
       <c r="F47" s="1" t="s">
@@ -5208,7 +5314,7 @@
         <v>560</v>
       </c>
     </row>
-    <row r="48" spans="1:15" ht="84" customHeight="1">
+    <row r="48" spans="1:15">
       <c r="A48" s="1" t="s">
         <v>561</v>
       </c>
@@ -5221,7 +5327,7 @@
       <c r="D48" s="1" t="s">
         <v>562</v>
       </c>
-      <c r="E48" s="2" t="s">
+      <c r="E48" s="1" t="s">
         <v>563</v>
       </c>
       <c r="F48" s="1" t="s">
@@ -5255,7 +5361,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="49" spans="1:15" ht="84" customHeight="1">
+    <row r="49" spans="1:15">
       <c r="A49" s="1" t="s">
         <v>569</v>
       </c>
@@ -5268,7 +5374,7 @@
       <c r="D49" s="1" t="s">
         <v>570</v>
       </c>
-      <c r="E49" s="2" t="s">
+      <c r="E49" s="1" t="s">
         <v>571</v>
       </c>
       <c r="F49" s="1" t="s">
@@ -5302,7 +5408,7 @@
         <v>576</v>
       </c>
     </row>
-    <row r="50" spans="1:15" ht="84" customHeight="1">
+    <row r="50" spans="1:15">
       <c r="A50" s="1" t="s">
         <v>577</v>
       </c>
@@ -5315,7 +5421,7 @@
       <c r="D50" s="1" t="s">
         <v>578</v>
       </c>
-      <c r="E50" s="2" t="s">
+      <c r="E50" s="1" t="s">
         <v>579</v>
       </c>
       <c r="F50" s="1" t="s">
@@ -5349,7 +5455,7 @@
         <v>585</v>
       </c>
     </row>
-    <row r="51" spans="1:15" ht="84" customHeight="1">
+    <row r="51" spans="1:15">
       <c r="A51" s="1" t="s">
         <v>586</v>
       </c>
@@ -5362,7 +5468,7 @@
       <c r="D51" s="1" t="s">
         <v>587</v>
       </c>
-      <c r="E51" s="2" t="s">
+      <c r="E51" s="1" t="s">
         <v>588</v>
       </c>
       <c r="F51" s="1" t="s">
@@ -5396,7 +5502,7 @@
         <v>593</v>
       </c>
     </row>
-    <row r="52" spans="1:15" ht="84" customHeight="1">
+    <row r="52" spans="1:15">
       <c r="A52" s="1" t="s">
         <v>594</v>
       </c>
@@ -5409,7 +5515,7 @@
       <c r="D52" s="1" t="s">
         <v>595</v>
       </c>
-      <c r="E52" s="2" t="s">
+      <c r="E52" s="1" t="s">
         <v>596</v>
       </c>
       <c r="F52" s="1" t="s">
@@ -5443,7 +5549,7 @@
         <v>601</v>
       </c>
     </row>
-    <row r="53" spans="1:15" ht="84" customHeight="1">
+    <row r="53" spans="1:15">
       <c r="A53" s="1" t="s">
         <v>602</v>
       </c>
@@ -5456,7 +5562,7 @@
       <c r="D53" s="1" t="s">
         <v>603</v>
       </c>
-      <c r="E53" s="2" t="s">
+      <c r="E53" s="1" t="s">
         <v>604</v>
       </c>
       <c r="F53" s="1" t="s">
@@ -5490,7 +5596,7 @@
         <v>609</v>
       </c>
     </row>
-    <row r="54" spans="1:15" ht="84" customHeight="1">
+    <row r="54" spans="1:15">
       <c r="A54" s="1" t="s">
         <v>610</v>
       </c>
@@ -5503,7 +5609,7 @@
       <c r="D54" s="1" t="s">
         <v>611</v>
       </c>
-      <c r="E54" s="2" t="s">
+      <c r="E54" s="1" t="s">
         <v>612</v>
       </c>
       <c r="F54" s="1" t="s">
@@ -5537,7 +5643,7 @@
         <v>617</v>
       </c>
     </row>
-    <row r="55" spans="1:15" ht="84" customHeight="1">
+    <row r="55" spans="1:15">
       <c r="A55" s="1" t="s">
         <v>618</v>
       </c>
@@ -5550,7 +5656,7 @@
       <c r="D55" s="1" t="s">
         <v>619</v>
       </c>
-      <c r="E55" s="2" t="s">
+      <c r="E55" s="1" t="s">
         <v>620</v>
       </c>
       <c r="F55" s="1" t="s">
@@ -5584,7 +5690,7 @@
         <v>625</v>
       </c>
     </row>
-    <row r="56" spans="1:15" ht="84" customHeight="1">
+    <row r="56" spans="1:15">
       <c r="A56" s="1" t="s">
         <v>626</v>
       </c>
@@ -5597,7 +5703,7 @@
       <c r="D56" s="1" t="s">
         <v>627</v>
       </c>
-      <c r="E56" s="2" t="s">
+      <c r="E56" s="1" t="s">
         <v>628</v>
       </c>
       <c r="F56" s="1" t="s">
@@ -5631,7 +5737,7 @@
         <v>633</v>
       </c>
     </row>
-    <row r="57" spans="1:15" ht="84" customHeight="1">
+    <row r="57" spans="1:15">
       <c r="A57" s="1" t="s">
         <v>634</v>
       </c>
@@ -5644,7 +5750,7 @@
       <c r="D57" s="1" t="s">
         <v>635</v>
       </c>
-      <c r="E57" s="2" t="s">
+      <c r="E57" s="1" t="s">
         <v>636</v>
       </c>
       <c r="F57" s="1" t="s">
@@ -5678,7 +5784,7 @@
         <v>641</v>
       </c>
     </row>
-    <row r="58" spans="1:15" ht="84" customHeight="1">
+    <row r="58" spans="1:15">
       <c r="A58" s="1" t="s">
         <v>642</v>
       </c>
@@ -5691,7 +5797,7 @@
       <c r="D58" s="1" t="s">
         <v>643</v>
       </c>
-      <c r="E58" s="2" t="s">
+      <c r="E58" s="1" t="s">
         <v>644</v>
       </c>
       <c r="F58" s="1" t="s">
@@ -5725,7 +5831,7 @@
         <v>648</v>
       </c>
     </row>
-    <row r="59" spans="1:15" ht="84" customHeight="1">
+    <row r="59" spans="1:15">
       <c r="A59" s="1" t="s">
         <v>649</v>
       </c>
@@ -5738,7 +5844,7 @@
       <c r="D59" s="1" t="s">
         <v>650</v>
       </c>
-      <c r="E59" s="2" t="s">
+      <c r="E59" s="1" t="s">
         <v>651</v>
       </c>
       <c r="F59" s="1" t="s">
@@ -5772,7 +5878,7 @@
         <v>656</v>
       </c>
     </row>
-    <row r="60" spans="1:15" ht="84" customHeight="1">
+    <row r="60" spans="1:15">
       <c r="A60" s="1" t="s">
         <v>657</v>
       </c>
@@ -5785,7 +5891,7 @@
       <c r="D60" s="1" t="s">
         <v>658</v>
       </c>
-      <c r="E60" s="2" t="s">
+      <c r="E60" s="1" t="s">
         <v>659</v>
       </c>
       <c r="F60" s="1" t="s">
@@ -5819,7 +5925,7 @@
         <v>664</v>
       </c>
     </row>
-    <row r="61" spans="1:15" ht="84" customHeight="1">
+    <row r="61" spans="1:15">
       <c r="A61" s="1" t="s">
         <v>665</v>
       </c>
@@ -5832,7 +5938,7 @@
       <c r="D61" s="1" t="s">
         <v>666</v>
       </c>
-      <c r="E61" s="2" t="s">
+      <c r="E61" s="1" t="s">
         <v>667</v>
       </c>
       <c r="F61" s="1" t="s">
@@ -5866,7 +5972,7 @@
         <v>671</v>
       </c>
     </row>
-    <row r="62" spans="1:15" ht="84" customHeight="1">
+    <row r="62" spans="1:15">
       <c r="A62" s="1" t="s">
         <v>672</v>
       </c>
@@ -5879,7 +5985,7 @@
       <c r="D62" s="1" t="s">
         <v>673</v>
       </c>
-      <c r="E62" s="2" t="s">
+      <c r="E62" s="1" t="s">
         <v>674</v>
       </c>
       <c r="F62" s="1" t="s">
@@ -5913,7 +6019,7 @@
         <v>679</v>
       </c>
     </row>
-    <row r="63" spans="1:15" ht="84" customHeight="1">
+    <row r="63" spans="1:15">
       <c r="A63" s="1" t="s">
         <v>680</v>
       </c>
@@ -5926,7 +6032,7 @@
       <c r="D63" s="1" t="s">
         <v>681</v>
       </c>
-      <c r="E63" s="2" t="s">
+      <c r="E63" s="1" t="s">
         <v>682</v>
       </c>
       <c r="F63" s="1" t="s">
@@ -5960,7 +6066,7 @@
         <v>687</v>
       </c>
     </row>
-    <row r="64" spans="1:15" ht="84" customHeight="1">
+    <row r="64" spans="1:15">
       <c r="A64" s="1" t="s">
         <v>688</v>
       </c>
@@ -5973,7 +6079,7 @@
       <c r="D64" s="1" t="s">
         <v>689</v>
       </c>
-      <c r="E64" s="2" t="s">
+      <c r="E64" s="1" t="s">
         <v>690</v>
       </c>
       <c r="F64" s="1" t="s">
@@ -6007,7 +6113,7 @@
         <v>695</v>
       </c>
     </row>
-    <row r="65" spans="1:15" ht="84" customHeight="1">
+    <row r="65" spans="1:15">
       <c r="A65" s="1" t="s">
         <v>696</v>
       </c>
@@ -6020,7 +6126,7 @@
       <c r="D65" s="1" t="s">
         <v>698</v>
       </c>
-      <c r="E65" s="2" t="s">
+      <c r="E65" s="1" t="s">
         <v>699</v>
       </c>
       <c r="F65" s="1" t="s">
@@ -6054,7 +6160,7 @@
         <v>704</v>
       </c>
     </row>
-    <row r="66" spans="1:15" ht="84" customHeight="1">
+    <row r="66" spans="1:15">
       <c r="A66" s="1" t="s">
         <v>705</v>
       </c>
@@ -6067,7 +6173,7 @@
       <c r="D66" s="1" t="s">
         <v>706</v>
       </c>
-      <c r="E66" s="2" t="s">
+      <c r="E66" s="1" t="s">
         <v>707</v>
       </c>
       <c r="F66" s="1" t="s">
@@ -6101,7 +6207,7 @@
         <v>712</v>
       </c>
     </row>
-    <row r="67" spans="1:15" ht="84" customHeight="1">
+    <row r="67" spans="1:15">
       <c r="A67" s="1" t="s">
         <v>713</v>
       </c>
@@ -6114,7 +6220,7 @@
       <c r="D67" s="1" t="s">
         <v>714</v>
       </c>
-      <c r="E67" s="2" t="s">
+      <c r="E67" s="1" t="s">
         <v>715</v>
       </c>
       <c r="F67" s="1" t="s">
@@ -6148,7 +6254,7 @@
         <v>719</v>
       </c>
     </row>
-    <row r="68" spans="1:15" ht="84" customHeight="1">
+    <row r="68" spans="1:15">
       <c r="A68" s="1" t="s">
         <v>720</v>
       </c>
@@ -6161,7 +6267,7 @@
       <c r="D68" s="1" t="s">
         <v>721</v>
       </c>
-      <c r="E68" s="2" t="s">
+      <c r="E68" s="1" t="s">
         <v>722</v>
       </c>
       <c r="F68" s="1" t="s">
@@ -6195,7 +6301,7 @@
         <v>727</v>
       </c>
     </row>
-    <row r="69" spans="1:15" ht="84" customHeight="1">
+    <row r="69" spans="1:15">
       <c r="A69" s="1" t="s">
         <v>728</v>
       </c>
@@ -6208,7 +6314,7 @@
       <c r="D69" s="1" t="s">
         <v>729</v>
       </c>
-      <c r="E69" s="2" t="s">
+      <c r="E69" s="1" t="s">
         <v>730</v>
       </c>
       <c r="F69" s="1" t="s">
@@ -6242,7 +6348,7 @@
         <v>735</v>
       </c>
     </row>
-    <row r="70" spans="1:15" ht="84" customHeight="1">
+    <row r="70" spans="1:15">
       <c r="A70" s="1" t="s">
         <v>736</v>
       </c>
@@ -6255,7 +6361,7 @@
       <c r="D70" s="1" t="s">
         <v>737</v>
       </c>
-      <c r="E70" s="2" t="s">
+      <c r="E70" s="1" t="s">
         <v>738</v>
       </c>
       <c r="F70" s="1" t="s">
@@ -6289,7 +6395,7 @@
         <v>743</v>
       </c>
     </row>
-    <row r="71" spans="1:15" ht="84" customHeight="1">
+    <row r="71" spans="1:15">
       <c r="A71" s="1" t="s">
         <v>744</v>
       </c>
@@ -6302,7 +6408,7 @@
       <c r="D71" s="1" t="s">
         <v>745</v>
       </c>
-      <c r="E71" s="2" t="s">
+      <c r="E71" s="1" t="s">
         <v>746</v>
       </c>
       <c r="F71" s="1" t="s">
@@ -6336,7 +6442,7 @@
         <v>750</v>
       </c>
     </row>
-    <row r="72" spans="1:15" ht="84" customHeight="1">
+    <row r="72" spans="1:15">
       <c r="A72" s="1" t="s">
         <v>751</v>
       </c>
@@ -6349,7 +6455,7 @@
       <c r="D72" s="1" t="s">
         <v>753</v>
       </c>
-      <c r="E72" s="2" t="s">
+      <c r="E72" s="1" t="s">
         <v>754</v>
       </c>
       <c r="F72" s="1" t="s">
@@ -6383,7 +6489,7 @@
         <v>763</v>
       </c>
     </row>
-    <row r="73" spans="1:15" ht="84" customHeight="1">
+    <row r="73" spans="1:15">
       <c r="A73" s="1" t="s">
         <v>764</v>
       </c>
@@ -6396,7 +6502,7 @@
       <c r="D73" s="1" t="s">
         <v>766</v>
       </c>
-      <c r="E73" s="2" t="s">
+      <c r="E73" s="1" t="s">
         <v>767</v>
       </c>
       <c r="F73" s="1" t="s">
@@ -6430,7 +6536,7 @@
         <v>776</v>
       </c>
     </row>
-    <row r="74" spans="1:15" ht="84" customHeight="1">
+    <row r="74" spans="1:15">
       <c r="A74" s="1" t="s">
         <v>777</v>
       </c>
@@ -6443,7 +6549,7 @@
       <c r="D74" s="1" t="s">
         <v>779</v>
       </c>
-      <c r="E74" s="2" t="s">
+      <c r="E74" s="1" t="s">
         <v>780</v>
       </c>
       <c r="F74" s="1" t="s">
@@ -6477,7 +6583,7 @@
         <v>784</v>
       </c>
     </row>
-    <row r="75" spans="1:15" ht="84" customHeight="1">
+    <row r="75" spans="1:15">
       <c r="A75" s="1" t="s">
         <v>785</v>
       </c>
@@ -6490,7 +6596,7 @@
       <c r="D75" s="1" t="s">
         <v>787</v>
       </c>
-      <c r="E75" s="2" t="s">
+      <c r="E75" s="1" t="s">
         <v>788</v>
       </c>
       <c r="F75" s="1" t="s">
@@ -6524,7 +6630,7 @@
         <v>795</v>
       </c>
     </row>
-    <row r="76" spans="1:15" ht="84" customHeight="1">
+    <row r="76" spans="1:15">
       <c r="A76" s="1" t="s">
         <v>796</v>
       </c>
@@ -6537,7 +6643,7 @@
       <c r="D76" s="1" t="s">
         <v>798</v>
       </c>
-      <c r="E76" s="2" t="s">
+      <c r="E76" s="1" t="s">
         <v>799</v>
       </c>
       <c r="F76" s="1" t="s">
@@ -6571,7 +6677,7 @@
         <v>808</v>
       </c>
     </row>
-    <row r="77" spans="1:15" ht="84" customHeight="1">
+    <row r="77" spans="1:15">
       <c r="A77" s="1" t="s">
         <v>809</v>
       </c>
@@ -6584,7 +6690,7 @@
       <c r="D77" s="1" t="s">
         <v>812</v>
       </c>
-      <c r="E77" s="2" t="s">
+      <c r="E77" s="1" t="s">
         <v>813</v>
       </c>
       <c r="F77" s="1" t="s">
@@ -6618,7 +6724,7 @@
         <v>821</v>
       </c>
     </row>
-    <row r="78" spans="1:15" ht="84" customHeight="1">
+    <row r="78" spans="1:15">
       <c r="A78" s="1" t="s">
         <v>822</v>
       </c>
@@ -6631,7 +6737,7 @@
       <c r="D78" s="1" t="s">
         <v>825</v>
       </c>
-      <c r="E78" s="2" t="s">
+      <c r="E78" s="1" t="s">
         <v>826</v>
       </c>
       <c r="F78" s="1" t="s">
@@ -6665,7 +6771,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="79" spans="1:15" ht="84" customHeight="1">
+    <row r="79" spans="1:15">
       <c r="A79" s="1" t="s">
         <v>835</v>
       </c>
@@ -6678,7 +6784,7 @@
       <c r="D79" s="1" t="s">
         <v>837</v>
       </c>
-      <c r="E79" s="2" t="s">
+      <c r="E79" s="1" t="s">
         <v>838</v>
       </c>
       <c r="F79" s="1" t="s">
@@ -6712,12 +6818,12 @@
         <v>847</v>
       </c>
     </row>
-    <row r="80" spans="1:15" ht="84" customHeight="1">
+    <row r="80" spans="1:15">
       <c r="A80" s="1" t="s">
         <v>848</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>441</v>
+        <v>101</v>
       </c>
       <c r="C80" s="1" t="s">
         <v>849</v>
@@ -6725,7 +6831,7 @@
       <c r="D80" s="1" t="s">
         <v>850</v>
       </c>
-      <c r="E80" s="2" t="s">
+      <c r="E80" s="1" t="s">
         <v>851</v>
       </c>
       <c r="F80" s="1" t="s">
@@ -6744,7 +6850,7 @@
         <v>856</v>
       </c>
       <c r="K80" s="1" t="s">
-        <v>450</v>
+        <v>110</v>
       </c>
       <c r="L80" s="1" t="s">
         <v>857</v>
@@ -6757,6 +6863,194 @@
       </c>
       <c r="O80" s="1" t="s">
         <v>860</v>
+      </c>
+    </row>
+    <row r="81" spans="1:15">
+      <c r="A81" s="1" t="s">
+        <v>861</v>
+      </c>
+      <c r="B81" s="1" t="s">
+        <v>862</v>
+      </c>
+      <c r="C81" s="1" t="s">
+        <v>863</v>
+      </c>
+      <c r="D81" s="1" t="s">
+        <v>864</v>
+      </c>
+      <c r="E81" s="1" t="s">
+        <v>865</v>
+      </c>
+      <c r="F81" s="1" t="s">
+        <v>866</v>
+      </c>
+      <c r="G81" s="1" t="s">
+        <v>867</v>
+      </c>
+      <c r="H81" s="1" t="s">
+        <v>868</v>
+      </c>
+      <c r="I81" s="1" t="s">
+        <v>869</v>
+      </c>
+      <c r="J81" s="1" t="s">
+        <v>870</v>
+      </c>
+      <c r="K81" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="L81" s="1" t="s">
+        <v>871</v>
+      </c>
+      <c r="M81" s="1" t="s">
+        <v>872</v>
+      </c>
+      <c r="N81" s="1" t="s">
+        <v>873</v>
+      </c>
+      <c r="O81" s="1" t="s">
+        <v>874</v>
+      </c>
+    </row>
+    <row r="82" spans="1:15">
+      <c r="A82" s="1" t="s">
+        <v>875</v>
+      </c>
+      <c r="B82" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="C82" s="1" t="s">
+        <v>876</v>
+      </c>
+      <c r="D82" s="1" t="s">
+        <v>877</v>
+      </c>
+      <c r="E82" s="1" t="s">
+        <v>878</v>
+      </c>
+      <c r="F82" s="1" t="s">
+        <v>879</v>
+      </c>
+      <c r="G82" s="1" t="s">
+        <v>880</v>
+      </c>
+      <c r="H82" s="1" t="s">
+        <v>881</v>
+      </c>
+      <c r="I82" s="1" t="s">
+        <v>882</v>
+      </c>
+      <c r="J82" s="1" t="s">
+        <v>883</v>
+      </c>
+      <c r="K82" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="L82" s="1" t="s">
+        <v>884</v>
+      </c>
+      <c r="M82" s="1" t="s">
+        <v>885</v>
+      </c>
+      <c r="N82" s="1" t="s">
+        <v>886</v>
+      </c>
+      <c r="O82" s="1" t="s">
+        <v>887</v>
+      </c>
+    </row>
+    <row r="83" spans="1:15">
+      <c r="A83" s="1" t="s">
+        <v>888</v>
+      </c>
+      <c r="B83" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="C83" s="1" t="s">
+        <v>876</v>
+      </c>
+      <c r="D83" s="1" t="s">
+        <v>889</v>
+      </c>
+      <c r="E83" s="1" t="s">
+        <v>890</v>
+      </c>
+      <c r="F83" s="1" t="s">
+        <v>879</v>
+      </c>
+      <c r="G83" s="1" t="s">
+        <v>880</v>
+      </c>
+      <c r="H83" s="1" t="s">
+        <v>891</v>
+      </c>
+      <c r="I83" s="1" t="s">
+        <v>892</v>
+      </c>
+      <c r="J83" s="1" t="s">
+        <v>893</v>
+      </c>
+      <c r="K83" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="L83" s="1" t="s">
+        <v>894</v>
+      </c>
+      <c r="M83" s="1" t="s">
+        <v>895</v>
+      </c>
+      <c r="N83" s="1" t="s">
+        <v>896</v>
+      </c>
+      <c r="O83" s="1" t="s">
+        <v>897</v>
+      </c>
+    </row>
+    <row r="84" spans="1:15">
+      <c r="A84" s="1" t="s">
+        <v>898</v>
+      </c>
+      <c r="B84" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="C84" s="1" t="s">
+        <v>876</v>
+      </c>
+      <c r="D84" s="1" t="s">
+        <v>899</v>
+      </c>
+      <c r="E84" s="1" t="s">
+        <v>900</v>
+      </c>
+      <c r="F84" s="1" t="s">
+        <v>879</v>
+      </c>
+      <c r="G84" s="1" t="s">
+        <v>880</v>
+      </c>
+      <c r="H84" s="1" t="s">
+        <v>891</v>
+      </c>
+      <c r="I84" s="1" t="s">
+        <v>901</v>
+      </c>
+      <c r="J84" s="1" t="s">
+        <v>902</v>
+      </c>
+      <c r="K84" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="L84" s="1" t="s">
+        <v>894</v>
+      </c>
+      <c r="M84" s="1" t="s">
+        <v>895</v>
+      </c>
+      <c r="N84" s="1" t="s">
+        <v>903</v>
+      </c>
+      <c r="O84" s="1" t="s">
+        <v>904</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Overboard a cappella source research
</commit_message>
<xml_diff>
--- a/dossier/source_dossier.xlsx
+++ b/dossier/source_dossier.xlsx
@@ -10,14 +10,14 @@
     <sheet name="source_dossier" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">source_dossier!$A$1:$O$84</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">source_dossier!$A$1:$O$85</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1260" uniqueCount="907">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1275" uniqueCount="921">
   <si>
     <t>id</t>
   </si>
@@ -2738,6 +2738,48 @@
   </si>
   <si>
     <t>{{cite web |title=CWAP 5/4/26 - Spring Town Meeting Debrief |url=https://www.youtube.com/watch?v=ClsjG0XI0_E |website=YouTube |publisher=Coffee with a Purpose, Natick MA |date=May 4, 2026 |access-date=June 9, 2026}}</t>
+  </si>
+  <si>
+    <t>HSJA1</t>
+  </si>
+  <si>
+    <t>2003-2011; 2026 page access</t>
+  </si>
+  <si>
+    <t>Harmony Sweepstakes / Wikipedia</t>
+  </si>
+  <si>
+    <t>Jeff Alderson a cappella activity, Overboard, and Integration by Parts source leads</t>
+  </si>
+  <si>
+    <t>https://www.harmony-sweepstakes.com/person/Jeff+Alderson</t>
+  </si>
+  <si>
+    <t>Competition/event records and Wikipedia group article</t>
+  </si>
+  <si>
+    <t>Mixed; mostly event records / source leads</t>
+  </si>
+  <si>
+    <t>Low for Alderson notability; direct for narrow a cappella participation facts</t>
+  </si>
+  <si>
+    <t>Harmony Sweepstakes person page lists Alderson with Overboard in 2008 as Boston Harmony Sweepstakes 3rd Place Winners and with Integration By Parts / Integration by Parts in 2003, 2004, and 2005. Overboard 2008 detail and Boston Regional pages list Alderson in the Overboard member roster. Wikipedia and Harmony pages verify Overboard's 2011 Boston Regional win, but the 2011 Overboard rosters do not include Alderson.</t>
+  </si>
+  <si>
+    <t>Alderson was listed as a member of Overboard in the 2008 Boston Regional Harmony Sweepstakes, where Overboard placed third; Alderson was also listed with Integration by Parts / Integration By Parts in 2003-2005 Boston Regional events; Overboard later won the 2011 Boston Regional, but the reviewed 2011 rosters do not list Alderson.</t>
+  </si>
+  <si>
+    <t>Dossier only unless a narrow music-background sentence is desired; do not cite Wikipedia in the article draft and do not claim Alderson was in Overboard's 2011 winning roster without another source.</t>
+  </si>
+  <si>
+    <t>Verified; HTML and raw wikitext captured where useful</t>
+  </si>
+  <si>
+    <t>Reviewed in sources/acappella_overboard_sources.md; local files data/harmony_sweepstakes_person_jeff_alderson.html, data/harmony_sweepstakes_details_48653_overboard_2008.html, data/harmony_sweepstakes_boston_2008.html, data/harmony_sweepstakes_boston_2011.html, data/harmony_sweepstakes_2011_national_finals.html, data/overboard_wikipedia.html, data/overboard_wikipedia_raw.wikitext, and Integration by Parts detail pages.</t>
+  </si>
+  <si>
+    <t>{{cite web |title=Jeff Alderson A Cappella Singer |url=https://www.harmony-sweepstakes.com/person/Jeff+Alderson |website=Harmony Sweepstakes A Cappella Festival |access-date=June 21, 2026}}</t>
   </si>
 </sst>
 </file>
@@ -2761,41 +2803,20 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFD9EAF7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -2804,7 +2825,7 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -3104,21 +3125,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O84"/>
+  <dimension ref="A1:O85"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="2" width="10.7109375" customWidth="1"/>
-    <col min="3" max="3" width="28.7109375" customWidth="1"/>
-    <col min="4" max="4" width="42.7109375" customWidth="1"/>
-    <col min="5" max="5" width="48.7109375" customWidth="1"/>
-    <col min="6" max="6" width="28.7109375" customWidth="1"/>
-    <col min="7" max="7" width="18.7109375" customWidth="1"/>
-    <col min="8" max="8" width="32.7109375" customWidth="1"/>
-    <col min="9" max="10" width="58.7109375" customWidth="1"/>
-    <col min="11" max="11" width="20.7109375" customWidth="1"/>
-    <col min="12" max="12" width="34.7109375" customWidth="1"/>
-    <col min="13" max="13" width="28.7109375" customWidth="1"/>
-    <col min="14" max="15" width="58.7109375" customWidth="1"/>
+    <col min="1" max="1" width="15.7109375" customWidth="1"/>
+    <col min="2" max="2" width="33.7109375" customWidth="1"/>
+    <col min="3" max="15" width="55.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15">
@@ -7069,8 +7081,55 @@
         <v>906</v>
       </c>
     </row>
+    <row r="85" spans="1:15">
+      <c r="A85" s="2" t="s">
+        <v>907</v>
+      </c>
+      <c r="B85" s="2" t="s">
+        <v>908</v>
+      </c>
+      <c r="C85" s="2" t="s">
+        <v>909</v>
+      </c>
+      <c r="D85" s="2" t="s">
+        <v>910</v>
+      </c>
+      <c r="E85" s="2" t="s">
+        <v>911</v>
+      </c>
+      <c r="F85" s="2" t="s">
+        <v>912</v>
+      </c>
+      <c r="G85" s="2" t="s">
+        <v>913</v>
+      </c>
+      <c r="H85" s="2" t="s">
+        <v>914</v>
+      </c>
+      <c r="I85" s="2" t="s">
+        <v>915</v>
+      </c>
+      <c r="J85" s="2" t="s">
+        <v>916</v>
+      </c>
+      <c r="K85" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="L85" s="2" t="s">
+        <v>917</v>
+      </c>
+      <c r="M85" s="2" t="s">
+        <v>918</v>
+      </c>
+      <c r="N85" s="2" t="s">
+        <v>919</v>
+      </c>
+      <c r="O85" s="2" t="s">
+        <v>920</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O84"/>
+  <autoFilter ref="A1:O85"/>
   <hyperlinks>
     <hyperlink ref="E2" r:id="rId1"/>
     <hyperlink ref="E3" r:id="rId2"/>
@@ -7155,6 +7214,7 @@
     <hyperlink ref="E82" r:id="rId81"/>
     <hyperlink ref="E83" r:id="rId82"/>
     <hyperlink ref="E84" r:id="rId83"/>
+    <hyperlink ref="E85" r:id="rId84"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>